<commit_message>
Add real-time stock prices and update timestamp to financial tracker
Integrate `yfinance` to fetch live stock prices, update `write_stock_row`, `build_tracker_sheet`, and `build_dashboard` to display prices and a "last fetched" timestamp.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 361222b0-77cf-4eeb-813e-f4be6db48368
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -993,7 +993,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 10:04 PM</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1480,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:04 PM</t>
         </is>
       </c>
     </row>
@@ -1603,7 +1603,7 @@
         </is>
       </c>
       <c r="E5" s="28" t="n">
-        <v>0</v>
+        <v>84.65000000000001</v>
       </c>
       <c r="F5" s="28" t="n">
         <v>0</v>
@@ -1746,7 +1746,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:04 PM</t>
         </is>
       </c>
     </row>
@@ -1869,7 +1869,7 @@
         </is>
       </c>
       <c r="E5" s="28" t="n">
-        <v>0</v>
+        <v>57.78</v>
       </c>
       <c r="F5" s="28" t="n">
         <v>0</v>
@@ -1938,7 +1938,7 @@
         </is>
       </c>
       <c r="E6" s="28" t="n">
-        <v>0</v>
+        <v>45.76</v>
       </c>
       <c r="F6" s="28" t="n">
         <v>0</v>
@@ -2339,7 +2339,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:04 PM</t>
         </is>
       </c>
     </row>
@@ -2462,7 +2462,7 @@
         </is>
       </c>
       <c r="E5" s="28" t="n">
-        <v>0</v>
+        <v>52.57</v>
       </c>
       <c r="F5" s="28" t="n">
         <v>0</v>
@@ -2531,7 +2531,7 @@
         </is>
       </c>
       <c r="E6" s="28" t="n">
-        <v>0</v>
+        <v>20.09</v>
       </c>
       <c r="F6" s="28" t="n">
         <v>0</v>
@@ -2600,7 +2600,7 @@
         </is>
       </c>
       <c r="E7" s="28" t="n">
-        <v>0</v>
+        <v>23.83</v>
       </c>
       <c r="F7" s="28" t="n">
         <v>0</v>
@@ -2743,7 +2743,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:04 PM</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
         </is>
       </c>
       <c r="E5" s="28" t="n">
-        <v>0</v>
+        <v>207.83</v>
       </c>
       <c r="F5" s="28" t="n">
         <v>0</v>
@@ -2935,7 +2935,7 @@
         </is>
       </c>
       <c r="E6" s="28" t="n">
-        <v>0</v>
+        <v>425.44</v>
       </c>
       <c r="F6" s="28" t="n">
         <v>0</v>
@@ -3004,7 +3004,7 @@
         </is>
       </c>
       <c r="E7" s="28" t="n">
-        <v>0</v>
+        <v>297.17</v>
       </c>
       <c r="F7" s="28" t="n">
         <v>0</v>
@@ -3073,7 +3073,7 @@
         </is>
       </c>
       <c r="E8" s="28" t="n">
-        <v>0</v>
+        <v>421.39</v>
       </c>
       <c r="F8" s="28" t="n">
         <v>0</v>
@@ -3142,7 +3142,7 @@
         </is>
       </c>
       <c r="E9" s="28" t="n">
-        <v>0</v>
+        <v>113.01</v>
       </c>
       <c r="F9" s="28" t="n">
         <v>0</v>
@@ -3211,7 +3211,7 @@
         </is>
       </c>
       <c r="E10" s="28" t="n">
-        <v>0</v>
+        <v>237.3</v>
       </c>
       <c r="F10" s="28" t="n">
         <v>0</v>
@@ -3354,7 +3354,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:04 PM</t>
         </is>
       </c>
     </row>
@@ -3477,7 +3477,7 @@
         </is>
       </c>
       <c r="E5" s="28" t="n">
-        <v>0</v>
+        <v>16.68</v>
       </c>
       <c r="F5" s="28" t="n">
         <v>0</v>
@@ -3546,7 +3546,7 @@
         </is>
       </c>
       <c r="E6" s="28" t="n">
-        <v>0</v>
+        <v>96.73</v>
       </c>
       <c r="F6" s="28" t="n">
         <v>0</v>
@@ -3615,7 +3615,7 @@
         </is>
       </c>
       <c r="E7" s="28" t="n">
-        <v>0</v>
+        <v>198.29</v>
       </c>
       <c r="F7" s="28" t="n">
         <v>0</v>
@@ -3684,7 +3684,7 @@
         </is>
       </c>
       <c r="E8" s="28" t="n">
-        <v>0</v>
+        <v>51.37</v>
       </c>
       <c r="F8" s="28" t="n">
         <v>0</v>
@@ -3753,7 +3753,7 @@
         </is>
       </c>
       <c r="E9" s="28" t="n">
-        <v>0</v>
+        <v>12.33</v>
       </c>
       <c r="F9" s="28" t="n">
         <v>0</v>
@@ -3822,7 +3822,7 @@
         </is>
       </c>
       <c r="E10" s="28" t="n">
-        <v>0</v>
+        <v>309.81</v>
       </c>
       <c r="F10" s="28" t="n">
         <v>0</v>
@@ -3891,7 +3891,7 @@
         </is>
       </c>
       <c r="E11" s="28" t="n">
-        <v>0</v>
+        <v>16.57</v>
       </c>
       <c r="F11" s="28" t="n">
         <v>0</v>
@@ -4034,7 +4034,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:04 PM</t>
         </is>
       </c>
     </row>
@@ -4157,7 +4157,7 @@
         </is>
       </c>
       <c r="E5" s="28" t="n">
-        <v>0</v>
+        <v>944.28</v>
       </c>
       <c r="F5" s="28" t="n">
         <v>0</v>
@@ -4300,7 +4300,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:04 PM</t>
         </is>
       </c>
     </row>
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="E5" s="28" t="n">
-        <v>0</v>
+        <v>926.9299999999999</v>
       </c>
       <c r="F5" s="28" t="n">
         <v>0</v>
@@ -4492,7 +4492,7 @@
         </is>
       </c>
       <c r="E6" s="28" t="n">
-        <v>0</v>
+        <v>2011.49</v>
       </c>
       <c r="F6" s="28" t="n">
         <v>0</v>
@@ -4561,7 +4561,7 @@
         </is>
       </c>
       <c r="E7" s="28" t="n">
-        <v>0</v>
+        <v>320.3</v>
       </c>
       <c r="F7" s="28" t="n">
         <v>0</v>
@@ -4630,7 +4630,7 @@
         </is>
       </c>
       <c r="E8" s="28" t="n">
-        <v>0</v>
+        <v>358.92</v>
       </c>
       <c r="F8" s="28" t="n">
         <v>0</v>
@@ -4773,7 +4773,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:04 PM</t>
         </is>
       </c>
     </row>
@@ -4896,7 +4896,7 @@
         </is>
       </c>
       <c r="E5" s="28" t="n">
-        <v>0</v>
+        <v>1118.96</v>
       </c>
       <c r="F5" s="28" t="n">
         <v>0</v>
@@ -4965,7 +4965,7 @@
         </is>
       </c>
       <c r="E6" s="28" t="n">
-        <v>0</v>
+        <v>785.24</v>
       </c>
       <c r="F6" s="28" t="n">
         <v>0</v>
@@ -5034,7 +5034,7 @@
         </is>
       </c>
       <c r="E7" s="28" t="n">
-        <v>0</v>
+        <v>285.47</v>
       </c>
       <c r="F7" s="28" t="n">
         <v>0</v>
@@ -5103,7 +5103,7 @@
         </is>
       </c>
       <c r="E8" s="28" t="n">
-        <v>0</v>
+        <v>79.62</v>
       </c>
       <c r="F8" s="28" t="n">
         <v>0</v>
@@ -5246,7 +5246,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:04 PM</t>
         </is>
       </c>
     </row>
@@ -5369,7 +5369,7 @@
         </is>
       </c>
       <c r="E5" s="28" t="n">
-        <v>0</v>
+        <v>195.09</v>
       </c>
       <c r="F5" s="28" t="n">
         <v>0</v>
@@ -5438,7 +5438,7 @@
         </is>
       </c>
       <c r="E6" s="28" t="n">
-        <v>0</v>
+        <v>133.79</v>
       </c>
       <c r="F6" s="28" t="n">
         <v>0</v>
@@ -5581,7 +5581,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:04 PM</t>
         </is>
       </c>
     </row>
@@ -5704,7 +5704,7 @@
         </is>
       </c>
       <c r="E5" s="28" t="n">
-        <v>0</v>
+        <v>9.34</v>
       </c>
       <c r="F5" s="28" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update financial tracker to show correct daily percentage change
Modify the price fetching logic to use `fast_info` and calculate today's percentage change based on `last_price` and `previous_close` for greater accuracy.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: ef4fd85f-8449-426c-938b-9ff4b49cc1c4
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1006,7 +1006,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 10:09 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
         </is>
       </c>
     </row>
@@ -1494,7 +1494,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:09 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
         </is>
       </c>
     </row>
@@ -1626,7 +1626,7 @@
         <v>84.65000000000001</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>0.07478414461518879</v>
+        <v>0.0787562320106908</v>
       </c>
       <c r="G5" s="28" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:09 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1902,7 @@
         <v>57.78</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>0.01137751967493678</v>
+        <v>0.004665116477114699</v>
       </c>
       <c r="G5" s="28" t="n">
         <v>0</v>
@@ -1974,7 +1974,7 @@
         <v>45.76</v>
       </c>
       <c r="F6" s="29" t="n">
-        <v>0.01983506598695283</v>
+        <v>0.01238934339675222</v>
       </c>
       <c r="G6" s="28" t="n">
         <v>0</v>
@@ -2376,7 +2376,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:09 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
         </is>
       </c>
     </row>
@@ -2508,7 +2508,7 @@
         <v>52.57</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>0.09520832697550456</v>
+        <v>0.09429641329775644</v>
       </c>
       <c r="G5" s="28" t="n">
         <v>0</v>
@@ -2580,7 +2580,7 @@
         <v>20.09</v>
       </c>
       <c r="F6" s="29" t="n">
-        <v>0.09961683903794465</v>
+        <v>0.1038522273522322</v>
       </c>
       <c r="G6" s="28" t="n">
         <v>0</v>
@@ -2652,7 +2652,7 @@
         <v>23.83</v>
       </c>
       <c r="F7" s="29" t="n">
-        <v>0.1063137841618168</v>
+        <v>0.1119925302709312</v>
       </c>
       <c r="G7" s="28" t="n">
         <v>0</v>
@@ -2796,7 +2796,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:09 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
         </is>
       </c>
     </row>
@@ -2928,7 +2928,7 @@
         <v>207.83</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>0.05765904239722487</v>
+        <v>0.05272809613927784</v>
       </c>
       <c r="G5" s="28" t="n">
         <v>0</v>
@@ -3000,7 +3000,7 @@
         <v>425.44</v>
       </c>
       <c r="F6" s="41" t="n">
-        <v>-0.004492659528188629</v>
+        <v>-0.01518517953378183</v>
       </c>
       <c r="G6" s="28" t="n">
         <v>0</v>
@@ -3072,7 +3072,7 @@
         <v>297.17</v>
       </c>
       <c r="F7" s="29" t="n">
-        <v>0.07748378020526668</v>
+        <v>0.06196624174582565</v>
       </c>
       <c r="G7" s="28" t="n">
         <v>0</v>
@@ -3144,7 +3144,7 @@
         <v>421.39</v>
       </c>
       <c r="F8" s="29" t="n">
-        <v>0.1861453669565576</v>
+        <v>0.017850276928593</v>
       </c>
       <c r="G8" s="28" t="n">
         <v>0</v>
@@ -3215,8 +3215,8 @@
       <c r="E9" s="28" t="n">
         <v>113.01</v>
       </c>
-      <c r="F9" s="29" t="n">
-        <v>0.04493759169470402</v>
+      <c r="F9" s="41" t="n">
+        <v>-0.002999540042077861</v>
       </c>
       <c r="G9" s="28" t="n">
         <v>0</v>
@@ -3288,7 +3288,7 @@
         <v>237.3</v>
       </c>
       <c r="F10" s="29" t="n">
-        <v>0.1362766099067566</v>
+        <v>0.04893251581027195</v>
       </c>
       <c r="G10" s="28" t="n">
         <v>0</v>
@@ -3432,7 +3432,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:09 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
         </is>
       </c>
     </row>
@@ -3563,8 +3563,8 @@
       <c r="E5" s="28" t="n">
         <v>16.68</v>
       </c>
-      <c r="F5" s="41" t="n">
-        <v>-0.04957259086641886</v>
+      <c r="F5" s="29" t="n">
+        <v>0.0127504739025976</v>
       </c>
       <c r="G5" s="28" t="n">
         <v>0</v>
@@ -3636,7 +3636,7 @@
         <v>96.73</v>
       </c>
       <c r="F6" s="29" t="n">
-        <v>0.06075228388207411</v>
+        <v>0.06176529155937345</v>
       </c>
       <c r="G6" s="28" t="n">
         <v>0</v>
@@ -3707,8 +3707,8 @@
       <c r="E7" s="28" t="n">
         <v>198.29</v>
       </c>
-      <c r="F7" s="29" t="n">
-        <v>0.02438387034830429</v>
+      <c r="F7" s="41" t="n">
+        <v>-0.001057968331824622</v>
       </c>
       <c r="G7" s="28" t="n">
         <v>0</v>
@@ -3780,7 +3780,7 @@
         <v>51.37</v>
       </c>
       <c r="F8" s="29" t="n">
-        <v>0.0340176855138408</v>
+        <v>0.027541779403253</v>
       </c>
       <c r="G8" s="28" t="n">
         <v>0</v>
@@ -3851,8 +3851,8 @@
       <c r="E9" s="28" t="n">
         <v>12.33</v>
       </c>
-      <c r="F9" s="29" t="n">
-        <v>0.01231523930804275</v>
+      <c r="F9" s="41" t="n">
+        <v>-0.002830576327856492</v>
       </c>
       <c r="G9" s="28" t="n">
         <v>0</v>
@@ -3924,7 +3924,7 @@
         <v>309.81</v>
       </c>
       <c r="F10" s="29" t="n">
-        <v>0.02055535818369094</v>
+        <v>0.0275621809571932</v>
       </c>
       <c r="G10" s="28" t="n">
         <v>0</v>
@@ -3996,7 +3996,7 @@
         <v>16.57</v>
       </c>
       <c r="F11" s="29" t="n">
-        <v>0.08727033751185366</v>
+        <v>0.07110534549607098</v>
       </c>
       <c r="G11" s="28" t="n">
         <v>0</v>
@@ -4140,7 +4140,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:09 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
         <v>944.28</v>
       </c>
       <c r="F5" s="41" t="n">
-        <v>-0.05055498751723778</v>
+        <v>-0.01642619728464659</v>
       </c>
       <c r="G5" s="28" t="n">
         <v>0</v>
@@ -4416,7 +4416,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:09 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
         </is>
       </c>
     </row>
@@ -4548,7 +4548,7 @@
         <v>926.9299999999999</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>0.02469623272099359</v>
+        <v>0.01762031516311836</v>
       </c>
       <c r="G5" s="28" t="n">
         <v>0</v>
@@ -4620,7 +4620,7 @@
         <v>2011.49</v>
       </c>
       <c r="F6" s="29" t="n">
-        <v>0.0224934427012782</v>
+        <v>0.01284503883945205</v>
       </c>
       <c r="G6" s="28" t="n">
         <v>0</v>
@@ -4692,7 +4692,7 @@
         <v>320.3</v>
       </c>
       <c r="F7" s="29" t="n">
-        <v>0.08690483266955953</v>
+        <v>0.06766662597656251</v>
       </c>
       <c r="G7" s="28" t="n">
         <v>0</v>
@@ -4764,7 +4764,7 @@
         <v>358.92</v>
       </c>
       <c r="F8" s="29" t="n">
-        <v>0.05248966333567288</v>
+        <v>0.02939746301010801</v>
       </c>
       <c r="G8" s="28" t="n">
         <v>0</v>
@@ -4908,7 +4908,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:09 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
         </is>
       </c>
     </row>
@@ -5040,7 +5040,7 @@
         <v>1118.96</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>0.02168533965822407</v>
+        <v>0.0171068781586888</v>
       </c>
       <c r="G5" s="28" t="n">
         <v>0</v>
@@ -5112,7 +5112,7 @@
         <v>785.24</v>
       </c>
       <c r="F6" s="29" t="n">
-        <v>0.01766437078519969</v>
+        <v>0.01881307604947841</v>
       </c>
       <c r="G6" s="28" t="n">
         <v>0</v>
@@ -5184,7 +5184,7 @@
         <v>285.47</v>
       </c>
       <c r="F7" s="41" t="n">
-        <v>-0.03312446665299534</v>
+        <v>-0.04067043441964675</v>
       </c>
       <c r="G7" s="28" t="n">
         <v>0</v>
@@ -5256,7 +5256,7 @@
         <v>79.62</v>
       </c>
       <c r="F8" s="29" t="n">
-        <v>0.1643756353412581</v>
+        <v>0.1715715530691883</v>
       </c>
       <c r="G8" s="28" t="n">
         <v>0</v>
@@ -5400,7 +5400,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:09 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
         <v>195.09</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>0.1089699770831929</v>
+        <v>0.1084973796863014</v>
       </c>
       <c r="G5" s="28" t="n">
         <v>0</v>
@@ -5604,7 +5604,7 @@
         <v>133.79</v>
       </c>
       <c r="F6" s="41" t="n">
-        <v>-0.01559863379333868</v>
+        <v>-0.01101424241474858</v>
       </c>
       <c r="G6" s="28" t="n">
         <v>0</v>
@@ -5748,7 +5748,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:09 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
         <v>9.34</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>0.001071835901780335</v>
+        <v>0.006595696920710679</v>
       </c>
       <c r="G5" s="28" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Correct daily percentage change calculation in financial tracker
Update the financial tracker script to store daily percentage changes as whole numbers and apply a literal percent sign in the cell format to prevent Excel from incorrectly multiplying the value by 100.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 77ea05e8-61b8-4da8-a339-b9da80179cae
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -29,7 +29,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="+0.00%;-0.00%;0.00%"/>
+    <numFmt numFmtId="165" formatCode="+0.00&quot;%&quot;;-0.00&quot;%&quot;;0.00&quot;%&quot;"/>
   </numFmts>
   <fonts count="23">
     <font>
@@ -1006,7 +1006,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
         </is>
       </c>
     </row>
@@ -1494,7 +1494,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
         </is>
       </c>
     </row>
@@ -1626,7 +1626,7 @@
         <v>84.65000000000001</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>0.0787562320106908</v>
+        <v>7.875623201069081</v>
       </c>
       <c r="G5" s="28" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1902,7 @@
         <v>57.78</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>0.004665116477114699</v>
+        <v>0.4665116477114699</v>
       </c>
       <c r="G5" s="28" t="n">
         <v>0</v>
@@ -1974,7 +1974,7 @@
         <v>45.76</v>
       </c>
       <c r="F6" s="29" t="n">
-        <v>0.01238934339675222</v>
+        <v>1.238934339675222</v>
       </c>
       <c r="G6" s="28" t="n">
         <v>0</v>
@@ -2376,7 +2376,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
         </is>
       </c>
     </row>
@@ -2508,7 +2508,7 @@
         <v>52.57</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>0.09429641329775644</v>
+        <v>9.429641329775643</v>
       </c>
       <c r="G5" s="28" t="n">
         <v>0</v>
@@ -2580,7 +2580,7 @@
         <v>20.09</v>
       </c>
       <c r="F6" s="29" t="n">
-        <v>0.1038522273522322</v>
+        <v>10.38522273522322</v>
       </c>
       <c r="G6" s="28" t="n">
         <v>0</v>
@@ -2652,7 +2652,7 @@
         <v>23.83</v>
       </c>
       <c r="F7" s="29" t="n">
-        <v>0.1119925302709312</v>
+        <v>11.19925302709312</v>
       </c>
       <c r="G7" s="28" t="n">
         <v>0</v>
@@ -2796,7 +2796,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
         </is>
       </c>
     </row>
@@ -2928,7 +2928,7 @@
         <v>207.83</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>0.05272809613927784</v>
+        <v>5.272809613927784</v>
       </c>
       <c r="G5" s="28" t="n">
         <v>0</v>
@@ -3000,7 +3000,7 @@
         <v>425.44</v>
       </c>
       <c r="F6" s="41" t="n">
-        <v>-0.01518517953378183</v>
+        <v>-1.518517953378183</v>
       </c>
       <c r="G6" s="28" t="n">
         <v>0</v>
@@ -3072,7 +3072,7 @@
         <v>297.17</v>
       </c>
       <c r="F7" s="29" t="n">
-        <v>0.06196624174582565</v>
+        <v>6.196624174582565</v>
       </c>
       <c r="G7" s="28" t="n">
         <v>0</v>
@@ -3144,7 +3144,7 @@
         <v>421.39</v>
       </c>
       <c r="F8" s="29" t="n">
-        <v>0.017850276928593</v>
+        <v>1.7850276928593</v>
       </c>
       <c r="G8" s="28" t="n">
         <v>0</v>
@@ -3216,7 +3216,7 @@
         <v>113.01</v>
       </c>
       <c r="F9" s="41" t="n">
-        <v>-0.002999540042077861</v>
+        <v>-0.2999540042077861</v>
       </c>
       <c r="G9" s="28" t="n">
         <v>0</v>
@@ -3288,7 +3288,7 @@
         <v>237.3</v>
       </c>
       <c r="F10" s="29" t="n">
-        <v>0.04893251581027195</v>
+        <v>4.893251581027195</v>
       </c>
       <c r="G10" s="28" t="n">
         <v>0</v>
@@ -3432,7 +3432,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
         </is>
       </c>
     </row>
@@ -3564,7 +3564,7 @@
         <v>16.68</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>0.0127504739025976</v>
+        <v>1.27504739025976</v>
       </c>
       <c r="G5" s="28" t="n">
         <v>0</v>
@@ -3636,7 +3636,7 @@
         <v>96.73</v>
       </c>
       <c r="F6" s="29" t="n">
-        <v>0.06176529155937345</v>
+        <v>6.176529155937345</v>
       </c>
       <c r="G6" s="28" t="n">
         <v>0</v>
@@ -3708,7 +3708,7 @@
         <v>198.29</v>
       </c>
       <c r="F7" s="41" t="n">
-        <v>-0.001057968331824622</v>
+        <v>-0.1057968331824622</v>
       </c>
       <c r="G7" s="28" t="n">
         <v>0</v>
@@ -3780,7 +3780,7 @@
         <v>51.37</v>
       </c>
       <c r="F8" s="29" t="n">
-        <v>0.027541779403253</v>
+        <v>2.7541779403253</v>
       </c>
       <c r="G8" s="28" t="n">
         <v>0</v>
@@ -3852,7 +3852,7 @@
         <v>12.33</v>
       </c>
       <c r="F9" s="41" t="n">
-        <v>-0.002830576327856492</v>
+        <v>-0.2830576327856492</v>
       </c>
       <c r="G9" s="28" t="n">
         <v>0</v>
@@ -3924,7 +3924,7 @@
         <v>309.81</v>
       </c>
       <c r="F10" s="29" t="n">
-        <v>0.0275621809571932</v>
+        <v>2.75621809571932</v>
       </c>
       <c r="G10" s="28" t="n">
         <v>0</v>
@@ -3996,7 +3996,7 @@
         <v>16.57</v>
       </c>
       <c r="F11" s="29" t="n">
-        <v>0.07110534549607098</v>
+        <v>7.110534549607098</v>
       </c>
       <c r="G11" s="28" t="n">
         <v>0</v>
@@ -4140,7 +4140,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
         <v>944.28</v>
       </c>
       <c r="F5" s="41" t="n">
-        <v>-0.01642619728464659</v>
+        <v>-1.642619728464659</v>
       </c>
       <c r="G5" s="28" t="n">
         <v>0</v>
@@ -4416,7 +4416,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
         </is>
       </c>
     </row>
@@ -4548,7 +4548,7 @@
         <v>926.9299999999999</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>0.01762031516311836</v>
+        <v>1.762031516311836</v>
       </c>
       <c r="G5" s="28" t="n">
         <v>0</v>
@@ -4620,7 +4620,7 @@
         <v>2011.49</v>
       </c>
       <c r="F6" s="29" t="n">
-        <v>0.01284503883945205</v>
+        <v>1.284503883945205</v>
       </c>
       <c r="G6" s="28" t="n">
         <v>0</v>
@@ -4692,7 +4692,7 @@
         <v>320.3</v>
       </c>
       <c r="F7" s="29" t="n">
-        <v>0.06766662597656251</v>
+        <v>6.766662597656251</v>
       </c>
       <c r="G7" s="28" t="n">
         <v>0</v>
@@ -4764,7 +4764,7 @@
         <v>358.92</v>
       </c>
       <c r="F8" s="29" t="n">
-        <v>0.02939746301010801</v>
+        <v>2.939746301010801</v>
       </c>
       <c r="G8" s="28" t="n">
         <v>0</v>
@@ -4908,7 +4908,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
         </is>
       </c>
     </row>
@@ -5040,7 +5040,7 @@
         <v>1118.96</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>0.0171068781586888</v>
+        <v>1.71068781586888</v>
       </c>
       <c r="G5" s="28" t="n">
         <v>0</v>
@@ -5112,7 +5112,7 @@
         <v>785.24</v>
       </c>
       <c r="F6" s="29" t="n">
-        <v>0.01881307604947841</v>
+        <v>1.881307604947841</v>
       </c>
       <c r="G6" s="28" t="n">
         <v>0</v>
@@ -5184,7 +5184,7 @@
         <v>285.47</v>
       </c>
       <c r="F7" s="41" t="n">
-        <v>-0.04067043441964675</v>
+        <v>-4.067043441964675</v>
       </c>
       <c r="G7" s="28" t="n">
         <v>0</v>
@@ -5256,7 +5256,7 @@
         <v>79.62</v>
       </c>
       <c r="F8" s="29" t="n">
-        <v>0.1715715530691883</v>
+        <v>17.15715530691883</v>
       </c>
       <c r="G8" s="28" t="n">
         <v>0</v>
@@ -5400,7 +5400,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
         <v>195.09</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>0.1084973796863014</v>
+        <v>10.84973796863014</v>
       </c>
       <c r="G5" s="28" t="n">
         <v>0</v>
@@ -5604,7 +5604,7 @@
         <v>133.79</v>
       </c>
       <c r="F6" s="41" t="n">
-        <v>-0.01101424241474858</v>
+        <v>-1.101424241474859</v>
       </c>
       <c r="G6" s="28" t="n">
         <v>0</v>
@@ -5748,7 +5748,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:11 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
         <v>9.34</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>0.006595696920710679</v>
+        <v>0.6595696920710679</v>
       </c>
       <c r="G5" s="28" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Organize investment notes below portfolio totals on each tab
Removes the "Investment Thesis / Notes" column and displays notes in a new, dedicated section below the portfolio totals for improved readability.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 608cae44-65ba-47aa-811b-aaeba7186851
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -31,7 +31,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="+0.00&quot;%&quot;;-0.00&quot;%&quot;;0.00&quot;%&quot;"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -166,6 +166,11 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <color rgb="001B2A4A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFD700"/>
       <sz val="14"/>
@@ -281,7 +286,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -317,11 +322,55 @@
         <color rgb="00AAAAAA"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -435,6 +484,23 @@
     <xf numFmtId="10" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -453,6 +519,9 @@
     <xf numFmtId="10" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -468,6 +537,9 @@
     <xf numFmtId="10" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -483,6 +555,9 @@
     <xf numFmtId="10" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -498,6 +573,9 @@
     <xf numFmtId="10" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -513,6 +591,9 @@
     <xf numFmtId="10" fontId="4" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -528,6 +609,9 @@
     <xf numFmtId="10" fontId="4" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -543,6 +627,9 @@
     <xf numFmtId="10" fontId="4" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -558,6 +645,9 @@
     <xf numFmtId="10" fontId="4" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -573,7 +663,10 @@
     <xf numFmtId="10" fontId="4" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1006,7 +1099,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
         </is>
       </c>
     </row>
@@ -1454,7 +1547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1474,11 +1567,10 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="50" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="75" t="inlineStr">
+      <c r="A1" s="89" t="inlineStr">
         <is>
           <t>🚀 Space Economy</t>
         </is>
@@ -1494,112 +1586,107 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="76" t="inlineStr">
+      <c r="A4" s="90" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="76" t="inlineStr">
+      <c r="B4" s="90" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="76" t="inlineStr">
+      <c r="C4" s="90" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="76" t="inlineStr">
+      <c r="D4" s="90" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="76" t="inlineStr">
+      <c r="E4" s="90" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="76" t="inlineStr">
+      <c r="F4" s="90" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="76" t="inlineStr">
+      <c r="G4" s="90" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="76" t="inlineStr">
+      <c r="H4" s="90" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="76" t="inlineStr">
+      <c r="I4" s="90" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="76" t="inlineStr">
+      <c r="J4" s="90" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="76" t="inlineStr">
+      <c r="K4" s="90" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="76" t="inlineStr">
+      <c r="L4" s="90" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="76" t="inlineStr">
+      <c r="M4" s="90" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="76" t="inlineStr">
+      <c r="N4" s="90" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="76" t="inlineStr">
+      <c r="O4" s="90" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="76" t="inlineStr">
+      <c r="P4" s="90" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="76" t="inlineStr">
+      <c r="Q4" s="90" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
         </is>
       </c>
-      <c r="R4" s="76" t="inlineStr">
-        <is>
-          <t>Investment Thesis / Notes</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
@@ -1667,41 +1754,94 @@
         <f>IFERROR(P5/E5-1,"")</f>
         <v/>
       </c>
-      <c r="R5" s="10" t="inlineStr">
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="91" t="inlineStr">
+        <is>
+          <t>PORTFOLIO TOTALS</t>
+        </is>
+      </c>
+      <c r="H7" s="92">
+        <f>SUM(H5:H5)</f>
+        <v/>
+      </c>
+      <c r="I7" s="92">
+        <f>SUM(I5:I5)</f>
+        <v/>
+      </c>
+      <c r="J7" s="92">
+        <f>SUM(J5:J5)</f>
+        <v/>
+      </c>
+      <c r="K7" s="93">
+        <f>IFERROR(J7/H7,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="94" t="inlineStr">
+        <is>
+          <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="40" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B10" s="40" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C10" s="41" t="inlineStr">
+        <is>
+          <t>Notes / Thesis</t>
+        </is>
+      </c>
+      <c r="D10" s="42" t="n"/>
+      <c r="E10" s="42" t="n"/>
+      <c r="F10" s="42" t="n"/>
+      <c r="G10" s="42" t="n"/>
+      <c r="H10" s="42" t="n"/>
+      <c r="I10" s="42" t="n"/>
+      <c r="J10" s="42" t="n"/>
+      <c r="K10" s="42" t="n"/>
+      <c r="L10" s="42" t="n"/>
+      <c r="M10" s="42" t="n"/>
+      <c r="N10" s="42" t="n"/>
+      <c r="O10" s="42" t="n"/>
+      <c r="P10" s="42" t="n"/>
+      <c r="Q10" s="43" t="n"/>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="B11" s="44" t="inlineStr">
+        <is>
+          <t>Rocket Lab USA</t>
+        </is>
+      </c>
+      <c r="C11" s="44" t="inlineStr">
         <is>
           <t>Huge future TAM over next decade+. Speculative but massive upside. Brilliant CEO. Near-term catalyst: SpaceX IPO in June.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="77" t="inlineStr">
-        <is>
-          <t>PORTFOLIO TOTALS</t>
-        </is>
-      </c>
-      <c r="H7" s="78">
-        <f>SUM(H5:H5)</f>
-        <v/>
-      </c>
-      <c r="I7" s="78">
-        <f>SUM(I5:I5)</f>
-        <v/>
-      </c>
-      <c r="J7" s="78">
-        <f>SUM(J5:J5)</f>
-        <v/>
-      </c>
-      <c r="K7" s="79">
-        <f>IFERROR(J7/H7,"")</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A3:R3"/>
-    <mergeCell ref="A2:R2"/>
-    <mergeCell ref="A1:R1"/>
+  <mergeCells count="7">
+    <mergeCell ref="A9:Q9"/>
+    <mergeCell ref="A3:Q3"/>
+    <mergeCell ref="C10:Q10"/>
+    <mergeCell ref="C11:Q11"/>
+    <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="J5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -1730,7 +1870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R8"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1750,11 +1890,10 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="50" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="80" t="inlineStr">
+      <c r="A1" s="95" t="inlineStr">
         <is>
           <t>🔭 Long Term Watchlist</t>
         </is>
@@ -1770,112 +1909,107 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="81" t="inlineStr">
+      <c r="A4" s="96" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="81" t="inlineStr">
+      <c r="B4" s="96" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="81" t="inlineStr">
+      <c r="C4" s="96" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="81" t="inlineStr">
+      <c r="D4" s="96" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="81" t="inlineStr">
+      <c r="E4" s="96" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="81" t="inlineStr">
+      <c r="F4" s="96" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="81" t="inlineStr">
+      <c r="G4" s="96" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="81" t="inlineStr">
+      <c r="H4" s="96" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="81" t="inlineStr">
+      <c r="I4" s="96" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="81" t="inlineStr">
+      <c r="J4" s="96" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="81" t="inlineStr">
+      <c r="K4" s="96" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="81" t="inlineStr">
+      <c r="L4" s="96" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="81" t="inlineStr">
+      <c r="M4" s="96" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="81" t="inlineStr">
+      <c r="N4" s="96" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="81" t="inlineStr">
+      <c r="O4" s="96" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="81" t="inlineStr">
+      <c r="P4" s="96" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="81" t="inlineStr">
+      <c r="Q4" s="96" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
         </is>
       </c>
-      <c r="R4" s="81" t="inlineStr">
-        <is>
-          <t>Investment Thesis / Notes</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
@@ -1943,11 +2077,6 @@
         <f>IFERROR(P5/E5-1,"")</f>
         <v/>
       </c>
-      <c r="R5" s="10" t="inlineStr">
-        <is>
-          <t>Long term investment research candidate.</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="33" t="inlineStr">
@@ -2015,41 +2144,112 @@
         <f>IFERROR(P6/E6-1,"")</f>
         <v/>
       </c>
-      <c r="R6" s="7" t="inlineStr">
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="97" t="inlineStr">
+        <is>
+          <t>PORTFOLIO TOTALS</t>
+        </is>
+      </c>
+      <c r="H8" s="98">
+        <f>SUM(H5:H6)</f>
+        <v/>
+      </c>
+      <c r="I8" s="98">
+        <f>SUM(I5:I6)</f>
+        <v/>
+      </c>
+      <c r="J8" s="98">
+        <f>SUM(J5:J6)</f>
+        <v/>
+      </c>
+      <c r="K8" s="99">
+        <f>IFERROR(J8/H8,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="100" t="inlineStr">
+        <is>
+          <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="40" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B11" s="40" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C11" s="41" t="inlineStr">
+        <is>
+          <t>Notes / Thesis</t>
+        </is>
+      </c>
+      <c r="D11" s="42" t="n"/>
+      <c r="E11" s="42" t="n"/>
+      <c r="F11" s="42" t="n"/>
+      <c r="G11" s="42" t="n"/>
+      <c r="H11" s="42" t="n"/>
+      <c r="I11" s="42" t="n"/>
+      <c r="J11" s="42" t="n"/>
+      <c r="K11" s="42" t="n"/>
+      <c r="L11" s="42" t="n"/>
+      <c r="M11" s="42" t="n"/>
+      <c r="N11" s="42" t="n"/>
+      <c r="O11" s="42" t="n"/>
+      <c r="P11" s="42" t="n"/>
+      <c r="Q11" s="43" t="n"/>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>RBRK</t>
+        </is>
+      </c>
+      <c r="B12" s="44" t="inlineStr">
+        <is>
+          <t>Rubrik Inc</t>
+        </is>
+      </c>
+      <c r="C12" s="44" t="inlineStr">
         <is>
           <t>Long term investment research candidate.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="82" t="inlineStr">
-        <is>
-          <t>PORTFOLIO TOTALS</t>
-        </is>
-      </c>
-      <c r="H8" s="83">
-        <f>SUM(H5:H6)</f>
-        <v/>
-      </c>
-      <c r="I8" s="83">
-        <f>SUM(I5:I6)</f>
-        <v/>
-      </c>
-      <c r="J8" s="83">
-        <f>SUM(J5:J6)</f>
-        <v/>
-      </c>
-      <c r="K8" s="84">
-        <f>IFERROR(J8/H8,"")</f>
-        <v/>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="27" t="inlineStr">
+        <is>
+          <t>NVO</t>
+        </is>
+      </c>
+      <c r="B13" s="45" t="inlineStr">
+        <is>
+          <t>Novo Nordisk</t>
+        </is>
+      </c>
+      <c r="C13" s="45" t="inlineStr">
+        <is>
+          <t>Long term investment research candidate.</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="8">
+    <mergeCell ref="A3:Q3"/>
     <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A3:R3"/>
-    <mergeCell ref="A2:R2"/>
-    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="C11:Q11"/>
+    <mergeCell ref="C13:Q13"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A10:Q10"/>
+    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="C12:Q12"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J6">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -2086,14 +2286,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="85" t="inlineStr">
+      <c r="A1" s="101" t="inlineStr">
         <is>
           <t>📝 RESEARCH NOTES &amp; INVESTMENT THESIS</t>
         </is>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1">
-      <c r="A2" s="86" t="inlineStr">
+      <c r="A2" s="102" t="inlineStr">
         <is>
           <t>401k To-Do</t>
         </is>
@@ -2106,7 +2306,7 @@
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="87" t="inlineStr">
+      <c r="A3" s="103" t="inlineStr">
         <is>
           <t>Savings Account</t>
         </is>
@@ -2118,7 +2318,7 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="86" t="inlineStr">
+      <c r="A4" s="102" t="inlineStr">
         <is>
           <t>Research Tools</t>
         </is>
@@ -2130,7 +2330,7 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="87" t="inlineStr">
+      <c r="A5" s="103" t="inlineStr">
         <is>
           <t>Quantum Thesis</t>
         </is>
@@ -2142,7 +2342,7 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="86" t="inlineStr">
+      <c r="A6" s="102" t="inlineStr">
         <is>
           <t>NVTS</t>
         </is>
@@ -2154,7 +2354,7 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="87" t="inlineStr">
+      <c r="A7" s="103" t="inlineStr">
         <is>
           <t>AEHR</t>
         </is>
@@ -2166,7 +2366,7 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="86" t="inlineStr">
+      <c r="A8" s="102" t="inlineStr">
         <is>
           <t>CRDO</t>
         </is>
@@ -2178,7 +2378,7 @@
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="87" t="inlineStr">
+      <c r="A9" s="103" t="inlineStr">
         <is>
           <t>ALGM</t>
         </is>
@@ -2190,7 +2390,7 @@
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="86" t="inlineStr">
+      <c r="A10" s="102" t="inlineStr">
         <is>
           <t>HIMX</t>
         </is>
@@ -2202,7 +2402,7 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="87" t="inlineStr">
+      <c r="A11" s="103" t="inlineStr">
         <is>
           <t>MTSI</t>
         </is>
@@ -2214,7 +2414,7 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="86" t="inlineStr">
+      <c r="A12" s="102" t="inlineStr">
         <is>
           <t>AEVA</t>
         </is>
@@ -2226,7 +2426,7 @@
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="87" t="inlineStr">
+      <c r="A13" s="103" t="inlineStr">
         <is>
           <t>AI Infrastructure</t>
         </is>
@@ -2238,7 +2438,7 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="86" t="inlineStr">
+      <c r="A14" s="102" t="inlineStr">
         <is>
           <t>LITE</t>
         </is>
@@ -2250,7 +2450,7 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="87" t="inlineStr">
+      <c r="A15" s="103" t="inlineStr">
         <is>
           <t>OKLO</t>
         </is>
@@ -2262,7 +2462,7 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="86" t="inlineStr">
+      <c r="A16" s="102" t="inlineStr">
         <is>
           <t>NBIS</t>
         </is>
@@ -2274,7 +2474,7 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="87" t="inlineStr">
+      <c r="A17" s="103" t="inlineStr">
         <is>
           <t>PLTR</t>
         </is>
@@ -2286,7 +2486,7 @@
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="86" t="inlineStr">
+      <c r="A18" s="102" t="inlineStr">
         <is>
           <t>ONDS</t>
         </is>
@@ -2298,7 +2498,7 @@
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="87" t="inlineStr">
+      <c r="A19" s="103" t="inlineStr">
         <is>
           <t>RKLB</t>
         </is>
@@ -2310,7 +2510,7 @@
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="86" t="inlineStr">
+      <c r="A20" s="102" t="inlineStr">
         <is>
           <t>Recommended Portfolio</t>
         </is>
@@ -2336,7 +2536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R9"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2356,7 +2556,6 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="50" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -2376,7 +2575,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
         </is>
       </c>
     </row>
@@ -2477,11 +2676,6 @@
 Target</t>
         </is>
       </c>
-      <c r="R4" s="26" t="inlineStr">
-        <is>
-          <t>Investment Thesis / Notes</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
@@ -2549,11 +2743,6 @@
         <f>IFERROR(P5/E5-1,"")</f>
         <v/>
       </c>
-      <c r="R5" s="10" t="inlineStr">
-        <is>
-          <t>Next quantum run candidate. Easy 10× within 2 years potential.</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="33" t="inlineStr">
@@ -2621,11 +2810,6 @@
         <f>IFERROR(P6/E6-1,"")</f>
         <v/>
       </c>
-      <c r="R6" s="7" t="inlineStr">
-        <is>
-          <t>Next quantum run candidate. Easy 10× within 2 years potential.</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
@@ -2693,11 +2877,6 @@
         <f>IFERROR(P7/E7-1,"")</f>
         <v/>
       </c>
-      <c r="R7" s="10" t="inlineStr">
-        <is>
-          <t>Next quantum run candidate. Easy 10× within 2 years potential.</t>
-        </is>
-      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="36" t="inlineStr">
@@ -2722,12 +2901,106 @@
         <v/>
       </c>
     </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="39" t="inlineStr">
+        <is>
+          <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="40" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B12" s="40" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C12" s="41" t="inlineStr">
+        <is>
+          <t>Notes / Thesis</t>
+        </is>
+      </c>
+      <c r="D12" s="42" t="n"/>
+      <c r="E12" s="42" t="n"/>
+      <c r="F12" s="42" t="n"/>
+      <c r="G12" s="42" t="n"/>
+      <c r="H12" s="42" t="n"/>
+      <c r="I12" s="42" t="n"/>
+      <c r="J12" s="42" t="n"/>
+      <c r="K12" s="42" t="n"/>
+      <c r="L12" s="42" t="n"/>
+      <c r="M12" s="42" t="n"/>
+      <c r="N12" s="42" t="n"/>
+      <c r="O12" s="42" t="n"/>
+      <c r="P12" s="42" t="n"/>
+      <c r="Q12" s="43" t="n"/>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>IONQ</t>
+        </is>
+      </c>
+      <c r="B13" s="44" t="inlineStr">
+        <is>
+          <t>IonQ Inc</t>
+        </is>
+      </c>
+      <c r="C13" s="44" t="inlineStr">
+        <is>
+          <t>Next quantum run candidate. Easy 10× within 2 years potential.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="27" t="inlineStr">
+        <is>
+          <t>RGTI</t>
+        </is>
+      </c>
+      <c r="B14" s="45" t="inlineStr">
+        <is>
+          <t>Rigetti Computing</t>
+        </is>
+      </c>
+      <c r="C14" s="45" t="inlineStr">
+        <is>
+          <t>Next quantum run candidate. Easy 10× within 2 years potential.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="33" t="inlineStr">
+        <is>
+          <t>QBTS</t>
+        </is>
+      </c>
+      <c r="B15" s="44" t="inlineStr">
+        <is>
+          <t>D-Wave Quantum</t>
+        </is>
+      </c>
+      <c r="C15" s="44" t="inlineStr">
+        <is>
+          <t>Next quantum run candidate. Easy 10× within 2 years potential.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A3:R3"/>
-    <mergeCell ref="A2:R2"/>
-    <mergeCell ref="A1:R1"/>
+  <mergeCells count="9">
+    <mergeCell ref="C15:Q15"/>
     <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A3:Q3"/>
+    <mergeCell ref="C14:Q14"/>
+    <mergeCell ref="C13:Q13"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A11:Q11"/>
+    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="C12:Q12"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J7">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -2756,7 +3029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R12"/>
+  <dimension ref="A1:Q21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2776,11 +3049,10 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="50" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="39" t="inlineStr">
+      <c r="A1" s="46" t="inlineStr">
         <is>
           <t>🖥️ Semiconductors &amp; Compute</t>
         </is>
@@ -2796,112 +3068,107 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="40" t="inlineStr">
+      <c r="A4" s="47" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="40" t="inlineStr">
+      <c r="B4" s="47" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="40" t="inlineStr">
+      <c r="C4" s="47" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="40" t="inlineStr">
+      <c r="D4" s="47" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="40" t="inlineStr">
+      <c r="E4" s="47" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="40" t="inlineStr">
+      <c r="F4" s="47" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="40" t="inlineStr">
+      <c r="G4" s="47" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="40" t="inlineStr">
+      <c r="H4" s="47" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="40" t="inlineStr">
+      <c r="I4" s="47" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="40" t="inlineStr">
+      <c r="J4" s="47" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="40" t="inlineStr">
+      <c r="K4" s="47" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="40" t="inlineStr">
+      <c r="L4" s="47" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="40" t="inlineStr">
+      <c r="M4" s="47" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="40" t="inlineStr">
+      <c r="N4" s="47" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="40" t="inlineStr">
+      <c r="O4" s="47" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="40" t="inlineStr">
+      <c r="P4" s="47" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="40" t="inlineStr">
+      <c r="Q4" s="47" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
         </is>
       </c>
-      <c r="R4" s="40" t="inlineStr">
-        <is>
-          <t>Investment Thesis / Notes</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
@@ -2969,11 +3236,6 @@
         <f>IFERROR(P5/E5-1,"")</f>
         <v/>
       </c>
-      <c r="R5" s="10" t="inlineStr">
-        <is>
-          <t>The AI compute king. Stability and steady compounder.</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="33" t="inlineStr">
@@ -2999,7 +3261,7 @@
       <c r="E6" s="28" t="n">
         <v>425.44</v>
       </c>
-      <c r="F6" s="41" t="n">
+      <c r="F6" s="48" t="n">
         <v>-1.518517953378183</v>
       </c>
       <c r="G6" s="28" t="n">
@@ -3041,11 +3303,6 @@
         <f>IFERROR(P6/E6-1,"")</f>
         <v/>
       </c>
-      <c r="R6" s="7" t="inlineStr">
-        <is>
-          <t>Stability and steady compounder.</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
@@ -3113,11 +3370,6 @@
         <f>IFERROR(P7/E7-1,"")</f>
         <v/>
       </c>
-      <c r="R7" s="10" t="inlineStr">
-        <is>
-          <t>Stability and steady compounder. DRAM equipment leader.</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="33" t="inlineStr">
@@ -3185,11 +3437,6 @@
         <f>IFERROR(P8/E8-1,"")</f>
         <v/>
       </c>
-      <c r="R8" s="7" t="inlineStr">
-        <is>
-          <t>CPU maker deep in the AI infrastructure stack.</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
@@ -3215,7 +3462,7 @@
       <c r="E9" s="28" t="n">
         <v>113.01</v>
       </c>
-      <c r="F9" s="41" t="n">
+      <c r="F9" s="48" t="n">
         <v>-0.2999540042077861</v>
       </c>
       <c r="G9" s="28" t="n">
@@ -3257,11 +3504,6 @@
         <f>IFERROR(P9/E9-1,"")</f>
         <v/>
       </c>
-      <c r="R9" s="10" t="inlineStr">
-        <is>
-          <t>CPU maker in AI infrastructure stack. Turnaround story.</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="33" t="inlineStr">
@@ -3329,41 +3571,184 @@
         <f>IFERROR(P10/E10-1,"")</f>
         <v/>
       </c>
-      <c r="R10" s="7" t="inlineStr">
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="49" t="inlineStr">
+        <is>
+          <t>PORTFOLIO TOTALS</t>
+        </is>
+      </c>
+      <c r="H12" s="50">
+        <f>SUM(H5:H10)</f>
+        <v/>
+      </c>
+      <c r="I12" s="50">
+        <f>SUM(I5:I10)</f>
+        <v/>
+      </c>
+      <c r="J12" s="50">
+        <f>SUM(J5:J10)</f>
+        <v/>
+      </c>
+      <c r="K12" s="51">
+        <f>IFERROR(J12/H12,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="52" t="inlineStr">
+        <is>
+          <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="40" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B15" s="40" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C15" s="41" t="inlineStr">
+        <is>
+          <t>Notes / Thesis</t>
+        </is>
+      </c>
+      <c r="D15" s="42" t="n"/>
+      <c r="E15" s="42" t="n"/>
+      <c r="F15" s="42" t="n"/>
+      <c r="G15" s="42" t="n"/>
+      <c r="H15" s="42" t="n"/>
+      <c r="I15" s="42" t="n"/>
+      <c r="J15" s="42" t="n"/>
+      <c r="K15" s="42" t="n"/>
+      <c r="L15" s="42" t="n"/>
+      <c r="M15" s="42" t="n"/>
+      <c r="N15" s="42" t="n"/>
+      <c r="O15" s="42" t="n"/>
+      <c r="P15" s="42" t="n"/>
+      <c r="Q15" s="43" t="n"/>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="33" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="B16" s="44" t="inlineStr">
+        <is>
+          <t>NVIDIA Corp</t>
+        </is>
+      </c>
+      <c r="C16" s="44" t="inlineStr">
+        <is>
+          <t>The AI compute king. Stability and steady compounder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="27" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="B17" s="45" t="inlineStr">
+        <is>
+          <t>Broadcom Inc</t>
+        </is>
+      </c>
+      <c r="C17" s="45" t="inlineStr">
+        <is>
+          <t>Stability and steady compounder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="33" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="B18" s="44" t="inlineStr">
+        <is>
+          <t>Lam Research</t>
+        </is>
+      </c>
+      <c r="C18" s="44" t="inlineStr">
+        <is>
+          <t>Stability and steady compounder. DRAM equipment leader.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="27" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B19" s="45" t="inlineStr">
+        <is>
+          <t>Advanced Micro Devices</t>
+        </is>
+      </c>
+      <c r="C19" s="45" t="inlineStr">
+        <is>
+          <t>CPU maker deep in the AI infrastructure stack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="33" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="B20" s="44" t="inlineStr">
+        <is>
+          <t>Intel Corp</t>
+        </is>
+      </c>
+      <c r="C20" s="44" t="inlineStr">
+        <is>
+          <t>CPU maker in AI infrastructure stack. Turnaround story.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" s="27" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="B21" s="45" t="inlineStr">
+        <is>
+          <t>Arm Holdings</t>
+        </is>
+      </c>
+      <c r="C21" s="45" t="inlineStr">
         <is>
           <t>Architecture behind most AI edge chips. Royalty model.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="42" t="inlineStr">
-        <is>
-          <t>PORTFOLIO TOTALS</t>
-        </is>
-      </c>
-      <c r="H12" s="43">
-        <f>SUM(H5:H10)</f>
-        <v/>
-      </c>
-      <c r="I12" s="43">
-        <f>SUM(I5:I10)</f>
-        <v/>
-      </c>
-      <c r="J12" s="43">
-        <f>SUM(J5:J10)</f>
-        <v/>
-      </c>
-      <c r="K12" s="44">
-        <f>IFERROR(J12/H12,"")</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A3:R3"/>
-    <mergeCell ref="A2:R2"/>
-    <mergeCell ref="A1:R1"/>
+  <mergeCells count="12">
+    <mergeCell ref="A14:Q14"/>
+    <mergeCell ref="C21:Q21"/>
+    <mergeCell ref="C20:Q20"/>
+    <mergeCell ref="C15:Q15"/>
+    <mergeCell ref="C17:Q17"/>
+    <mergeCell ref="A3:Q3"/>
+    <mergeCell ref="C16:Q16"/>
     <mergeCell ref="A12:G12"/>
+    <mergeCell ref="C19:Q19"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="C18:Q18"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J10">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -3392,7 +3777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R13"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3412,11 +3797,10 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="50" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="45" t="inlineStr">
+      <c r="A1" s="53" t="inlineStr">
         <is>
           <t>⚙️ AI Picks &amp; Shovels</t>
         </is>
@@ -3432,112 +3816,107 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="46" t="inlineStr">
+      <c r="A4" s="54" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="46" t="inlineStr">
+      <c r="B4" s="54" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="46" t="inlineStr">
+      <c r="C4" s="54" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="46" t="inlineStr">
+      <c r="D4" s="54" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="46" t="inlineStr">
+      <c r="E4" s="54" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="46" t="inlineStr">
+      <c r="F4" s="54" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="46" t="inlineStr">
+      <c r="G4" s="54" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="46" t="inlineStr">
+      <c r="H4" s="54" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="46" t="inlineStr">
+      <c r="I4" s="54" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="46" t="inlineStr">
+      <c r="J4" s="54" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="46" t="inlineStr">
+      <c r="K4" s="54" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="46" t="inlineStr">
+      <c r="L4" s="54" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="46" t="inlineStr">
+      <c r="M4" s="54" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="46" t="inlineStr">
+      <c r="N4" s="54" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="46" t="inlineStr">
+      <c r="O4" s="54" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="46" t="inlineStr">
+      <c r="P4" s="54" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="46" t="inlineStr">
+      <c r="Q4" s="54" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
         </is>
       </c>
-      <c r="R4" s="46" t="inlineStr">
-        <is>
-          <t>Investment Thesis / Notes</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
@@ -3605,11 +3984,6 @@
         <f>IFERROR(P5/E5-1,"")</f>
         <v/>
       </c>
-      <c r="R5" s="10" t="inlineStr">
-        <is>
-          <t>AI data centers need radically more efficient power delivery. Picks-and-shovels for compute growth.</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="33" t="inlineStr">
@@ -3677,11 +4051,6 @@
         <f>IFERROR(P6/E6-1,"")</f>
         <v/>
       </c>
-      <c r="R6" s="7" t="inlineStr">
-        <is>
-          <t>Classic shovels in a gold rush. More AI chips = more testing bottleneck demand.</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
@@ -3707,7 +4076,7 @@
       <c r="E7" s="28" t="n">
         <v>198.29</v>
       </c>
-      <c r="F7" s="41" t="n">
+      <c r="F7" s="48" t="n">
         <v>-0.1057968331824622</v>
       </c>
       <c r="G7" s="28" t="n">
@@ -3749,11 +4118,6 @@
         <f>IFERROR(P7/E7-1,"")</f>
         <v/>
       </c>
-      <c r="R7" s="10" t="inlineStr">
-        <is>
-          <t>GPUs don't matter if data can't move between them. Cleanest AI infrastructure picks-and-shovels name.</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="33" t="inlineStr">
@@ -3821,11 +4185,6 @@
         <f>IFERROR(P8/E8-1,"")</f>
         <v/>
       </c>
-      <c r="R8" s="7" t="inlineStr">
-        <is>
-          <t>Electrification + AI hardware power efficiency. Quiet compounder, early in AI rerating narrative.</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
@@ -3851,7 +4210,7 @@
       <c r="E9" s="28" t="n">
         <v>12.33</v>
       </c>
-      <c r="F9" s="41" t="n">
+      <c r="F9" s="48" t="n">
         <v>-0.2830576327856492</v>
       </c>
       <c r="G9" s="28" t="n">
@@ -3893,11 +4252,6 @@
         <f>IFERROR(P9/E9-1,"")</f>
         <v/>
       </c>
-      <c r="R9" s="10" t="inlineStr">
-        <is>
-          <t>Exposure to AI edge devices + optics. Higher volatility, historically rerates fast on cycles.</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="33" t="inlineStr">
@@ -3965,11 +4319,6 @@
         <f>IFERROR(P10/E10-1,"")</f>
         <v/>
       </c>
-      <c r="R10" s="7" t="inlineStr">
-        <is>
-          <t>AI datacenter interconnect + telecom backbone. Less hype, more industrial AI backbone exposure.</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
@@ -4037,41 +4386,202 @@
         <f>IFERROR(P11/E11-1,"")</f>
         <v/>
       </c>
-      <c r="R11" s="10" t="inlineStr">
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="55" t="inlineStr">
+        <is>
+          <t>PORTFOLIO TOTALS</t>
+        </is>
+      </c>
+      <c r="H13" s="56">
+        <f>SUM(H5:H11)</f>
+        <v/>
+      </c>
+      <c r="I13" s="56">
+        <f>SUM(I5:I11)</f>
+        <v/>
+      </c>
+      <c r="J13" s="56">
+        <f>SUM(J5:J11)</f>
+        <v/>
+      </c>
+      <c r="K13" s="57">
+        <f>IFERROR(J13/H13,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="58" t="inlineStr">
+        <is>
+          <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="40" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B16" s="40" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C16" s="41" t="inlineStr">
+        <is>
+          <t>Notes / Thesis</t>
+        </is>
+      </c>
+      <c r="D16" s="42" t="n"/>
+      <c r="E16" s="42" t="n"/>
+      <c r="F16" s="42" t="n"/>
+      <c r="G16" s="42" t="n"/>
+      <c r="H16" s="42" t="n"/>
+      <c r="I16" s="42" t="n"/>
+      <c r="J16" s="42" t="n"/>
+      <c r="K16" s="42" t="n"/>
+      <c r="L16" s="42" t="n"/>
+      <c r="M16" s="42" t="n"/>
+      <c r="N16" s="42" t="n"/>
+      <c r="O16" s="42" t="n"/>
+      <c r="P16" s="42" t="n"/>
+      <c r="Q16" s="43" t="n"/>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="33" t="inlineStr">
+        <is>
+          <t>NVTS</t>
+        </is>
+      </c>
+      <c r="B17" s="44" t="inlineStr">
+        <is>
+          <t>Navitas Semiconductor</t>
+        </is>
+      </c>
+      <c r="C17" s="44" t="inlineStr">
+        <is>
+          <t>AI data centers need radically more efficient power delivery. Picks-and-shovels for compute growth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="27" t="inlineStr">
+        <is>
+          <t>AEHR</t>
+        </is>
+      </c>
+      <c r="B18" s="45" t="inlineStr">
+        <is>
+          <t>AEHR Test Systems</t>
+        </is>
+      </c>
+      <c r="C18" s="45" t="inlineStr">
+        <is>
+          <t>Classic shovels in a gold rush. More AI chips = more testing bottleneck demand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="33" t="inlineStr">
+        <is>
+          <t>CRDO</t>
+        </is>
+      </c>
+      <c r="B19" s="44" t="inlineStr">
+        <is>
+          <t>Credo Technology</t>
+        </is>
+      </c>
+      <c r="C19" s="44" t="inlineStr">
+        <is>
+          <t>GPUs don't matter if data can't move between them. Cleanest AI infrastructure picks-and-shovels name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="27" t="inlineStr">
+        <is>
+          <t>ALGM</t>
+        </is>
+      </c>
+      <c r="B20" s="45" t="inlineStr">
+        <is>
+          <t>Allegro MicroSystems</t>
+        </is>
+      </c>
+      <c r="C20" s="45" t="inlineStr">
+        <is>
+          <t>Electrification + AI hardware power efficiency. Quiet compounder, early in AI rerating narrative.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" s="33" t="inlineStr">
+        <is>
+          <t>HIMX</t>
+        </is>
+      </c>
+      <c r="B21" s="44" t="inlineStr">
+        <is>
+          <t>Himax Technologies</t>
+        </is>
+      </c>
+      <c r="C21" s="44" t="inlineStr">
+        <is>
+          <t>Exposure to AI edge devices + optics. Higher volatility, historically rerates fast on cycles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="48" customHeight="1">
+      <c r="A22" s="27" t="inlineStr">
+        <is>
+          <t>MTSI</t>
+        </is>
+      </c>
+      <c r="B22" s="45" t="inlineStr">
+        <is>
+          <t>MACOM Technology</t>
+        </is>
+      </c>
+      <c r="C22" s="45" t="inlineStr">
+        <is>
+          <t>AI datacenter interconnect + telecom backbone. Less hype, more industrial AI backbone exposure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="48" customHeight="1">
+      <c r="A23" s="33" t="inlineStr">
+        <is>
+          <t>AEVA</t>
+        </is>
+      </c>
+      <c r="B23" s="44" t="inlineStr">
+        <is>
+          <t>Aeva Technologies</t>
+        </is>
+      </c>
+      <c r="C23" s="44" t="inlineStr">
         <is>
           <t>Autonomous systems + robotics long tail. Pure asymmetric bet: low probability, high upside.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="47" t="inlineStr">
-        <is>
-          <t>PORTFOLIO TOTALS</t>
-        </is>
-      </c>
-      <c r="H13" s="48">
-        <f>SUM(H5:H11)</f>
-        <v/>
-      </c>
-      <c r="I13" s="48">
-        <f>SUM(I5:I11)</f>
-        <v/>
-      </c>
-      <c r="J13" s="48">
-        <f>SUM(J5:J11)</f>
-        <v/>
-      </c>
-      <c r="K13" s="49">
-        <f>IFERROR(J13/H13,"")</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A3:R3"/>
-    <mergeCell ref="A2:R2"/>
+  <mergeCells count="13">
     <mergeCell ref="A13:G13"/>
-    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="C21:Q21"/>
+    <mergeCell ref="C20:Q20"/>
+    <mergeCell ref="C17:Q17"/>
+    <mergeCell ref="A3:Q3"/>
+    <mergeCell ref="C16:Q16"/>
+    <mergeCell ref="C19:Q19"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A15:Q15"/>
+    <mergeCell ref="C23:Q23"/>
+    <mergeCell ref="C22:Q22"/>
+    <mergeCell ref="C18:Q18"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J11">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -4100,7 +4610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4120,11 +4630,10 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="50" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="50" t="inlineStr">
+      <c r="A1" s="59" t="inlineStr">
         <is>
           <t>💡 Photonics &amp; Optics</t>
         </is>
@@ -4140,112 +4649,107 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="51" t="inlineStr">
+      <c r="A4" s="60" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="51" t="inlineStr">
+      <c r="B4" s="60" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="51" t="inlineStr">
+      <c r="C4" s="60" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="51" t="inlineStr">
+      <c r="D4" s="60" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="51" t="inlineStr">
+      <c r="E4" s="60" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="51" t="inlineStr">
+      <c r="F4" s="60" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="51" t="inlineStr">
+      <c r="G4" s="60" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="51" t="inlineStr">
+      <c r="H4" s="60" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="51" t="inlineStr">
+      <c r="I4" s="60" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="51" t="inlineStr">
+      <c r="J4" s="60" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="51" t="inlineStr">
+      <c r="K4" s="60" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="51" t="inlineStr">
+      <c r="L4" s="60" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="51" t="inlineStr">
+      <c r="M4" s="60" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="51" t="inlineStr">
+      <c r="N4" s="60" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="51" t="inlineStr">
+      <c r="O4" s="60" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="51" t="inlineStr">
+      <c r="P4" s="60" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="51" t="inlineStr">
+      <c r="Q4" s="60" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
         </is>
       </c>
-      <c r="R4" s="51" t="inlineStr">
-        <is>
-          <t>Investment Thesis / Notes</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
@@ -4271,7 +4775,7 @@
       <c r="E5" s="28" t="n">
         <v>944.28</v>
       </c>
-      <c r="F5" s="41" t="n">
+      <c r="F5" s="48" t="n">
         <v>-1.642619728464659</v>
       </c>
       <c r="G5" s="28" t="n">
@@ -4313,41 +4817,94 @@
         <f>IFERROR(P5/E5-1,"")</f>
         <v/>
       </c>
-      <c r="R5" s="10" t="inlineStr">
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="61" t="inlineStr">
+        <is>
+          <t>PORTFOLIO TOTALS</t>
+        </is>
+      </c>
+      <c r="H7" s="62">
+        <f>SUM(H5:H5)</f>
+        <v/>
+      </c>
+      <c r="I7" s="62">
+        <f>SUM(I5:I5)</f>
+        <v/>
+      </c>
+      <c r="J7" s="62">
+        <f>SUM(J5:J5)</f>
+        <v/>
+      </c>
+      <c r="K7" s="63">
+        <f>IFERROR(J7/H7,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="64" t="inlineStr">
+        <is>
+          <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="40" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B10" s="40" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C10" s="41" t="inlineStr">
+        <is>
+          <t>Notes / Thesis</t>
+        </is>
+      </c>
+      <c r="D10" s="42" t="n"/>
+      <c r="E10" s="42" t="n"/>
+      <c r="F10" s="42" t="n"/>
+      <c r="G10" s="42" t="n"/>
+      <c r="H10" s="42" t="n"/>
+      <c r="I10" s="42" t="n"/>
+      <c r="J10" s="42" t="n"/>
+      <c r="K10" s="42" t="n"/>
+      <c r="L10" s="42" t="n"/>
+      <c r="M10" s="42" t="n"/>
+      <c r="N10" s="42" t="n"/>
+      <c r="O10" s="42" t="n"/>
+      <c r="P10" s="42" t="n"/>
+      <c r="Q10" s="43" t="n"/>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>LITE</t>
+        </is>
+      </c>
+      <c r="B11" s="44" t="inlineStr">
+        <is>
+          <t>Lumentum Holdings</t>
+        </is>
+      </c>
+      <c r="C11" s="44" t="inlineStr">
         <is>
           <t>King of Photonics. Could moonshot. Key bottleneck in AI data movement. Critical infrastructure.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="52" t="inlineStr">
-        <is>
-          <t>PORTFOLIO TOTALS</t>
-        </is>
-      </c>
-      <c r="H7" s="53">
-        <f>SUM(H5:H5)</f>
-        <v/>
-      </c>
-      <c r="I7" s="53">
-        <f>SUM(I5:I5)</f>
-        <v/>
-      </c>
-      <c r="J7" s="53">
-        <f>SUM(J5:J5)</f>
-        <v/>
-      </c>
-      <c r="K7" s="54">
-        <f>IFERROR(J7/H7,"")</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A3:R3"/>
-    <mergeCell ref="A2:R2"/>
-    <mergeCell ref="A1:R1"/>
+  <mergeCells count="7">
+    <mergeCell ref="A9:Q9"/>
+    <mergeCell ref="A3:Q3"/>
+    <mergeCell ref="C10:Q10"/>
+    <mergeCell ref="C11:Q11"/>
+    <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="J5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -4376,7 +4933,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R10"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4396,11 +4953,10 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="50" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="55" t="inlineStr">
+      <c r="A1" s="65" t="inlineStr">
         <is>
           <t>🏗️ DC Builders &amp; Cooling</t>
         </is>
@@ -4416,112 +4972,107 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="56" t="inlineStr">
+      <c r="A4" s="66" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="56" t="inlineStr">
+      <c r="B4" s="66" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="56" t="inlineStr">
+      <c r="C4" s="66" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="56" t="inlineStr">
+      <c r="D4" s="66" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="56" t="inlineStr">
+      <c r="E4" s="66" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="56" t="inlineStr">
+      <c r="F4" s="66" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="56" t="inlineStr">
+      <c r="G4" s="66" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="56" t="inlineStr">
+      <c r="H4" s="66" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="56" t="inlineStr">
+      <c r="I4" s="66" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="56" t="inlineStr">
+      <c r="J4" s="66" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="56" t="inlineStr">
+      <c r="K4" s="66" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="56" t="inlineStr">
+      <c r="L4" s="66" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="56" t="inlineStr">
+      <c r="M4" s="66" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="56" t="inlineStr">
+      <c r="N4" s="66" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="56" t="inlineStr">
+      <c r="O4" s="66" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="56" t="inlineStr">
+      <c r="P4" s="66" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="56" t="inlineStr">
+      <c r="Q4" s="66" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
         </is>
       </c>
-      <c r="R4" s="56" t="inlineStr">
-        <is>
-          <t>Investment Thesis / Notes</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
@@ -4589,11 +5140,6 @@
         <f>IFERROR(P5/E5-1,"")</f>
         <v/>
       </c>
-      <c r="R5" s="10" t="inlineStr">
-        <is>
-          <t>Actual builder and materials company in the AI data center trade.</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="33" t="inlineStr">
@@ -4661,11 +5207,6 @@
         <f>IFERROR(P6/E6-1,"")</f>
         <v/>
       </c>
-      <c r="R6" s="7" t="inlineStr">
-        <is>
-          <t>Builder AND cooling company. AI data center HVAC &amp; MEP systems. Major growing bottleneck.</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
@@ -4733,11 +5274,6 @@
         <f>IFERROR(P7/E7-1,"")</f>
         <v/>
       </c>
-      <c r="R7" s="10" t="inlineStr">
-        <is>
-          <t>Electrical infrastructure builder for AI data centers.</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="33" t="inlineStr">
@@ -4805,40 +5341,147 @@
         <f>IFERROR(P8/E8-1,"")</f>
         <v/>
       </c>
-      <c r="R8" s="7" t="inlineStr">
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="67" t="inlineStr">
+        <is>
+          <t>PORTFOLIO TOTALS</t>
+        </is>
+      </c>
+      <c r="H10" s="68">
+        <f>SUM(H5:H8)</f>
+        <v/>
+      </c>
+      <c r="I10" s="68">
+        <f>SUM(I5:I8)</f>
+        <v/>
+      </c>
+      <c r="J10" s="68">
+        <f>SUM(J5:J8)</f>
+        <v/>
+      </c>
+      <c r="K10" s="69">
+        <f>IFERROR(J10/H10,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="70" t="inlineStr">
+        <is>
+          <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="40" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B13" s="40" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C13" s="41" t="inlineStr">
+        <is>
+          <t>Notes / Thesis</t>
+        </is>
+      </c>
+      <c r="D13" s="42" t="n"/>
+      <c r="E13" s="42" t="n"/>
+      <c r="F13" s="42" t="n"/>
+      <c r="G13" s="42" t="n"/>
+      <c r="H13" s="42" t="n"/>
+      <c r="I13" s="42" t="n"/>
+      <c r="J13" s="42" t="n"/>
+      <c r="K13" s="42" t="n"/>
+      <c r="L13" s="42" t="n"/>
+      <c r="M13" s="42" t="n"/>
+      <c r="N13" s="42" t="n"/>
+      <c r="O13" s="42" t="n"/>
+      <c r="P13" s="42" t="n"/>
+      <c r="Q13" s="43" t="n"/>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="33" t="inlineStr">
+        <is>
+          <t>CAT</t>
+        </is>
+      </c>
+      <c r="B14" s="44" t="inlineStr">
+        <is>
+          <t>Caterpillar Inc</t>
+        </is>
+      </c>
+      <c r="C14" s="44" t="inlineStr">
+        <is>
+          <t>Actual builder and materials company in the AI data center trade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="27" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="B15" s="45" t="inlineStr">
+        <is>
+          <t>Comfort Systems USA</t>
+        </is>
+      </c>
+      <c r="C15" s="45" t="inlineStr">
+        <is>
+          <t>Builder AND cooling company. AI data center HVAC &amp; MEP systems. Major growing bottleneck.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="33" t="inlineStr">
+        <is>
+          <t>POWL</t>
+        </is>
+      </c>
+      <c r="B16" s="44" t="inlineStr">
+        <is>
+          <t>Powell Industries</t>
+        </is>
+      </c>
+      <c r="C16" s="44" t="inlineStr">
+        <is>
+          <t>Electrical infrastructure builder for AI data centers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="27" t="inlineStr">
+        <is>
+          <t>VRT</t>
+        </is>
+      </c>
+      <c r="B17" s="45" t="inlineStr">
+        <is>
+          <t>Vertiv Holdings</t>
+        </is>
+      </c>
+      <c r="C17" s="45" t="inlineStr">
         <is>
           <t>Premier AI data center cooling play. Cooling is a growing bottleneck.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="57" t="inlineStr">
-        <is>
-          <t>PORTFOLIO TOTALS</t>
-        </is>
-      </c>
-      <c r="H10" s="58">
-        <f>SUM(H5:H8)</f>
-        <v/>
-      </c>
-      <c r="I10" s="58">
-        <f>SUM(I5:I8)</f>
-        <v/>
-      </c>
-      <c r="J10" s="58">
-        <f>SUM(J5:J8)</f>
-        <v/>
-      </c>
-      <c r="K10" s="59">
-        <f>IFERROR(J10/H10,"")</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A3:R3"/>
-    <mergeCell ref="A2:R2"/>
-    <mergeCell ref="A1:R1"/>
+  <mergeCells count="10">
+    <mergeCell ref="C15:Q15"/>
+    <mergeCell ref="C17:Q17"/>
+    <mergeCell ref="A3:Q3"/>
+    <mergeCell ref="C16:Q16"/>
+    <mergeCell ref="A12:Q12"/>
+    <mergeCell ref="C14:Q14"/>
+    <mergeCell ref="C13:Q13"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A10:G10"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J8">
@@ -4868,7 +5511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R10"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4888,11 +5531,10 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="50" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="60" t="inlineStr">
+      <c r="A1" s="71" t="inlineStr">
         <is>
           <t>⚡ Power &amp; Energy</t>
         </is>
@@ -4908,112 +5550,107 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="61" t="inlineStr">
+      <c r="A4" s="72" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="61" t="inlineStr">
+      <c r="B4" s="72" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="61" t="inlineStr">
+      <c r="C4" s="72" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="61" t="inlineStr">
+      <c r="D4" s="72" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="61" t="inlineStr">
+      <c r="E4" s="72" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="61" t="inlineStr">
+      <c r="F4" s="72" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="61" t="inlineStr">
+      <c r="G4" s="72" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="61" t="inlineStr">
+      <c r="H4" s="72" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="61" t="inlineStr">
+      <c r="I4" s="72" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="61" t="inlineStr">
+      <c r="J4" s="72" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="61" t="inlineStr">
+      <c r="K4" s="72" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="61" t="inlineStr">
+      <c r="L4" s="72" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="61" t="inlineStr">
+      <c r="M4" s="72" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="61" t="inlineStr">
+      <c r="N4" s="72" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="61" t="inlineStr">
+      <c r="O4" s="72" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="61" t="inlineStr">
+      <c r="P4" s="72" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="61" t="inlineStr">
+      <c r="Q4" s="72" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
         </is>
       </c>
-      <c r="R4" s="61" t="inlineStr">
-        <is>
-          <t>Investment Thesis / Notes</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
@@ -5081,11 +5718,6 @@
         <f>IFERROR(P5/E5-1,"")</f>
         <v/>
       </c>
-      <c r="R5" s="10" t="inlineStr">
-        <is>
-          <t>Stability and steady compounder. Power and grid maintenance for AI buildout.</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="33" t="inlineStr">
@@ -5153,11 +5785,6 @@
         <f>IFERROR(P6/E6-1,"")</f>
         <v/>
       </c>
-      <c r="R6" s="7" t="inlineStr">
-        <is>
-          <t>Power generation and grid maintenance. Growing bottleneck for AI buildout.</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
@@ -5183,7 +5810,7 @@
       <c r="E7" s="28" t="n">
         <v>285.47</v>
       </c>
-      <c r="F7" s="41" t="n">
+      <c r="F7" s="48" t="n">
         <v>-4.067043441964675</v>
       </c>
       <c r="G7" s="28" t="n">
@@ -5225,11 +5852,6 @@
         <f>IFERROR(P7/E7-1,"")</f>
         <v/>
       </c>
-      <c r="R7" s="10" t="inlineStr">
-        <is>
-          <t>Moonshot potential if hydrogen &amp; fuel cell technology takes off.</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="33" t="inlineStr">
@@ -5297,40 +5919,147 @@
         <f>IFERROR(P8/E8-1,"")</f>
         <v/>
       </c>
-      <c r="R8" s="7" t="inlineStr">
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="73" t="inlineStr">
+        <is>
+          <t>PORTFOLIO TOTALS</t>
+        </is>
+      </c>
+      <c r="H10" s="74">
+        <f>SUM(H5:H8)</f>
+        <v/>
+      </c>
+      <c r="I10" s="74">
+        <f>SUM(I5:I8)</f>
+        <v/>
+      </c>
+      <c r="J10" s="74">
+        <f>SUM(J5:J8)</f>
+        <v/>
+      </c>
+      <c r="K10" s="75">
+        <f>IFERROR(J10/H10,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="76" t="inlineStr">
+        <is>
+          <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="40" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B13" s="40" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C13" s="41" t="inlineStr">
+        <is>
+          <t>Notes / Thesis</t>
+        </is>
+      </c>
+      <c r="D13" s="42" t="n"/>
+      <c r="E13" s="42" t="n"/>
+      <c r="F13" s="42" t="n"/>
+      <c r="G13" s="42" t="n"/>
+      <c r="H13" s="42" t="n"/>
+      <c r="I13" s="42" t="n"/>
+      <c r="J13" s="42" t="n"/>
+      <c r="K13" s="42" t="n"/>
+      <c r="L13" s="42" t="n"/>
+      <c r="M13" s="42" t="n"/>
+      <c r="N13" s="42" t="n"/>
+      <c r="O13" s="42" t="n"/>
+      <c r="P13" s="42" t="n"/>
+      <c r="Q13" s="43" t="n"/>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="33" t="inlineStr">
+        <is>
+          <t>GEV</t>
+        </is>
+      </c>
+      <c r="B14" s="44" t="inlineStr">
+        <is>
+          <t>GE Vernova</t>
+        </is>
+      </c>
+      <c r="C14" s="44" t="inlineStr">
+        <is>
+          <t>Stability and steady compounder. Power and grid maintenance for AI buildout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="27" t="inlineStr">
+        <is>
+          <t>PWR</t>
+        </is>
+      </c>
+      <c r="B15" s="45" t="inlineStr">
+        <is>
+          <t>Quanta Services</t>
+        </is>
+      </c>
+      <c r="C15" s="45" t="inlineStr">
+        <is>
+          <t>Power generation and grid maintenance. Growing bottleneck for AI buildout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="33" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="B16" s="44" t="inlineStr">
+        <is>
+          <t>Bloom Energy</t>
+        </is>
+      </c>
+      <c r="C16" s="44" t="inlineStr">
+        <is>
+          <t>Moonshot potential if hydrogen &amp; fuel cell technology takes off.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="27" t="inlineStr">
+        <is>
+          <t>OKLO</t>
+        </is>
+      </c>
+      <c r="B17" s="45" t="inlineStr">
+        <is>
+          <t>Oklo Inc</t>
+        </is>
+      </c>
+      <c r="C17" s="45" t="inlineStr">
         <is>
           <t>Massive moonshot potential. Big regulatory &amp; execution risk. Worth a small % of portfolio given massive potential.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="62" t="inlineStr">
-        <is>
-          <t>PORTFOLIO TOTALS</t>
-        </is>
-      </c>
-      <c r="H10" s="63">
-        <f>SUM(H5:H8)</f>
-        <v/>
-      </c>
-      <c r="I10" s="63">
-        <f>SUM(I5:I8)</f>
-        <v/>
-      </c>
-      <c r="J10" s="63">
-        <f>SUM(J5:J8)</f>
-        <v/>
-      </c>
-      <c r="K10" s="64">
-        <f>IFERROR(J10/H10,"")</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A3:R3"/>
-    <mergeCell ref="A2:R2"/>
-    <mergeCell ref="A1:R1"/>
+  <mergeCells count="10">
+    <mergeCell ref="C15:Q15"/>
+    <mergeCell ref="C17:Q17"/>
+    <mergeCell ref="A3:Q3"/>
+    <mergeCell ref="C16:Q16"/>
+    <mergeCell ref="A12:Q12"/>
+    <mergeCell ref="C14:Q14"/>
+    <mergeCell ref="C13:Q13"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A10:G10"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J8">
@@ -5360,7 +6089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R8"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5380,11 +6109,10 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="50" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="65" t="inlineStr">
+      <c r="A1" s="77" t="inlineStr">
         <is>
           <t>☁️ Neoclouds &amp; AI Software</t>
         </is>
@@ -5400,112 +6128,107 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="66" t="inlineStr">
+      <c r="A4" s="78" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="66" t="inlineStr">
+      <c r="B4" s="78" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="66" t="inlineStr">
+      <c r="C4" s="78" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="66" t="inlineStr">
+      <c r="D4" s="78" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="66" t="inlineStr">
+      <c r="E4" s="78" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="66" t="inlineStr">
+      <c r="F4" s="78" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="66" t="inlineStr">
+      <c r="G4" s="78" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="66" t="inlineStr">
+      <c r="H4" s="78" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="66" t="inlineStr">
+      <c r="I4" s="78" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="66" t="inlineStr">
+      <c r="J4" s="78" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="66" t="inlineStr">
+      <c r="K4" s="78" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="66" t="inlineStr">
+      <c r="L4" s="78" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="66" t="inlineStr">
+      <c r="M4" s="78" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="66" t="inlineStr">
+      <c r="N4" s="78" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="66" t="inlineStr">
+      <c r="O4" s="78" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="66" t="inlineStr">
+      <c r="P4" s="78" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="66" t="inlineStr">
+      <c r="Q4" s="78" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
         </is>
       </c>
-      <c r="R4" s="66" t="inlineStr">
-        <is>
-          <t>Investment Thesis / Notes</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
@@ -5573,11 +6296,6 @@
         <f>IFERROR(P5/E5-1,"")</f>
         <v/>
       </c>
-      <c r="R5" s="10" t="inlineStr">
-        <is>
-          <t>Leading Neocloud with multiple revenue streams (Clickhouse, AV Ride). Modern Amazon/Google style company. Could become a future Hyperscaler.</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="33" t="inlineStr">
@@ -5603,7 +6321,7 @@
       <c r="E6" s="28" t="n">
         <v>133.79</v>
       </c>
-      <c r="F6" s="41" t="n">
+      <c r="F6" s="48" t="n">
         <v>-1.101424241474859</v>
       </c>
       <c r="G6" s="28" t="n">
@@ -5645,41 +6363,112 @@
         <f>IFERROR(P6/E6-1,"")</f>
         <v/>
       </c>
-      <c r="R6" s="7" t="inlineStr">
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="79" t="inlineStr">
+        <is>
+          <t>PORTFOLIO TOTALS</t>
+        </is>
+      </c>
+      <c r="H8" s="80">
+        <f>SUM(H5:H6)</f>
+        <v/>
+      </c>
+      <c r="I8" s="80">
+        <f>SUM(I5:I6)</f>
+        <v/>
+      </c>
+      <c r="J8" s="80">
+        <f>SUM(J5:J6)</f>
+        <v/>
+      </c>
+      <c r="K8" s="81">
+        <f>IFERROR(J8/H8,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="82" t="inlineStr">
+        <is>
+          <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="40" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B11" s="40" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C11" s="41" t="inlineStr">
+        <is>
+          <t>Notes / Thesis</t>
+        </is>
+      </c>
+      <c r="D11" s="42" t="n"/>
+      <c r="E11" s="42" t="n"/>
+      <c r="F11" s="42" t="n"/>
+      <c r="G11" s="42" t="n"/>
+      <c r="H11" s="42" t="n"/>
+      <c r="I11" s="42" t="n"/>
+      <c r="J11" s="42" t="n"/>
+      <c r="K11" s="42" t="n"/>
+      <c r="L11" s="42" t="n"/>
+      <c r="M11" s="42" t="n"/>
+      <c r="N11" s="42" t="n"/>
+      <c r="O11" s="42" t="n"/>
+      <c r="P11" s="42" t="n"/>
+      <c r="Q11" s="43" t="n"/>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>NBIS</t>
+        </is>
+      </c>
+      <c r="B12" s="44" t="inlineStr">
+        <is>
+          <t>Nebius Group</t>
+        </is>
+      </c>
+      <c r="C12" s="44" t="inlineStr">
+        <is>
+          <t>Leading Neocloud with multiple revenue streams (Clickhouse, AV Ride). Modern Amazon/Google style company. Could become a future Hyperscaler.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="27" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="B13" s="45" t="inlineStr">
+        <is>
+          <t>Palantir Technologies</t>
+        </is>
+      </c>
+      <c r="C13" s="45" t="inlineStr">
         <is>
           <t>Integral to the entire government AI stack. Not going anywhere. AI Software outlier outside the data center trade.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="67" t="inlineStr">
-        <is>
-          <t>PORTFOLIO TOTALS</t>
-        </is>
-      </c>
-      <c r="H8" s="68">
-        <f>SUM(H5:H6)</f>
-        <v/>
-      </c>
-      <c r="I8" s="68">
-        <f>SUM(I5:I6)</f>
-        <v/>
-      </c>
-      <c r="J8" s="68">
-        <f>SUM(J5:J6)</f>
-        <v/>
-      </c>
-      <c r="K8" s="69">
-        <f>IFERROR(J8/H8,"")</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="8">
+    <mergeCell ref="A3:Q3"/>
     <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A3:R3"/>
-    <mergeCell ref="A2:R2"/>
-    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="C11:Q11"/>
+    <mergeCell ref="C13:Q13"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A10:Q10"/>
+    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="C12:Q12"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J6">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -5708,7 +6497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5728,11 +6517,10 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="50" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="70" t="inlineStr">
+      <c r="A1" s="83" t="inlineStr">
         <is>
           <t>🛡️ Defense &amp; Drones</t>
         </is>
@@ -5748,112 +6536,107 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:14 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="71" t="inlineStr">
+      <c r="A4" s="84" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="71" t="inlineStr">
+      <c r="B4" s="84" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="71" t="inlineStr">
+      <c r="C4" s="84" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="71" t="inlineStr">
+      <c r="D4" s="84" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="71" t="inlineStr">
+      <c r="E4" s="84" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="71" t="inlineStr">
+      <c r="F4" s="84" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="71" t="inlineStr">
+      <c r="G4" s="84" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="71" t="inlineStr">
+      <c r="H4" s="84" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="71" t="inlineStr">
+      <c r="I4" s="84" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="71" t="inlineStr">
+      <c r="J4" s="84" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="71" t="inlineStr">
+      <c r="K4" s="84" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="71" t="inlineStr">
+      <c r="L4" s="84" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="71" t="inlineStr">
+      <c r="M4" s="84" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="71" t="inlineStr">
+      <c r="N4" s="84" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="71" t="inlineStr">
+      <c r="O4" s="84" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="71" t="inlineStr">
+      <c r="P4" s="84" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="71" t="inlineStr">
+      <c r="Q4" s="84" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
         </is>
       </c>
-      <c r="R4" s="71" t="inlineStr">
-        <is>
-          <t>Investment Thesis / Notes</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
@@ -5921,41 +6704,94 @@
         <f>IFERROR(P5/E5-1,"")</f>
         <v/>
       </c>
-      <c r="R5" s="10" t="inlineStr">
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="85" t="inlineStr">
+        <is>
+          <t>PORTFOLIO TOTALS</t>
+        </is>
+      </c>
+      <c r="H7" s="86">
+        <f>SUM(H5:H5)</f>
+        <v/>
+      </c>
+      <c r="I7" s="86">
+        <f>SUM(I5:I5)</f>
+        <v/>
+      </c>
+      <c r="J7" s="86">
+        <f>SUM(J5:J5)</f>
+        <v/>
+      </c>
+      <c r="K7" s="87">
+        <f>IFERROR(J7/H7,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="88" t="inlineStr">
+        <is>
+          <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="40" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B10" s="40" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C10" s="41" t="inlineStr">
+        <is>
+          <t>Notes / Thesis</t>
+        </is>
+      </c>
+      <c r="D10" s="42" t="n"/>
+      <c r="E10" s="42" t="n"/>
+      <c r="F10" s="42" t="n"/>
+      <c r="G10" s="42" t="n"/>
+      <c r="H10" s="42" t="n"/>
+      <c r="I10" s="42" t="n"/>
+      <c r="J10" s="42" t="n"/>
+      <c r="K10" s="42" t="n"/>
+      <c r="L10" s="42" t="n"/>
+      <c r="M10" s="42" t="n"/>
+      <c r="N10" s="42" t="n"/>
+      <c r="O10" s="42" t="n"/>
+      <c r="P10" s="42" t="n"/>
+      <c r="Q10" s="43" t="n"/>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>ONDS</t>
+        </is>
+      </c>
+      <c r="B11" s="44" t="inlineStr">
+        <is>
+          <t>Ondas Holdings</t>
+        </is>
+      </c>
+      <c r="C11" s="44" t="inlineStr">
         <is>
           <t>$1.5T defense budget, $56B to drones/counter-drones via DAWG Program. Best chance to scale after March 2026 acquisitions &amp; partnerships. Very speculative.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="72" t="inlineStr">
-        <is>
-          <t>PORTFOLIO TOTALS</t>
-        </is>
-      </c>
-      <c r="H7" s="73">
-        <f>SUM(H5:H5)</f>
-        <v/>
-      </c>
-      <c r="I7" s="73">
-        <f>SUM(I5:I5)</f>
-        <v/>
-      </c>
-      <c r="J7" s="73">
-        <f>SUM(J5:J5)</f>
-        <v/>
-      </c>
-      <c r="K7" s="74">
-        <f>IFERROR(J7/H7,"")</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A3:R3"/>
-    <mergeCell ref="A2:R2"/>
-    <mergeCell ref="A1:R1"/>
+  <mergeCells count="7">
+    <mergeCell ref="A9:Q9"/>
+    <mergeCell ref="A3:Q3"/>
+    <mergeCell ref="C10:Q10"/>
+    <mergeCell ref="C11:Q11"/>
+    <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="J5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">

</xml_diff>

<commit_message>
Adjust cell heights to fully display all notes
Dynamically calculate and set row heights in `scripts/generate_financial_tracker.py` to accommodate varying lengths of stock notes, replacing fixed heights.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 9f7d38a1-7a28-4675-865b-9257b35f4ceb
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1099,7 +1099,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
         </is>
       </c>
     </row>
@@ -1586,7 +1586,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
         </is>
       </c>
     </row>
@@ -1816,7 +1816,7 @@
       <c r="P10" s="42" t="n"/>
       <c r="Q10" s="43" t="n"/>
     </row>
-    <row r="11" ht="48" customHeight="1">
+    <row r="11" ht="40" customHeight="1">
       <c r="A11" s="33" t="inlineStr">
         <is>
           <t>RKLB</t>
@@ -1909,7 +1909,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       <c r="P11" s="42" t="n"/>
       <c r="Q11" s="43" t="n"/>
     </row>
-    <row r="12" ht="48" customHeight="1">
+    <row r="12" ht="40" customHeight="1">
       <c r="A12" s="33" t="inlineStr">
         <is>
           <t>RBRK</t>
@@ -2223,7 +2223,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="48" customHeight="1">
+    <row r="13" ht="40" customHeight="1">
       <c r="A13" s="27" t="inlineStr">
         <is>
           <t>NVO</t>
@@ -2575,7 +2575,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
         </is>
       </c>
     </row>
@@ -2939,7 +2939,7 @@
       <c r="P12" s="42" t="n"/>
       <c r="Q12" s="43" t="n"/>
     </row>
-    <row r="13" ht="48" customHeight="1">
+    <row r="13" ht="40" customHeight="1">
       <c r="A13" s="33" t="inlineStr">
         <is>
           <t>IONQ</t>
@@ -2956,7 +2956,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="48" customHeight="1">
+    <row r="14" ht="40" customHeight="1">
       <c r="A14" s="27" t="inlineStr">
         <is>
           <t>RGTI</t>
@@ -2973,7 +2973,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="48" customHeight="1">
+    <row r="15" ht="40" customHeight="1">
       <c r="A15" s="33" t="inlineStr">
         <is>
           <t>QBTS</t>
@@ -3068,7 +3068,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
         </is>
       </c>
     </row>
@@ -3633,7 +3633,7 @@
       <c r="P15" s="42" t="n"/>
       <c r="Q15" s="43" t="n"/>
     </row>
-    <row r="16" ht="48" customHeight="1">
+    <row r="16" ht="40" customHeight="1">
       <c r="A16" s="33" t="inlineStr">
         <is>
           <t>NVDA</t>
@@ -3650,7 +3650,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="48" customHeight="1">
+    <row r="17" ht="40" customHeight="1">
       <c r="A17" s="27" t="inlineStr">
         <is>
           <t>AVGO</t>
@@ -3667,7 +3667,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="48" customHeight="1">
+    <row r="18" ht="40" customHeight="1">
       <c r="A18" s="33" t="inlineStr">
         <is>
           <t>LRCX</t>
@@ -3684,7 +3684,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="48" customHeight="1">
+    <row r="19" ht="40" customHeight="1">
       <c r="A19" s="27" t="inlineStr">
         <is>
           <t>AMD</t>
@@ -3701,7 +3701,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="48" customHeight="1">
+    <row r="20" ht="40" customHeight="1">
       <c r="A20" s="33" t="inlineStr">
         <is>
           <t>INTC</t>
@@ -3718,7 +3718,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="48" customHeight="1">
+    <row r="21" ht="40" customHeight="1">
       <c r="A21" s="27" t="inlineStr">
         <is>
           <t>ARM</t>
@@ -3816,7 +3816,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
         </is>
       </c>
     </row>
@@ -4448,7 +4448,7 @@
       <c r="P16" s="42" t="n"/>
       <c r="Q16" s="43" t="n"/>
     </row>
-    <row r="17" ht="48" customHeight="1">
+    <row r="17" ht="40" customHeight="1">
       <c r="A17" s="33" t="inlineStr">
         <is>
           <t>NVTS</t>
@@ -4465,7 +4465,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="48" customHeight="1">
+    <row r="18" ht="40" customHeight="1">
       <c r="A18" s="27" t="inlineStr">
         <is>
           <t>AEHR</t>
@@ -4482,7 +4482,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="48" customHeight="1">
+    <row r="19" ht="40" customHeight="1">
       <c r="A19" s="33" t="inlineStr">
         <is>
           <t>CRDO</t>
@@ -4499,7 +4499,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="48" customHeight="1">
+    <row r="20" ht="40" customHeight="1">
       <c r="A20" s="27" t="inlineStr">
         <is>
           <t>ALGM</t>
@@ -4516,7 +4516,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="48" customHeight="1">
+    <row r="21" ht="40" customHeight="1">
       <c r="A21" s="33" t="inlineStr">
         <is>
           <t>HIMX</t>
@@ -4533,7 +4533,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="48" customHeight="1">
+    <row r="22" ht="40" customHeight="1">
       <c r="A22" s="27" t="inlineStr">
         <is>
           <t>MTSI</t>
@@ -4550,7 +4550,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="48" customHeight="1">
+    <row r="23" ht="40" customHeight="1">
       <c r="A23" s="33" t="inlineStr">
         <is>
           <t>AEVA</t>
@@ -4649,7 +4649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
         </is>
       </c>
     </row>
@@ -4879,7 +4879,7 @@
       <c r="P10" s="42" t="n"/>
       <c r="Q10" s="43" t="n"/>
     </row>
-    <row r="11" ht="48" customHeight="1">
+    <row r="11" ht="40" customHeight="1">
       <c r="A11" s="33" t="inlineStr">
         <is>
           <t>LITE</t>
@@ -4972,7 +4972,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
         </is>
       </c>
     </row>
@@ -5403,7 +5403,7 @@
       <c r="P13" s="42" t="n"/>
       <c r="Q13" s="43" t="n"/>
     </row>
-    <row r="14" ht="48" customHeight="1">
+    <row r="14" ht="40" customHeight="1">
       <c r="A14" s="33" t="inlineStr">
         <is>
           <t>CAT</t>
@@ -5420,7 +5420,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="48" customHeight="1">
+    <row r="15" ht="40" customHeight="1">
       <c r="A15" s="27" t="inlineStr">
         <is>
           <t>FIX</t>
@@ -5437,7 +5437,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="48" customHeight="1">
+    <row r="16" ht="40" customHeight="1">
       <c r="A16" s="33" t="inlineStr">
         <is>
           <t>POWL</t>
@@ -5454,7 +5454,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="48" customHeight="1">
+    <row r="17" ht="40" customHeight="1">
       <c r="A17" s="27" t="inlineStr">
         <is>
           <t>VRT</t>
@@ -5550,7 +5550,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
         </is>
       </c>
     </row>
@@ -5981,7 +5981,7 @@
       <c r="P13" s="42" t="n"/>
       <c r="Q13" s="43" t="n"/>
     </row>
-    <row r="14" ht="48" customHeight="1">
+    <row r="14" ht="40" customHeight="1">
       <c r="A14" s="33" t="inlineStr">
         <is>
           <t>GEV</t>
@@ -5998,7 +5998,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="48" customHeight="1">
+    <row r="15" ht="40" customHeight="1">
       <c r="A15" s="27" t="inlineStr">
         <is>
           <t>PWR</t>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="48" customHeight="1">
+    <row r="16" ht="40" customHeight="1">
       <c r="A16" s="33" t="inlineStr">
         <is>
           <t>BE</t>
@@ -6032,7 +6032,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="48" customHeight="1">
+    <row r="17" ht="40" customHeight="1">
       <c r="A17" s="27" t="inlineStr">
         <is>
           <t>OKLO</t>
@@ -6128,7 +6128,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
         </is>
       </c>
     </row>
@@ -6425,7 +6425,7 @@
       <c r="P11" s="42" t="n"/>
       <c r="Q11" s="43" t="n"/>
     </row>
-    <row r="12" ht="48" customHeight="1">
+    <row r="12" ht="40" customHeight="1">
       <c r="A12" s="33" t="inlineStr">
         <is>
           <t>NBIS</t>
@@ -6442,7 +6442,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="48" customHeight="1">
+    <row r="13" ht="40" customHeight="1">
       <c r="A13" s="27" t="inlineStr">
         <is>
           <t>PLTR</t>
@@ -6536,7 +6536,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:17 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
         </is>
       </c>
     </row>
@@ -6766,7 +6766,7 @@
       <c r="P10" s="42" t="n"/>
       <c r="Q10" s="43" t="n"/>
     </row>
-    <row r="11" ht="48" customHeight="1">
+    <row r="11" ht="40" customHeight="1">
       <c r="A11" s="33" t="inlineStr">
         <is>
           <t>ONDS</t>

</xml_diff>

<commit_message>
Restructure notes section to span entire row width
Modify the Python script to make the notes section for each stock span all columns, resolving text truncation issues in merged cells.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 1e64165d-ed2e-4a21-9606-4c849060239a
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -286,7 +286,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -323,54 +323,32 @@
       </bottom>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="thin">
+      <left style="medium">
+        <color rgb="00AAAAAA"/>
+      </left>
+      <right style="medium">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="medium">
         <color rgb="00AAAAAA"/>
       </top>
-      <bottom/>
-      <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
+      <left style="medium">
+        <color rgb="00AAAAAA"/>
+      </left>
+      <right style="medium">
         <color rgb="00AAAAAA"/>
       </right>
-      <top style="thin">
-        <color rgb="00AAAAAA"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00AAAAAA"/>
-      </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color rgb="00AAAAAA"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00AAAAAA"/>
-      </right>
-      <top style="thin">
-        <color rgb="00AAAAAA"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00AAAAAA"/>
-      </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -487,18 +465,13 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1099,7 +1072,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
         </is>
       </c>
     </row>
@@ -1570,7 +1543,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="89" t="inlineStr">
+      <c r="A1" s="86" t="inlineStr">
         <is>
           <t>🚀 Space Economy</t>
         </is>
@@ -1586,102 +1559,102 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="90" t="inlineStr">
+      <c r="A4" s="87" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="90" t="inlineStr">
+      <c r="B4" s="87" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="90" t="inlineStr">
+      <c r="C4" s="87" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="90" t="inlineStr">
+      <c r="D4" s="87" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="90" t="inlineStr">
+      <c r="E4" s="87" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="90" t="inlineStr">
+      <c r="F4" s="87" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="90" t="inlineStr">
+      <c r="G4" s="87" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="90" t="inlineStr">
+      <c r="H4" s="87" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="90" t="inlineStr">
+      <c r="I4" s="87" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="90" t="inlineStr">
+      <c r="J4" s="87" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="90" t="inlineStr">
+      <c r="K4" s="87" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="90" t="inlineStr">
+      <c r="L4" s="87" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="90" t="inlineStr">
+      <c r="M4" s="87" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="90" t="inlineStr">
+      <c r="N4" s="87" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="90" t="inlineStr">
+      <c r="O4" s="87" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="90" t="inlineStr">
+      <c r="P4" s="87" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="90" t="inlineStr">
+      <c r="Q4" s="87" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
@@ -1756,78 +1729,44 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="91" t="inlineStr">
+      <c r="A7" s="88" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H7" s="92">
+      <c r="H7" s="89">
         <f>SUM(H5:H5)</f>
         <v/>
       </c>
-      <c r="I7" s="92">
+      <c r="I7" s="89">
         <f>SUM(I5:I5)</f>
         <v/>
       </c>
-      <c r="J7" s="92">
+      <c r="J7" s="89">
         <f>SUM(J5:J5)</f>
         <v/>
       </c>
-      <c r="K7" s="93">
+      <c r="K7" s="90">
         <f>IFERROR(J7/H7,"")</f>
         <v/>
       </c>
     </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="94" t="inlineStr">
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="91" t="inlineStr">
         <is>
           <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="16" customHeight="1">
+    <row r="10" ht="18" customHeight="1">
       <c r="A10" s="40" t="inlineStr">
         <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B10" s="40" t="inlineStr">
-        <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="C10" s="41" t="inlineStr">
-        <is>
-          <t>Notes / Thesis</t>
-        </is>
-      </c>
-      <c r="D10" s="42" t="n"/>
-      <c r="E10" s="42" t="n"/>
-      <c r="F10" s="42" t="n"/>
-      <c r="G10" s="42" t="n"/>
-      <c r="H10" s="42" t="n"/>
-      <c r="I10" s="42" t="n"/>
-      <c r="J10" s="42" t="n"/>
-      <c r="K10" s="42" t="n"/>
-      <c r="L10" s="42" t="n"/>
-      <c r="M10" s="42" t="n"/>
-      <c r="N10" s="42" t="n"/>
-      <c r="O10" s="42" t="n"/>
-      <c r="P10" s="42" t="n"/>
-      <c r="Q10" s="43" t="n"/>
-    </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="33" t="inlineStr">
-        <is>
-          <t>RKLB</t>
-        </is>
-      </c>
-      <c r="B11" s="44" t="inlineStr">
-        <is>
-          <t>Rocket Lab USA</t>
-        </is>
-      </c>
-      <c r="C11" s="44" t="inlineStr">
+          <t xml:space="preserve">  RKLB  —  Rocket Lab USA  |  Risk: High</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="52" customHeight="1">
+      <c r="A11" s="41" t="inlineStr">
         <is>
           <t>Huge future TAM over next decade+. Speculative but massive upside. Brilliant CEO. Near-term catalyst: SpaceX IPO in June.</t>
         </is>
@@ -1837,10 +1776,10 @@
   <mergeCells count="7">
     <mergeCell ref="A9:Q9"/>
     <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="C10:Q10"/>
-    <mergeCell ref="C11:Q11"/>
     <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A10:Q10"/>
     <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A11:Q11"/>
     <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="J5">
@@ -1870,7 +1809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1893,7 +1832,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="95" t="inlineStr">
+      <c r="A1" s="92" t="inlineStr">
         <is>
           <t>🔭 Long Term Watchlist</t>
         </is>
@@ -1909,102 +1848,102 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="96" t="inlineStr">
+      <c r="A4" s="93" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="96" t="inlineStr">
+      <c r="B4" s="93" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="96" t="inlineStr">
+      <c r="C4" s="93" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="96" t="inlineStr">
+      <c r="D4" s="93" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="96" t="inlineStr">
+      <c r="E4" s="93" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="96" t="inlineStr">
+      <c r="F4" s="93" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="96" t="inlineStr">
+      <c r="G4" s="93" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="96" t="inlineStr">
+      <c r="H4" s="93" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="96" t="inlineStr">
+      <c r="I4" s="93" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="96" t="inlineStr">
+      <c r="J4" s="93" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="96" t="inlineStr">
+      <c r="K4" s="93" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="96" t="inlineStr">
+      <c r="L4" s="93" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="96" t="inlineStr">
+      <c r="M4" s="93" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="96" t="inlineStr">
+      <c r="N4" s="93" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="96" t="inlineStr">
+      <c r="O4" s="93" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="96" t="inlineStr">
+      <c r="P4" s="93" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="96" t="inlineStr">
+      <c r="Q4" s="93" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
@@ -2146,110 +2085,74 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="97" t="inlineStr">
+      <c r="A8" s="94" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H8" s="98">
+      <c r="H8" s="95">
         <f>SUM(H5:H6)</f>
         <v/>
       </c>
-      <c r="I8" s="98">
+      <c r="I8" s="95">
         <f>SUM(I5:I6)</f>
         <v/>
       </c>
-      <c r="J8" s="98">
+      <c r="J8" s="95">
         <f>SUM(J5:J6)</f>
         <v/>
       </c>
-      <c r="K8" s="99">
+      <c r="K8" s="96">
         <f>IFERROR(J8/H8,"")</f>
         <v/>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="100" t="inlineStr">
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="97" t="inlineStr">
         <is>
           <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="16" customHeight="1">
+    <row r="11" ht="18" customHeight="1">
       <c r="A11" s="40" t="inlineStr">
         <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B11" s="40" t="inlineStr">
-        <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="C11" s="41" t="inlineStr">
-        <is>
-          <t>Notes / Thesis</t>
-        </is>
-      </c>
-      <c r="D11" s="42" t="n"/>
-      <c r="E11" s="42" t="n"/>
-      <c r="F11" s="42" t="n"/>
-      <c r="G11" s="42" t="n"/>
-      <c r="H11" s="42" t="n"/>
-      <c r="I11" s="42" t="n"/>
-      <c r="J11" s="42" t="n"/>
-      <c r="K11" s="42" t="n"/>
-      <c r="L11" s="42" t="n"/>
-      <c r="M11" s="42" t="n"/>
-      <c r="N11" s="42" t="n"/>
-      <c r="O11" s="42" t="n"/>
-      <c r="P11" s="42" t="n"/>
-      <c r="Q11" s="43" t="n"/>
-    </row>
-    <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="33" t="inlineStr">
-        <is>
-          <t>RBRK</t>
-        </is>
-      </c>
-      <c r="B12" s="44" t="inlineStr">
-        <is>
-          <t>Rubrik Inc</t>
-        </is>
-      </c>
-      <c r="C12" s="44" t="inlineStr">
+          <t xml:space="preserve">  RBRK  —  Rubrik Inc  |  Risk: Med-High</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="52" customHeight="1">
+      <c r="A12" s="41" t="inlineStr">
         <is>
           <t>Long term investment research candidate.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="27" t="inlineStr">
-        <is>
-          <t>NVO</t>
-        </is>
-      </c>
-      <c r="B13" s="45" t="inlineStr">
-        <is>
-          <t>Novo Nordisk</t>
-        </is>
-      </c>
-      <c r="C13" s="45" t="inlineStr">
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NVO  —  Novo Nordisk  |  Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="52" customHeight="1">
+      <c r="A14" s="42" t="inlineStr">
         <is>
           <t>Long term investment research candidate.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
+    <mergeCell ref="A14:Q14"/>
     <mergeCell ref="A3:Q3"/>
     <mergeCell ref="A8:G8"/>
-    <mergeCell ref="C11:Q11"/>
-    <mergeCell ref="C13:Q13"/>
+    <mergeCell ref="A12:Q12"/>
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A10:Q10"/>
+    <mergeCell ref="A11:Q11"/>
     <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="C12:Q12"/>
+    <mergeCell ref="A13:Q13"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J6">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -2286,14 +2189,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="101" t="inlineStr">
+      <c r="A1" s="98" t="inlineStr">
         <is>
           <t>📝 RESEARCH NOTES &amp; INVESTMENT THESIS</t>
         </is>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1">
-      <c r="A2" s="102" t="inlineStr">
+      <c r="A2" s="99" t="inlineStr">
         <is>
           <t>401k To-Do</t>
         </is>
@@ -2306,7 +2209,7 @@
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="103" t="inlineStr">
+      <c r="A3" s="100" t="inlineStr">
         <is>
           <t>Savings Account</t>
         </is>
@@ -2318,7 +2221,7 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="102" t="inlineStr">
+      <c r="A4" s="99" t="inlineStr">
         <is>
           <t>Research Tools</t>
         </is>
@@ -2330,7 +2233,7 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="103" t="inlineStr">
+      <c r="A5" s="100" t="inlineStr">
         <is>
           <t>Quantum Thesis</t>
         </is>
@@ -2342,7 +2245,7 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="102" t="inlineStr">
+      <c r="A6" s="99" t="inlineStr">
         <is>
           <t>NVTS</t>
         </is>
@@ -2354,7 +2257,7 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="103" t="inlineStr">
+      <c r="A7" s="100" t="inlineStr">
         <is>
           <t>AEHR</t>
         </is>
@@ -2366,7 +2269,7 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="102" t="inlineStr">
+      <c r="A8" s="99" t="inlineStr">
         <is>
           <t>CRDO</t>
         </is>
@@ -2378,7 +2281,7 @@
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="103" t="inlineStr">
+      <c r="A9" s="100" t="inlineStr">
         <is>
           <t>ALGM</t>
         </is>
@@ -2390,7 +2293,7 @@
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="102" t="inlineStr">
+      <c r="A10" s="99" t="inlineStr">
         <is>
           <t>HIMX</t>
         </is>
@@ -2402,7 +2305,7 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="103" t="inlineStr">
+      <c r="A11" s="100" t="inlineStr">
         <is>
           <t>MTSI</t>
         </is>
@@ -2414,7 +2317,7 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="102" t="inlineStr">
+      <c r="A12" s="99" t="inlineStr">
         <is>
           <t>AEVA</t>
         </is>
@@ -2426,7 +2329,7 @@
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="103" t="inlineStr">
+      <c r="A13" s="100" t="inlineStr">
         <is>
           <t>AI Infrastructure</t>
         </is>
@@ -2438,7 +2341,7 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="102" t="inlineStr">
+      <c r="A14" s="99" t="inlineStr">
         <is>
           <t>LITE</t>
         </is>
@@ -2450,7 +2353,7 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="103" t="inlineStr">
+      <c r="A15" s="100" t="inlineStr">
         <is>
           <t>OKLO</t>
         </is>
@@ -2462,7 +2365,7 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="102" t="inlineStr">
+      <c r="A16" s="99" t="inlineStr">
         <is>
           <t>NBIS</t>
         </is>
@@ -2474,7 +2377,7 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="103" t="inlineStr">
+      <c r="A17" s="100" t="inlineStr">
         <is>
           <t>PLTR</t>
         </is>
@@ -2486,7 +2389,7 @@
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="102" t="inlineStr">
+      <c r="A18" s="99" t="inlineStr">
         <is>
           <t>ONDS</t>
         </is>
@@ -2498,7 +2401,7 @@
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="103" t="inlineStr">
+      <c r="A19" s="100" t="inlineStr">
         <is>
           <t>RKLB</t>
         </is>
@@ -2510,7 +2413,7 @@
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="102" t="inlineStr">
+      <c r="A20" s="99" t="inlineStr">
         <is>
           <t>Recommended Portfolio</t>
         </is>
@@ -2536,7 +2439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2575,7 +2478,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
         </is>
       </c>
     </row>
@@ -2901,106 +2804,68 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1">
+    <row r="11" ht="22" customHeight="1">
       <c r="A11" s="39" t="inlineStr">
         <is>
           <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="16" customHeight="1">
+    <row r="12" ht="18" customHeight="1">
       <c r="A12" s="40" t="inlineStr">
         <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B12" s="40" t="inlineStr">
-        <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="C12" s="41" t="inlineStr">
-        <is>
-          <t>Notes / Thesis</t>
-        </is>
-      </c>
-      <c r="D12" s="42" t="n"/>
-      <c r="E12" s="42" t="n"/>
-      <c r="F12" s="42" t="n"/>
-      <c r="G12" s="42" t="n"/>
-      <c r="H12" s="42" t="n"/>
-      <c r="I12" s="42" t="n"/>
-      <c r="J12" s="42" t="n"/>
-      <c r="K12" s="42" t="n"/>
-      <c r="L12" s="42" t="n"/>
-      <c r="M12" s="42" t="n"/>
-      <c r="N12" s="42" t="n"/>
-      <c r="O12" s="42" t="n"/>
-      <c r="P12" s="42" t="n"/>
-      <c r="Q12" s="43" t="n"/>
-    </row>
-    <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="33" t="inlineStr">
-        <is>
-          <t>IONQ</t>
-        </is>
-      </c>
-      <c r="B13" s="44" t="inlineStr">
-        <is>
-          <t>IonQ Inc</t>
-        </is>
-      </c>
-      <c r="C13" s="44" t="inlineStr">
+          <t xml:space="preserve">  IONQ  —  IonQ Inc  |  Risk: Very High</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="52" customHeight="1">
+      <c r="A13" s="41" t="inlineStr">
         <is>
           <t>Next quantum run candidate. Easy 10× within 2 years potential.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="27" t="inlineStr">
-        <is>
-          <t>RGTI</t>
-        </is>
-      </c>
-      <c r="B14" s="45" t="inlineStr">
-        <is>
-          <t>Rigetti Computing</t>
-        </is>
-      </c>
-      <c r="C14" s="45" t="inlineStr">
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  RGTI  —  Rigetti Computing  |  Risk: Very High</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="52" customHeight="1">
+      <c r="A15" s="42" t="inlineStr">
         <is>
           <t>Next quantum run candidate. Easy 10× within 2 years potential.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="33" t="inlineStr">
-        <is>
-          <t>QBTS</t>
-        </is>
-      </c>
-      <c r="B15" s="44" t="inlineStr">
-        <is>
-          <t>D-Wave Quantum</t>
-        </is>
-      </c>
-      <c r="C15" s="44" t="inlineStr">
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  QBTS  —  D-Wave Quantum  |  Risk: Very High</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="52" customHeight="1">
+      <c r="A17" s="41" t="inlineStr">
         <is>
           <t>Next quantum run candidate. Easy 10× within 2 years potential.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="C15:Q15"/>
+  <mergeCells count="11">
+    <mergeCell ref="A14:Q14"/>
+    <mergeCell ref="A17:Q17"/>
     <mergeCell ref="A9:G9"/>
     <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="C14:Q14"/>
-    <mergeCell ref="C13:Q13"/>
+    <mergeCell ref="A12:Q12"/>
     <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A16:Q16"/>
+    <mergeCell ref="A15:Q15"/>
     <mergeCell ref="A11:Q11"/>
     <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="C12:Q12"/>
+    <mergeCell ref="A13:Q13"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J7">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -3029,7 +2894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q21"/>
+  <dimension ref="A1:Q26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3052,7 +2917,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="46" t="inlineStr">
+      <c r="A1" s="43" t="inlineStr">
         <is>
           <t>🖥️ Semiconductors &amp; Compute</t>
         </is>
@@ -3068,102 +2933,102 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="47" t="inlineStr">
+      <c r="A4" s="44" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="47" t="inlineStr">
+      <c r="B4" s="44" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="47" t="inlineStr">
+      <c r="C4" s="44" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="47" t="inlineStr">
+      <c r="D4" s="44" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="47" t="inlineStr">
+      <c r="E4" s="44" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="47" t="inlineStr">
+      <c r="F4" s="44" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="47" t="inlineStr">
+      <c r="G4" s="44" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="47" t="inlineStr">
+      <c r="H4" s="44" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="47" t="inlineStr">
+      <c r="I4" s="44" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="47" t="inlineStr">
+      <c r="J4" s="44" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="47" t="inlineStr">
+      <c r="K4" s="44" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="47" t="inlineStr">
+      <c r="L4" s="44" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="47" t="inlineStr">
+      <c r="M4" s="44" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="47" t="inlineStr">
+      <c r="N4" s="44" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="47" t="inlineStr">
+      <c r="O4" s="44" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="47" t="inlineStr">
+      <c r="P4" s="44" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="47" t="inlineStr">
+      <c r="Q4" s="44" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
@@ -3261,7 +3126,7 @@
       <c r="E6" s="28" t="n">
         <v>425.44</v>
       </c>
-      <c r="F6" s="48" t="n">
+      <c r="F6" s="45" t="n">
         <v>-1.518517953378183</v>
       </c>
       <c r="G6" s="28" t="n">
@@ -3462,7 +3327,7 @@
       <c r="E9" s="28" t="n">
         <v>113.01</v>
       </c>
-      <c r="F9" s="48" t="n">
+      <c r="F9" s="45" t="n">
         <v>-0.2999540042077861</v>
       </c>
       <c r="G9" s="28" t="n">
@@ -3573,182 +3438,138 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="49" t="inlineStr">
+      <c r="A12" s="46" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H12" s="50">
+      <c r="H12" s="47">
         <f>SUM(H5:H10)</f>
         <v/>
       </c>
-      <c r="I12" s="50">
+      <c r="I12" s="47">
         <f>SUM(I5:I10)</f>
         <v/>
       </c>
-      <c r="J12" s="50">
+      <c r="J12" s="47">
         <f>SUM(J5:J10)</f>
         <v/>
       </c>
-      <c r="K12" s="51">
+      <c r="K12" s="48">
         <f>IFERROR(J12/H12,"")</f>
         <v/>
       </c>
     </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="52" t="inlineStr">
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="49" t="inlineStr">
         <is>
           <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="16" customHeight="1">
+    <row r="15" ht="18" customHeight="1">
       <c r="A15" s="40" t="inlineStr">
         <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B15" s="40" t="inlineStr">
-        <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="C15" s="41" t="inlineStr">
-        <is>
-          <t>Notes / Thesis</t>
-        </is>
-      </c>
-      <c r="D15" s="42" t="n"/>
-      <c r="E15" s="42" t="n"/>
-      <c r="F15" s="42" t="n"/>
-      <c r="G15" s="42" t="n"/>
-      <c r="H15" s="42" t="n"/>
-      <c r="I15" s="42" t="n"/>
-      <c r="J15" s="42" t="n"/>
-      <c r="K15" s="42" t="n"/>
-      <c r="L15" s="42" t="n"/>
-      <c r="M15" s="42" t="n"/>
-      <c r="N15" s="42" t="n"/>
-      <c r="O15" s="42" t="n"/>
-      <c r="P15" s="42" t="n"/>
-      <c r="Q15" s="43" t="n"/>
-    </row>
-    <row r="16" ht="40" customHeight="1">
-      <c r="A16" s="33" t="inlineStr">
-        <is>
-          <t>NVDA</t>
-        </is>
-      </c>
-      <c r="B16" s="44" t="inlineStr">
-        <is>
-          <t>NVIDIA Corp</t>
-        </is>
-      </c>
-      <c r="C16" s="44" t="inlineStr">
+          <t xml:space="preserve">  NVDA  —  NVIDIA Corp  |  Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="52" customHeight="1">
+      <c r="A16" s="41" t="inlineStr">
         <is>
           <t>The AI compute king. Stability and steady compounder.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="27" t="inlineStr">
-        <is>
-          <t>AVGO</t>
-        </is>
-      </c>
-      <c r="B17" s="45" t="inlineStr">
-        <is>
-          <t>Broadcom Inc</t>
-        </is>
-      </c>
-      <c r="C17" s="45" t="inlineStr">
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AVGO  —  Broadcom Inc  |  Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="52" customHeight="1">
+      <c r="A18" s="42" t="inlineStr">
         <is>
           <t>Stability and steady compounder.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="40" customHeight="1">
-      <c r="A18" s="33" t="inlineStr">
-        <is>
-          <t>LRCX</t>
-        </is>
-      </c>
-      <c r="B18" s="44" t="inlineStr">
-        <is>
-          <t>Lam Research</t>
-        </is>
-      </c>
-      <c r="C18" s="44" t="inlineStr">
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  LRCX  —  Lam Research  |  Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="52" customHeight="1">
+      <c r="A20" s="41" t="inlineStr">
         <is>
           <t>Stability and steady compounder. DRAM equipment leader.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="40" customHeight="1">
-      <c r="A19" s="27" t="inlineStr">
-        <is>
-          <t>AMD</t>
-        </is>
-      </c>
-      <c r="B19" s="45" t="inlineStr">
-        <is>
-          <t>Advanced Micro Devices</t>
-        </is>
-      </c>
-      <c r="C19" s="45" t="inlineStr">
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AMD  —  Advanced Micro Devices  |  Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="52" customHeight="1">
+      <c r="A22" s="42" t="inlineStr">
         <is>
           <t>CPU maker deep in the AI infrastructure stack.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="40" customHeight="1">
-      <c r="A20" s="33" t="inlineStr">
-        <is>
-          <t>INTC</t>
-        </is>
-      </c>
-      <c r="B20" s="44" t="inlineStr">
-        <is>
-          <t>Intel Corp</t>
-        </is>
-      </c>
-      <c r="C20" s="44" t="inlineStr">
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  INTC  —  Intel Corp  |  Risk: Med-High</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="52" customHeight="1">
+      <c r="A24" s="41" t="inlineStr">
         <is>
           <t>CPU maker in AI infrastructure stack. Turnaround story.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="40" customHeight="1">
-      <c r="A21" s="27" t="inlineStr">
-        <is>
-          <t>ARM</t>
-        </is>
-      </c>
-      <c r="B21" s="45" t="inlineStr">
-        <is>
-          <t>Arm Holdings</t>
-        </is>
-      </c>
-      <c r="C21" s="45" t="inlineStr">
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ARM  —  Arm Holdings  |  Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="52" customHeight="1">
+      <c r="A26" s="42" t="inlineStr">
         <is>
           <t>Architecture behind most AI edge chips. Royalty model.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="17">
     <mergeCell ref="A14:Q14"/>
-    <mergeCell ref="C21:Q21"/>
-    <mergeCell ref="C20:Q20"/>
-    <mergeCell ref="C15:Q15"/>
-    <mergeCell ref="C17:Q17"/>
+    <mergeCell ref="A22:Q22"/>
+    <mergeCell ref="A17:Q17"/>
+    <mergeCell ref="A18:Q18"/>
     <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="C16:Q16"/>
+    <mergeCell ref="A21:Q21"/>
     <mergeCell ref="A12:G12"/>
-    <mergeCell ref="C19:Q19"/>
+    <mergeCell ref="A20:Q20"/>
+    <mergeCell ref="A24:Q24"/>
     <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="C18:Q18"/>
+    <mergeCell ref="A16:Q16"/>
+    <mergeCell ref="A15:Q15"/>
+    <mergeCell ref="A26:Q26"/>
+    <mergeCell ref="A25:Q25"/>
+    <mergeCell ref="A19:Q19"/>
     <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A23:Q23"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J10">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -3777,7 +3598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:Q29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3800,7 +3621,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="53" t="inlineStr">
+      <c r="A1" s="50" t="inlineStr">
         <is>
           <t>⚙️ AI Picks &amp; Shovels</t>
         </is>
@@ -3816,102 +3637,102 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="54" t="inlineStr">
+      <c r="A4" s="51" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="54" t="inlineStr">
+      <c r="B4" s="51" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="54" t="inlineStr">
+      <c r="C4" s="51" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="54" t="inlineStr">
+      <c r="D4" s="51" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="54" t="inlineStr">
+      <c r="E4" s="51" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="54" t="inlineStr">
+      <c r="F4" s="51" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="54" t="inlineStr">
+      <c r="G4" s="51" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="54" t="inlineStr">
+      <c r="H4" s="51" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="54" t="inlineStr">
+      <c r="I4" s="51" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="54" t="inlineStr">
+      <c r="J4" s="51" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="54" t="inlineStr">
+      <c r="K4" s="51" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="54" t="inlineStr">
+      <c r="L4" s="51" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="54" t="inlineStr">
+      <c r="M4" s="51" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="54" t="inlineStr">
+      <c r="N4" s="51" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="54" t="inlineStr">
+      <c r="O4" s="51" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="54" t="inlineStr">
+      <c r="P4" s="51" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="54" t="inlineStr">
+      <c r="Q4" s="51" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
@@ -4076,7 +3897,7 @@
       <c r="E7" s="28" t="n">
         <v>198.29</v>
       </c>
-      <c r="F7" s="48" t="n">
+      <c r="F7" s="45" t="n">
         <v>-0.1057968331824622</v>
       </c>
       <c r="G7" s="28" t="n">
@@ -4210,7 +4031,7 @@
       <c r="E9" s="28" t="n">
         <v>12.33</v>
       </c>
-      <c r="F9" s="48" t="n">
+      <c r="F9" s="45" t="n">
         <v>-0.2830576327856492</v>
       </c>
       <c r="G9" s="28" t="n">
@@ -4388,200 +4209,154 @@
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="55" t="inlineStr">
+      <c r="A13" s="52" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H13" s="56">
+      <c r="H13" s="53">
         <f>SUM(H5:H11)</f>
         <v/>
       </c>
-      <c r="I13" s="56">
+      <c r="I13" s="53">
         <f>SUM(I5:I11)</f>
         <v/>
       </c>
-      <c r="J13" s="56">
+      <c r="J13" s="53">
         <f>SUM(J5:J11)</f>
         <v/>
       </c>
-      <c r="K13" s="57">
+      <c r="K13" s="54">
         <f>IFERROR(J13/H13,"")</f>
         <v/>
       </c>
     </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="58" t="inlineStr">
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="55" t="inlineStr">
         <is>
           <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="16" customHeight="1">
+    <row r="16" ht="18" customHeight="1">
       <c r="A16" s="40" t="inlineStr">
         <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B16" s="40" t="inlineStr">
-        <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="C16" s="41" t="inlineStr">
-        <is>
-          <t>Notes / Thesis</t>
-        </is>
-      </c>
-      <c r="D16" s="42" t="n"/>
-      <c r="E16" s="42" t="n"/>
-      <c r="F16" s="42" t="n"/>
-      <c r="G16" s="42" t="n"/>
-      <c r="H16" s="42" t="n"/>
-      <c r="I16" s="42" t="n"/>
-      <c r="J16" s="42" t="n"/>
-      <c r="K16" s="42" t="n"/>
-      <c r="L16" s="42" t="n"/>
-      <c r="M16" s="42" t="n"/>
-      <c r="N16" s="42" t="n"/>
-      <c r="O16" s="42" t="n"/>
-      <c r="P16" s="42" t="n"/>
-      <c r="Q16" s="43" t="n"/>
-    </row>
-    <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="33" t="inlineStr">
-        <is>
-          <t>NVTS</t>
-        </is>
-      </c>
-      <c r="B17" s="44" t="inlineStr">
-        <is>
-          <t>Navitas Semiconductor</t>
-        </is>
-      </c>
-      <c r="C17" s="44" t="inlineStr">
+          <t xml:space="preserve">  NVTS  —  Navitas Semiconductor  |  Risk: High</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="52" customHeight="1">
+      <c r="A17" s="41" t="inlineStr">
         <is>
           <t>AI data centers need radically more efficient power delivery. Picks-and-shovels for compute growth.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="40" customHeight="1">
-      <c r="A18" s="27" t="inlineStr">
-        <is>
-          <t>AEHR</t>
-        </is>
-      </c>
-      <c r="B18" s="45" t="inlineStr">
-        <is>
-          <t>AEHR Test Systems</t>
-        </is>
-      </c>
-      <c r="C18" s="45" t="inlineStr">
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AEHR  —  AEHR Test Systems  |  Risk: High</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="52" customHeight="1">
+      <c r="A19" s="42" t="inlineStr">
         <is>
           <t>Classic shovels in a gold rush. More AI chips = more testing bottleneck demand.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="40" customHeight="1">
-      <c r="A19" s="33" t="inlineStr">
-        <is>
-          <t>CRDO</t>
-        </is>
-      </c>
-      <c r="B19" s="44" t="inlineStr">
-        <is>
-          <t>Credo Technology</t>
-        </is>
-      </c>
-      <c r="C19" s="44" t="inlineStr">
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CRDO  —  Credo Technology  |  Risk: High</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="52" customHeight="1">
+      <c r="A21" s="41" t="inlineStr">
         <is>
           <t>GPUs don't matter if data can't move between them. Cleanest AI infrastructure picks-and-shovels name.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="40" customHeight="1">
-      <c r="A20" s="27" t="inlineStr">
-        <is>
-          <t>ALGM</t>
-        </is>
-      </c>
-      <c r="B20" s="45" t="inlineStr">
-        <is>
-          <t>Allegro MicroSystems</t>
-        </is>
-      </c>
-      <c r="C20" s="45" t="inlineStr">
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ALGM  —  Allegro MicroSystems  |  Risk: Med-High</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="52" customHeight="1">
+      <c r="A23" s="42" t="inlineStr">
         <is>
           <t>Electrification + AI hardware power efficiency. Quiet compounder, early in AI rerating narrative.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="40" customHeight="1">
-      <c r="A21" s="33" t="inlineStr">
-        <is>
-          <t>HIMX</t>
-        </is>
-      </c>
-      <c r="B21" s="44" t="inlineStr">
-        <is>
-          <t>Himax Technologies</t>
-        </is>
-      </c>
-      <c r="C21" s="44" t="inlineStr">
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  HIMX  —  Himax Technologies  |  Risk: High</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="52" customHeight="1">
+      <c r="A25" s="41" t="inlineStr">
         <is>
           <t>Exposure to AI edge devices + optics. Higher volatility, historically rerates fast on cycles.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="40" customHeight="1">
-      <c r="A22" s="27" t="inlineStr">
-        <is>
-          <t>MTSI</t>
-        </is>
-      </c>
-      <c r="B22" s="45" t="inlineStr">
-        <is>
-          <t>MACOM Technology</t>
-        </is>
-      </c>
-      <c r="C22" s="45" t="inlineStr">
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MTSI  —  MACOM Technology  |  Risk: Med-High</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="52" customHeight="1">
+      <c r="A27" s="42" t="inlineStr">
         <is>
           <t>AI datacenter interconnect + telecom backbone. Less hype, more industrial AI backbone exposure.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="40" customHeight="1">
-      <c r="A23" s="33" t="inlineStr">
-        <is>
-          <t>AEVA</t>
-        </is>
-      </c>
-      <c r="B23" s="44" t="inlineStr">
-        <is>
-          <t>Aeva Technologies</t>
-        </is>
-      </c>
-      <c r="C23" s="44" t="inlineStr">
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AEVA  —  Aeva Technologies  |  Risk: Very High</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="52" customHeight="1">
+      <c r="A29" s="41" t="inlineStr">
         <is>
           <t>Autonomous systems + robotics long tail. Pure asymmetric bet: low probability, high upside.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="19">
+    <mergeCell ref="A24:Q24"/>
+    <mergeCell ref="A15:Q15"/>
+    <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A13:G13"/>
-    <mergeCell ref="C21:Q21"/>
-    <mergeCell ref="C20:Q20"/>
-    <mergeCell ref="C17:Q17"/>
+    <mergeCell ref="A16:Q16"/>
+    <mergeCell ref="A25:Q25"/>
+    <mergeCell ref="A18:Q18"/>
+    <mergeCell ref="A27:Q27"/>
     <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="C16:Q16"/>
-    <mergeCell ref="C19:Q19"/>
+    <mergeCell ref="A21:Q21"/>
+    <mergeCell ref="A26:Q26"/>
     <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A15:Q15"/>
-    <mergeCell ref="C23:Q23"/>
-    <mergeCell ref="C22:Q22"/>
-    <mergeCell ref="C18:Q18"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A23:Q23"/>
+    <mergeCell ref="A22:Q22"/>
+    <mergeCell ref="A17:Q17"/>
+    <mergeCell ref="A29:Q29"/>
+    <mergeCell ref="A20:Q20"/>
+    <mergeCell ref="A28:Q28"/>
+    <mergeCell ref="A19:Q19"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J11">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -4633,7 +4408,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="59" t="inlineStr">
+      <c r="A1" s="56" t="inlineStr">
         <is>
           <t>💡 Photonics &amp; Optics</t>
         </is>
@@ -4649,102 +4424,102 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="60" t="inlineStr">
+      <c r="A4" s="57" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="60" t="inlineStr">
+      <c r="B4" s="57" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="60" t="inlineStr">
+      <c r="C4" s="57" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="60" t="inlineStr">
+      <c r="D4" s="57" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="60" t="inlineStr">
+      <c r="E4" s="57" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="60" t="inlineStr">
+      <c r="F4" s="57" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="60" t="inlineStr">
+      <c r="G4" s="57" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="60" t="inlineStr">
+      <c r="H4" s="57" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="60" t="inlineStr">
+      <c r="I4" s="57" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="60" t="inlineStr">
+      <c r="J4" s="57" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="60" t="inlineStr">
+      <c r="K4" s="57" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="60" t="inlineStr">
+      <c r="L4" s="57" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="60" t="inlineStr">
+      <c r="M4" s="57" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="60" t="inlineStr">
+      <c r="N4" s="57" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="60" t="inlineStr">
+      <c r="O4" s="57" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="60" t="inlineStr">
+      <c r="P4" s="57" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="60" t="inlineStr">
+      <c r="Q4" s="57" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
@@ -4775,7 +4550,7 @@
       <c r="E5" s="28" t="n">
         <v>944.28</v>
       </c>
-      <c r="F5" s="48" t="n">
+      <c r="F5" s="45" t="n">
         <v>-1.642619728464659</v>
       </c>
       <c r="G5" s="28" t="n">
@@ -4819,78 +4594,44 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="61" t="inlineStr">
+      <c r="A7" s="58" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H7" s="62">
+      <c r="H7" s="59">
         <f>SUM(H5:H5)</f>
         <v/>
       </c>
-      <c r="I7" s="62">
+      <c r="I7" s="59">
         <f>SUM(I5:I5)</f>
         <v/>
       </c>
-      <c r="J7" s="62">
+      <c r="J7" s="59">
         <f>SUM(J5:J5)</f>
         <v/>
       </c>
-      <c r="K7" s="63">
+      <c r="K7" s="60">
         <f>IFERROR(J7/H7,"")</f>
         <v/>
       </c>
     </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="64" t="inlineStr">
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="61" t="inlineStr">
         <is>
           <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="16" customHeight="1">
+    <row r="10" ht="18" customHeight="1">
       <c r="A10" s="40" t="inlineStr">
         <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B10" s="40" t="inlineStr">
-        <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="C10" s="41" t="inlineStr">
-        <is>
-          <t>Notes / Thesis</t>
-        </is>
-      </c>
-      <c r="D10" s="42" t="n"/>
-      <c r="E10" s="42" t="n"/>
-      <c r="F10" s="42" t="n"/>
-      <c r="G10" s="42" t="n"/>
-      <c r="H10" s="42" t="n"/>
-      <c r="I10" s="42" t="n"/>
-      <c r="J10" s="42" t="n"/>
-      <c r="K10" s="42" t="n"/>
-      <c r="L10" s="42" t="n"/>
-      <c r="M10" s="42" t="n"/>
-      <c r="N10" s="42" t="n"/>
-      <c r="O10" s="42" t="n"/>
-      <c r="P10" s="42" t="n"/>
-      <c r="Q10" s="43" t="n"/>
-    </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="33" t="inlineStr">
-        <is>
-          <t>LITE</t>
-        </is>
-      </c>
-      <c r="B11" s="44" t="inlineStr">
-        <is>
-          <t>Lumentum Holdings</t>
-        </is>
-      </c>
-      <c r="C11" s="44" t="inlineStr">
+          <t xml:space="preserve">  LITE  —  Lumentum Holdings  |  Risk: High</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="52" customHeight="1">
+      <c r="A11" s="41" t="inlineStr">
         <is>
           <t>King of Photonics. Could moonshot. Key bottleneck in AI data movement. Critical infrastructure.</t>
         </is>
@@ -4900,10 +4641,10 @@
   <mergeCells count="7">
     <mergeCell ref="A9:Q9"/>
     <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="C10:Q10"/>
-    <mergeCell ref="C11:Q11"/>
     <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A10:Q10"/>
     <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A11:Q11"/>
     <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="J5">
@@ -4933,7 +4674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4956,7 +4697,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="65" t="inlineStr">
+      <c r="A1" s="62" t="inlineStr">
         <is>
           <t>🏗️ DC Builders &amp; Cooling</t>
         </is>
@@ -4972,102 +4713,102 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="66" t="inlineStr">
+      <c r="A4" s="63" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="66" t="inlineStr">
+      <c r="B4" s="63" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="66" t="inlineStr">
+      <c r="C4" s="63" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="66" t="inlineStr">
+      <c r="D4" s="63" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="66" t="inlineStr">
+      <c r="E4" s="63" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="66" t="inlineStr">
+      <c r="F4" s="63" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="66" t="inlineStr">
+      <c r="G4" s="63" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="66" t="inlineStr">
+      <c r="H4" s="63" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="66" t="inlineStr">
+      <c r="I4" s="63" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="66" t="inlineStr">
+      <c r="J4" s="63" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="66" t="inlineStr">
+      <c r="K4" s="63" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="66" t="inlineStr">
+      <c r="L4" s="63" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="66" t="inlineStr">
+      <c r="M4" s="63" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="66" t="inlineStr">
+      <c r="N4" s="63" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="66" t="inlineStr">
+      <c r="O4" s="63" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="66" t="inlineStr">
+      <c r="P4" s="63" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="66" t="inlineStr">
+      <c r="Q4" s="63" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
@@ -5343,146 +5084,106 @@
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="67" t="inlineStr">
+      <c r="A10" s="64" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H10" s="68">
+      <c r="H10" s="65">
         <f>SUM(H5:H8)</f>
         <v/>
       </c>
-      <c r="I10" s="68">
+      <c r="I10" s="65">
         <f>SUM(I5:I8)</f>
         <v/>
       </c>
-      <c r="J10" s="68">
+      <c r="J10" s="65">
         <f>SUM(J5:J8)</f>
         <v/>
       </c>
-      <c r="K10" s="69">
+      <c r="K10" s="66">
         <f>IFERROR(J10/H10,"")</f>
         <v/>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="70" t="inlineStr">
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="67" t="inlineStr">
         <is>
           <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="16" customHeight="1">
+    <row r="13" ht="18" customHeight="1">
       <c r="A13" s="40" t="inlineStr">
         <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B13" s="40" t="inlineStr">
-        <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="C13" s="41" t="inlineStr">
-        <is>
-          <t>Notes / Thesis</t>
-        </is>
-      </c>
-      <c r="D13" s="42" t="n"/>
-      <c r="E13" s="42" t="n"/>
-      <c r="F13" s="42" t="n"/>
-      <c r="G13" s="42" t="n"/>
-      <c r="H13" s="42" t="n"/>
-      <c r="I13" s="42" t="n"/>
-      <c r="J13" s="42" t="n"/>
-      <c r="K13" s="42" t="n"/>
-      <c r="L13" s="42" t="n"/>
-      <c r="M13" s="42" t="n"/>
-      <c r="N13" s="42" t="n"/>
-      <c r="O13" s="42" t="n"/>
-      <c r="P13" s="42" t="n"/>
-      <c r="Q13" s="43" t="n"/>
-    </row>
-    <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="33" t="inlineStr">
-        <is>
-          <t>CAT</t>
-        </is>
-      </c>
-      <c r="B14" s="44" t="inlineStr">
-        <is>
-          <t>Caterpillar Inc</t>
-        </is>
-      </c>
-      <c r="C14" s="44" t="inlineStr">
+          <t xml:space="preserve">  CAT  —  Caterpillar Inc  |  Risk: Low-Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="52" customHeight="1">
+      <c r="A14" s="41" t="inlineStr">
         <is>
           <t>Actual builder and materials company in the AI data center trade.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="27" t="inlineStr">
-        <is>
-          <t>FIX</t>
-        </is>
-      </c>
-      <c r="B15" s="45" t="inlineStr">
-        <is>
-          <t>Comfort Systems USA</t>
-        </is>
-      </c>
-      <c r="C15" s="45" t="inlineStr">
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  FIX  —  Comfort Systems USA  |  Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="52" customHeight="1">
+      <c r="A16" s="42" t="inlineStr">
         <is>
           <t>Builder AND cooling company. AI data center HVAC &amp; MEP systems. Major growing bottleneck.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="40" customHeight="1">
-      <c r="A16" s="33" t="inlineStr">
-        <is>
-          <t>POWL</t>
-        </is>
-      </c>
-      <c r="B16" s="44" t="inlineStr">
-        <is>
-          <t>Powell Industries</t>
-        </is>
-      </c>
-      <c r="C16" s="44" t="inlineStr">
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  POWL  —  Powell Industries  |  Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="52" customHeight="1">
+      <c r="A18" s="41" t="inlineStr">
         <is>
           <t>Electrical infrastructure builder for AI data centers.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="27" t="inlineStr">
-        <is>
-          <t>VRT</t>
-        </is>
-      </c>
-      <c r="B17" s="45" t="inlineStr">
-        <is>
-          <t>Vertiv Holdings</t>
-        </is>
-      </c>
-      <c r="C17" s="45" t="inlineStr">
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  VRT  —  Vertiv Holdings  |  Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="52" customHeight="1">
+      <c r="A20" s="42" t="inlineStr">
         <is>
           <t>Premier AI data center cooling play. Cooling is a growing bottleneck.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="C15:Q15"/>
-    <mergeCell ref="C17:Q17"/>
+  <mergeCells count="13">
+    <mergeCell ref="A14:Q14"/>
+    <mergeCell ref="A17:Q17"/>
+    <mergeCell ref="A18:Q18"/>
     <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="C16:Q16"/>
     <mergeCell ref="A12:Q12"/>
-    <mergeCell ref="C14:Q14"/>
-    <mergeCell ref="C13:Q13"/>
+    <mergeCell ref="A20:Q20"/>
     <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A16:Q16"/>
+    <mergeCell ref="A15:Q15"/>
+    <mergeCell ref="A19:Q19"/>
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A13:Q13"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J8">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -5511,7 +5212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5534,7 +5235,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="71" t="inlineStr">
+      <c r="A1" s="68" t="inlineStr">
         <is>
           <t>⚡ Power &amp; Energy</t>
         </is>
@@ -5550,102 +5251,102 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="72" t="inlineStr">
+      <c r="A4" s="69" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="72" t="inlineStr">
+      <c r="B4" s="69" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="72" t="inlineStr">
+      <c r="C4" s="69" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="72" t="inlineStr">
+      <c r="D4" s="69" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="72" t="inlineStr">
+      <c r="E4" s="69" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="72" t="inlineStr">
+      <c r="F4" s="69" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="72" t="inlineStr">
+      <c r="G4" s="69" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="72" t="inlineStr">
+      <c r="H4" s="69" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="72" t="inlineStr">
+      <c r="I4" s="69" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="72" t="inlineStr">
+      <c r="J4" s="69" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="72" t="inlineStr">
+      <c r="K4" s="69" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="72" t="inlineStr">
+      <c r="L4" s="69" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="72" t="inlineStr">
+      <c r="M4" s="69" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="72" t="inlineStr">
+      <c r="N4" s="69" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="72" t="inlineStr">
+      <c r="O4" s="69" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="72" t="inlineStr">
+      <c r="P4" s="69" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="72" t="inlineStr">
+      <c r="Q4" s="69" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
@@ -5810,7 +5511,7 @@
       <c r="E7" s="28" t="n">
         <v>285.47</v>
       </c>
-      <c r="F7" s="48" t="n">
+      <c r="F7" s="45" t="n">
         <v>-4.067043441964675</v>
       </c>
       <c r="G7" s="28" t="n">
@@ -5921,146 +5622,106 @@
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="73" t="inlineStr">
+      <c r="A10" s="70" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H10" s="74">
+      <c r="H10" s="71">
         <f>SUM(H5:H8)</f>
         <v/>
       </c>
-      <c r="I10" s="74">
+      <c r="I10" s="71">
         <f>SUM(I5:I8)</f>
         <v/>
       </c>
-      <c r="J10" s="74">
+      <c r="J10" s="71">
         <f>SUM(J5:J8)</f>
         <v/>
       </c>
-      <c r="K10" s="75">
+      <c r="K10" s="72">
         <f>IFERROR(J10/H10,"")</f>
         <v/>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="76" t="inlineStr">
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="73" t="inlineStr">
         <is>
           <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="16" customHeight="1">
+    <row r="13" ht="18" customHeight="1">
       <c r="A13" s="40" t="inlineStr">
         <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B13" s="40" t="inlineStr">
-        <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="C13" s="41" t="inlineStr">
-        <is>
-          <t>Notes / Thesis</t>
-        </is>
-      </c>
-      <c r="D13" s="42" t="n"/>
-      <c r="E13" s="42" t="n"/>
-      <c r="F13" s="42" t="n"/>
-      <c r="G13" s="42" t="n"/>
-      <c r="H13" s="42" t="n"/>
-      <c r="I13" s="42" t="n"/>
-      <c r="J13" s="42" t="n"/>
-      <c r="K13" s="42" t="n"/>
-      <c r="L13" s="42" t="n"/>
-      <c r="M13" s="42" t="n"/>
-      <c r="N13" s="42" t="n"/>
-      <c r="O13" s="42" t="n"/>
-      <c r="P13" s="42" t="n"/>
-      <c r="Q13" s="43" t="n"/>
-    </row>
-    <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="33" t="inlineStr">
-        <is>
-          <t>GEV</t>
-        </is>
-      </c>
-      <c r="B14" s="44" t="inlineStr">
-        <is>
-          <t>GE Vernova</t>
-        </is>
-      </c>
-      <c r="C14" s="44" t="inlineStr">
+          <t xml:space="preserve">  GEV  —  GE Vernova  |  Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="52" customHeight="1">
+      <c r="A14" s="41" t="inlineStr">
         <is>
           <t>Stability and steady compounder. Power and grid maintenance for AI buildout.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="27" t="inlineStr">
-        <is>
-          <t>PWR</t>
-        </is>
-      </c>
-      <c r="B15" s="45" t="inlineStr">
-        <is>
-          <t>Quanta Services</t>
-        </is>
-      </c>
-      <c r="C15" s="45" t="inlineStr">
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PWR  —  Quanta Services  |  Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="52" customHeight="1">
+      <c r="A16" s="42" t="inlineStr">
         <is>
           <t>Power generation and grid maintenance. Growing bottleneck for AI buildout.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="40" customHeight="1">
-      <c r="A16" s="33" t="inlineStr">
-        <is>
-          <t>BE</t>
-        </is>
-      </c>
-      <c r="B16" s="44" t="inlineStr">
-        <is>
-          <t>Bloom Energy</t>
-        </is>
-      </c>
-      <c r="C16" s="44" t="inlineStr">
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  BE  —  Bloom Energy  |  Risk: High</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="52" customHeight="1">
+      <c r="A18" s="41" t="inlineStr">
         <is>
           <t>Moonshot potential if hydrogen &amp; fuel cell technology takes off.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="27" t="inlineStr">
-        <is>
-          <t>OKLO</t>
-        </is>
-      </c>
-      <c r="B17" s="45" t="inlineStr">
-        <is>
-          <t>Oklo Inc</t>
-        </is>
-      </c>
-      <c r="C17" s="45" t="inlineStr">
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  OKLO  —  Oklo Inc  |  Risk: Very High</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="52" customHeight="1">
+      <c r="A20" s="42" t="inlineStr">
         <is>
           <t>Massive moonshot potential. Big regulatory &amp; execution risk. Worth a small % of portfolio given massive potential.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="C15:Q15"/>
-    <mergeCell ref="C17:Q17"/>
+  <mergeCells count="13">
+    <mergeCell ref="A14:Q14"/>
+    <mergeCell ref="A17:Q17"/>
+    <mergeCell ref="A18:Q18"/>
     <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="C16:Q16"/>
     <mergeCell ref="A12:Q12"/>
-    <mergeCell ref="C14:Q14"/>
-    <mergeCell ref="C13:Q13"/>
+    <mergeCell ref="A20:Q20"/>
     <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A16:Q16"/>
+    <mergeCell ref="A15:Q15"/>
+    <mergeCell ref="A19:Q19"/>
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A13:Q13"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J8">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -6089,7 +5750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6112,7 +5773,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="77" t="inlineStr">
+      <c r="A1" s="74" t="inlineStr">
         <is>
           <t>☁️ Neoclouds &amp; AI Software</t>
         </is>
@@ -6128,102 +5789,102 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="78" t="inlineStr">
+      <c r="A4" s="75" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="78" t="inlineStr">
+      <c r="B4" s="75" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="78" t="inlineStr">
+      <c r="C4" s="75" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="78" t="inlineStr">
+      <c r="D4" s="75" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="78" t="inlineStr">
+      <c r="E4" s="75" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="78" t="inlineStr">
+      <c r="F4" s="75" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="78" t="inlineStr">
+      <c r="G4" s="75" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="78" t="inlineStr">
+      <c r="H4" s="75" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="78" t="inlineStr">
+      <c r="I4" s="75" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="78" t="inlineStr">
+      <c r="J4" s="75" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="78" t="inlineStr">
+      <c r="K4" s="75" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="78" t="inlineStr">
+      <c r="L4" s="75" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="78" t="inlineStr">
+      <c r="M4" s="75" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="78" t="inlineStr">
+      <c r="N4" s="75" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="78" t="inlineStr">
+      <c r="O4" s="75" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="78" t="inlineStr">
+      <c r="P4" s="75" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="78" t="inlineStr">
+      <c r="Q4" s="75" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
@@ -6321,7 +5982,7 @@
       <c r="E6" s="28" t="n">
         <v>133.79</v>
       </c>
-      <c r="F6" s="48" t="n">
+      <c r="F6" s="45" t="n">
         <v>-1.101424241474859</v>
       </c>
       <c r="G6" s="28" t="n">
@@ -6365,110 +6026,74 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="79" t="inlineStr">
+      <c r="A8" s="76" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H8" s="80">
+      <c r="H8" s="77">
         <f>SUM(H5:H6)</f>
         <v/>
       </c>
-      <c r="I8" s="80">
+      <c r="I8" s="77">
         <f>SUM(I5:I6)</f>
         <v/>
       </c>
-      <c r="J8" s="80">
+      <c r="J8" s="77">
         <f>SUM(J5:J6)</f>
         <v/>
       </c>
-      <c r="K8" s="81">
+      <c r="K8" s="78">
         <f>IFERROR(J8/H8,"")</f>
         <v/>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="82" t="inlineStr">
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="79" t="inlineStr">
         <is>
           <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="16" customHeight="1">
+    <row r="11" ht="18" customHeight="1">
       <c r="A11" s="40" t="inlineStr">
         <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B11" s="40" t="inlineStr">
-        <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="C11" s="41" t="inlineStr">
-        <is>
-          <t>Notes / Thesis</t>
-        </is>
-      </c>
-      <c r="D11" s="42" t="n"/>
-      <c r="E11" s="42" t="n"/>
-      <c r="F11" s="42" t="n"/>
-      <c r="G11" s="42" t="n"/>
-      <c r="H11" s="42" t="n"/>
-      <c r="I11" s="42" t="n"/>
-      <c r="J11" s="42" t="n"/>
-      <c r="K11" s="42" t="n"/>
-      <c r="L11" s="42" t="n"/>
-      <c r="M11" s="42" t="n"/>
-      <c r="N11" s="42" t="n"/>
-      <c r="O11" s="42" t="n"/>
-      <c r="P11" s="42" t="n"/>
-      <c r="Q11" s="43" t="n"/>
-    </row>
-    <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="33" t="inlineStr">
-        <is>
-          <t>NBIS</t>
-        </is>
-      </c>
-      <c r="B12" s="44" t="inlineStr">
-        <is>
-          <t>Nebius Group</t>
-        </is>
-      </c>
-      <c r="C12" s="44" t="inlineStr">
+          <t xml:space="preserve">  NBIS  —  Nebius Group  |  Risk: High</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="52" customHeight="1">
+      <c r="A12" s="41" t="inlineStr">
         <is>
           <t>Leading Neocloud with multiple revenue streams (Clickhouse, AV Ride). Modern Amazon/Google style company. Could become a future Hyperscaler.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="27" t="inlineStr">
-        <is>
-          <t>PLTR</t>
-        </is>
-      </c>
-      <c r="B13" s="45" t="inlineStr">
-        <is>
-          <t>Palantir Technologies</t>
-        </is>
-      </c>
-      <c r="C13" s="45" t="inlineStr">
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PLTR  —  Palantir Technologies  |  Risk: Med-High</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="52" customHeight="1">
+      <c r="A14" s="42" t="inlineStr">
         <is>
           <t>Integral to the entire government AI stack. Not going anywhere. AI Software outlier outside the data center trade.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
+    <mergeCell ref="A14:Q14"/>
     <mergeCell ref="A3:Q3"/>
     <mergeCell ref="A8:G8"/>
-    <mergeCell ref="C11:Q11"/>
-    <mergeCell ref="C13:Q13"/>
+    <mergeCell ref="A12:Q12"/>
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A10:Q10"/>
+    <mergeCell ref="A11:Q11"/>
     <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="C12:Q12"/>
+    <mergeCell ref="A13:Q13"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J6">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -6520,7 +6145,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="83" t="inlineStr">
+      <c r="A1" s="80" t="inlineStr">
         <is>
           <t>🛡️ Defense &amp; Drones</t>
         </is>
@@ -6536,102 +6161,102 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:24 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="84" t="inlineStr">
+      <c r="A4" s="81" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="84" t="inlineStr">
+      <c r="B4" s="81" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="84" t="inlineStr">
+      <c r="C4" s="81" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="84" t="inlineStr">
+      <c r="D4" s="81" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="84" t="inlineStr">
+      <c r="E4" s="81" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="84" t="inlineStr">
+      <c r="F4" s="81" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="84" t="inlineStr">
+      <c r="G4" s="81" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="84" t="inlineStr">
+      <c r="H4" s="81" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="84" t="inlineStr">
+      <c r="I4" s="81" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="84" t="inlineStr">
+      <c r="J4" s="81" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="84" t="inlineStr">
+      <c r="K4" s="81" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="84" t="inlineStr">
+      <c r="L4" s="81" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="84" t="inlineStr">
+      <c r="M4" s="81" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="84" t="inlineStr">
+      <c r="N4" s="81" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="84" t="inlineStr">
+      <c r="O4" s="81" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="84" t="inlineStr">
+      <c r="P4" s="81" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="84" t="inlineStr">
+      <c r="Q4" s="81" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
@@ -6706,78 +6331,44 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="85" t="inlineStr">
+      <c r="A7" s="82" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H7" s="86">
+      <c r="H7" s="83">
         <f>SUM(H5:H5)</f>
         <v/>
       </c>
-      <c r="I7" s="86">
+      <c r="I7" s="83">
         <f>SUM(I5:I5)</f>
         <v/>
       </c>
-      <c r="J7" s="86">
+      <c r="J7" s="83">
         <f>SUM(J5:J5)</f>
         <v/>
       </c>
-      <c r="K7" s="87">
+      <c r="K7" s="84">
         <f>IFERROR(J7/H7,"")</f>
         <v/>
       </c>
     </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="88" t="inlineStr">
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="85" t="inlineStr">
         <is>
           <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="16" customHeight="1">
+    <row r="10" ht="18" customHeight="1">
       <c r="A10" s="40" t="inlineStr">
         <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B10" s="40" t="inlineStr">
-        <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="C10" s="41" t="inlineStr">
-        <is>
-          <t>Notes / Thesis</t>
-        </is>
-      </c>
-      <c r="D10" s="42" t="n"/>
-      <c r="E10" s="42" t="n"/>
-      <c r="F10" s="42" t="n"/>
-      <c r="G10" s="42" t="n"/>
-      <c r="H10" s="42" t="n"/>
-      <c r="I10" s="42" t="n"/>
-      <c r="J10" s="42" t="n"/>
-      <c r="K10" s="42" t="n"/>
-      <c r="L10" s="42" t="n"/>
-      <c r="M10" s="42" t="n"/>
-      <c r="N10" s="42" t="n"/>
-      <c r="O10" s="42" t="n"/>
-      <c r="P10" s="42" t="n"/>
-      <c r="Q10" s="43" t="n"/>
-    </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="33" t="inlineStr">
-        <is>
-          <t>ONDS</t>
-        </is>
-      </c>
-      <c r="B11" s="44" t="inlineStr">
-        <is>
-          <t>Ondas Holdings</t>
-        </is>
-      </c>
-      <c r="C11" s="44" t="inlineStr">
+          <t xml:space="preserve">  ONDS  —  Ondas Holdings  |  Risk: Very High</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="52" customHeight="1">
+      <c r="A11" s="41" t="inlineStr">
         <is>
           <t>$1.5T defense budget, $56B to drones/counter-drones via DAWG Program. Best chance to scale after March 2026 acquisitions &amp; partnerships. Very speculative.</t>
         </is>
@@ -6787,10 +6378,10 @@
   <mergeCells count="7">
     <mergeCell ref="A9:Q9"/>
     <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="C10:Q10"/>
-    <mergeCell ref="C11:Q11"/>
     <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A10:Q10"/>
     <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A11:Q11"/>
     <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="J5">

</xml_diff>

<commit_message>
Improve display of investment notes to span entire row
Update script to use explicit merge cell arguments and increase row height to ensure notes display across the full width of the sheet.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: b37bbd1d-3cee-4cf1-82d7-fb06ea342597
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -31,7 +31,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="+0.00&quot;%&quot;;-0.00&quot;%&quot;;0.00&quot;%&quot;"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -166,6 +166,12 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001B2A4A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <color rgb="001B2A4A"/>
       <sz val="10"/>
     </font>
@@ -286,7 +292,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -322,28 +328,6 @@
         <color rgb="00AAAAAA"/>
       </bottom>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="00AAAAAA"/>
-      </left>
-      <right style="medium">
-        <color rgb="00AAAAAA"/>
-      </right>
-      <top style="medium">
-        <color rgb="00AAAAAA"/>
-      </top>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="00AAAAAA"/>
-      </left>
-      <right style="medium">
-        <color rgb="00AAAAAA"/>
-      </right>
-      <bottom style="medium">
-        <color rgb="00AAAAAA"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -463,15 +447,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -493,7 +477,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -511,7 +495,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -529,7 +513,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -547,7 +531,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -565,7 +549,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -583,7 +567,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -601,7 +585,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -619,7 +603,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -637,9 +621,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1072,7 +1056,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1543,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
         </is>
       </c>
     </row>
@@ -1758,14 +1742,14 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1">
+    <row r="10" ht="20" customHeight="1">
       <c r="A10" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  RKLB  —  Rocket Lab USA  |  Risk: High</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="52" customHeight="1">
+    <row r="11" ht="409" customHeight="1">
       <c r="A11" s="41" t="inlineStr">
         <is>
           <t>Huge future TAM over next decade+. Speculative but massive upside. Brilliant CEO. Near-term catalyst: SpaceX IPO in June.</t>
@@ -1848,7 +1832,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
         </is>
       </c>
     </row>
@@ -2114,28 +2098,28 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1">
+    <row r="11" ht="20" customHeight="1">
       <c r="A11" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  RBRK  —  Rubrik Inc  |  Risk: Med-High</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="52" customHeight="1">
+    <row r="12" ht="409" customHeight="1">
       <c r="A12" s="41" t="inlineStr">
         <is>
           <t>Long term investment research candidate.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
+    <row r="13" ht="20" customHeight="1">
       <c r="A13" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  NVO  —  Novo Nordisk  |  Risk: Medium</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="52" customHeight="1">
+    <row r="14" ht="409" customHeight="1">
       <c r="A14" s="42" t="inlineStr">
         <is>
           <t>Long term investment research candidate.</t>
@@ -2478,7 +2462,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
         </is>
       </c>
     </row>
@@ -2811,42 +2795,42 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1">
+    <row r="12" ht="20" customHeight="1">
       <c r="A12" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  IONQ  —  IonQ Inc  |  Risk: Very High</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="52" customHeight="1">
+    <row r="13" ht="409" customHeight="1">
       <c r="A13" s="41" t="inlineStr">
         <is>
           <t>Next quantum run candidate. Easy 10× within 2 years potential.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1">
+    <row r="14" ht="20" customHeight="1">
       <c r="A14" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  RGTI  —  Rigetti Computing  |  Risk: Very High</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="52" customHeight="1">
+    <row r="15" ht="409" customHeight="1">
       <c r="A15" s="42" t="inlineStr">
         <is>
           <t>Next quantum run candidate. Easy 10× within 2 years potential.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1">
+    <row r="16" ht="20" customHeight="1">
       <c r="A16" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  QBTS  —  D-Wave Quantum  |  Risk: Very High</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="52" customHeight="1">
+    <row r="17" ht="409" customHeight="1">
       <c r="A17" s="41" t="inlineStr">
         <is>
           <t>Next quantum run candidate. Easy 10× within 2 years potential.</t>
@@ -2933,7 +2917,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
         </is>
       </c>
     </row>
@@ -3467,84 +3451,84 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1">
+    <row r="15" ht="20" customHeight="1">
       <c r="A15" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  NVDA  —  NVIDIA Corp  |  Risk: Medium</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="52" customHeight="1">
+    <row r="16" ht="409" customHeight="1">
       <c r="A16" s="41" t="inlineStr">
         <is>
           <t>The AI compute king. Stability and steady compounder.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1">
+    <row r="17" ht="20" customHeight="1">
       <c r="A17" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  AVGO  —  Broadcom Inc  |  Risk: Medium</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="52" customHeight="1">
+    <row r="18" ht="409" customHeight="1">
       <c r="A18" s="42" t="inlineStr">
         <is>
           <t>Stability and steady compounder.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1">
+    <row r="19" ht="20" customHeight="1">
       <c r="A19" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  LRCX  —  Lam Research  |  Risk: Medium</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="52" customHeight="1">
+    <row r="20" ht="409" customHeight="1">
       <c r="A20" s="41" t="inlineStr">
         <is>
           <t>Stability and steady compounder. DRAM equipment leader.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="18" customHeight="1">
+    <row r="21" ht="20" customHeight="1">
       <c r="A21" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  AMD  —  Advanced Micro Devices  |  Risk: Medium</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="52" customHeight="1">
+    <row r="22" ht="409" customHeight="1">
       <c r="A22" s="42" t="inlineStr">
         <is>
           <t>CPU maker deep in the AI infrastructure stack.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="18" customHeight="1">
+    <row r="23" ht="20" customHeight="1">
       <c r="A23" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  INTC  —  Intel Corp  |  Risk: Med-High</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="52" customHeight="1">
+    <row r="24" ht="409" customHeight="1">
       <c r="A24" s="41" t="inlineStr">
         <is>
           <t>CPU maker in AI infrastructure stack. Turnaround story.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="18" customHeight="1">
+    <row r="25" ht="20" customHeight="1">
       <c r="A25" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  ARM  —  Arm Holdings  |  Risk: Medium</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="52" customHeight="1">
+    <row r="26" ht="409" customHeight="1">
       <c r="A26" s="42" t="inlineStr">
         <is>
           <t>Architecture behind most AI edge chips. Royalty model.</t>
@@ -3637,7 +3621,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
         </is>
       </c>
     </row>
@@ -4238,98 +4222,98 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1">
+    <row r="16" ht="20" customHeight="1">
       <c r="A16" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  NVTS  —  Navitas Semiconductor  |  Risk: High</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="52" customHeight="1">
+    <row r="17" ht="409" customHeight="1">
       <c r="A17" s="41" t="inlineStr">
         <is>
           <t>AI data centers need radically more efficient power delivery. Picks-and-shovels for compute growth.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="18" customHeight="1">
+    <row r="18" ht="20" customHeight="1">
       <c r="A18" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  AEHR  —  AEHR Test Systems  |  Risk: High</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="52" customHeight="1">
+    <row r="19" ht="409" customHeight="1">
       <c r="A19" s="42" t="inlineStr">
         <is>
           <t>Classic shovels in a gold rush. More AI chips = more testing bottleneck demand.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="18" customHeight="1">
+    <row r="20" ht="20" customHeight="1">
       <c r="A20" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  CRDO  —  Credo Technology  |  Risk: High</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="52" customHeight="1">
+    <row r="21" ht="409" customHeight="1">
       <c r="A21" s="41" t="inlineStr">
         <is>
           <t>GPUs don't matter if data can't move between them. Cleanest AI infrastructure picks-and-shovels name.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="18" customHeight="1">
+    <row r="22" ht="20" customHeight="1">
       <c r="A22" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  ALGM  —  Allegro MicroSystems  |  Risk: Med-High</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="52" customHeight="1">
+    <row r="23" ht="409" customHeight="1">
       <c r="A23" s="42" t="inlineStr">
         <is>
           <t>Electrification + AI hardware power efficiency. Quiet compounder, early in AI rerating narrative.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="18" customHeight="1">
+    <row r="24" ht="20" customHeight="1">
       <c r="A24" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  HIMX  —  Himax Technologies  |  Risk: High</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="52" customHeight="1">
+    <row r="25" ht="409" customHeight="1">
       <c r="A25" s="41" t="inlineStr">
         <is>
           <t>Exposure to AI edge devices + optics. Higher volatility, historically rerates fast on cycles.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="18" customHeight="1">
+    <row r="26" ht="20" customHeight="1">
       <c r="A26" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  MTSI  —  MACOM Technology  |  Risk: Med-High</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="52" customHeight="1">
+    <row r="27" ht="409" customHeight="1">
       <c r="A27" s="42" t="inlineStr">
         <is>
           <t>AI datacenter interconnect + telecom backbone. Less hype, more industrial AI backbone exposure.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="18" customHeight="1">
+    <row r="28" ht="20" customHeight="1">
       <c r="A28" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  AEVA  —  Aeva Technologies  |  Risk: Very High</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="52" customHeight="1">
+    <row r="29" ht="409" customHeight="1">
       <c r="A29" s="41" t="inlineStr">
         <is>
           <t>Autonomous systems + robotics long tail. Pure asymmetric bet: low probability, high upside.</t>
@@ -4424,7 +4408,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
         </is>
       </c>
     </row>
@@ -4623,14 +4607,14 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1">
+    <row r="10" ht="20" customHeight="1">
       <c r="A10" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  LITE  —  Lumentum Holdings  |  Risk: High</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="52" customHeight="1">
+    <row r="11" ht="409" customHeight="1">
       <c r="A11" s="41" t="inlineStr">
         <is>
           <t>King of Photonics. Could moonshot. Key bottleneck in AI data movement. Critical infrastructure.</t>
@@ -4713,7 +4697,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
         </is>
       </c>
     </row>
@@ -5113,56 +5097,56 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
+    <row r="13" ht="20" customHeight="1">
       <c r="A13" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  CAT  —  Caterpillar Inc  |  Risk: Low-Med</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="52" customHeight="1">
+    <row r="14" ht="409" customHeight="1">
       <c r="A14" s="41" t="inlineStr">
         <is>
           <t>Actual builder and materials company in the AI data center trade.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1">
+    <row r="15" ht="20" customHeight="1">
       <c r="A15" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  FIX  —  Comfort Systems USA  |  Risk: Medium</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="52" customHeight="1">
+    <row r="16" ht="409" customHeight="1">
       <c r="A16" s="42" t="inlineStr">
         <is>
           <t>Builder AND cooling company. AI data center HVAC &amp; MEP systems. Major growing bottleneck.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1">
+    <row r="17" ht="20" customHeight="1">
       <c r="A17" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  POWL  —  Powell Industries  |  Risk: Medium</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="52" customHeight="1">
+    <row r="18" ht="409" customHeight="1">
       <c r="A18" s="41" t="inlineStr">
         <is>
           <t>Electrical infrastructure builder for AI data centers.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1">
+    <row r="19" ht="20" customHeight="1">
       <c r="A19" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  VRT  —  Vertiv Holdings  |  Risk: Medium</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="52" customHeight="1">
+    <row r="20" ht="409" customHeight="1">
       <c r="A20" s="42" t="inlineStr">
         <is>
           <t>Premier AI data center cooling play. Cooling is a growing bottleneck.</t>
@@ -5251,7 +5235,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
         </is>
       </c>
     </row>
@@ -5651,56 +5635,56 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
+    <row r="13" ht="20" customHeight="1">
       <c r="A13" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  GEV  —  GE Vernova  |  Risk: Medium</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="52" customHeight="1">
+    <row r="14" ht="409" customHeight="1">
       <c r="A14" s="41" t="inlineStr">
         <is>
           <t>Stability and steady compounder. Power and grid maintenance for AI buildout.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1">
+    <row r="15" ht="20" customHeight="1">
       <c r="A15" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  PWR  —  Quanta Services  |  Risk: Medium</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="52" customHeight="1">
+    <row r="16" ht="409" customHeight="1">
       <c r="A16" s="42" t="inlineStr">
         <is>
           <t>Power generation and grid maintenance. Growing bottleneck for AI buildout.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1">
+    <row r="17" ht="20" customHeight="1">
       <c r="A17" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  BE  —  Bloom Energy  |  Risk: High</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="52" customHeight="1">
+    <row r="18" ht="409" customHeight="1">
       <c r="A18" s="41" t="inlineStr">
         <is>
           <t>Moonshot potential if hydrogen &amp; fuel cell technology takes off.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1">
+    <row r="19" ht="20" customHeight="1">
       <c r="A19" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  OKLO  —  Oklo Inc  |  Risk: Very High</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="52" customHeight="1">
+    <row r="20" ht="409" customHeight="1">
       <c r="A20" s="42" t="inlineStr">
         <is>
           <t>Massive moonshot potential. Big regulatory &amp; execution risk. Worth a small % of portfolio given massive potential.</t>
@@ -5789,7 +5773,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
         </is>
       </c>
     </row>
@@ -6055,28 +6039,28 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1">
+    <row r="11" ht="20" customHeight="1">
       <c r="A11" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  NBIS  —  Nebius Group  |  Risk: High</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="52" customHeight="1">
+    <row r="12" ht="409" customHeight="1">
       <c r="A12" s="41" t="inlineStr">
         <is>
           <t>Leading Neocloud with multiple revenue streams (Clickhouse, AV Ride). Modern Amazon/Google style company. Could become a future Hyperscaler.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
+    <row r="13" ht="20" customHeight="1">
       <c r="A13" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  PLTR  —  Palantir Technologies  |  Risk: Med-High</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="52" customHeight="1">
+    <row r="14" ht="409" customHeight="1">
       <c r="A14" s="42" t="inlineStr">
         <is>
           <t>Integral to the entire government AI stack. Not going anywhere. AI Software outlier outside the data center trade.</t>
@@ -6161,7 +6145,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:30 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
         </is>
       </c>
     </row>
@@ -6360,14 +6344,14 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1">
+    <row r="10" ht="20" customHeight="1">
       <c r="A10" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  ONDS  —  Ondas Holdings  |  Risk: Very High</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="52" customHeight="1">
+    <row r="11" ht="409" customHeight="1">
       <c r="A11" s="41" t="inlineStr">
         <is>
           <t>$1.5T defense budget, $56B to drones/counter-drones via DAWG Program. Best chance to scale after March 2026 acquisitions &amp; partnerships. Very speculative.</t>

</xml_diff>

<commit_message>
Fix notes display by writing them as plain text across multiple rows
Remove merged cells and text wrapping dependency for notes; instead, split notes into individual lines and write each to its own row in column B, which is then widened to accommodate the text. Update section header styling and ensure background color extends across all columns.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 8cddc9b3-d5c5-4f72-97e0-844384cc90e5
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -332,7 +332,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -449,14 +449,20 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="23" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="23" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -479,6 +485,7 @@
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -497,6 +504,7 @@
     <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -515,6 +523,7 @@
     <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -533,6 +542,7 @@
     <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -551,6 +561,7 @@
     <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -569,6 +580,7 @@
     <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -587,6 +599,7 @@
     <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -605,6 +618,7 @@
     <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -623,6 +637,7 @@
     <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="24" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1056,7 +1071,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
         </is>
       </c>
     </row>
@@ -1504,11 +1519,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="130" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -1527,7 +1542,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="86" t="inlineStr">
+      <c r="A1" s="97" t="inlineStr">
         <is>
           <t>🚀 Space Economy</t>
         </is>
@@ -1543,102 +1558,102 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="87" t="inlineStr">
+      <c r="A4" s="98" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="87" t="inlineStr">
+      <c r="B4" s="98" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="87" t="inlineStr">
+      <c r="C4" s="98" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="87" t="inlineStr">
+      <c r="D4" s="98" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="87" t="inlineStr">
+      <c r="E4" s="98" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="87" t="inlineStr">
+      <c r="F4" s="98" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="87" t="inlineStr">
+      <c r="G4" s="98" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="87" t="inlineStr">
+      <c r="H4" s="98" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="87" t="inlineStr">
+      <c r="I4" s="98" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="87" t="inlineStr">
+      <c r="J4" s="98" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="87" t="inlineStr">
+      <c r="K4" s="98" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="87" t="inlineStr">
+      <c r="L4" s="98" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="87" t="inlineStr">
+      <c r="M4" s="98" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="87" t="inlineStr">
+      <c r="N4" s="98" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="87" t="inlineStr">
+      <c r="O4" s="98" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="87" t="inlineStr">
+      <c r="P4" s="98" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="87" t="inlineStr">
+      <c r="Q4" s="98" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
@@ -1713,58 +1728,81 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="88" t="inlineStr">
+      <c r="A7" s="99" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H7" s="89">
+      <c r="H7" s="100">
         <f>SUM(H5:H5)</f>
         <v/>
       </c>
-      <c r="I7" s="89">
+      <c r="I7" s="100">
         <f>SUM(I5:I5)</f>
         <v/>
       </c>
-      <c r="J7" s="89">
+      <c r="J7" s="100">
         <f>SUM(J5:J5)</f>
         <v/>
       </c>
-      <c r="K7" s="90">
+      <c r="K7" s="101">
         <f>IFERROR(J7/H7,"")</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="91" t="inlineStr">
-        <is>
-          <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
-        </is>
-      </c>
+      <c r="A9" s="102" t="inlineStr">
+        <is>
+          <t>INVESTMENT THESIS &amp; RESEARCH NOTES</t>
+        </is>
+      </c>
+      <c r="B9" s="103" t="n"/>
+      <c r="C9" s="103" t="n"/>
+      <c r="D9" s="103" t="n"/>
+      <c r="E9" s="103" t="n"/>
+      <c r="F9" s="103" t="n"/>
+      <c r="G9" s="103" t="n"/>
+      <c r="H9" s="103" t="n"/>
+      <c r="I9" s="103" t="n"/>
+      <c r="J9" s="103" t="n"/>
+      <c r="K9" s="103" t="n"/>
+      <c r="L9" s="103" t="n"/>
+      <c r="M9" s="103" t="n"/>
+      <c r="N9" s="103" t="n"/>
+      <c r="O9" s="103" t="n"/>
+      <c r="P9" s="103" t="n"/>
+      <c r="Q9" s="103" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  RKLB  —  Rocket Lab USA  |  Risk: High</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="409" customHeight="1">
-      <c r="A11" s="41" t="inlineStr">
-        <is>
-          <t>Huge future TAM over next decade+. Speculative but massive upside. Brilliant CEO. Near-term catalyst: SpaceX IPO in June.</t>
-        </is>
-      </c>
+      <c r="A10" s="41" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="B10" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Rocket Lab USA   |   Risk: High</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="43" t="n"/>
+      <c r="B11" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Huge future TAM over next decade+. Speculative but massive upside. Brilliant CEO. Near-term catalyst: SpaceX IPO in June.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="6" customHeight="1">
+      <c r="A12" s="45" t="n"/>
+      <c r="B12" s="45" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A9:Q9"/>
+  <mergeCells count="4">
     <mergeCell ref="A3:Q3"/>
     <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A10:Q10"/>
+    <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A7:G7"/>
-    <mergeCell ref="A11:Q11"/>
-    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="J5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -1793,11 +1831,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q14"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="130" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -1816,7 +1854,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="92" t="inlineStr">
+      <c r="A1" s="104" t="inlineStr">
         <is>
           <t>🔭 Long Term Watchlist</t>
         </is>
@@ -1832,102 +1870,102 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="93" t="inlineStr">
+      <c r="A4" s="105" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="93" t="inlineStr">
+      <c r="B4" s="105" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="93" t="inlineStr">
+      <c r="C4" s="105" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="93" t="inlineStr">
+      <c r="D4" s="105" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="93" t="inlineStr">
+      <c r="E4" s="105" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="93" t="inlineStr">
+      <c r="F4" s="105" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="93" t="inlineStr">
+      <c r="G4" s="105" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="93" t="inlineStr">
+      <c r="H4" s="105" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="93" t="inlineStr">
+      <c r="I4" s="105" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="93" t="inlineStr">
+      <c r="J4" s="105" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="93" t="inlineStr">
+      <c r="K4" s="105" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="93" t="inlineStr">
+      <c r="L4" s="105" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="93" t="inlineStr">
+      <c r="M4" s="105" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="93" t="inlineStr">
+      <c r="N4" s="105" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="93" t="inlineStr">
+      <c r="O4" s="105" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="93" t="inlineStr">
+      <c r="P4" s="105" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="93" t="inlineStr">
+      <c r="Q4" s="105" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
@@ -2069,74 +2107,105 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="94" t="inlineStr">
+      <c r="A8" s="106" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H8" s="95">
+      <c r="H8" s="107">
         <f>SUM(H5:H6)</f>
         <v/>
       </c>
-      <c r="I8" s="95">
+      <c r="I8" s="107">
         <f>SUM(I5:I6)</f>
         <v/>
       </c>
-      <c r="J8" s="95">
+      <c r="J8" s="107">
         <f>SUM(J5:J6)</f>
         <v/>
       </c>
-      <c r="K8" s="96">
+      <c r="K8" s="108">
         <f>IFERROR(J8/H8,"")</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="97" t="inlineStr">
-        <is>
-          <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
-        </is>
-      </c>
+      <c r="A10" s="109" t="inlineStr">
+        <is>
+          <t>INVESTMENT THESIS &amp; RESEARCH NOTES</t>
+        </is>
+      </c>
+      <c r="B10" s="110" t="n"/>
+      <c r="C10" s="110" t="n"/>
+      <c r="D10" s="110" t="n"/>
+      <c r="E10" s="110" t="n"/>
+      <c r="F10" s="110" t="n"/>
+      <c r="G10" s="110" t="n"/>
+      <c r="H10" s="110" t="n"/>
+      <c r="I10" s="110" t="n"/>
+      <c r="J10" s="110" t="n"/>
+      <c r="K10" s="110" t="n"/>
+      <c r="L10" s="110" t="n"/>
+      <c r="M10" s="110" t="n"/>
+      <c r="N10" s="110" t="n"/>
+      <c r="O10" s="110" t="n"/>
+      <c r="P10" s="110" t="n"/>
+      <c r="Q10" s="110" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  RBRK  —  Rubrik Inc  |  Risk: Med-High</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="409" customHeight="1">
-      <c r="A12" s="41" t="inlineStr">
-        <is>
-          <t>Long term investment research candidate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  NVO  —  Novo Nordisk  |  Risk: Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="409" customHeight="1">
-      <c r="A14" s="42" t="inlineStr">
-        <is>
-          <t>Long term investment research candidate.</t>
-        </is>
-      </c>
+      <c r="A11" s="41" t="inlineStr">
+        <is>
+          <t>RBRK</t>
+        </is>
+      </c>
+      <c r="B11" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Rubrik Inc   |   Risk: Med-High</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="43" t="n"/>
+      <c r="B12" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Long term investment research candidate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="6" customHeight="1">
+      <c r="A13" s="45" t="n"/>
+      <c r="B13" s="45" t="n"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="41" t="inlineStr">
+        <is>
+          <t>NVO</t>
+        </is>
+      </c>
+      <c r="B14" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Novo Nordisk   |   Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="45" t="n"/>
+      <c r="B15" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Long term investment research candidate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="6" customHeight="1">
+      <c r="A16" s="45" t="n"/>
+      <c r="B16" s="45" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A14:Q14"/>
+  <mergeCells count="4">
     <mergeCell ref="A3:Q3"/>
+    <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A12:Q12"/>
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A10:Q10"/>
-    <mergeCell ref="A11:Q11"/>
     <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="A13:Q13"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J6">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -2173,14 +2242,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="98" t="inlineStr">
+      <c r="A1" s="111" t="inlineStr">
         <is>
           <t>📝 RESEARCH NOTES &amp; INVESTMENT THESIS</t>
         </is>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1">
-      <c r="A2" s="99" t="inlineStr">
+      <c r="A2" s="112" t="inlineStr">
         <is>
           <t>401k To-Do</t>
         </is>
@@ -2193,7 +2262,7 @@
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="100" t="inlineStr">
+      <c r="A3" s="113" t="inlineStr">
         <is>
           <t>Savings Account</t>
         </is>
@@ -2205,7 +2274,7 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="99" t="inlineStr">
+      <c r="A4" s="112" t="inlineStr">
         <is>
           <t>Research Tools</t>
         </is>
@@ -2217,7 +2286,7 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="100" t="inlineStr">
+      <c r="A5" s="113" t="inlineStr">
         <is>
           <t>Quantum Thesis</t>
         </is>
@@ -2229,7 +2298,7 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="99" t="inlineStr">
+      <c r="A6" s="112" t="inlineStr">
         <is>
           <t>NVTS</t>
         </is>
@@ -2241,7 +2310,7 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="100" t="inlineStr">
+      <c r="A7" s="113" t="inlineStr">
         <is>
           <t>AEHR</t>
         </is>
@@ -2253,7 +2322,7 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="99" t="inlineStr">
+      <c r="A8" s="112" t="inlineStr">
         <is>
           <t>CRDO</t>
         </is>
@@ -2265,7 +2334,7 @@
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="100" t="inlineStr">
+      <c r="A9" s="113" t="inlineStr">
         <is>
           <t>ALGM</t>
         </is>
@@ -2277,7 +2346,7 @@
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="99" t="inlineStr">
+      <c r="A10" s="112" t="inlineStr">
         <is>
           <t>HIMX</t>
         </is>
@@ -2289,7 +2358,7 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="100" t="inlineStr">
+      <c r="A11" s="113" t="inlineStr">
         <is>
           <t>MTSI</t>
         </is>
@@ -2301,7 +2370,7 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="99" t="inlineStr">
+      <c r="A12" s="112" t="inlineStr">
         <is>
           <t>AEVA</t>
         </is>
@@ -2313,7 +2382,7 @@
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="100" t="inlineStr">
+      <c r="A13" s="113" t="inlineStr">
         <is>
           <t>AI Infrastructure</t>
         </is>
@@ -2325,7 +2394,7 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="99" t="inlineStr">
+      <c r="A14" s="112" t="inlineStr">
         <is>
           <t>LITE</t>
         </is>
@@ -2337,7 +2406,7 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="100" t="inlineStr">
+      <c r="A15" s="113" t="inlineStr">
         <is>
           <t>OKLO</t>
         </is>
@@ -2349,7 +2418,7 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="99" t="inlineStr">
+      <c r="A16" s="112" t="inlineStr">
         <is>
           <t>NBIS</t>
         </is>
@@ -2361,7 +2430,7 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="100" t="inlineStr">
+      <c r="A17" s="113" t="inlineStr">
         <is>
           <t>PLTR</t>
         </is>
@@ -2373,7 +2442,7 @@
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="99" t="inlineStr">
+      <c r="A18" s="112" t="inlineStr">
         <is>
           <t>ONDS</t>
         </is>
@@ -2385,7 +2454,7 @@
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="100" t="inlineStr">
+      <c r="A19" s="113" t="inlineStr">
         <is>
           <t>RKLB</t>
         </is>
@@ -2397,7 +2466,7 @@
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="99" t="inlineStr">
+      <c r="A20" s="112" t="inlineStr">
         <is>
           <t>Recommended Portfolio</t>
         </is>
@@ -2423,11 +2492,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="130" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -2462,7 +2531,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
         </is>
       </c>
     </row>
@@ -2791,65 +2860,104 @@
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="39" t="inlineStr">
         <is>
-          <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
-        </is>
-      </c>
+          <t>INVESTMENT THESIS &amp; RESEARCH NOTES</t>
+        </is>
+      </c>
+      <c r="B11" s="40" t="n"/>
+      <c r="C11" s="40" t="n"/>
+      <c r="D11" s="40" t="n"/>
+      <c r="E11" s="40" t="n"/>
+      <c r="F11" s="40" t="n"/>
+      <c r="G11" s="40" t="n"/>
+      <c r="H11" s="40" t="n"/>
+      <c r="I11" s="40" t="n"/>
+      <c r="J11" s="40" t="n"/>
+      <c r="K11" s="40" t="n"/>
+      <c r="L11" s="40" t="n"/>
+      <c r="M11" s="40" t="n"/>
+      <c r="N11" s="40" t="n"/>
+      <c r="O11" s="40" t="n"/>
+      <c r="P11" s="40" t="n"/>
+      <c r="Q11" s="40" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  IONQ  —  IonQ Inc  |  Risk: Very High</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="409" customHeight="1">
-      <c r="A13" s="41" t="inlineStr">
-        <is>
-          <t>Next quantum run candidate. Easy 10× within 2 years potential.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  RGTI  —  Rigetti Computing  |  Risk: Very High</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="409" customHeight="1">
-      <c r="A15" s="42" t="inlineStr">
-        <is>
-          <t>Next quantum run candidate. Easy 10× within 2 years potential.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  QBTS  —  D-Wave Quantum  |  Risk: Very High</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="409" customHeight="1">
-      <c r="A17" s="41" t="inlineStr">
-        <is>
-          <t>Next quantum run candidate. Easy 10× within 2 years potential.</t>
-        </is>
-      </c>
+      <c r="A12" s="41" t="inlineStr">
+        <is>
+          <t>IONQ</t>
+        </is>
+      </c>
+      <c r="B12" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  IonQ Inc   |   Risk: Very High</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="43" t="n"/>
+      <c r="B13" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Next quantum run candidate. Easy 10× within 2 years potential.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="6" customHeight="1">
+      <c r="A14" s="45" t="n"/>
+      <c r="B14" s="45" t="n"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="41" t="inlineStr">
+        <is>
+          <t>RGTI</t>
+        </is>
+      </c>
+      <c r="B15" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Rigetti Computing   |   Risk: Very High</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="45" t="n"/>
+      <c r="B16" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Next quantum run candidate. Easy 10× within 2 years potential.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="6" customHeight="1">
+      <c r="A17" s="45" t="n"/>
+      <c r="B17" s="45" t="n"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="41" t="inlineStr">
+        <is>
+          <t>QBTS</t>
+        </is>
+      </c>
+      <c r="B18" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  D-Wave Quantum   |   Risk: Very High</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="43" t="n"/>
+      <c r="B19" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Next quantum run candidate. Easy 10× within 2 years potential.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="6" customHeight="1">
+      <c r="A20" s="45" t="n"/>
+      <c r="B20" s="45" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A14:Q14"/>
-    <mergeCell ref="A17:Q17"/>
+  <mergeCells count="4">
+    <mergeCell ref="A3:Q3"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A9:G9"/>
-    <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="A12:Q12"/>
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A16:Q16"/>
-    <mergeCell ref="A15:Q15"/>
-    <mergeCell ref="A11:Q11"/>
-    <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="A13:Q13"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J7">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -2878,11 +2986,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q26"/>
+  <dimension ref="A1:Q32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="130" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -2901,7 +3009,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="43" t="inlineStr">
+      <c r="A1" s="47" t="inlineStr">
         <is>
           <t>🖥️ Semiconductors &amp; Compute</t>
         </is>
@@ -2917,102 +3025,102 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="44" t="inlineStr">
+      <c r="A4" s="48" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="44" t="inlineStr">
+      <c r="B4" s="48" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="44" t="inlineStr">
+      <c r="C4" s="48" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="44" t="inlineStr">
+      <c r="D4" s="48" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="44" t="inlineStr">
+      <c r="E4" s="48" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="44" t="inlineStr">
+      <c r="F4" s="48" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="44" t="inlineStr">
+      <c r="G4" s="48" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="44" t="inlineStr">
+      <c r="H4" s="48" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="44" t="inlineStr">
+      <c r="I4" s="48" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="44" t="inlineStr">
+      <c r="J4" s="48" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="44" t="inlineStr">
+      <c r="K4" s="48" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="44" t="inlineStr">
+      <c r="L4" s="48" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="44" t="inlineStr">
+      <c r="M4" s="48" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="44" t="inlineStr">
+      <c r="N4" s="48" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="44" t="inlineStr">
+      <c r="O4" s="48" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="44" t="inlineStr">
+      <c r="P4" s="48" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="44" t="inlineStr">
+      <c r="Q4" s="48" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
@@ -3110,7 +3218,7 @@
       <c r="E6" s="28" t="n">
         <v>425.44</v>
       </c>
-      <c r="F6" s="45" t="n">
+      <c r="F6" s="49" t="n">
         <v>-1.518517953378183</v>
       </c>
       <c r="G6" s="28" t="n">
@@ -3311,7 +3419,7 @@
       <c r="E9" s="28" t="n">
         <v>113.01</v>
       </c>
-      <c r="F9" s="45" t="n">
+      <c r="F9" s="49" t="n">
         <v>-0.2999540042077861</v>
       </c>
       <c r="G9" s="28" t="n">
@@ -3422,138 +3530,201 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="46" t="inlineStr">
+      <c r="A12" s="50" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H12" s="47">
+      <c r="H12" s="51">
         <f>SUM(H5:H10)</f>
         <v/>
       </c>
-      <c r="I12" s="47">
+      <c r="I12" s="51">
         <f>SUM(I5:I10)</f>
         <v/>
       </c>
-      <c r="J12" s="47">
+      <c r="J12" s="51">
         <f>SUM(J5:J10)</f>
         <v/>
       </c>
-      <c r="K12" s="48">
+      <c r="K12" s="52">
         <f>IFERROR(J12/H12,"")</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="49" t="inlineStr">
-        <is>
-          <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
-        </is>
-      </c>
+      <c r="A14" s="53" t="inlineStr">
+        <is>
+          <t>INVESTMENT THESIS &amp; RESEARCH NOTES</t>
+        </is>
+      </c>
+      <c r="B14" s="54" t="n"/>
+      <c r="C14" s="54" t="n"/>
+      <c r="D14" s="54" t="n"/>
+      <c r="E14" s="54" t="n"/>
+      <c r="F14" s="54" t="n"/>
+      <c r="G14" s="54" t="n"/>
+      <c r="H14" s="54" t="n"/>
+      <c r="I14" s="54" t="n"/>
+      <c r="J14" s="54" t="n"/>
+      <c r="K14" s="54" t="n"/>
+      <c r="L14" s="54" t="n"/>
+      <c r="M14" s="54" t="n"/>
+      <c r="N14" s="54" t="n"/>
+      <c r="O14" s="54" t="n"/>
+      <c r="P14" s="54" t="n"/>
+      <c r="Q14" s="54" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  NVDA  —  NVIDIA Corp  |  Risk: Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="409" customHeight="1">
-      <c r="A16" s="41" t="inlineStr">
-        <is>
-          <t>The AI compute king. Stability and steady compounder.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  AVGO  —  Broadcom Inc  |  Risk: Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="409" customHeight="1">
-      <c r="A18" s="42" t="inlineStr">
-        <is>
-          <t>Stability and steady compounder.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  LRCX  —  Lam Research  |  Risk: Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="409" customHeight="1">
-      <c r="A20" s="41" t="inlineStr">
-        <is>
-          <t>Stability and steady compounder. DRAM equipment leader.</t>
-        </is>
-      </c>
+      <c r="A15" s="41" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="B15" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NVIDIA Corp   |   Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="43" t="n"/>
+      <c r="B16" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  The AI compute king. Stability and steady compounder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="6" customHeight="1">
+      <c r="A17" s="45" t="n"/>
+      <c r="B17" s="45" t="n"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="41" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="B18" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Broadcom Inc   |   Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="45" t="n"/>
+      <c r="B19" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Stability and steady compounder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="6" customHeight="1">
+      <c r="A20" s="45" t="n"/>
+      <c r="B20" s="45" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  AMD  —  Advanced Micro Devices  |  Risk: Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="409" customHeight="1">
-      <c r="A22" s="42" t="inlineStr">
-        <is>
-          <t>CPU maker deep in the AI infrastructure stack.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  INTC  —  Intel Corp  |  Risk: Med-High</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="409" customHeight="1">
+      <c r="A21" s="41" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="B21" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lam Research   |   Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="43" t="n"/>
+      <c r="B22" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Stability and steady compounder. DRAM equipment leader.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="6" customHeight="1">
+      <c r="A23" s="45" t="n"/>
+      <c r="B23" s="45" t="n"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
       <c r="A24" s="41" t="inlineStr">
         <is>
-          <t>CPU maker in AI infrastructure stack. Turnaround story.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ARM  —  Arm Holdings  |  Risk: Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="409" customHeight="1">
-      <c r="A26" s="42" t="inlineStr">
-        <is>
-          <t>Architecture behind most AI edge chips. Royalty model.</t>
-        </is>
-      </c>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B24" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Advanced Micro Devices   |   Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="16" customHeight="1">
+      <c r="A25" s="45" t="n"/>
+      <c r="B25" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CPU maker deep in the AI infrastructure stack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="6" customHeight="1">
+      <c r="A26" s="45" t="n"/>
+      <c r="B26" s="45" t="n"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="41" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="B27" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Intel Corp   |   Risk: Med-High</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="16" customHeight="1">
+      <c r="A28" s="43" t="n"/>
+      <c r="B28" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CPU maker in AI infrastructure stack. Turnaround story.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="6" customHeight="1">
+      <c r="A29" s="45" t="n"/>
+      <c r="B29" s="45" t="n"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="41" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="B30" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Arm Holdings   |   Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="16" customHeight="1">
+      <c r="A31" s="45" t="n"/>
+      <c r="B31" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Architecture behind most AI edge chips. Royalty model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="6" customHeight="1">
+      <c r="A32" s="45" t="n"/>
+      <c r="B32" s="45" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="A14:Q14"/>
-    <mergeCell ref="A22:Q22"/>
-    <mergeCell ref="A17:Q17"/>
-    <mergeCell ref="A18:Q18"/>
+  <mergeCells count="4">
     <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="A21:Q21"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A12:G12"/>
-    <mergeCell ref="A20:Q20"/>
-    <mergeCell ref="A24:Q24"/>
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A16:Q16"/>
-    <mergeCell ref="A15:Q15"/>
-    <mergeCell ref="A26:Q26"/>
-    <mergeCell ref="A25:Q25"/>
-    <mergeCell ref="A19:Q19"/>
-    <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="A23:Q23"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J10">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -3582,11 +3753,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q29"/>
+  <dimension ref="A1:Q36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="130" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -3605,7 +3776,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="50" t="inlineStr">
+      <c r="A1" s="55" t="inlineStr">
         <is>
           <t>⚙️ AI Picks &amp; Shovels</t>
         </is>
@@ -3621,102 +3792,102 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="51" t="inlineStr">
+      <c r="A4" s="56" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="51" t="inlineStr">
+      <c r="B4" s="56" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="51" t="inlineStr">
+      <c r="C4" s="56" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="51" t="inlineStr">
+      <c r="D4" s="56" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="51" t="inlineStr">
+      <c r="E4" s="56" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="51" t="inlineStr">
+      <c r="F4" s="56" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="51" t="inlineStr">
+      <c r="G4" s="56" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="51" t="inlineStr">
+      <c r="H4" s="56" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="51" t="inlineStr">
+      <c r="I4" s="56" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="51" t="inlineStr">
+      <c r="J4" s="56" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="51" t="inlineStr">
+      <c r="K4" s="56" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="51" t="inlineStr">
+      <c r="L4" s="56" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="51" t="inlineStr">
+      <c r="M4" s="56" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="51" t="inlineStr">
+      <c r="N4" s="56" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="51" t="inlineStr">
+      <c r="O4" s="56" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="51" t="inlineStr">
+      <c r="P4" s="56" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="51" t="inlineStr">
+      <c r="Q4" s="56" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
@@ -3881,7 +4052,7 @@
       <c r="E7" s="28" t="n">
         <v>198.29</v>
       </c>
-      <c r="F7" s="45" t="n">
+      <c r="F7" s="49" t="n">
         <v>-0.1057968331824622</v>
       </c>
       <c r="G7" s="28" t="n">
@@ -4015,7 +4186,7 @@
       <c r="E9" s="28" t="n">
         <v>12.33</v>
       </c>
-      <c r="F9" s="45" t="n">
+      <c r="F9" s="49" t="n">
         <v>-0.2830576327856492</v>
       </c>
       <c r="G9" s="28" t="n">
@@ -4193,154 +4364,225 @@
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="52" t="inlineStr">
+      <c r="A13" s="57" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H13" s="53">
+      <c r="H13" s="58">
         <f>SUM(H5:H11)</f>
         <v/>
       </c>
-      <c r="I13" s="53">
+      <c r="I13" s="58">
         <f>SUM(I5:I11)</f>
         <v/>
       </c>
-      <c r="J13" s="53">
+      <c r="J13" s="58">
         <f>SUM(J5:J11)</f>
         <v/>
       </c>
-      <c r="K13" s="54">
+      <c r="K13" s="59">
         <f>IFERROR(J13/H13,"")</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="55" t="inlineStr">
-        <is>
-          <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
-        </is>
-      </c>
+      <c r="A15" s="60" t="inlineStr">
+        <is>
+          <t>INVESTMENT THESIS &amp; RESEARCH NOTES</t>
+        </is>
+      </c>
+      <c r="B15" s="61" t="n"/>
+      <c r="C15" s="61" t="n"/>
+      <c r="D15" s="61" t="n"/>
+      <c r="E15" s="61" t="n"/>
+      <c r="F15" s="61" t="n"/>
+      <c r="G15" s="61" t="n"/>
+      <c r="H15" s="61" t="n"/>
+      <c r="I15" s="61" t="n"/>
+      <c r="J15" s="61" t="n"/>
+      <c r="K15" s="61" t="n"/>
+      <c r="L15" s="61" t="n"/>
+      <c r="M15" s="61" t="n"/>
+      <c r="N15" s="61" t="n"/>
+      <c r="O15" s="61" t="n"/>
+      <c r="P15" s="61" t="n"/>
+      <c r="Q15" s="61" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  NVTS  —  Navitas Semiconductor  |  Risk: High</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="409" customHeight="1">
-      <c r="A17" s="41" t="inlineStr">
-        <is>
-          <t>AI data centers need radically more efficient power delivery. Picks-and-shovels for compute growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  AEHR  —  AEHR Test Systems  |  Risk: High</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="409" customHeight="1">
-      <c r="A19" s="42" t="inlineStr">
-        <is>
-          <t>Classic shovels in a gold rush. More AI chips = more testing bottleneck demand.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  CRDO  —  Credo Technology  |  Risk: High</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="409" customHeight="1">
-      <c r="A21" s="41" t="inlineStr">
-        <is>
-          <t>GPUs don't matter if data can't move between them. Cleanest AI infrastructure picks-and-shovels name.</t>
-        </is>
-      </c>
+      <c r="A16" s="41" t="inlineStr">
+        <is>
+          <t>NVTS</t>
+        </is>
+      </c>
+      <c r="B16" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Navitas Semiconductor   |   Risk: High</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="43" t="n"/>
+      <c r="B17" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AI data centers need radically more efficient power delivery. Picks-and-shovels for compute growth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="6" customHeight="1">
+      <c r="A18" s="45" t="n"/>
+      <c r="B18" s="45" t="n"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="41" t="inlineStr">
+        <is>
+          <t>AEHR</t>
+        </is>
+      </c>
+      <c r="B19" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AEHR Test Systems   |   Risk: High</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="45" t="n"/>
+      <c r="B20" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Classic shovels in a gold rush. More AI chips = more testing bottleneck demand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="6" customHeight="1">
+      <c r="A21" s="45" t="n"/>
+      <c r="B21" s="45" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ALGM  —  Allegro MicroSystems  |  Risk: Med-High</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="409" customHeight="1">
-      <c r="A23" s="42" t="inlineStr">
-        <is>
-          <t>Electrification + AI hardware power efficiency. Quiet compounder, early in AI rerating narrative.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  HIMX  —  Himax Technologies  |  Risk: High</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="409" customHeight="1">
+      <c r="A22" s="41" t="inlineStr">
+        <is>
+          <t>CRDO</t>
+        </is>
+      </c>
+      <c r="B22" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Credo Technology   |   Risk: High</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="43" t="n"/>
+      <c r="B23" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  GPUs don't matter if data can't move between them. Cleanest AI infrastructure picks-and-shovels name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="6" customHeight="1">
+      <c r="A24" s="45" t="n"/>
+      <c r="B24" s="45" t="n"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
       <c r="A25" s="41" t="inlineStr">
         <is>
-          <t>Exposure to AI edge devices + optics. Higher volatility, historically rerates fast on cycles.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  MTSI  —  MACOM Technology  |  Risk: Med-High</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="409" customHeight="1">
-      <c r="A27" s="42" t="inlineStr">
-        <is>
-          <t>AI datacenter interconnect + telecom backbone. Less hype, more industrial AI backbone exposure.</t>
-        </is>
-      </c>
+          <t>ALGM</t>
+        </is>
+      </c>
+      <c r="B25" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Allegro MicroSystems   |   Risk: Med-High</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="45" t="n"/>
+      <c r="B26" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Electrification + AI hardware power efficiency. Quiet compounder, early in AI rerating narrative.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="6" customHeight="1">
+      <c r="A27" s="45" t="n"/>
+      <c r="B27" s="45" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  AEVA  —  Aeva Technologies  |  Risk: Very High</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="409" customHeight="1">
-      <c r="A29" s="41" t="inlineStr">
-        <is>
-          <t>Autonomous systems + robotics long tail. Pure asymmetric bet: low probability, high upside.</t>
-        </is>
-      </c>
+      <c r="A28" s="41" t="inlineStr">
+        <is>
+          <t>HIMX</t>
+        </is>
+      </c>
+      <c r="B28" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Himax Technologies   |   Risk: High</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="16" customHeight="1">
+      <c r="A29" s="43" t="n"/>
+      <c r="B29" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Exposure to AI edge devices + optics. Higher volatility, historically rerates fast on cycles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="6" customHeight="1">
+      <c r="A30" s="45" t="n"/>
+      <c r="B30" s="45" t="n"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="41" t="inlineStr">
+        <is>
+          <t>MTSI</t>
+        </is>
+      </c>
+      <c r="B31" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MACOM Technology   |   Risk: Med-High</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="16" customHeight="1">
+      <c r="A32" s="45" t="n"/>
+      <c r="B32" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AI datacenter interconnect + telecom backbone. Less hype, more industrial AI backbone exposure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="6" customHeight="1">
+      <c r="A33" s="45" t="n"/>
+      <c r="B33" s="45" t="n"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="41" t="inlineStr">
+        <is>
+          <t>AEVA</t>
+        </is>
+      </c>
+      <c r="B34" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Aeva Technologies   |   Risk: Very High</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="A35" s="43" t="n"/>
+      <c r="B35" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Autonomous systems + robotics long tail. Pure asymmetric bet: low probability, high upside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="6" customHeight="1">
+      <c r="A36" s="45" t="n"/>
+      <c r="B36" s="45" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="A24:Q24"/>
-    <mergeCell ref="A15:Q15"/>
+  <mergeCells count="4">
+    <mergeCell ref="A3:Q3"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A13:G13"/>
     <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="A13:G13"/>
-    <mergeCell ref="A16:Q16"/>
-    <mergeCell ref="A25:Q25"/>
-    <mergeCell ref="A18:Q18"/>
-    <mergeCell ref="A27:Q27"/>
-    <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="A21:Q21"/>
-    <mergeCell ref="A26:Q26"/>
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A23:Q23"/>
-    <mergeCell ref="A22:Q22"/>
-    <mergeCell ref="A17:Q17"/>
-    <mergeCell ref="A29:Q29"/>
-    <mergeCell ref="A20:Q20"/>
-    <mergeCell ref="A28:Q28"/>
-    <mergeCell ref="A19:Q19"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J11">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -4369,11 +4611,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="130" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -4392,7 +4634,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="56" t="inlineStr">
+      <c r="A1" s="62" t="inlineStr">
         <is>
           <t>💡 Photonics &amp; Optics</t>
         </is>
@@ -4408,102 +4650,102 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="57" t="inlineStr">
+      <c r="A4" s="63" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="57" t="inlineStr">
+      <c r="B4" s="63" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="57" t="inlineStr">
+      <c r="C4" s="63" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="57" t="inlineStr">
+      <c r="D4" s="63" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="57" t="inlineStr">
+      <c r="E4" s="63" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="57" t="inlineStr">
+      <c r="F4" s="63" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="57" t="inlineStr">
+      <c r="G4" s="63" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="57" t="inlineStr">
+      <c r="H4" s="63" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="57" t="inlineStr">
+      <c r="I4" s="63" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="57" t="inlineStr">
+      <c r="J4" s="63" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="57" t="inlineStr">
+      <c r="K4" s="63" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="57" t="inlineStr">
+      <c r="L4" s="63" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="57" t="inlineStr">
+      <c r="M4" s="63" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="57" t="inlineStr">
+      <c r="N4" s="63" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="57" t="inlineStr">
+      <c r="O4" s="63" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="57" t="inlineStr">
+      <c r="P4" s="63" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="57" t="inlineStr">
+      <c r="Q4" s="63" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
@@ -4534,7 +4776,7 @@
       <c r="E5" s="28" t="n">
         <v>944.28</v>
       </c>
-      <c r="F5" s="45" t="n">
+      <c r="F5" s="49" t="n">
         <v>-1.642619728464659</v>
       </c>
       <c r="G5" s="28" t="n">
@@ -4578,58 +4820,81 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="58" t="inlineStr">
+      <c r="A7" s="64" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H7" s="59">
+      <c r="H7" s="65">
         <f>SUM(H5:H5)</f>
         <v/>
       </c>
-      <c r="I7" s="59">
+      <c r="I7" s="65">
         <f>SUM(I5:I5)</f>
         <v/>
       </c>
-      <c r="J7" s="59">
+      <c r="J7" s="65">
         <f>SUM(J5:J5)</f>
         <v/>
       </c>
-      <c r="K7" s="60">
+      <c r="K7" s="66">
         <f>IFERROR(J7/H7,"")</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="61" t="inlineStr">
-        <is>
-          <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
-        </is>
-      </c>
+      <c r="A9" s="67" t="inlineStr">
+        <is>
+          <t>INVESTMENT THESIS &amp; RESEARCH NOTES</t>
+        </is>
+      </c>
+      <c r="B9" s="68" t="n"/>
+      <c r="C9" s="68" t="n"/>
+      <c r="D9" s="68" t="n"/>
+      <c r="E9" s="68" t="n"/>
+      <c r="F9" s="68" t="n"/>
+      <c r="G9" s="68" t="n"/>
+      <c r="H9" s="68" t="n"/>
+      <c r="I9" s="68" t="n"/>
+      <c r="J9" s="68" t="n"/>
+      <c r="K9" s="68" t="n"/>
+      <c r="L9" s="68" t="n"/>
+      <c r="M9" s="68" t="n"/>
+      <c r="N9" s="68" t="n"/>
+      <c r="O9" s="68" t="n"/>
+      <c r="P9" s="68" t="n"/>
+      <c r="Q9" s="68" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  LITE  —  Lumentum Holdings  |  Risk: High</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="409" customHeight="1">
-      <c r="A11" s="41" t="inlineStr">
-        <is>
-          <t>King of Photonics. Could moonshot. Key bottleneck in AI data movement. Critical infrastructure.</t>
-        </is>
-      </c>
+      <c r="A10" s="41" t="inlineStr">
+        <is>
+          <t>LITE</t>
+        </is>
+      </c>
+      <c r="B10" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lumentum Holdings   |   Risk: High</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="43" t="n"/>
+      <c r="B11" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  King of Photonics. Could moonshot. Key bottleneck in AI data movement. Critical infrastructure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="6" customHeight="1">
+      <c r="A12" s="45" t="n"/>
+      <c r="B12" s="45" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A9:Q9"/>
+  <mergeCells count="4">
     <mergeCell ref="A3:Q3"/>
     <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A10:Q10"/>
+    <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A7:G7"/>
-    <mergeCell ref="A11:Q11"/>
-    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="J5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -4658,11 +4923,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:Q24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="130" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -4681,7 +4946,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="62" t="inlineStr">
+      <c r="A1" s="69" t="inlineStr">
         <is>
           <t>🏗️ DC Builders &amp; Cooling</t>
         </is>
@@ -4697,102 +4962,102 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="63" t="inlineStr">
+      <c r="A4" s="70" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="63" t="inlineStr">
+      <c r="B4" s="70" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="63" t="inlineStr">
+      <c r="C4" s="70" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="63" t="inlineStr">
+      <c r="D4" s="70" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="63" t="inlineStr">
+      <c r="E4" s="70" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="63" t="inlineStr">
+      <c r="F4" s="70" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="63" t="inlineStr">
+      <c r="G4" s="70" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="63" t="inlineStr">
+      <c r="H4" s="70" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="63" t="inlineStr">
+      <c r="I4" s="70" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="63" t="inlineStr">
+      <c r="J4" s="70" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="63" t="inlineStr">
+      <c r="K4" s="70" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="63" t="inlineStr">
+      <c r="L4" s="70" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="63" t="inlineStr">
+      <c r="M4" s="70" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="63" t="inlineStr">
+      <c r="N4" s="70" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="63" t="inlineStr">
+      <c r="O4" s="70" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="63" t="inlineStr">
+      <c r="P4" s="70" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="63" t="inlineStr">
+      <c r="Q4" s="70" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
@@ -5068,106 +5333,153 @@
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="64" t="inlineStr">
+      <c r="A10" s="71" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H10" s="65">
+      <c r="H10" s="72">
         <f>SUM(H5:H8)</f>
         <v/>
       </c>
-      <c r="I10" s="65">
+      <c r="I10" s="72">
         <f>SUM(I5:I8)</f>
         <v/>
       </c>
-      <c r="J10" s="65">
+      <c r="J10" s="72">
         <f>SUM(J5:J8)</f>
         <v/>
       </c>
-      <c r="K10" s="66">
+      <c r="K10" s="73">
         <f>IFERROR(J10/H10,"")</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="67" t="inlineStr">
-        <is>
-          <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
-        </is>
-      </c>
+      <c r="A12" s="74" t="inlineStr">
+        <is>
+          <t>INVESTMENT THESIS &amp; RESEARCH NOTES</t>
+        </is>
+      </c>
+      <c r="B12" s="75" t="n"/>
+      <c r="C12" s="75" t="n"/>
+      <c r="D12" s="75" t="n"/>
+      <c r="E12" s="75" t="n"/>
+      <c r="F12" s="75" t="n"/>
+      <c r="G12" s="75" t="n"/>
+      <c r="H12" s="75" t="n"/>
+      <c r="I12" s="75" t="n"/>
+      <c r="J12" s="75" t="n"/>
+      <c r="K12" s="75" t="n"/>
+      <c r="L12" s="75" t="n"/>
+      <c r="M12" s="75" t="n"/>
+      <c r="N12" s="75" t="n"/>
+      <c r="O12" s="75" t="n"/>
+      <c r="P12" s="75" t="n"/>
+      <c r="Q12" s="75" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  CAT  —  Caterpillar Inc  |  Risk: Low-Med</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="409" customHeight="1">
-      <c r="A14" s="41" t="inlineStr">
-        <is>
-          <t>Actual builder and materials company in the AI data center trade.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  FIX  —  Comfort Systems USA  |  Risk: Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="409" customHeight="1">
-      <c r="A16" s="42" t="inlineStr">
-        <is>
-          <t>Builder AND cooling company. AI data center HVAC &amp; MEP systems. Major growing bottleneck.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  POWL  —  Powell Industries  |  Risk: Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="409" customHeight="1">
-      <c r="A18" s="41" t="inlineStr">
-        <is>
-          <t>Electrical infrastructure builder for AI data centers.</t>
-        </is>
-      </c>
+      <c r="A13" s="41" t="inlineStr">
+        <is>
+          <t>CAT</t>
+        </is>
+      </c>
+      <c r="B13" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Caterpillar Inc   |   Risk: Low-Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="43" t="n"/>
+      <c r="B14" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Actual builder and materials company in the AI data center trade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="6" customHeight="1">
+      <c r="A15" s="45" t="n"/>
+      <c r="B15" s="45" t="n"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="41" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="B16" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Comfort Systems USA   |   Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="45" t="n"/>
+      <c r="B17" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Builder AND cooling company. AI data center HVAC &amp; MEP systems. Major growing bottleneck.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="6" customHeight="1">
+      <c r="A18" s="45" t="n"/>
+      <c r="B18" s="45" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  VRT  —  Vertiv Holdings  |  Risk: Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="409" customHeight="1">
-      <c r="A20" s="42" t="inlineStr">
-        <is>
-          <t>Premier AI data center cooling play. Cooling is a growing bottleneck.</t>
-        </is>
-      </c>
+      <c r="A19" s="41" t="inlineStr">
+        <is>
+          <t>POWL</t>
+        </is>
+      </c>
+      <c r="B19" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Powell Industries   |   Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="43" t="n"/>
+      <c r="B20" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Electrical infrastructure builder for AI data centers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="6" customHeight="1">
+      <c r="A21" s="45" t="n"/>
+      <c r="B21" s="45" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="41" t="inlineStr">
+        <is>
+          <t>VRT</t>
+        </is>
+      </c>
+      <c r="B22" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Vertiv Holdings   |   Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="45" t="n"/>
+      <c r="B23" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Premier AI data center cooling play. Cooling is a growing bottleneck.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="6" customHeight="1">
+      <c r="A24" s="45" t="n"/>
+      <c r="B24" s="45" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="A14:Q14"/>
-    <mergeCell ref="A17:Q17"/>
-    <mergeCell ref="A18:Q18"/>
+  <mergeCells count="4">
     <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="A12:Q12"/>
-    <mergeCell ref="A20:Q20"/>
     <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A16:Q16"/>
-    <mergeCell ref="A15:Q15"/>
-    <mergeCell ref="A19:Q19"/>
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A10:G10"/>
-    <mergeCell ref="A13:Q13"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J8">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -5196,11 +5508,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:Q24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="130" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -5219,7 +5531,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="68" t="inlineStr">
+      <c r="A1" s="76" t="inlineStr">
         <is>
           <t>⚡ Power &amp; Energy</t>
         </is>
@@ -5235,102 +5547,102 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="69" t="inlineStr">
+      <c r="A4" s="77" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="69" t="inlineStr">
+      <c r="B4" s="77" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="69" t="inlineStr">
+      <c r="C4" s="77" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="69" t="inlineStr">
+      <c r="D4" s="77" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="69" t="inlineStr">
+      <c r="E4" s="77" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="69" t="inlineStr">
+      <c r="F4" s="77" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="69" t="inlineStr">
+      <c r="G4" s="77" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="69" t="inlineStr">
+      <c r="H4" s="77" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="69" t="inlineStr">
+      <c r="I4" s="77" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="69" t="inlineStr">
+      <c r="J4" s="77" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="69" t="inlineStr">
+      <c r="K4" s="77" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="69" t="inlineStr">
+      <c r="L4" s="77" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="69" t="inlineStr">
+      <c r="M4" s="77" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="69" t="inlineStr">
+      <c r="N4" s="77" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="69" t="inlineStr">
+      <c r="O4" s="77" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="69" t="inlineStr">
+      <c r="P4" s="77" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="69" t="inlineStr">
+      <c r="Q4" s="77" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
@@ -5495,7 +5807,7 @@
       <c r="E7" s="28" t="n">
         <v>285.47</v>
       </c>
-      <c r="F7" s="45" t="n">
+      <c r="F7" s="49" t="n">
         <v>-4.067043441964675</v>
       </c>
       <c r="G7" s="28" t="n">
@@ -5606,106 +5918,153 @@
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="70" t="inlineStr">
+      <c r="A10" s="78" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H10" s="71">
+      <c r="H10" s="79">
         <f>SUM(H5:H8)</f>
         <v/>
       </c>
-      <c r="I10" s="71">
+      <c r="I10" s="79">
         <f>SUM(I5:I8)</f>
         <v/>
       </c>
-      <c r="J10" s="71">
+      <c r="J10" s="79">
         <f>SUM(J5:J8)</f>
         <v/>
       </c>
-      <c r="K10" s="72">
+      <c r="K10" s="80">
         <f>IFERROR(J10/H10,"")</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="73" t="inlineStr">
-        <is>
-          <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
-        </is>
-      </c>
+      <c r="A12" s="81" t="inlineStr">
+        <is>
+          <t>INVESTMENT THESIS &amp; RESEARCH NOTES</t>
+        </is>
+      </c>
+      <c r="B12" s="82" t="n"/>
+      <c r="C12" s="82" t="n"/>
+      <c r="D12" s="82" t="n"/>
+      <c r="E12" s="82" t="n"/>
+      <c r="F12" s="82" t="n"/>
+      <c r="G12" s="82" t="n"/>
+      <c r="H12" s="82" t="n"/>
+      <c r="I12" s="82" t="n"/>
+      <c r="J12" s="82" t="n"/>
+      <c r="K12" s="82" t="n"/>
+      <c r="L12" s="82" t="n"/>
+      <c r="M12" s="82" t="n"/>
+      <c r="N12" s="82" t="n"/>
+      <c r="O12" s="82" t="n"/>
+      <c r="P12" s="82" t="n"/>
+      <c r="Q12" s="82" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  GEV  —  GE Vernova  |  Risk: Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="409" customHeight="1">
-      <c r="A14" s="41" t="inlineStr">
-        <is>
-          <t>Stability and steady compounder. Power and grid maintenance for AI buildout.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  PWR  —  Quanta Services  |  Risk: Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="409" customHeight="1">
-      <c r="A16" s="42" t="inlineStr">
-        <is>
-          <t>Power generation and grid maintenance. Growing bottleneck for AI buildout.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  BE  —  Bloom Energy  |  Risk: High</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="409" customHeight="1">
-      <c r="A18" s="41" t="inlineStr">
-        <is>
-          <t>Moonshot potential if hydrogen &amp; fuel cell technology takes off.</t>
-        </is>
-      </c>
+      <c r="A13" s="41" t="inlineStr">
+        <is>
+          <t>GEV</t>
+        </is>
+      </c>
+      <c r="B13" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  GE Vernova   |   Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="43" t="n"/>
+      <c r="B14" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Stability and steady compounder. Power and grid maintenance for AI buildout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="6" customHeight="1">
+      <c r="A15" s="45" t="n"/>
+      <c r="B15" s="45" t="n"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="41" t="inlineStr">
+        <is>
+          <t>PWR</t>
+        </is>
+      </c>
+      <c r="B16" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Quanta Services   |   Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="45" t="n"/>
+      <c r="B17" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Power generation and grid maintenance. Growing bottleneck for AI buildout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="6" customHeight="1">
+      <c r="A18" s="45" t="n"/>
+      <c r="B18" s="45" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  OKLO  —  Oklo Inc  |  Risk: Very High</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="409" customHeight="1">
-      <c r="A20" s="42" t="inlineStr">
-        <is>
-          <t>Massive moonshot potential. Big regulatory &amp; execution risk. Worth a small % of portfolio given massive potential.</t>
-        </is>
-      </c>
+      <c r="A19" s="41" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="B19" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Bloom Energy   |   Risk: High</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="43" t="n"/>
+      <c r="B20" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Moonshot potential if hydrogen &amp; fuel cell technology takes off.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="6" customHeight="1">
+      <c r="A21" s="45" t="n"/>
+      <c r="B21" s="45" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="41" t="inlineStr">
+        <is>
+          <t>OKLO</t>
+        </is>
+      </c>
+      <c r="B22" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Oklo Inc   |   Risk: Very High</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="45" t="n"/>
+      <c r="B23" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Massive moonshot potential. Big regulatory &amp; execution risk. Worth a small % of portfolio given massive potential.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="6" customHeight="1">
+      <c r="A24" s="45" t="n"/>
+      <c r="B24" s="45" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="A14:Q14"/>
-    <mergeCell ref="A17:Q17"/>
-    <mergeCell ref="A18:Q18"/>
+  <mergeCells count="4">
     <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="A12:Q12"/>
-    <mergeCell ref="A20:Q20"/>
     <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A16:Q16"/>
-    <mergeCell ref="A15:Q15"/>
-    <mergeCell ref="A19:Q19"/>
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A10:G10"/>
-    <mergeCell ref="A13:Q13"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J8">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -5734,11 +6093,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q14"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="130" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -5757,7 +6116,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="74" t="inlineStr">
+      <c r="A1" s="83" t="inlineStr">
         <is>
           <t>☁️ Neoclouds &amp; AI Software</t>
         </is>
@@ -5773,102 +6132,102 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="75" t="inlineStr">
+      <c r="A4" s="84" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="75" t="inlineStr">
+      <c r="B4" s="84" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="75" t="inlineStr">
+      <c r="C4" s="84" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="75" t="inlineStr">
+      <c r="D4" s="84" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="75" t="inlineStr">
+      <c r="E4" s="84" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="75" t="inlineStr">
+      <c r="F4" s="84" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="75" t="inlineStr">
+      <c r="G4" s="84" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="75" t="inlineStr">
+      <c r="H4" s="84" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="75" t="inlineStr">
+      <c r="I4" s="84" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="75" t="inlineStr">
+      <c r="J4" s="84" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="75" t="inlineStr">
+      <c r="K4" s="84" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="75" t="inlineStr">
+      <c r="L4" s="84" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="75" t="inlineStr">
+      <c r="M4" s="84" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="75" t="inlineStr">
+      <c r="N4" s="84" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="75" t="inlineStr">
+      <c r="O4" s="84" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="75" t="inlineStr">
+      <c r="P4" s="84" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="75" t="inlineStr">
+      <c r="Q4" s="84" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
@@ -5966,7 +6325,7 @@
       <c r="E6" s="28" t="n">
         <v>133.79</v>
       </c>
-      <c r="F6" s="45" t="n">
+      <c r="F6" s="49" t="n">
         <v>-1.101424241474859</v>
       </c>
       <c r="G6" s="28" t="n">
@@ -6010,74 +6369,113 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="76" t="inlineStr">
+      <c r="A8" s="85" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H8" s="77">
+      <c r="H8" s="86">
         <f>SUM(H5:H6)</f>
         <v/>
       </c>
-      <c r="I8" s="77">
+      <c r="I8" s="86">
         <f>SUM(I5:I6)</f>
         <v/>
       </c>
-      <c r="J8" s="77">
+      <c r="J8" s="86">
         <f>SUM(J5:J6)</f>
         <v/>
       </c>
-      <c r="K8" s="78">
+      <c r="K8" s="87">
         <f>IFERROR(J8/H8,"")</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="79" t="inlineStr">
-        <is>
-          <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
-        </is>
-      </c>
+      <c r="A10" s="88" t="inlineStr">
+        <is>
+          <t>INVESTMENT THESIS &amp; RESEARCH NOTES</t>
+        </is>
+      </c>
+      <c r="B10" s="89" t="n"/>
+      <c r="C10" s="89" t="n"/>
+      <c r="D10" s="89" t="n"/>
+      <c r="E10" s="89" t="n"/>
+      <c r="F10" s="89" t="n"/>
+      <c r="G10" s="89" t="n"/>
+      <c r="H10" s="89" t="n"/>
+      <c r="I10" s="89" t="n"/>
+      <c r="J10" s="89" t="n"/>
+      <c r="K10" s="89" t="n"/>
+      <c r="L10" s="89" t="n"/>
+      <c r="M10" s="89" t="n"/>
+      <c r="N10" s="89" t="n"/>
+      <c r="O10" s="89" t="n"/>
+      <c r="P10" s="89" t="n"/>
+      <c r="Q10" s="89" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  NBIS  —  Nebius Group  |  Risk: High</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="409" customHeight="1">
-      <c r="A12" s="41" t="inlineStr">
-        <is>
-          <t>Leading Neocloud with multiple revenue streams (Clickhouse, AV Ride). Modern Amazon/Google style company. Could become a future Hyperscaler.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  PLTR  —  Palantir Technologies  |  Risk: Med-High</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="409" customHeight="1">
-      <c r="A14" s="42" t="inlineStr">
-        <is>
-          <t>Integral to the entire government AI stack. Not going anywhere. AI Software outlier outside the data center trade.</t>
-        </is>
-      </c>
+      <c r="A11" s="41" t="inlineStr">
+        <is>
+          <t>NBIS</t>
+        </is>
+      </c>
+      <c r="B11" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Nebius Group   |   Risk: High</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="43" t="n"/>
+      <c r="B12" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Leading Neocloud with multiple revenue streams (Clickhouse, AV Ride). Modern Amazon/Google style company. Could become a future</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="43" t="n"/>
+      <c r="B13" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Hyperscaler.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="6" customHeight="1">
+      <c r="A14" s="45" t="n"/>
+      <c r="B14" s="45" t="n"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="41" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="B15" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Palantir Technologies   |   Risk: Med-High</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="45" t="n"/>
+      <c r="B16" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Integral to the entire government AI stack. Not going anywhere. AI Software outlier outside the data center trade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="6" customHeight="1">
+      <c r="A17" s="45" t="n"/>
+      <c r="B17" s="45" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A14:Q14"/>
+  <mergeCells count="4">
     <mergeCell ref="A3:Q3"/>
+    <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A12:Q12"/>
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A10:Q10"/>
-    <mergeCell ref="A11:Q11"/>
     <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="A13:Q13"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J6">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -6106,11 +6504,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="130" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -6129,7 +6527,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="80" t="inlineStr">
+      <c r="A1" s="90" t="inlineStr">
         <is>
           <t>🛡️ Defense &amp; Drones</t>
         </is>
@@ -6145,102 +6543,102 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:33 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="81" t="inlineStr">
+      <c r="A4" s="91" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="81" t="inlineStr">
+      <c r="B4" s="91" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="81" t="inlineStr">
+      <c r="C4" s="91" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="81" t="inlineStr">
+      <c r="D4" s="91" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="81" t="inlineStr">
+      <c r="E4" s="91" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="81" t="inlineStr">
+      <c r="F4" s="91" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="81" t="inlineStr">
+      <c r="G4" s="91" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="81" t="inlineStr">
+      <c r="H4" s="91" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="81" t="inlineStr">
+      <c r="I4" s="91" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="81" t="inlineStr">
+      <c r="J4" s="91" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="81" t="inlineStr">
+      <c r="K4" s="91" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="81" t="inlineStr">
+      <c r="L4" s="91" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="81" t="inlineStr">
+      <c r="M4" s="91" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="81" t="inlineStr">
+      <c r="N4" s="91" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="81" t="inlineStr">
+      <c r="O4" s="91" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="81" t="inlineStr">
+      <c r="P4" s="91" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="81" t="inlineStr">
+      <c r="Q4" s="91" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
@@ -6315,58 +6713,89 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="82" t="inlineStr">
+      <c r="A7" s="92" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H7" s="83">
+      <c r="H7" s="93">
         <f>SUM(H5:H5)</f>
         <v/>
       </c>
-      <c r="I7" s="83">
+      <c r="I7" s="93">
         <f>SUM(I5:I5)</f>
         <v/>
       </c>
-      <c r="J7" s="83">
+      <c r="J7" s="93">
         <f>SUM(J5:J5)</f>
         <v/>
       </c>
-      <c r="K7" s="84">
+      <c r="K7" s="94">
         <f>IFERROR(J7/H7,"")</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="85" t="inlineStr">
-        <is>
-          <t>📌  INVESTMENT THESIS &amp; RESEARCH NOTES</t>
-        </is>
-      </c>
+      <c r="A9" s="95" t="inlineStr">
+        <is>
+          <t>INVESTMENT THESIS &amp; RESEARCH NOTES</t>
+        </is>
+      </c>
+      <c r="B9" s="96" t="n"/>
+      <c r="C9" s="96" t="n"/>
+      <c r="D9" s="96" t="n"/>
+      <c r="E9" s="96" t="n"/>
+      <c r="F9" s="96" t="n"/>
+      <c r="G9" s="96" t="n"/>
+      <c r="H9" s="96" t="n"/>
+      <c r="I9" s="96" t="n"/>
+      <c r="J9" s="96" t="n"/>
+      <c r="K9" s="96" t="n"/>
+      <c r="L9" s="96" t="n"/>
+      <c r="M9" s="96" t="n"/>
+      <c r="N9" s="96" t="n"/>
+      <c r="O9" s="96" t="n"/>
+      <c r="P9" s="96" t="n"/>
+      <c r="Q9" s="96" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ONDS  —  Ondas Holdings  |  Risk: Very High</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="409" customHeight="1">
-      <c r="A11" s="41" t="inlineStr">
-        <is>
-          <t>$1.5T defense budget, $56B to drones/counter-drones via DAWG Program. Best chance to scale after March 2026 acquisitions &amp; partnerships. Very speculative.</t>
-        </is>
-      </c>
+      <c r="A10" s="41" t="inlineStr">
+        <is>
+          <t>ONDS</t>
+        </is>
+      </c>
+      <c r="B10" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Ondas Holdings   |   Risk: Very High</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="43" t="n"/>
+      <c r="B11" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  $1.5T defense budget, $56B to drones/counter-drones via DAWG Program. Best chance to scale after March 2026 acquisitions &amp;</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="43" t="n"/>
+      <c r="B12" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  partnerships. Very speculative.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="6" customHeight="1">
+      <c r="A13" s="45" t="n"/>
+      <c r="B13" s="45" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A9:Q9"/>
+  <mergeCells count="4">
     <mergeCell ref="A3:Q3"/>
     <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A10:Q10"/>
+    <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A7:G7"/>
-    <mergeCell ref="A11:Q11"/>
-    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="J5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">

</xml_diff>

<commit_message>
Expand investment thesis notes for all stock categories
Updates the `.agents/agent_assets_metadata.toml` file to reflect a change in the title of the stock tracker. It also modifies `scripts/generate_financial_tracker.py` to include expanded and detailed notes for stocks within the "Quantum computing" and "Core semiconductor & compute names" categories.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 1fb81a51-bd60-4e30-b8b1-02cf3807d410
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1071,7 +1071,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1558,7 +1558,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
         </is>
       </c>
     </row>
@@ -1789,13 +1789,69 @@
       <c r="A11" s="43" t="n"/>
       <c r="B11" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Huge future TAM over next decade+. Speculative but massive upside. Brilliant CEO. Near-term catalyst: SpaceX IPO in June.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="6" customHeight="1">
-      <c r="A12" s="45" t="n"/>
-      <c r="B12" s="45" t="n"/>
+          <t xml:space="preserve">  Space economy and space infrastructure — huge future TAM over the next decade and beyond. Rocket Lab is the second most active</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="43" t="n"/>
+      <c r="B12" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  launch company in the world (after SpaceX) and is the only credible alternative for small and medium satellite launches. Their</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="43" t="n"/>
+      <c r="B13" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Electron rocket has an exceptional launch record, and the larger Neutron rocket (in development) is designed to compete with</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="43" t="n"/>
+      <c r="B14" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SpaceX's Falcon 9 for medium payloads. The CEO (Peter Beck) is brilliant and has consistently delivered on technical milestones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="43" t="n"/>
+      <c r="B15" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Near-term catalyst: the SpaceX IPO (expected June 2026) will drive massive media attention to the space economy, and RKLB will</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="43" t="n"/>
+      <c r="B16" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  benefit as the most investable public proxy. Longer term, Rocket Lab is building a vertically integrated space company</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="43" t="n"/>
+      <c r="B17" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (satellites, components, software, launch) which gives them multiple revenue streams. Speculative but with massive compounding</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="43" t="n"/>
+      <c r="B18" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  upside if they execute over the next 5-10 years.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="6" customHeight="1">
+      <c r="A19" s="45" t="n"/>
+      <c r="B19" s="45" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1831,7 +1887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:Q27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1870,7 +1926,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
         </is>
       </c>
     </row>
@@ -2168,37 +2224,125 @@
       <c r="A12" s="43" t="n"/>
       <c r="B12" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Long term investment research candidate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="6" customHeight="1">
-      <c r="A13" s="45" t="n"/>
-      <c r="B13" s="45" t="n"/>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="41" t="inlineStr">
+          <t xml:space="preserve">  Under active long-term evaluation. Rubrik is a cybersecurity and data management company focused on data resilience — protecting</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="43" t="n"/>
+      <c r="B13" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  enterprise data from ransomware, ensuring recoverability, and managing data across hybrid cloud environments. As AI adoption</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="43" t="n"/>
+      <c r="B14" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  accelerates, the volume and value of enterprise data explodes, making data protection and recovery increasingly critical. Rubrik</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="43" t="n"/>
+      <c r="B15" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  has a subscription-based revenue model (good for predictability) and is growing fast. The risk: the cybersecurity market is</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="43" t="n"/>
+      <c r="B16" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  crowded and competitive, and the valuation already prices in significant growth. Watch for: revenue acceleration, margin</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="43" t="n"/>
+      <c r="B17" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  improvement, and any signs of customer concentration. Add on weakness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="6" customHeight="1">
+      <c r="A18" s="45" t="n"/>
+      <c r="B18" s="45" t="n"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="41" t="inlineStr">
         <is>
           <t>NVO</t>
         </is>
       </c>
-      <c r="B14" s="42" t="inlineStr">
+      <c r="B19" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  Novo Nordisk   |   Risk: Medium</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="45" t="n"/>
-      <c r="B15" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Long term investment research candidate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="6" customHeight="1">
-      <c r="A16" s="45" t="n"/>
-      <c r="B16" s="45" t="n"/>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="45" t="n"/>
+      <c r="B20" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Under active long-term evaluation. Novo Nordisk is the global leader in GLP-1 drugs (Ozempic, Wegovy) for diabetes and obesity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="45" t="n"/>
+      <c r="B21" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  The obesity drug market is potentially the largest pharmaceutical market ever — hundreds of millions of people globally are</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="45" t="n"/>
+      <c r="B22" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  candidates for GLP-1 treatment, and early data suggests these drugs also reduce cardiovascular events, sleep apnea, and other</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="45" t="n"/>
+      <c r="B23" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  conditions beyond weight loss. Novo has the manufacturing scale, the brand recognition, and the clinical data to dominate this</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="45" t="n"/>
+      <c r="B24" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  market for years. The stock has pulled back significantly from its highs as competition from Eli Lilly (Mounjaro/Zepbound) has</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="16" customHeight="1">
+      <c r="A25" s="45" t="n"/>
+      <c r="B25" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  intensified — which creates a potentially attractive entry point. A long-term compounder in healthcare, completely uncorrelated to</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="45" t="n"/>
+      <c r="B26" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  the AI trade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="6" customHeight="1">
+      <c r="A27" s="45" t="n"/>
+      <c r="B27" s="45" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2492,7 +2636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:Q32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2531,7 +2675,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
         </is>
       </c>
     </row>
@@ -2896,61 +3040,157 @@
       <c r="A13" s="43" t="n"/>
       <c r="B13" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Next quantum run candidate. Easy 10× within 2 years potential.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="6" customHeight="1">
-      <c r="A14" s="45" t="n"/>
-      <c r="B14" s="45" t="n"/>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="41" t="inlineStr">
+          <t xml:space="preserve">  Next quantum run candidate. The belief: 'Buy IONQ, RGTI, and QBTS — easy 10x within 2 years.' IonQ is the most commercially</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="43" t="n"/>
+      <c r="B14" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  advanced pure-play quantum computing company, using trapped-ion technology which is considered one of the most promising paths to</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="43" t="n"/>
+      <c r="B15" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  fault-tolerant quantum computers. They already have paying customers (government, pharma, finance) and are generating real</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="43" t="n"/>
+      <c r="B16" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  revenue. When the next quantum hype cycle hits, IonQ will be the headline name that institutions pile into. Very speculative —</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="43" t="n"/>
+      <c r="B17" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  treat as a high-risk asymmetric bet and size position accordingly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="6" customHeight="1">
+      <c r="A18" s="45" t="n"/>
+      <c r="B18" s="45" t="n"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="41" t="inlineStr">
         <is>
           <t>RGTI</t>
         </is>
       </c>
-      <c r="B15" s="42" t="inlineStr">
+      <c r="B19" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rigetti Computing   |   Risk: Very High</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="45" t="n"/>
-      <c r="B16" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Next quantum run candidate. Easy 10× within 2 years potential.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="6" customHeight="1">
-      <c r="A17" s="45" t="n"/>
-      <c r="B17" s="45" t="n"/>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="41" t="inlineStr">
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="45" t="n"/>
+      <c r="B20" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Next quantum run candidate alongside IONQ and QBTS. Rigetti builds its own quantum processors and offers cloud-based quantum</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="45" t="n"/>
+      <c r="B21" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  computing access. It's a smaller, scrappier name than IonQ, which means more volatility but also more upside if they execute. The</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="45" t="n"/>
+      <c r="B22" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  company has been building out its QPU (quantum processing unit) roadmap and targeting commercial applications in chemistry,</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="45" t="n"/>
+      <c r="B23" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  logistics, and finance. When the next quantum narrative cycle accelerates, RGTI tends to move fast and hard. Pure asymmetric bet —</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="45" t="n"/>
+      <c r="B24" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  small position, high conviction on timing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="6" customHeight="1">
+      <c r="A25" s="45" t="n"/>
+      <c r="B25" s="45" t="n"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="41" t="inlineStr">
         <is>
           <t>QBTS</t>
         </is>
       </c>
-      <c r="B18" s="42" t="inlineStr">
+      <c r="B26" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  D-Wave Quantum   |   Risk: Very High</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="43" t="n"/>
-      <c r="B19" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Next quantum run candidate. Easy 10× within 2 years potential.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="6" customHeight="1">
-      <c r="A20" s="45" t="n"/>
-      <c r="B20" s="45" t="n"/>
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="43" t="n"/>
+      <c r="B27" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Next quantum run candidate alongside IONQ and RGTI. D-Wave is unique in that it uses quantum annealing rather than gate-based</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="16" customHeight="1">
+      <c r="A28" s="43" t="n"/>
+      <c r="B28" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  quantum computing, which makes it commercially viable TODAY for specific optimization problems — logistics, scheduling, materials</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="16" customHeight="1">
+      <c r="A29" s="43" t="n"/>
+      <c r="B29" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  discovery — that classical computers struggle with. It already has real enterprise customers generating recurring revenue. The</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="16" customHeight="1">
+      <c r="A30" s="43" t="n"/>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  commercial viability argument is stronger than most quantum names. Easy 10x potential if the next quantum hype cycle materializes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="16" customHeight="1">
+      <c r="A31" s="43" t="n"/>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Very speculative — size position accordingly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="6" customHeight="1">
+      <c r="A32" s="45" t="n"/>
+      <c r="B32" s="45" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2986,7 +3226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q32"/>
+  <dimension ref="A1:Q57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3025,7 +3265,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
         </is>
       </c>
     </row>
@@ -3591,71 +3831,71 @@
       <c r="A16" s="43" t="n"/>
       <c r="B16" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  The AI compute king. Stability and steady compounder.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="6" customHeight="1">
-      <c r="A17" s="45" t="n"/>
-      <c r="B17" s="45" t="n"/>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="41" t="inlineStr">
+          <t xml:space="preserve">  The AI compute king and the core stability position in this portfolio. NVIDIA doesn't just make GPUs — it has built the dominant</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="43" t="n"/>
+      <c r="B17" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  software ecosystem (CUDA) that makes its hardware nearly impossible to replace even if competitors close the hardware gap. Every</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="43" t="n"/>
+      <c r="B18" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  major hyperscaler (Google, Amazon, Microsoft, Meta) depends on NVIDIA for AI training. As AI spending continues to accelerate,</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="43" t="n"/>
+      <c r="B19" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NVIDIA captures the most direct revenue from every dollar spent on AI compute. This is a steady compounder that also has massive</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="43" t="n"/>
+      <c r="B20" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  upside as the AI buildout continues. Hold as a core long-term position.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="6" customHeight="1">
+      <c r="A21" s="45" t="n"/>
+      <c r="B21" s="45" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="41" t="inlineStr">
         <is>
           <t>AVGO</t>
         </is>
       </c>
-      <c r="B18" s="42" t="inlineStr">
+      <c r="B22" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  Broadcom Inc   |   Risk: Medium</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="45" t="n"/>
-      <c r="B19" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Stability and steady compounder.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="6" customHeight="1">
-      <c r="A20" s="45" t="n"/>
-      <c r="B20" s="45" t="n"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="41" t="inlineStr">
-        <is>
-          <t>LRCX</t>
-        </is>
-      </c>
-      <c r="B21" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Lam Research   |   Risk: Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="43" t="n"/>
-      <c r="B22" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Stability and steady compounder. DRAM equipment leader.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="6" customHeight="1">
+    <row r="23" ht="16" customHeight="1">
       <c r="A23" s="45" t="n"/>
-      <c r="B23" s="45" t="n"/>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="41" t="inlineStr">
-        <is>
-          <t>AMD</t>
-        </is>
-      </c>
-      <c r="B24" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Advanced Micro Devices   |   Risk: Medium</t>
+      <c r="B23" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Stability and steady compounder — one of the most reliable semiconductor businesses in the world. Broadcom makes the networking</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="45" t="n"/>
+      <c r="B24" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  chips that connect all the GPUs inside hyperscaler data centers. As AI clusters scale to hundreds of thousands of GPUs, the</t>
         </is>
       </c>
     </row>
@@ -3663,61 +3903,261 @@
       <c r="A25" s="45" t="n"/>
       <c r="B25" s="46" t="inlineStr">
         <is>
-          <t xml:space="preserve">  CPU maker deep in the AI infrastructure stack.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="6" customHeight="1">
+          <t xml:space="preserve">  networking infrastructure connecting them becomes more valuable and more complex. Broadcom also has a massive software revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1">
       <c r="A26" s="45" t="n"/>
-      <c r="B26" s="45" t="n"/>
-    </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="41" t="inlineStr">
+      <c r="B26" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  stream from its VMware acquisition that provides recurring cash flow stability. Management is world-class at capital allocation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="45" t="n"/>
+      <c r="B27" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  This is a core hold that compounds quietly while the AI buildout accelerates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="6" customHeight="1">
+      <c r="A28" s="45" t="n"/>
+      <c r="B28" s="45" t="n"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="41" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="B29" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lam Research   |   Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="16" customHeight="1">
+      <c r="A30" s="43" t="n"/>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Stability and steady compounder — DRAM equipment leader. Lam Research makes the etch and deposition equipment that builds memory</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="16" customHeight="1">
+      <c r="A31" s="43" t="n"/>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  chips (DRAM and NAND). AI requires massive amounts of high-bandwidth memory (HBM), and every HBM chip that gets manufactured</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="16" customHeight="1">
+      <c r="A32" s="43" t="n"/>
+      <c r="B32" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  requires Lam's tools. This gives Lam direct and durable exposure to the AI memory build-out without the volatility of owning the</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="A33" s="43" t="n"/>
+      <c r="B33" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  memory chipmakers directly. The business is highly recurring (installed base + consumables) and grows every time wafer starts</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="16" customHeight="1">
+      <c r="A34" s="43" t="n"/>
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  increase. A core picks-and-shovels play for the AI infrastructure trade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="6" customHeight="1">
+      <c r="A35" s="45" t="n"/>
+      <c r="B35" s="45" t="n"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="41" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B36" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Advanced Micro Devices   |   Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="16" customHeight="1">
+      <c r="A37" s="45" t="n"/>
+      <c r="B37" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CPU maker deep in the AI infrastructure stack and the only credible challenger to NVIDIA in AI accelerators. AMD's MI300X GPU is</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="16" customHeight="1">
+      <c r="A38" s="45" t="n"/>
+      <c r="B38" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  winning meaningful enterprise AI workloads, particularly inference, where customers want a cheaper alternative to NVIDIA's</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="16" customHeight="1">
+      <c r="A39" s="45" t="n"/>
+      <c r="B39" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  H100/H200. On the CPU side, AMD's EPYC chips power a huge share of hyperscaler server infrastructure. The AI narrative is also</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="16" customHeight="1">
+      <c r="A40" s="45" t="n"/>
+      <c r="B40" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  shifting down-stack into CPU makers — AMD benefits from both trends simultaneously. Risk: NVIDIA's software moat (CUDA) is still</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="16" customHeight="1">
+      <c r="A41" s="45" t="n"/>
+      <c r="B41" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  wide. But as a compounder and a hedge on NVIDIA dominance, AMD belongs in the portfolio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="6" customHeight="1">
+      <c r="A42" s="45" t="n"/>
+      <c r="B42" s="45" t="n"/>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="41" t="inlineStr">
         <is>
           <t>INTC</t>
         </is>
       </c>
-      <c r="B27" s="42" t="inlineStr">
+      <c r="B43" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  Intel Corp   |   Risk: Med-High</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="43" t="n"/>
-      <c r="B28" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  CPU maker in AI infrastructure stack. Turnaround story.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="6" customHeight="1">
-      <c r="A29" s="45" t="n"/>
-      <c r="B29" s="45" t="n"/>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="41" t="inlineStr">
+    <row r="44" ht="16" customHeight="1">
+      <c r="A44" s="43" t="n"/>
+      <c r="B44" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CPU maker in the AI infrastructure stack and the most controversial turnaround story in semiconductors. Intel lost its</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="16" customHeight="1">
+      <c r="A45" s="43" t="n"/>
+      <c r="B45" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  manufacturing lead to TSMC and its AI accelerator business to NVIDIA and AMD. The thesis here is a turnaround: new management,</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="16" customHeight="1">
+      <c r="A46" s="43" t="n"/>
+      <c r="B46" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  massive government subsidies via the CHIPS Act, and a path to reclaiming leading-edge manufacturing through its Intel Foundry</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="16" customHeight="1">
+      <c r="A47" s="43" t="n"/>
+      <c r="B47" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Services (IFS) division. If the turnaround works, INTC is deeply undervalued. If it doesn't, the downside is meaningful. This is a</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="16" customHeight="1">
+      <c r="A48" s="43" t="n"/>
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  higher-risk position — size it as a speculative turnaround bet, not a core hold. The AI infrastructure narrative (CPU makers</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="16" customHeight="1">
+      <c r="A49" s="43" t="n"/>
+      <c r="B49" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  shifting down-stack) gives it a tailwind even without a full recovery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="6" customHeight="1">
+      <c r="A50" s="45" t="n"/>
+      <c r="B50" s="45" t="n"/>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="41" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
-      <c r="B30" s="42" t="inlineStr">
+      <c r="B51" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  Arm Holdings   |   Risk: Medium</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="45" t="n"/>
-      <c r="B31" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Architecture behind most AI edge chips. Royalty model.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="6" customHeight="1">
-      <c r="A32" s="45" t="n"/>
-      <c r="B32" s="45" t="n"/>
+    <row r="52" ht="16" customHeight="1">
+      <c r="A52" s="45" t="n"/>
+      <c r="B52" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  The architecture behind nearly every AI chip that isn't an x86 CPU. ARM licenses its instruction set architecture to Apple,</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="16" customHeight="1">
+      <c r="A53" s="45" t="n"/>
+      <c r="B53" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Qualcomm, Amazon (Graviton), Google, NVIDIA, and dozens of others. Every time an AI edge chip, smartphone chip, or custom</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="16" customHeight="1">
+      <c r="A54" s="45" t="n"/>
+      <c r="B54" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  datacenter chip gets designed and sold, ARM earns a royalty. This is a pure royalty business model — no manufacturing risk, no</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="16" customHeight="1">
+      <c r="A55" s="45" t="n"/>
+      <c r="B55" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  inventory risk — just IP licensing that scales with every chip shipped globally. As AI moves to the edge (phones, cars, robots),</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="16" customHeight="1">
+      <c r="A56" s="45" t="n"/>
+      <c r="B56" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ARM's exposure compounds. The royalty rate per chip is also increasing as designs get more complex. A core compounder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="6" customHeight="1">
+      <c r="A57" s="45" t="n"/>
+      <c r="B57" s="45" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -3753,7 +4193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q36"/>
+  <dimension ref="A1:Q68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3792,7 +4232,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
         </is>
       </c>
     </row>
@@ -4425,71 +4865,71 @@
       <c r="A17" s="43" t="n"/>
       <c r="B17" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AI data centers need radically more efficient power delivery. Picks-and-shovels for compute growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="6" customHeight="1">
-      <c r="A18" s="45" t="n"/>
-      <c r="B18" s="45" t="n"/>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="41" t="inlineStr">
+          <t xml:space="preserve">  The NVDA-parallel picks-and-shovels bet for AI power. Navitas makes GaN (gallium nitride) power chips that are radically more</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="43" t="n"/>
+      <c r="B18" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  efficient than traditional silicon-based power delivery. AI data centers are hitting a hard wall on power density — the amount of</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="43" t="n"/>
+      <c r="B19" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  electricity you can push into a rack is physically limited by current power conversion technology. GaN solves this by converting</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="43" t="n"/>
+      <c r="B20" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  power more efficiently and at higher frequencies, enabling denser, cooler, more power-efficient data centers. As hyperscalers</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="43" t="n"/>
+      <c r="B21" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  build out hundreds of gigawatts of AI compute, NVTS stands to be a critical infrastructure supplier. High-risk, asymmetric upside</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="43" t="n"/>
+      <c r="B22" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  — the kind of bet that looks obvious in hindsight.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="6" customHeight="1">
+      <c r="A23" s="45" t="n"/>
+      <c r="B23" s="45" t="n"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="41" t="inlineStr">
         <is>
           <t>AEHR</t>
         </is>
       </c>
-      <c r="B19" s="42" t="inlineStr">
+      <c r="B24" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  AEHR Test Systems   |   Risk: High</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="45" t="n"/>
-      <c r="B20" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Classic shovels in a gold rush. More AI chips = more testing bottleneck demand.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="6" customHeight="1">
-      <c r="A21" s="45" t="n"/>
-      <c r="B21" s="45" t="n"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="41" t="inlineStr">
-        <is>
-          <t>CRDO</t>
-        </is>
-      </c>
-      <c r="B22" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Credo Technology   |   Risk: High</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="43" t="n"/>
-      <c r="B23" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  GPUs don't matter if data can't move between them. Cleanest AI infrastructure picks-and-shovels name.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="6" customHeight="1">
-      <c r="A24" s="45" t="n"/>
-      <c r="B24" s="45" t="n"/>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="41" t="inlineStr">
-        <is>
-          <t>ALGM</t>
-        </is>
-      </c>
-      <c r="B25" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Allegro MicroSystems   |   Risk: Med-High</t>
+    <row r="25" ht="16" customHeight="1">
+      <c r="A25" s="45" t="n"/>
+      <c r="B25" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Classic shovels-in-a-gold-rush setup. AEHR makes specialized semiconductor burn-in and test equipment used to stress-test chips</t>
         </is>
       </c>
     </row>
@@ -4497,31 +4937,31 @@
       <c r="A26" s="45" t="n"/>
       <c r="B26" s="46" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Electrification + AI hardware power efficiency. Quiet compounder, early in AI rerating narrative.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="6" customHeight="1">
+          <t xml:space="preserve">  before they ship. As AI chips become more complex and expensive (each H100 costs $30k+), the cost of shipping a defective chip</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="16" customHeight="1">
       <c r="A27" s="45" t="n"/>
-      <c r="B27" s="45" t="n"/>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="41" t="inlineStr">
-        <is>
-          <t>HIMX</t>
-        </is>
-      </c>
-      <c r="B28" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Himax Technologies   |   Risk: High</t>
+      <c r="B27" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  becomes enormous — which means chip manufacturers are investing heavily in advanced testing. More AI chips manufactured = more</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="16" customHeight="1">
+      <c r="A28" s="45" t="n"/>
+      <c r="B28" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  testing bottleneck demand = more AEHR revenue. The business is lumpy (large equipment orders), which creates volatility, but the</t>
         </is>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="43" t="n"/>
-      <c r="B29" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Exposure to AI edge devices + optics. Higher volatility, historically rerates fast on cycles.</t>
+      <c r="A29" s="45" t="n"/>
+      <c r="B29" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  long-term tailwind is durable. A pure picks-and-shovels beneficiary of the AI chip production ramp.</t>
         </is>
       </c>
     </row>
@@ -4532,36 +4972,36 @@
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="41" t="inlineStr">
         <is>
-          <t>MTSI</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B31" s="42" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MACOM Technology   |   Risk: Med-High</t>
+          <t xml:space="preserve">  Credo Technology   |   Risk: High</t>
         </is>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="45" t="n"/>
-      <c r="B32" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  AI datacenter interconnect + telecom backbone. Less hype, more industrial AI backbone exposure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="6" customHeight="1">
-      <c r="A33" s="45" t="n"/>
-      <c r="B33" s="45" t="n"/>
-    </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="41" t="inlineStr">
-        <is>
-          <t>AEVA</t>
-        </is>
-      </c>
-      <c r="B34" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Aeva Technologies   |   Risk: Very High</t>
+      <c r="A32" s="43" t="n"/>
+      <c r="B32" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  One of the cleanest AI infrastructure picks-and-shovels names available. GPUs are useless if the data can't move between them fast</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="A33" s="43" t="n"/>
+      <c r="B33" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  enough. Credo makes high-speed SerDes (serializer/deserializer) connectivity chips that are the plumbing inside AI data centers —</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="16" customHeight="1">
+      <c r="A34" s="43" t="n"/>
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  connecting GPUs to memory, switches, and storage at speeds that match the compute throughput. As AI clusters scale from thousands</t>
         </is>
       </c>
     </row>
@@ -4569,13 +5009,269 @@
       <c r="A35" s="43" t="n"/>
       <c r="B35" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Autonomous systems + robotics long tail. Pure asymmetric bet: low probability, high upside.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="6" customHeight="1">
-      <c r="A36" s="45" t="n"/>
-      <c r="B36" s="45" t="n"/>
+          <t xml:space="preserve">  to hundreds of thousands of GPUs, the interconnect bandwidth requirement explodes. Credo has direct customer relationships with</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="16" customHeight="1">
+      <c r="A36" s="43" t="n"/>
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  hyperscalers and is already generating real revenue from the AI buildout. Strong execution, growing bookings, and a durable</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="16" customHeight="1">
+      <c r="A37" s="43" t="n"/>
+      <c r="B37" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  structural tailwind.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="6" customHeight="1">
+      <c r="A38" s="45" t="n"/>
+      <c r="B38" s="45" t="n"/>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="41" t="inlineStr">
+        <is>
+          <t>ALGM</t>
+        </is>
+      </c>
+      <c r="B39" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Allegro MicroSystems   |   Risk: Med-High</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="16" customHeight="1">
+      <c r="A40" s="45" t="n"/>
+      <c r="B40" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A quiet compounder that is early in its AI rerating narrative. Allegro makes power management and sensing semiconductors used in</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="16" customHeight="1">
+      <c r="A41" s="45" t="n"/>
+      <c r="B41" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  automotive, industrial, and increasingly AI hardware applications. As AI hardware demands more precise power delivery and thermal</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="16" customHeight="1">
+      <c r="A42" s="45" t="n"/>
+      <c r="B42" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  sensing, Allegro's chips become more embedded in the data center infrastructure. The automotive exposure (EV power management)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="16" customHeight="1">
+      <c r="A43" s="45" t="n"/>
+      <c r="B43" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  provides a separate growth vector. Less hype than the pure-play AI names, which means it hasn't been fully rerated yet — creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="16" customHeight="1">
+      <c r="A44" s="45" t="n"/>
+      <c r="B44" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  a potential catch-up opportunity. More of a steady grower than a moonshot, but with meaningful upside as the narrative broadens.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="6" customHeight="1">
+      <c r="A45" s="45" t="n"/>
+      <c r="B45" s="45" t="n"/>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="41" t="inlineStr">
+        <is>
+          <t>HIMX</t>
+        </is>
+      </c>
+      <c r="B46" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Himax Technologies   |   Risk: High</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="16" customHeight="1">
+      <c r="A47" s="43" t="n"/>
+      <c r="B47" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  An often-overlooked ADR with cyclical breakout behavior. Himax makes display driver ICs and AI vision chips used in AR/VR devices,</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="16" customHeight="1">
+      <c r="A48" s="43" t="n"/>
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  automotive displays, and AI edge sensing applications. When AI edge device cycles accelerate — smartphones, AR glasses, smart</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="16" customHeight="1">
+      <c r="A49" s="43" t="n"/>
+      <c r="B49" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  cameras — Himax tends to move fast. It's historically undervalued relative to its revenue and has a pattern of sharp re-ratings on</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="16" customHeight="1">
+      <c r="A50" s="43" t="n"/>
+      <c r="B50" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  earnings beats during upcycles. The AR/AI vision chip exposure is genuinely interesting as AI moves from the cloud to the edge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="16" customHeight="1">
+      <c r="A51" s="43" t="n"/>
+      <c r="B51" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Higher volatility, but the kind of name that can double in a single cycle. Treat as a tactical position sized for the volatility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="6" customHeight="1">
+      <c r="A52" s="45" t="n"/>
+      <c r="B52" s="45" t="n"/>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="41" t="inlineStr">
+        <is>
+          <t>MTSI</t>
+        </is>
+      </c>
+      <c r="B53" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MACOM Technology   |   Risk: Med-High</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="16" customHeight="1">
+      <c r="A54" s="45" t="n"/>
+      <c r="B54" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Less hype, more industrial AI backbone. MACOM makes RF, microwave, and high-speed analog chips used in data center interconnects,</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="16" customHeight="1">
+      <c r="A55" s="45" t="n"/>
+      <c r="B55" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  telecom backbones, and defense systems. As AI data centers demand ever-higher bandwidth between racks and buildings, MACOM's</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="16" customHeight="1">
+      <c r="A56" s="45" t="n"/>
+      <c r="B56" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  optical and RF interconnect chips become critical infrastructure. The telecom angle also gives it exposure to 5G buildout and the</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="16" customHeight="1">
+      <c r="A57" s="45" t="n"/>
+      <c r="B57" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  long-term bandwidth expansion required to support AI inference at the edge. Not a headline name, but a steady grower with durable</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="16" customHeight="1">
+      <c r="A58" s="45" t="n"/>
+      <c r="B58" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  end-market demand. The kind of stock that compounds quietly while the hype goes elsewhere, then re-rates when the market catches</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="16" customHeight="1">
+      <c r="A59" s="45" t="n"/>
+      <c r="B59" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="6" customHeight="1">
+      <c r="A60" s="45" t="n"/>
+      <c r="B60" s="45" t="n"/>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="41" t="inlineStr">
+        <is>
+          <t>AEVA</t>
+        </is>
+      </c>
+      <c r="B61" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Aeva Technologies   |   Risk: Very High</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="16" customHeight="1">
+      <c r="A62" s="43" t="n"/>
+      <c r="B62" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Pure asymmetric bet — low probability, high upside if they execute. Aeva makes FMCW (frequency-modulated continuous-wave) lidar</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="16" customHeight="1">
+      <c r="A63" s="43" t="n"/>
+      <c r="B63" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  sensors for autonomous vehicles and robotics. Their approach is technically differentiated — FMCW lidar can detect velocity</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="16" customHeight="1">
+      <c r="A64" s="43" t="n"/>
+      <c r="B64" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  directly (not just position) and works better in adverse conditions than traditional lidar. The autonomous vehicle and robotics</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="16" customHeight="1">
+      <c r="A65" s="43" t="n"/>
+      <c r="B65" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  market is massive if it materializes, and Aeva would be a key sensing supplier. Still in early commercialization — revenue is</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="16" customHeight="1">
+      <c r="A66" s="43" t="n"/>
+      <c r="B66" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  minimal and the path to profitability is long. This is a speculative moonshot, not a core position. Size it as a lottery ticket:</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="16" customHeight="1">
+      <c r="A67" s="43" t="n"/>
+      <c r="B67" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  accept that it could go to zero, but the upside if robotics/AV take off is 10-20x.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="6" customHeight="1">
+      <c r="A68" s="45" t="n"/>
+      <c r="B68" s="45" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -4611,7 +5307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4650,7 +5346,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
         </is>
       </c>
     </row>
@@ -4881,13 +5577,61 @@
       <c r="A11" s="43" t="n"/>
       <c r="B11" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  King of Photonics. Could moonshot. Key bottleneck in AI data movement. Critical infrastructure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="6" customHeight="1">
-      <c r="A12" s="45" t="n"/>
-      <c r="B12" s="45" t="n"/>
+          <t xml:space="preserve">  King of Photonics — and this could be a genuine moonshot. Lumentum makes the optical components (lasers, transceivers, photonic</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="43" t="n"/>
+      <c r="B12" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  integrated circuits) that transmit data at the speed of light inside and between AI data centers. As AI clusters scale to hundreds</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="43" t="n"/>
+      <c r="B13" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  of thousands of GPUs spread across multiple buildings, the optical interconnect becomes the critical bottleneck — you can't run</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="43" t="n"/>
+      <c r="B14" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  copper cables at those distances and speeds. Lumentum is one of the few companies with the technology and scale to supply this</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="43" t="n"/>
+      <c r="B15" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  infrastructure. The AI tailwind here is massive and underappreciated. Photonics is the next big narrative after GPUs and power —</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="43" t="n"/>
+      <c r="B16" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  when the market wakes up to the data movement bottleneck, LITE is the headline name. High conviction, high risk, moonshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="43" t="n"/>
+      <c r="B17" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  potential.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="6" customHeight="1">
+      <c r="A18" s="45" t="n"/>
+      <c r="B18" s="45" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -4923,7 +5667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:Q44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4962,7 +5706,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
         </is>
       </c>
     </row>
@@ -5394,71 +6138,71 @@
       <c r="A14" s="43" t="n"/>
       <c r="B14" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Actual builder and materials company in the AI data center trade.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="6" customHeight="1">
-      <c r="A15" s="45" t="n"/>
-      <c r="B15" s="45" t="n"/>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="41" t="inlineStr">
+          <t xml:space="preserve">  The actual builder and materials company in the AI data center trade. AI data centers are physical buildings requiring massive</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="43" t="n"/>
+      <c r="B15" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  earthmoving, foundation work, and construction equipment — and Caterpillar is the dominant supplier of that heavy equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="43" t="n"/>
+      <c r="B16" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  globally. Every hyperscaler campus that Meta, Google, Microsoft, and Amazon builds requires CAT equipment on site. This is a</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="43" t="n"/>
+      <c r="B17" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  steadier, lower-volatility way to play the AI infrastructure buildout than the semiconductor names. CAT also benefits from</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="43" t="n"/>
+      <c r="B18" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  infrastructure spending more broadly (roads, bridges, energy projects) which provides diversification. A solid core position —</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="43" t="n"/>
+      <c r="B19" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  steady compounder with the AI tailwind as a bonus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="6" customHeight="1">
+      <c r="A20" s="45" t="n"/>
+      <c r="B20" s="45" t="n"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="41" t="inlineStr">
         <is>
           <t>FIX</t>
         </is>
       </c>
-      <c r="B16" s="42" t="inlineStr">
+      <c r="B21" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  Comfort Systems USA   |   Risk: Medium</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="45" t="n"/>
-      <c r="B17" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Builder AND cooling company. AI data center HVAC &amp; MEP systems. Major growing bottleneck.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="6" customHeight="1">
-      <c r="A18" s="45" t="n"/>
-      <c r="B18" s="45" t="n"/>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="41" t="inlineStr">
-        <is>
-          <t>POWL</t>
-        </is>
-      </c>
-      <c r="B19" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Powell Industries   |   Risk: Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="43" t="n"/>
-      <c r="B20" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Electrical infrastructure builder for AI data centers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="6" customHeight="1">
-      <c r="A21" s="45" t="n"/>
-      <c r="B21" s="45" t="n"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="41" t="inlineStr">
-        <is>
-          <t>VRT</t>
-        </is>
-      </c>
-      <c r="B22" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Vertiv Holdings   |   Risk: Medium</t>
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="45" t="n"/>
+      <c r="B22" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Builder AND cooling company — one of the best-positioned picks-and-shovels plays in the AI buildout. Comfort Systems provides</t>
         </is>
       </c>
     </row>
@@ -5466,13 +6210,173 @@
       <c r="A23" s="45" t="n"/>
       <c r="B23" s="46" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Premier AI data center cooling play. Cooling is a growing bottleneck.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="6" customHeight="1">
+          <t xml:space="preserve">  HVAC, mechanical, plumbing, and electrical systems for commercial buildings, including AI data centers. Cooling is a MAJOR and</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1">
       <c r="A24" s="45" t="n"/>
-      <c r="B24" s="45" t="n"/>
+      <c r="B24" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  growing bottleneck in AI data centers — every GPU cluster generates enormous heat that must be managed. FIX designs and installs</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="16" customHeight="1">
+      <c r="A25" s="45" t="n"/>
+      <c r="B25" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  the entire MEP (mechanical, electrical, plumbing) system that keeps these facilities running. They have direct contracts with</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="45" t="n"/>
+      <c r="B26" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  hyperscalers and are seeing demand accelerate as AI data center construction ramps. A quality business with real earnings growth,</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="45" t="n"/>
+      <c r="B27" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  not a speculative bet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="6" customHeight="1">
+      <c r="A28" s="45" t="n"/>
+      <c r="B28" s="45" t="n"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="41" t="inlineStr">
+        <is>
+          <t>POWL</t>
+        </is>
+      </c>
+      <c r="B29" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Powell Industries   |   Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="16" customHeight="1">
+      <c r="A30" s="43" t="n"/>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Electrical infrastructure builder for AI data centers — the company that builds the switchgear, motor control centers, and power</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="16" customHeight="1">
+      <c r="A31" s="43" t="n"/>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  distribution equipment that routes electricity inside data centers and industrial facilities. As AI data centers require ever-</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="16" customHeight="1">
+      <c r="A32" s="43" t="n"/>
+      <c r="B32" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  larger amounts of power (some campus projects exceed 1 GW), the electrical infrastructure to safely distribute that power becomes</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="A33" s="43" t="n"/>
+      <c r="B33" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  a critical bottleneck. Powell has a backlog-heavy business model with long-cycle orders, which means revenue visibility is strong.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="16" customHeight="1">
+      <c r="A34" s="43" t="n"/>
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Less volatile than the semiconductor names because of the order backlog and industrial nature of the business. A solid mid-cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="A35" s="43" t="n"/>
+      <c r="B35" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  infrastructure pick with a genuine AI tailwind.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="6" customHeight="1">
+      <c r="A36" s="45" t="n"/>
+      <c r="B36" s="45" t="n"/>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="41" t="inlineStr">
+        <is>
+          <t>VRT</t>
+        </is>
+      </c>
+      <c r="B37" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Vertiv Holdings   |   Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="16" customHeight="1">
+      <c r="A38" s="45" t="n"/>
+      <c r="B38" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  The premier AI data center cooling play and one of the most direct beneficiaries of the AI buildout. Vertiv makes thermal</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="16" customHeight="1">
+      <c r="A39" s="45" t="n"/>
+      <c r="B39" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  management systems (liquid cooling, air cooling, heat exchangers) along with power distribution infrastructure for data centers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="16" customHeight="1">
+      <c r="A40" s="45" t="n"/>
+      <c r="B40" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Cooling is not optional — you cannot run a GPU cluster without solving the thermal problem, and as GPU power consumption has</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="16" customHeight="1">
+      <c r="A41" s="45" t="n"/>
+      <c r="B41" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  exploded from 300W to 700W per chip, existing cooling infrastructure is completely inadequate. Every new AI data center that gets</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="16" customHeight="1">
+      <c r="A42" s="45" t="n"/>
+      <c r="B42" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  built needs Vertiv's systems. The company has multi-year backlog, growing margins, and is adding capacity to meet demand. A high-</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="16" customHeight="1">
+      <c r="A43" s="45" t="n"/>
+      <c r="B43" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  conviction hold in the AI infrastructure basket.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="6" customHeight="1">
+      <c r="A44" s="45" t="n"/>
+      <c r="B44" s="45" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -5508,7 +6412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:Q46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5547,7 +6451,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
         </is>
       </c>
     </row>
@@ -5979,71 +6883,71 @@
       <c r="A14" s="43" t="n"/>
       <c r="B14" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Stability and steady compounder. Power and grid maintenance for AI buildout.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="6" customHeight="1">
-      <c r="A15" s="45" t="n"/>
-      <c r="B15" s="45" t="n"/>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="41" t="inlineStr">
+          <t xml:space="preserve">  Stability and steady compounder — the premier power generation and grid equipment company spun out of GE. GE Vernova makes gas</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="43" t="n"/>
+      <c r="B15" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  turbines, wind turbines, grid software, and electrification equipment. AI data centers are consuming power at a rate that is</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="43" t="n"/>
+      <c r="B16" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  straining the US electrical grid, and new power generation capacity takes years to build. GE Vernova is one of the few companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="43" t="n"/>
+      <c r="B17" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  with the scale and installed base to actually supply that new capacity fast. Their gas turbine backlog is multi-year and growing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="43" t="n"/>
+      <c r="B18" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  This is not a speculative bet — it's a high-quality industrial compounder with a very real and durable demand tailwind from AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="43" t="n"/>
+      <c r="B19" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  power needs. A core long-term hold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="6" customHeight="1">
+      <c r="A20" s="45" t="n"/>
+      <c r="B20" s="45" t="n"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="41" t="inlineStr">
         <is>
           <t>PWR</t>
         </is>
       </c>
-      <c r="B16" s="42" t="inlineStr">
+      <c r="B21" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  Quanta Services   |   Risk: Medium</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="45" t="n"/>
-      <c r="B17" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Power generation and grid maintenance. Growing bottleneck for AI buildout.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="6" customHeight="1">
-      <c r="A18" s="45" t="n"/>
-      <c r="B18" s="45" t="n"/>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="41" t="inlineStr">
-        <is>
-          <t>BE</t>
-        </is>
-      </c>
-      <c r="B19" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Bloom Energy   |   Risk: High</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="43" t="n"/>
-      <c r="B20" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Moonshot potential if hydrogen &amp; fuel cell technology takes off.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="6" customHeight="1">
-      <c r="A21" s="45" t="n"/>
-      <c r="B21" s="45" t="n"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="41" t="inlineStr">
-        <is>
-          <t>OKLO</t>
-        </is>
-      </c>
-      <c r="B22" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Oklo Inc   |   Risk: Very High</t>
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="45" t="n"/>
+      <c r="B22" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Power grid infrastructure and maintenance — a growing bottleneck for the AI buildout. Quanta Services is the largest specialty</t>
         </is>
       </c>
     </row>
@@ -6051,13 +6955,189 @@
       <c r="A23" s="45" t="n"/>
       <c r="B23" s="46" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Massive moonshot potential. Big regulatory &amp; execution risk. Worth a small % of portfolio given massive potential.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="6" customHeight="1">
+          <t xml:space="preserve">  contractor for electric power infrastructure in North America. They build and maintain power lines, substations, and grid</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1">
       <c r="A24" s="45" t="n"/>
-      <c r="B24" s="45" t="n"/>
+      <c r="B24" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  connections that are essential to delivering electricity to AI data centers. Every new data center campus needs a grid connection,</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="16" customHeight="1">
+      <c r="A25" s="45" t="n"/>
+      <c r="B25" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  often requiring new transmission lines and substations — all of which Quanta builds. The company has multi-year visibility through</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="45" t="n"/>
+      <c r="B26" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  its backlog and framework agreements with utilities. A steady, high-quality compounder that benefits directly and durably from the</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="45" t="n"/>
+      <c r="B27" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AI power demand surge. Lower volatility than the semiconductor names with a comparably strong tailwind.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="6" customHeight="1">
+      <c r="A28" s="45" t="n"/>
+      <c r="B28" s="45" t="n"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="41" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="B29" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Bloom Energy   |   Risk: High</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="16" customHeight="1">
+      <c r="A30" s="43" t="n"/>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Moonshot potential if hydrogen and fuel cell technology takes off — and the AI power crisis is accelerating the timeline. Bloom</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="16" customHeight="1">
+      <c r="A31" s="43" t="n"/>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Energy makes solid oxide fuel cells that generate electricity on-site without connecting to the grid. For AI data centers that</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="16" customHeight="1">
+      <c r="A32" s="43" t="n"/>
+      <c r="B32" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  need reliable, clean, on-site power (especially in areas with grid congestion), Bloom's solution is genuinely compelling. They're</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="A33" s="43" t="n"/>
+      <c r="B33" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  already selling to data centers and have partnerships with major tech companies. The bull case: AI power demand is so acute that</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="16" customHeight="1">
+      <c r="A34" s="43" t="n"/>
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  on-site generation becomes mandatory, and Bloom is uniquely positioned. The bear case: fuel cells are expensive and hydrogen</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="A35" s="43" t="n"/>
+      <c r="B35" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  infrastructure is still nascent. Worth holding a position — the upside if they win even a small share of the AI power market is</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="16" customHeight="1">
+      <c r="A36" s="43" t="n"/>
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  very large.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="6" customHeight="1">
+      <c r="A37" s="45" t="n"/>
+      <c r="B37" s="45" t="n"/>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="41" t="inlineStr">
+        <is>
+          <t>OKLO</t>
+        </is>
+      </c>
+      <c r="B38" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Oklo Inc   |   Risk: Very High</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="16" customHeight="1">
+      <c r="A39" s="45" t="n"/>
+      <c r="B39" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Nuclear SMRs and nuclear fuel waste company with massive moonshot potential — but big regulatory and execution risk. Oklo is</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="16" customHeight="1">
+      <c r="A40" s="45" t="n"/>
+      <c r="B40" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  building small modular nuclear reactors (SMRs) that could provide clean, always-on baseload power for AI data centers at scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="16" customHeight="1">
+      <c r="A41" s="45" t="n"/>
+      <c r="B41" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Several major tech companies (including Microsoft) have already signed nuclear power agreements, signaling that nuclear is being</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="16" customHeight="1">
+      <c r="A42" s="45" t="n"/>
+      <c r="B42" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  taken seriously as an AI power solution. Oklo also has a fuel recycling angle (using spent nuclear fuel) that could be a</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="16" customHeight="1">
+      <c r="A43" s="45" t="n"/>
+      <c r="B43" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  significant business in itself. The regulatory path is long and uncertain, and Oklo has not yet built a commercial reactor. This</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="16" customHeight="1">
+      <c r="A44" s="45" t="n"/>
+      <c r="B44" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  is a small-% portfolio position — accept that it could go to zero, but the upside if nuclear SMRs get commercially deployed is</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="16" customHeight="1">
+      <c r="A45" s="45" t="n"/>
+      <c r="B45" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  enormous and the valuation reflects very little of that potential today.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="6" customHeight="1">
+      <c r="A46" s="45" t="n"/>
+      <c r="B46" s="45" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -6093,7 +7173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6132,7 +7212,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
         </is>
       </c>
     </row>
@@ -6430,7 +7510,7 @@
       <c r="A12" s="43" t="n"/>
       <c r="B12" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Leading Neocloud with multiple revenue streams (Clickhouse, AV Ride). Modern Amazon/Google style company. Could become a future</t>
+          <t xml:space="preserve">  The leading Neocloud and one of the most interesting companies in this portfolio. Nebius is a modern Amazon/Google-style company:</t>
         </is>
       </c>
     </row>
@@ -6438,37 +7518,125 @@
       <c r="A13" s="43" t="n"/>
       <c r="B13" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Hyperscaler.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="6" customHeight="1">
-      <c r="A14" s="45" t="n"/>
-      <c r="B14" s="45" t="n"/>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="41" t="inlineStr">
+          <t xml:space="preserve">  it has a primary product (GPU cloud computing for AI companies that can't get capacity from AWS/Azure/GCP) AND multiple other</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="43" t="n"/>
+      <c r="B14" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  revenue streams that could each become massive independently — Clickhouse (high-performance analytics database used by thousands</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="43" t="n"/>
+      <c r="B15" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  of companies), AV Ride (autonomous vehicle tech), and others. The neocloud thesis: hyperscalers are capacity-constrained and have</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="43" t="n"/>
+      <c r="B16" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  long waitlists for GPU compute, creating a massive opening for alternative cloud providers. NBIS is the best-positioned name to</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="43" t="n"/>
+      <c r="B17" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  fill that gap. I believe this company could become a future Hyperscaler in the same way Amazon AWS or Google Cloud became defining</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="43" t="n"/>
+      <c r="B18" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  infrastructure businesses. High conviction, long-term hold — this is the kind of company you look back on in 10 years and wish you</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="43" t="n"/>
+      <c r="B19" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  owned more of.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="6" customHeight="1">
+      <c r="A20" s="45" t="n"/>
+      <c r="B20" s="45" t="n"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="41" t="inlineStr">
         <is>
           <t>PLTR</t>
         </is>
       </c>
-      <c r="B15" s="42" t="inlineStr">
+      <c r="B21" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  Palantir Technologies   |   Risk: Med-High</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="45" t="n"/>
-      <c r="B16" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Integral to the entire government AI stack. Not going anywhere. AI Software outlier outside the data center trade.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="6" customHeight="1">
-      <c r="A17" s="45" t="n"/>
-      <c r="B17" s="45" t="n"/>
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="45" t="n"/>
+      <c r="B22" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  So integral to the entire US government AI stack that it is effectively a national security asset. Palantir's software (Gotham for</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="45" t="n"/>
+      <c r="B23" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  government, Foundry for enterprise, AIP for AI) is deeply embedded in the Department of Defense, intelligence agencies, and dozens</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="45" t="n"/>
+      <c r="B24" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  of federal programs. You don't rip out Palantir — agencies build entire workflows on top of it. The AI Platform (AIP) is now being</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="16" customHeight="1">
+      <c r="A25" s="45" t="n"/>
+      <c r="B25" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  adopted by commercial enterprises as well, opening a second growth vector. The $1.5T defense budget and accelerating government AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="45" t="n"/>
+      <c r="B26" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  spending is a direct tailwind. Yes, the valuation is demanding, but for a company this strategically embedded, the premium is</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="45" t="n"/>
+      <c r="B27" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  arguably justified. An outlier name outside the data center trade that belongs in a long-term AI portfolio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="6" customHeight="1">
+      <c r="A28" s="45" t="n"/>
+      <c r="B28" s="45" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -6504,7 +7672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6543,7 +7711,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:38 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
         </is>
       </c>
     </row>
@@ -6774,7 +7942,7 @@
       <c r="A11" s="43" t="n"/>
       <c r="B11" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  $1.5T defense budget, $56B to drones/counter-drones via DAWG Program. Best chance to scale after March 2026 acquisitions &amp;</t>
+          <t xml:space="preserve">  Drones and defense tech — very speculative but with a massive catalyst behind it. The US government just announced a $1.5 trillion</t>
         </is>
       </c>
     </row>
@@ -6782,13 +7950,53 @@
       <c r="A12" s="43" t="n"/>
       <c r="B12" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  partnerships. Very speculative.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="6" customHeight="1">
-      <c r="A13" s="45" t="n"/>
-      <c r="B13" s="45" t="n"/>
+          <t xml:space="preserve">  defense budget with $56 billion going specifically to drones and counter-drones through the DAWG (Drone and Autonomous Warfare</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="43" t="n"/>
+      <c r="B13" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Group) program. Ondas is one of the few small-cap companies with actual drone technology, recent acquisitions in the space, and</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="43" t="n"/>
+      <c r="B14" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  partnerships that position them to compete for these contracts. Their March 2026 acquisitions and partnerships were specifically</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="43" t="n"/>
+      <c r="B15" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  designed to make them a stronger DAWG program competitor. This is not a guaranteed win — it's a very speculative bet on a small</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="43" t="n"/>
+      <c r="B16" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  company winning government contracts in a highly competitive space. But if they win even a small slice of the $56B drone budget,</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="43" t="n"/>
+      <c r="B17" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  the upside from current levels is enormous. Size it appropriately — this could go to zero or it could 5-10x.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="6" customHeight="1">
+      <c r="A18" s="45" t="n"/>
+      <c r="B18" s="45" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Display full investment notes in financial tracker
Update script to ensure all text in the 'notes' column of the Financial_Stock_Tracker.xlsx is fully visible by enabling text wrapping and increasing row height.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: c95ceed4-127f-4b36-9a74-43bcd86517dc
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -458,11 +458,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="23" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="23" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1071,7 +1071,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q19"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1558,7 +1558,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
         </is>
       </c>
     </row>
@@ -1785,74 +1785,15 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="16" customHeight="1">
+    <row r="11" ht="250" customHeight="1">
       <c r="A11" s="43" t="n"/>
       <c r="B11" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Space economy and space infrastructure — huge future TAM over the next decade and beyond. Rocket Lab is the second most active</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="43" t="n"/>
-      <c r="B12" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  launch company in the world (after SpaceX) and is the only credible alternative for small and medium satellite launches. Their</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="43" t="n"/>
-      <c r="B13" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Electron rocket has an exceptional launch record, and the larger Neutron rocket (in development) is designed to compete with</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="43" t="n"/>
-      <c r="B14" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SpaceX's Falcon 9 for medium payloads. The CEO (Peter Beck) is brilliant and has consistently delivered on technical milestones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="43" t="n"/>
-      <c r="B15" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Near-term catalyst: the SpaceX IPO (expected June 2026) will drive massive media attention to the space economy, and RKLB will</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="43" t="n"/>
-      <c r="B16" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  benefit as the most investable public proxy. Longer term, Rocket Lab is building a vertically integrated space company</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="43" t="n"/>
-      <c r="B17" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  (satellites, components, software, launch) which gives them multiple revenue streams. Speculative but with massive compounding</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="43" t="n"/>
-      <c r="B18" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  upside if they execute over the next 5-10 years.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="6" customHeight="1">
-      <c r="A19" s="45" t="n"/>
-      <c r="B19" s="45" t="n"/>
-    </row>
+          <t>Space economy and space infrastructure — huge future TAM over the next decade and beyond. Rocket Lab is the second most active launch company in the world (after SpaceX) and is the only credible alternative for small and medium satellite launches. Their Electron rocket has an exceptional launch record, and the larger Neutron rocket (in development) is designed to compete with SpaceX's Falcon 9 for medium payloads. The CEO (Peter Beck) is brilliant and has consistently delivered on technical milestones. Near-term catalyst: the SpaceX IPO (expected June 2026) will drive massive media attention to the space economy, and RKLB will benefit as the most investable public proxy. Longer term, Rocket Lab is building a vertically integrated space company (satellites, components, software, launch) which gives them multiple revenue streams. Speculative but with massive compounding upside if they execute over the next 5-10 years.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A3:Q3"/>
@@ -1887,7 +1828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q27"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1926,7 +1867,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
         </is>
       </c>
     </row>
@@ -2220,130 +2161,36 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="16" customHeight="1">
+    <row r="12" ht="250" customHeight="1">
       <c r="A12" s="43" t="n"/>
       <c r="B12" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Under active long-term evaluation. Rubrik is a cybersecurity and data management company focused on data resilience — protecting</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="43" t="n"/>
-      <c r="B13" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  enterprise data from ransomware, ensuring recoverability, and managing data across hybrid cloud environments. As AI adoption</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="43" t="n"/>
-      <c r="B14" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  accelerates, the volume and value of enterprise data explodes, making data protection and recovery increasingly critical. Rubrik</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="43" t="n"/>
-      <c r="B15" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  has a subscription-based revenue model (good for predictability) and is growing fast. The risk: the cybersecurity market is</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="43" t="n"/>
-      <c r="B16" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  crowded and competitive, and the valuation already prices in significant growth. Watch for: revenue acceleration, margin</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="43" t="n"/>
-      <c r="B17" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  improvement, and any signs of customer concentration. Add on weakness.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="6" customHeight="1">
-      <c r="A18" s="45" t="n"/>
-      <c r="B18" s="45" t="n"/>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="41" t="inlineStr">
+          <t>Under active long-term evaluation. Rubrik is a cybersecurity and data management company focused on data resilience — protecting enterprise data from ransomware, ensuring recoverability, and managing data across hybrid cloud environments. As AI adoption accelerates, the volume and value of enterprise data explodes, making data protection and recovery increasingly critical. Rubrik has a subscription-based revenue model (good for predictability) and is growing fast. The risk: the cybersecurity market is crowded and competitive, and the valuation already prices in significant growth. Watch for: revenue acceleration, margin improvement, and any signs of customer concentration. Add on weakness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="8" customHeight="1"/>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="41" t="inlineStr">
         <is>
           <t>NVO</t>
         </is>
       </c>
-      <c r="B19" s="42" t="inlineStr">
+      <c r="B14" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  Novo Nordisk   |   Risk: Medium</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="45" t="n"/>
-      <c r="B20" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Under active long-term evaluation. Novo Nordisk is the global leader in GLP-1 drugs (Ozempic, Wegovy) for diabetes and obesity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="45" t="n"/>
-      <c r="B21" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  The obesity drug market is potentially the largest pharmaceutical market ever — hundreds of millions of people globally are</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="45" t="n"/>
-      <c r="B22" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  candidates for GLP-1 treatment, and early data suggests these drugs also reduce cardiovascular events, sleep apnea, and other</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="45" t="n"/>
-      <c r="B23" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  conditions beyond weight loss. Novo has the manufacturing scale, the brand recognition, and the clinical data to dominate this</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="45" t="n"/>
-      <c r="B24" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  market for years. The stock has pulled back significantly from its highs as competition from Eli Lilly (Mounjaro/Zepbound) has</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="45" t="n"/>
-      <c r="B25" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  intensified — which creates a potentially attractive entry point. A long-term compounder in healthcare, completely uncorrelated to</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="45" t="n"/>
-      <c r="B26" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  the AI trade.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="6" customHeight="1">
-      <c r="A27" s="45" t="n"/>
-      <c r="B27" s="45" t="n"/>
-    </row>
+    <row r="15" ht="250" customHeight="1">
+      <c r="A15" s="45" t="n"/>
+      <c r="B15" s="46" t="inlineStr">
+        <is>
+          <t>Under active long-term evaluation. Novo Nordisk is the global leader in GLP-1 drugs (Ozempic, Wegovy) for diabetes and obesity. The obesity drug market is potentially the largest pharmaceutical market ever — hundreds of millions of people globally are candidates for GLP-1 treatment, and early data suggests these drugs also reduce cardiovascular events, sleep apnea, and other conditions beyond weight loss. Novo has the manufacturing scale, the brand recognition, and the clinical data to dominate this market for years. The stock has pulled back significantly from its highs as competition from Eli Lilly (Mounjaro/Zepbound) has intensified — which creates a potentially attractive entry point. A long-term compounder in healthcare, completely uncorrelated to the AI trade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A3:Q3"/>
@@ -2636,7 +2483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q32"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2675,7 +2522,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
         </is>
       </c>
     </row>
@@ -3036,162 +2883,57 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="16" customHeight="1">
+    <row r="13" ht="250" customHeight="1">
       <c r="A13" s="43" t="n"/>
       <c r="B13" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Next quantum run candidate. The belief: 'Buy IONQ, RGTI, and QBTS — easy 10x within 2 years.' IonQ is the most commercially</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="43" t="n"/>
-      <c r="B14" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  advanced pure-play quantum computing company, using trapped-ion technology which is considered one of the most promising paths to</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="43" t="n"/>
-      <c r="B15" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  fault-tolerant quantum computers. They already have paying customers (government, pharma, finance) and are generating real</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="43" t="n"/>
-      <c r="B16" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  revenue. When the next quantum hype cycle hits, IonQ will be the headline name that institutions pile into. Very speculative —</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="43" t="n"/>
-      <c r="B17" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  treat as a high-risk asymmetric bet and size position accordingly.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="6" customHeight="1">
-      <c r="A18" s="45" t="n"/>
-      <c r="B18" s="45" t="n"/>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="41" t="inlineStr">
+          <t>Next quantum run candidate. The belief: 'Buy IONQ, RGTI, and QBTS — easy 10x within 2 years.' IonQ is the most commercially advanced pure-play quantum computing company, using trapped-ion technology which is considered one of the most promising paths to fault-tolerant quantum computers. They already have paying customers (government, pharma, finance) and are generating real revenue. When the next quantum hype cycle hits, IonQ will be the headline name that institutions pile into. Very speculative — treat as a high-risk asymmetric bet and size position accordingly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="8" customHeight="1"/>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="41" t="inlineStr">
         <is>
           <t>RGTI</t>
         </is>
       </c>
-      <c r="B19" s="42" t="inlineStr">
+      <c r="B15" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rigetti Computing   |   Risk: Very High</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="45" t="n"/>
-      <c r="B20" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Next quantum run candidate alongside IONQ and QBTS. Rigetti builds its own quantum processors and offers cloud-based quantum</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="45" t="n"/>
-      <c r="B21" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  computing access. It's a smaller, scrappier name than IonQ, which means more volatility but also more upside if they execute. The</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="45" t="n"/>
-      <c r="B22" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  company has been building out its QPU (quantum processing unit) roadmap and targeting commercial applications in chemistry,</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="45" t="n"/>
-      <c r="B23" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  logistics, and finance. When the next quantum narrative cycle accelerates, RGTI tends to move fast and hard. Pure asymmetric bet —</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="45" t="n"/>
-      <c r="B24" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  small position, high conviction on timing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="6" customHeight="1">
-      <c r="A25" s="45" t="n"/>
-      <c r="B25" s="45" t="n"/>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="41" t="inlineStr">
+    <row r="16" ht="250" customHeight="1">
+      <c r="A16" s="45" t="n"/>
+      <c r="B16" s="46" t="inlineStr">
+        <is>
+          <t>Next quantum run candidate alongside IONQ and QBTS. Rigetti builds its own quantum processors and offers cloud-based quantum computing access. It's a smaller, scrappier name than IonQ, which means more volatility but also more upside if they execute. The company has been building out its QPU (quantum processing unit) roadmap and targeting commercial applications in chemistry, logistics, and finance. When the next quantum narrative cycle accelerates, RGTI tends to move fast and hard. Pure asymmetric bet — small position, high conviction on timing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="8" customHeight="1"/>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="41" t="inlineStr">
         <is>
           <t>QBTS</t>
         </is>
       </c>
-      <c r="B26" s="42" t="inlineStr">
+      <c r="B18" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  D-Wave Quantum   |   Risk: Very High</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="43" t="n"/>
-      <c r="B27" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Next quantum run candidate alongside IONQ and RGTI. D-Wave is unique in that it uses quantum annealing rather than gate-based</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="43" t="n"/>
-      <c r="B28" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  quantum computing, which makes it commercially viable TODAY for specific optimization problems — logistics, scheduling, materials</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="43" t="n"/>
-      <c r="B29" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  discovery — that classical computers struggle with. It already has real enterprise customers generating recurring revenue. The</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="43" t="n"/>
-      <c r="B30" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  commercial viability argument is stronger than most quantum names. Easy 10x potential if the next quantum hype cycle materializes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="43" t="n"/>
-      <c r="B31" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Very speculative — size position accordingly.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="6" customHeight="1">
-      <c r="A32" s="45" t="n"/>
-      <c r="B32" s="45" t="n"/>
-    </row>
+    <row r="19" ht="250" customHeight="1">
+      <c r="A19" s="43" t="n"/>
+      <c r="B19" s="44" t="inlineStr">
+        <is>
+          <t>Next quantum run candidate alongside IONQ and RGTI. D-Wave is unique in that it uses quantum annealing rather than gate-based quantum computing, which makes it commercially viable TODAY for specific optimization problems — logistics, scheduling, materials discovery — that classical computers struggle with. It already has real enterprise customers generating recurring revenue. The commercial viability argument is stronger than most quantum names. Easy 10x potential if the next quantum hype cycle materializes. Very speculative — size position accordingly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A3:Q3"/>
@@ -3226,7 +2968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q57"/>
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3265,7 +3007,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
         </is>
       </c>
     </row>
@@ -3827,338 +3569,120 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="16" customHeight="1">
+    <row r="16" ht="250" customHeight="1">
       <c r="A16" s="43" t="n"/>
       <c r="B16" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  The AI compute king and the core stability position in this portfolio. NVIDIA doesn't just make GPUs — it has built the dominant</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="43" t="n"/>
-      <c r="B17" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  software ecosystem (CUDA) that makes its hardware nearly impossible to replace even if competitors close the hardware gap. Every</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="43" t="n"/>
-      <c r="B18" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  major hyperscaler (Google, Amazon, Microsoft, Meta) depends on NVIDIA for AI training. As AI spending continues to accelerate,</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="43" t="n"/>
-      <c r="B19" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  NVIDIA captures the most direct revenue from every dollar spent on AI compute. This is a steady compounder that also has massive</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="43" t="n"/>
-      <c r="B20" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  upside as the AI buildout continues. Hold as a core long-term position.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="6" customHeight="1">
-      <c r="A21" s="45" t="n"/>
-      <c r="B21" s="45" t="n"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="41" t="inlineStr">
+          <t>The AI compute king and the core stability position in this portfolio. NVIDIA doesn't just make GPUs — it has built the dominant software ecosystem (CUDA) that makes its hardware nearly impossible to replace even if competitors close the hardware gap. Every major hyperscaler (Google, Amazon, Microsoft, Meta) depends on NVIDIA for AI training. As AI spending continues to accelerate, NVIDIA captures the most direct revenue from every dollar spent on AI compute. This is a steady compounder that also has massive upside as the AI buildout continues. Hold as a core long-term position.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="8" customHeight="1"/>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="41" t="inlineStr">
         <is>
           <t>AVGO</t>
         </is>
       </c>
-      <c r="B22" s="42" t="inlineStr">
+      <c r="B18" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  Broadcom Inc   |   Risk: Medium</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="45" t="n"/>
-      <c r="B23" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Stability and steady compounder — one of the most reliable semiconductor businesses in the world. Broadcom makes the networking</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="45" t="n"/>
-      <c r="B24" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  chips that connect all the GPUs inside hyperscaler data centers. As AI clusters scale to hundreds of thousands of GPUs, the</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="16" customHeight="1">
+    <row r="19" ht="250" customHeight="1">
+      <c r="A19" s="45" t="n"/>
+      <c r="B19" s="46" t="inlineStr">
+        <is>
+          <t>Stability and steady compounder — one of the most reliable semiconductor businesses in the world. Broadcom makes the networking chips that connect all the GPUs inside hyperscaler data centers. As AI clusters scale to hundreds of thousands of GPUs, the networking infrastructure connecting them becomes more valuable and more complex. Broadcom also has a massive software revenue stream from its VMware acquisition that provides recurring cash flow stability. Management is world-class at capital allocation. This is a core hold that compounds quietly while the AI buildout accelerates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="8" customHeight="1"/>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="41" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="B21" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lam Research   |   Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="250" customHeight="1">
+      <c r="A22" s="43" t="n"/>
+      <c r="B22" s="44" t="inlineStr">
+        <is>
+          <t>Stability and steady compounder — DRAM equipment leader. Lam Research makes the etch and deposition equipment that builds memory chips (DRAM and NAND). AI requires massive amounts of high-bandwidth memory (HBM), and every HBM chip that gets manufactured requires Lam's tools. This gives Lam direct and durable exposure to the AI memory build-out without the volatility of owning the memory chipmakers directly. The business is highly recurring (installed base + consumables) and grows every time wafer starts increase. A core picks-and-shovels play for the AI infrastructure trade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="8" customHeight="1"/>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="41" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B24" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Advanced Micro Devices   |   Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="250" customHeight="1">
       <c r="A25" s="45" t="n"/>
       <c r="B25" s="46" t="inlineStr">
         <is>
-          <t xml:space="preserve">  networking infrastructure connecting them becomes more valuable and more complex. Broadcom also has a massive software revenue</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="45" t="n"/>
-      <c r="B26" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  stream from its VMware acquisition that provides recurring cash flow stability. Management is world-class at capital allocation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="45" t="n"/>
-      <c r="B27" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  This is a core hold that compounds quietly while the AI buildout accelerates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="6" customHeight="1">
-      <c r="A28" s="45" t="n"/>
-      <c r="B28" s="45" t="n"/>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="41" t="inlineStr">
-        <is>
-          <t>LRCX</t>
-        </is>
-      </c>
-      <c r="B29" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Lam Research   |   Risk: Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="43" t="n"/>
-      <c r="B30" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Stability and steady compounder — DRAM equipment leader. Lam Research makes the etch and deposition equipment that builds memory</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="43" t="n"/>
-      <c r="B31" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  chips (DRAM and NAND). AI requires massive amounts of high-bandwidth memory (HBM), and every HBM chip that gets manufactured</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="43" t="n"/>
-      <c r="B32" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  requires Lam's tools. This gives Lam direct and durable exposure to the AI memory build-out without the volatility of owning the</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="43" t="n"/>
-      <c r="B33" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  memory chipmakers directly. The business is highly recurring (installed base + consumables) and grows every time wafer starts</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="43" t="n"/>
-      <c r="B34" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  increase. A core picks-and-shovels play for the AI infrastructure trade.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="6" customHeight="1">
-      <c r="A35" s="45" t="n"/>
-      <c r="B35" s="45" t="n"/>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="41" t="inlineStr">
-        <is>
-          <t>AMD</t>
-        </is>
-      </c>
-      <c r="B36" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Advanced Micro Devices   |   Risk: Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="16" customHeight="1">
-      <c r="A37" s="45" t="n"/>
-      <c r="B37" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  CPU maker deep in the AI infrastructure stack and the only credible challenger to NVIDIA in AI accelerators. AMD's MI300X GPU is</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="16" customHeight="1">
-      <c r="A38" s="45" t="n"/>
-      <c r="B38" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  winning meaningful enterprise AI workloads, particularly inference, where customers want a cheaper alternative to NVIDIA's</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="45" t="n"/>
-      <c r="B39" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  H100/H200. On the CPU side, AMD's EPYC chips power a huge share of hyperscaler server infrastructure. The AI narrative is also</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="45" t="n"/>
-      <c r="B40" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  shifting down-stack into CPU makers — AMD benefits from both trends simultaneously. Risk: NVIDIA's software moat (CUDA) is still</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="45" t="n"/>
-      <c r="B41" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  wide. But as a compounder and a hedge on NVIDIA dominance, AMD belongs in the portfolio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="6" customHeight="1">
-      <c r="A42" s="45" t="n"/>
-      <c r="B42" s="45" t="n"/>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="41" t="inlineStr">
+          <t>CPU maker deep in the AI infrastructure stack and the only credible challenger to NVIDIA in AI accelerators. AMD's MI300X GPU is winning meaningful enterprise AI workloads, particularly inference, where customers want a cheaper alternative to NVIDIA's H100/H200. On the CPU side, AMD's EPYC chips power a huge share of hyperscaler server infrastructure. The AI narrative is also shifting down-stack into CPU makers — AMD benefits from both trends simultaneously. Risk: NVIDIA's software moat (CUDA) is still wide. But as a compounder and a hedge on NVIDIA dominance, AMD belongs in the portfolio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="8" customHeight="1"/>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="41" t="inlineStr">
         <is>
           <t>INTC</t>
         </is>
       </c>
-      <c r="B43" s="42" t="inlineStr">
+      <c r="B27" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  Intel Corp   |   Risk: Med-High</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="16" customHeight="1">
-      <c r="A44" s="43" t="n"/>
-      <c r="B44" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  CPU maker in the AI infrastructure stack and the most controversial turnaround story in semiconductors. Intel lost its</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="16" customHeight="1">
-      <c r="A45" s="43" t="n"/>
-      <c r="B45" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  manufacturing lead to TSMC and its AI accelerator business to NVIDIA and AMD. The thesis here is a turnaround: new management,</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="16" customHeight="1">
-      <c r="A46" s="43" t="n"/>
-      <c r="B46" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  massive government subsidies via the CHIPS Act, and a path to reclaiming leading-edge manufacturing through its Intel Foundry</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="16" customHeight="1">
-      <c r="A47" s="43" t="n"/>
-      <c r="B47" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Services (IFS) division. If the turnaround works, INTC is deeply undervalued. If it doesn't, the downside is meaningful. This is a</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="16" customHeight="1">
-      <c r="A48" s="43" t="n"/>
-      <c r="B48" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  higher-risk position — size it as a speculative turnaround bet, not a core hold. The AI infrastructure narrative (CPU makers</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="16" customHeight="1">
-      <c r="A49" s="43" t="n"/>
-      <c r="B49" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  shifting down-stack) gives it a tailwind even without a full recovery.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="6" customHeight="1">
-      <c r="A50" s="45" t="n"/>
-      <c r="B50" s="45" t="n"/>
-    </row>
-    <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="41" t="inlineStr">
+    <row r="28" ht="250" customHeight="1">
+      <c r="A28" s="43" t="n"/>
+      <c r="B28" s="44" t="inlineStr">
+        <is>
+          <t>CPU maker in the AI infrastructure stack and the most controversial turnaround story in semiconductors. Intel lost its manufacturing lead to TSMC and its AI accelerator business to NVIDIA and AMD. The thesis here is a turnaround: new management, massive government subsidies via the CHIPS Act, and a path to reclaiming leading-edge manufacturing through its Intel Foundry Services (IFS) division. If the turnaround works, INTC is deeply undervalued. If it doesn't, the downside is meaningful. This is a higher-risk position — size it as a speculative turnaround bet, not a core hold. The AI infrastructure narrative (CPU makers shifting down-stack) gives it a tailwind even without a full recovery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="8" customHeight="1"/>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="41" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
-      <c r="B51" s="42" t="inlineStr">
+      <c r="B30" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  Arm Holdings   |   Risk: Medium</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="16" customHeight="1">
-      <c r="A52" s="45" t="n"/>
-      <c r="B52" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  The architecture behind nearly every AI chip that isn't an x86 CPU. ARM licenses its instruction set architecture to Apple,</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="16" customHeight="1">
-      <c r="A53" s="45" t="n"/>
-      <c r="B53" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Qualcomm, Amazon (Graviton), Google, NVIDIA, and dozens of others. Every time an AI edge chip, smartphone chip, or custom</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="16" customHeight="1">
-      <c r="A54" s="45" t="n"/>
-      <c r="B54" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  datacenter chip gets designed and sold, ARM earns a royalty. This is a pure royalty business model — no manufacturing risk, no</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="16" customHeight="1">
-      <c r="A55" s="45" t="n"/>
-      <c r="B55" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  inventory risk — just IP licensing that scales with every chip shipped globally. As AI moves to the edge (phones, cars, robots),</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="16" customHeight="1">
-      <c r="A56" s="45" t="n"/>
-      <c r="B56" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ARM's exposure compounds. The royalty rate per chip is also increasing as designs get more complex. A core compounder.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="6" customHeight="1">
-      <c r="A57" s="45" t="n"/>
-      <c r="B57" s="45" t="n"/>
-    </row>
+    <row r="31" ht="250" customHeight="1">
+      <c r="A31" s="45" t="n"/>
+      <c r="B31" s="46" t="inlineStr">
+        <is>
+          <t>The architecture behind nearly every AI chip that isn't an x86 CPU. ARM licenses its instruction set architecture to Apple, Qualcomm, Amazon (Graviton), Google, NVIDIA, and dozens of others. Every time an AI edge chip, smartphone chip, or custom datacenter chip gets designed and sold, ARM earns a royalty. This is a pure royalty business model — no manufacturing risk, no inventory risk — just IP licensing that scales with every chip shipped globally. As AI moves to the edge (phones, cars, robots), ARM's exposure compounds. The royalty rate per chip is also increasing as designs get more complex. A core compounder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A3:Q3"/>
@@ -4193,7 +3717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q68"/>
+  <dimension ref="A1:Q35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4232,7 +3756,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
         </is>
       </c>
     </row>
@@ -4861,418 +4385,141 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="16" customHeight="1">
+    <row r="17" ht="250" customHeight="1">
       <c r="A17" s="43" t="n"/>
       <c r="B17" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  The NVDA-parallel picks-and-shovels bet for AI power. Navitas makes GaN (gallium nitride) power chips that are radically more</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="43" t="n"/>
-      <c r="B18" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  efficient than traditional silicon-based power delivery. AI data centers are hitting a hard wall on power density — the amount of</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="43" t="n"/>
-      <c r="B19" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  electricity you can push into a rack is physically limited by current power conversion technology. GaN solves this by converting</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="43" t="n"/>
-      <c r="B20" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  power more efficiently and at higher frequencies, enabling denser, cooler, more power-efficient data centers. As hyperscalers</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="43" t="n"/>
-      <c r="B21" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  build out hundreds of gigawatts of AI compute, NVTS stands to be a critical infrastructure supplier. High-risk, asymmetric upside</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="43" t="n"/>
-      <c r="B22" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  — the kind of bet that looks obvious in hindsight.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="6" customHeight="1">
-      <c r="A23" s="45" t="n"/>
-      <c r="B23" s="45" t="n"/>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="41" t="inlineStr">
+          <t>The NVDA-parallel picks-and-shovels bet for AI power. Navitas makes GaN (gallium nitride) power chips that are radically more efficient than traditional silicon-based power delivery. AI data centers are hitting a hard wall on power density — the amount of electricity you can push into a rack is physically limited by current power conversion technology. GaN solves this by converting power more efficiently and at higher frequencies, enabling denser, cooler, more power-efficient data centers. As hyperscalers build out hundreds of gigawatts of AI compute, NVTS stands to be a critical infrastructure supplier. High-risk, asymmetric upside — the kind of bet that looks obvious in hindsight.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="8" customHeight="1"/>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="41" t="inlineStr">
         <is>
           <t>AEHR</t>
         </is>
       </c>
-      <c r="B24" s="42" t="inlineStr">
+      <c r="B19" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  AEHR Test Systems   |   Risk: High</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="45" t="n"/>
-      <c r="B25" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Classic shovels-in-a-gold-rush setup. AEHR makes specialized semiconductor burn-in and test equipment used to stress-test chips</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="16" customHeight="1">
+    <row r="20" ht="250" customHeight="1">
+      <c r="A20" s="45" t="n"/>
+      <c r="B20" s="46" t="inlineStr">
+        <is>
+          <t>Classic shovels-in-a-gold-rush setup. AEHR makes specialized semiconductor burn-in and test equipment used to stress-test chips before they ship. As AI chips become more complex and expensive (each H100 costs $30k+), the cost of shipping a defective chip becomes enormous — which means chip manufacturers are investing heavily in advanced testing. More AI chips manufactured = more testing bottleneck demand = more AEHR revenue. The business is lumpy (large equipment orders), which creates volatility, but the long-term tailwind is durable. A pure picks-and-shovels beneficiary of the AI chip production ramp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="8" customHeight="1"/>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="41" t="inlineStr">
+        <is>
+          <t>CRDO</t>
+        </is>
+      </c>
+      <c r="B22" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Credo Technology   |   Risk: High</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="250" customHeight="1">
+      <c r="A23" s="43" t="n"/>
+      <c r="B23" s="44" t="inlineStr">
+        <is>
+          <t>One of the cleanest AI infrastructure picks-and-shovels names available. GPUs are useless if the data can't move between them fast enough. Credo makes high-speed SerDes (serializer/deserializer) connectivity chips that are the plumbing inside AI data centers — connecting GPUs to memory, switches, and storage at speeds that match the compute throughput. As AI clusters scale from thousands to hundreds of thousands of GPUs, the interconnect bandwidth requirement explodes. Credo has direct customer relationships with hyperscalers and is already generating real revenue from the AI buildout. Strong execution, growing bookings, and a durable structural tailwind.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="8" customHeight="1"/>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="41" t="inlineStr">
+        <is>
+          <t>ALGM</t>
+        </is>
+      </c>
+      <c r="B25" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Allegro MicroSystems   |   Risk: Med-High</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="250" customHeight="1">
       <c r="A26" s="45" t="n"/>
       <c r="B26" s="46" t="inlineStr">
         <is>
-          <t xml:space="preserve">  before they ship. As AI chips become more complex and expensive (each H100 costs $30k+), the cost of shipping a defective chip</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="45" t="n"/>
-      <c r="B27" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  becomes enormous — which means chip manufacturers are investing heavily in advanced testing. More AI chips manufactured = more</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="45" t="n"/>
-      <c r="B28" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  testing bottleneck demand = more AEHR revenue. The business is lumpy (large equipment orders), which creates volatility, but the</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="45" t="n"/>
-      <c r="B29" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  long-term tailwind is durable. A pure picks-and-shovels beneficiary of the AI chip production ramp.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="6" customHeight="1">
-      <c r="A30" s="45" t="n"/>
-      <c r="B30" s="45" t="n"/>
-    </row>
+          <t>A quiet compounder that is early in its AI rerating narrative. Allegro makes power management and sensing semiconductors used in automotive, industrial, and increasingly AI hardware applications. As AI hardware demands more precise power delivery and thermal sensing, Allegro's chips become more embedded in the data center infrastructure. The automotive exposure (EV power management) provides a separate growth vector. Less hype than the pure-play AI names, which means it hasn't been fully rerated yet — creating a potential catch-up opportunity. More of a steady grower than a moonshot, but with meaningful upside as the narrative broadens.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="8" customHeight="1"/>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="41" t="inlineStr">
+        <is>
+          <t>HIMX</t>
+        </is>
+      </c>
+      <c r="B28" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Himax Technologies   |   Risk: High</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="250" customHeight="1">
+      <c r="A29" s="43" t="n"/>
+      <c r="B29" s="44" t="inlineStr">
+        <is>
+          <t>An often-overlooked ADR with cyclical breakout behavior. Himax makes display driver ICs and AI vision chips used in AR/VR devices, automotive displays, and AI edge sensing applications. When AI edge device cycles accelerate — smartphones, AR glasses, smart cameras — Himax tends to move fast. It's historically undervalued relative to its revenue and has a pattern of sharp re-ratings on earnings beats during upcycles. The AR/AI vision chip exposure is genuinely interesting as AI moves from the cloud to the edge. Higher volatility, but the kind of name that can double in a single cycle. Treat as a tactical position sized for the volatility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="8" customHeight="1"/>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="41" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>MTSI</t>
         </is>
       </c>
       <c r="B31" s="42" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Credo Technology   |   Risk: High</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="43" t="n"/>
-      <c r="B32" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  One of the cleanest AI infrastructure picks-and-shovels names available. GPUs are useless if the data can't move between them fast</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="43" t="n"/>
-      <c r="B33" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  enough. Credo makes high-speed SerDes (serializer/deserializer) connectivity chips that are the plumbing inside AI data centers —</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="43" t="n"/>
-      <c r="B34" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  connecting GPUs to memory, switches, and storage at speeds that match the compute throughput. As AI clusters scale from thousands</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="16" customHeight="1">
+          <t xml:space="preserve">  MACOM Technology   |   Risk: Med-High</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="250" customHeight="1">
+      <c r="A32" s="45" t="n"/>
+      <c r="B32" s="46" t="inlineStr">
+        <is>
+          <t>Less hype, more industrial AI backbone. MACOM makes RF, microwave, and high-speed analog chips used in data center interconnects, telecom backbones, and defense systems. As AI data centers demand ever-higher bandwidth between racks and buildings, MACOM's optical and RF interconnect chips become critical infrastructure. The telecom angle also gives it exposure to 5G buildout and the long-term bandwidth expansion required to support AI inference at the edge. Not a headline name, but a steady grower with durable end-market demand. The kind of stock that compounds quietly while the hype goes elsewhere, then re-rates when the market catches up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="8" customHeight="1"/>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="41" t="inlineStr">
+        <is>
+          <t>AEVA</t>
+        </is>
+      </c>
+      <c r="B34" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Aeva Technologies   |   Risk: Very High</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="250" customHeight="1">
       <c r="A35" s="43" t="n"/>
       <c r="B35" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  to hundreds of thousands of GPUs, the interconnect bandwidth requirement explodes. Credo has direct customer relationships with</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="43" t="n"/>
-      <c r="B36" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  hyperscalers and is already generating real revenue from the AI buildout. Strong execution, growing bookings, and a durable</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="16" customHeight="1">
-      <c r="A37" s="43" t="n"/>
-      <c r="B37" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  structural tailwind.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="6" customHeight="1">
-      <c r="A38" s="45" t="n"/>
-      <c r="B38" s="45" t="n"/>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="41" t="inlineStr">
-        <is>
-          <t>ALGM</t>
-        </is>
-      </c>
-      <c r="B39" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Allegro MicroSystems   |   Risk: Med-High</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="45" t="n"/>
-      <c r="B40" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  A quiet compounder that is early in its AI rerating narrative. Allegro makes power management and sensing semiconductors used in</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="45" t="n"/>
-      <c r="B41" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  automotive, industrial, and increasingly AI hardware applications. As AI hardware demands more precise power delivery and thermal</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="16" customHeight="1">
-      <c r="A42" s="45" t="n"/>
-      <c r="B42" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  sensing, Allegro's chips become more embedded in the data center infrastructure. The automotive exposure (EV power management)</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="16" customHeight="1">
-      <c r="A43" s="45" t="n"/>
-      <c r="B43" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  provides a separate growth vector. Less hype than the pure-play AI names, which means it hasn't been fully rerated yet — creating</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="16" customHeight="1">
-      <c r="A44" s="45" t="n"/>
-      <c r="B44" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  a potential catch-up opportunity. More of a steady grower than a moonshot, but with meaningful upside as the narrative broadens.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="6" customHeight="1">
-      <c r="A45" s="45" t="n"/>
-      <c r="B45" s="45" t="n"/>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="41" t="inlineStr">
-        <is>
-          <t>HIMX</t>
-        </is>
-      </c>
-      <c r="B46" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Himax Technologies   |   Risk: High</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="16" customHeight="1">
-      <c r="A47" s="43" t="n"/>
-      <c r="B47" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  An often-overlooked ADR with cyclical breakout behavior. Himax makes display driver ICs and AI vision chips used in AR/VR devices,</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="16" customHeight="1">
-      <c r="A48" s="43" t="n"/>
-      <c r="B48" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  automotive displays, and AI edge sensing applications. When AI edge device cycles accelerate — smartphones, AR glasses, smart</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="16" customHeight="1">
-      <c r="A49" s="43" t="n"/>
-      <c r="B49" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  cameras — Himax tends to move fast. It's historically undervalued relative to its revenue and has a pattern of sharp re-ratings on</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="16" customHeight="1">
-      <c r="A50" s="43" t="n"/>
-      <c r="B50" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  earnings beats during upcycles. The AR/AI vision chip exposure is genuinely interesting as AI moves from the cloud to the edge.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="16" customHeight="1">
-      <c r="A51" s="43" t="n"/>
-      <c r="B51" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Higher volatility, but the kind of name that can double in a single cycle. Treat as a tactical position sized for the volatility.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="6" customHeight="1">
-      <c r="A52" s="45" t="n"/>
-      <c r="B52" s="45" t="n"/>
-    </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="41" t="inlineStr">
-        <is>
-          <t>MTSI</t>
-        </is>
-      </c>
-      <c r="B53" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  MACOM Technology   |   Risk: Med-High</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="16" customHeight="1">
-      <c r="A54" s="45" t="n"/>
-      <c r="B54" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Less hype, more industrial AI backbone. MACOM makes RF, microwave, and high-speed analog chips used in data center interconnects,</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="16" customHeight="1">
-      <c r="A55" s="45" t="n"/>
-      <c r="B55" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  telecom backbones, and defense systems. As AI data centers demand ever-higher bandwidth between racks and buildings, MACOM's</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="16" customHeight="1">
-      <c r="A56" s="45" t="n"/>
-      <c r="B56" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  optical and RF interconnect chips become critical infrastructure. The telecom angle also gives it exposure to 5G buildout and the</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="16" customHeight="1">
-      <c r="A57" s="45" t="n"/>
-      <c r="B57" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  long-term bandwidth expansion required to support AI inference at the edge. Not a headline name, but a steady grower with durable</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="16" customHeight="1">
-      <c r="A58" s="45" t="n"/>
-      <c r="B58" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  end-market demand. The kind of stock that compounds quietly while the hype goes elsewhere, then re-rates when the market catches</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="16" customHeight="1">
-      <c r="A59" s="45" t="n"/>
-      <c r="B59" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  up.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="6" customHeight="1">
-      <c r="A60" s="45" t="n"/>
-      <c r="B60" s="45" t="n"/>
-    </row>
-    <row r="61" ht="20" customHeight="1">
-      <c r="A61" s="41" t="inlineStr">
-        <is>
-          <t>AEVA</t>
-        </is>
-      </c>
-      <c r="B61" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Aeva Technologies   |   Risk: Very High</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="16" customHeight="1">
-      <c r="A62" s="43" t="n"/>
-      <c r="B62" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Pure asymmetric bet — low probability, high upside if they execute. Aeva makes FMCW (frequency-modulated continuous-wave) lidar</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="16" customHeight="1">
-      <c r="A63" s="43" t="n"/>
-      <c r="B63" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  sensors for autonomous vehicles and robotics. Their approach is technically differentiated — FMCW lidar can detect velocity</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="16" customHeight="1">
-      <c r="A64" s="43" t="n"/>
-      <c r="B64" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  directly (not just position) and works better in adverse conditions than traditional lidar. The autonomous vehicle and robotics</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="16" customHeight="1">
-      <c r="A65" s="43" t="n"/>
-      <c r="B65" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  market is massive if it materializes, and Aeva would be a key sensing supplier. Still in early commercialization — revenue is</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="16" customHeight="1">
-      <c r="A66" s="43" t="n"/>
-      <c r="B66" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  minimal and the path to profitability is long. This is a speculative moonshot, not a core position. Size it as a lottery ticket:</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="16" customHeight="1">
-      <c r="A67" s="43" t="n"/>
-      <c r="B67" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  accept that it could go to zero, but the upside if robotics/AV take off is 10-20x.</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="6" customHeight="1">
-      <c r="A68" s="45" t="n"/>
-      <c r="B68" s="45" t="n"/>
-    </row>
+          <t>Pure asymmetric bet — low probability, high upside if they execute. Aeva makes FMCW (frequency-modulated continuous-wave) lidar sensors for autonomous vehicles and robotics. Their approach is technically differentiated — FMCW lidar can detect velocity directly (not just position) and works better in adverse conditions than traditional lidar. The autonomous vehicle and robotics market is massive if it materializes, and Aeva would be a key sensing supplier. Still in early commercialization — revenue is minimal and the path to profitability is long. This is a speculative moonshot, not a core position. Size it as a lottery ticket: accept that it could go to zero, but the upside if robotics/AV take off is 10-20x.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A3:Q3"/>
@@ -5307,7 +4554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q18"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5346,7 +4593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
         </is>
       </c>
     </row>
@@ -5573,66 +4820,15 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="16" customHeight="1">
+    <row r="11" ht="250" customHeight="1">
       <c r="A11" s="43" t="n"/>
       <c r="B11" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  King of Photonics — and this could be a genuine moonshot. Lumentum makes the optical components (lasers, transceivers, photonic</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="43" t="n"/>
-      <c r="B12" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  integrated circuits) that transmit data at the speed of light inside and between AI data centers. As AI clusters scale to hundreds</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="43" t="n"/>
-      <c r="B13" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  of thousands of GPUs spread across multiple buildings, the optical interconnect becomes the critical bottleneck — you can't run</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="43" t="n"/>
-      <c r="B14" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  copper cables at those distances and speeds. Lumentum is one of the few companies with the technology and scale to supply this</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="43" t="n"/>
-      <c r="B15" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  infrastructure. The AI tailwind here is massive and underappreciated. Photonics is the next big narrative after GPUs and power —</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="43" t="n"/>
-      <c r="B16" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  when the market wakes up to the data movement bottleneck, LITE is the headline name. High conviction, high risk, moonshot</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="43" t="n"/>
-      <c r="B17" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  potential.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="6" customHeight="1">
-      <c r="A18" s="45" t="n"/>
-      <c r="B18" s="45" t="n"/>
-    </row>
+          <t>King of Photonics — and this could be a genuine moonshot. Lumentum makes the optical components (lasers, transceivers, photonic integrated circuits) that transmit data at the speed of light inside and between AI data centers. As AI clusters scale to hundreds of thousands of GPUs spread across multiple buildings, the optical interconnect becomes the critical bottleneck — you can't run copper cables at those distances and speeds. Lumentum is one of the few companies with the technology and scale to supply this infrastructure. The AI tailwind here is massive and underappreciated. Photonics is the next big narrative after GPUs and power — when the market wakes up to the data movement bottleneck, LITE is the headline name. High conviction, high risk, moonshot potential.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A3:Q3"/>
@@ -5667,7 +4863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q44"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5706,7 +4902,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
         </is>
       </c>
     </row>
@@ -6134,250 +5330,78 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="16" customHeight="1">
+    <row r="14" ht="250" customHeight="1">
       <c r="A14" s="43" t="n"/>
       <c r="B14" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  The actual builder and materials company in the AI data center trade. AI data centers are physical buildings requiring massive</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="43" t="n"/>
-      <c r="B15" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  earthmoving, foundation work, and construction equipment — and Caterpillar is the dominant supplier of that heavy equipment</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="43" t="n"/>
-      <c r="B16" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  globally. Every hyperscaler campus that Meta, Google, Microsoft, and Amazon builds requires CAT equipment on site. This is a</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="43" t="n"/>
-      <c r="B17" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  steadier, lower-volatility way to play the AI infrastructure buildout than the semiconductor names. CAT also benefits from</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="43" t="n"/>
-      <c r="B18" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  infrastructure spending more broadly (roads, bridges, energy projects) which provides diversification. A solid core position —</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="43" t="n"/>
-      <c r="B19" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  steady compounder with the AI tailwind as a bonus.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="6" customHeight="1">
-      <c r="A20" s="45" t="n"/>
-      <c r="B20" s="45" t="n"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="41" t="inlineStr">
+          <t>The actual builder and materials company in the AI data center trade. AI data centers are physical buildings requiring massive earthmoving, foundation work, and construction equipment — and Caterpillar is the dominant supplier of that heavy equipment globally. Every hyperscaler campus that Meta, Google, Microsoft, and Amazon builds requires CAT equipment on site. This is a steadier, lower-volatility way to play the AI infrastructure buildout than the semiconductor names. CAT also benefits from infrastructure spending more broadly (roads, bridges, energy projects) which provides diversification. A solid core position — steady compounder with the AI tailwind as a bonus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="8" customHeight="1"/>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="41" t="inlineStr">
         <is>
           <t>FIX</t>
         </is>
       </c>
-      <c r="B21" s="42" t="inlineStr">
+      <c r="B16" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  Comfort Systems USA   |   Risk: Medium</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="45" t="n"/>
-      <c r="B22" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Builder AND cooling company — one of the best-positioned picks-and-shovels plays in the AI buildout. Comfort Systems provides</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="16" customHeight="1">
+    <row r="17" ht="250" customHeight="1">
+      <c r="A17" s="45" t="n"/>
+      <c r="B17" s="46" t="inlineStr">
+        <is>
+          <t>Builder AND cooling company — one of the best-positioned picks-and-shovels plays in the AI buildout. Comfort Systems provides HVAC, mechanical, plumbing, and electrical systems for commercial buildings, including AI data centers. Cooling is a MAJOR and growing bottleneck in AI data centers — every GPU cluster generates enormous heat that must be managed. FIX designs and installs the entire MEP (mechanical, electrical, plumbing) system that keeps these facilities running. They have direct contracts with hyperscalers and are seeing demand accelerate as AI data center construction ramps. A quality business with real earnings growth, not a speculative bet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="8" customHeight="1"/>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="41" t="inlineStr">
+        <is>
+          <t>POWL</t>
+        </is>
+      </c>
+      <c r="B19" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Powell Industries   |   Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="250" customHeight="1">
+      <c r="A20" s="43" t="n"/>
+      <c r="B20" s="44" t="inlineStr">
+        <is>
+          <t>Electrical infrastructure builder for AI data centers — the company that builds the switchgear, motor control centers, and power distribution equipment that routes electricity inside data centers and industrial facilities. As AI data centers require ever-larger amounts of power (some campus projects exceed 1 GW), the electrical infrastructure to safely distribute that power becomes a critical bottleneck. Powell has a backlog-heavy business model with long-cycle orders, which means revenue visibility is strong. Less volatile than the semiconductor names because of the order backlog and industrial nature of the business. A solid mid-cap infrastructure pick with a genuine AI tailwind.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="8" customHeight="1"/>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="41" t="inlineStr">
+        <is>
+          <t>VRT</t>
+        </is>
+      </c>
+      <c r="B22" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Vertiv Holdings   |   Risk: Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="250" customHeight="1">
       <c r="A23" s="45" t="n"/>
       <c r="B23" s="46" t="inlineStr">
         <is>
-          <t xml:space="preserve">  HVAC, mechanical, plumbing, and electrical systems for commercial buildings, including AI data centers. Cooling is a MAJOR and</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="45" t="n"/>
-      <c r="B24" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  growing bottleneck in AI data centers — every GPU cluster generates enormous heat that must be managed. FIX designs and installs</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="45" t="n"/>
-      <c r="B25" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  the entire MEP (mechanical, electrical, plumbing) system that keeps these facilities running. They have direct contracts with</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="45" t="n"/>
-      <c r="B26" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  hyperscalers and are seeing demand accelerate as AI data center construction ramps. A quality business with real earnings growth,</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="45" t="n"/>
-      <c r="B27" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  not a speculative bet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="6" customHeight="1">
-      <c r="A28" s="45" t="n"/>
-      <c r="B28" s="45" t="n"/>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="41" t="inlineStr">
-        <is>
-          <t>POWL</t>
-        </is>
-      </c>
-      <c r="B29" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Powell Industries   |   Risk: Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="43" t="n"/>
-      <c r="B30" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Electrical infrastructure builder for AI data centers — the company that builds the switchgear, motor control centers, and power</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="43" t="n"/>
-      <c r="B31" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  distribution equipment that routes electricity inside data centers and industrial facilities. As AI data centers require ever-</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="43" t="n"/>
-      <c r="B32" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  larger amounts of power (some campus projects exceed 1 GW), the electrical infrastructure to safely distribute that power becomes</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="43" t="n"/>
-      <c r="B33" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  a critical bottleneck. Powell has a backlog-heavy business model with long-cycle orders, which means revenue visibility is strong.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="43" t="n"/>
-      <c r="B34" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Less volatile than the semiconductor names because of the order backlog and industrial nature of the business. A solid mid-cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="43" t="n"/>
-      <c r="B35" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  infrastructure pick with a genuine AI tailwind.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="6" customHeight="1">
-      <c r="A36" s="45" t="n"/>
-      <c r="B36" s="45" t="n"/>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="41" t="inlineStr">
-        <is>
-          <t>VRT</t>
-        </is>
-      </c>
-      <c r="B37" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Vertiv Holdings   |   Risk: Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="16" customHeight="1">
-      <c r="A38" s="45" t="n"/>
-      <c r="B38" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  The premier AI data center cooling play and one of the most direct beneficiaries of the AI buildout. Vertiv makes thermal</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="45" t="n"/>
-      <c r="B39" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  management systems (liquid cooling, air cooling, heat exchangers) along with power distribution infrastructure for data centers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="45" t="n"/>
-      <c r="B40" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Cooling is not optional — you cannot run a GPU cluster without solving the thermal problem, and as GPU power consumption has</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="45" t="n"/>
-      <c r="B41" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  exploded from 300W to 700W per chip, existing cooling infrastructure is completely inadequate. Every new AI data center that gets</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="16" customHeight="1">
-      <c r="A42" s="45" t="n"/>
-      <c r="B42" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  built needs Vertiv's systems. The company has multi-year backlog, growing margins, and is adding capacity to meet demand. A high-</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="16" customHeight="1">
-      <c r="A43" s="45" t="n"/>
-      <c r="B43" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  conviction hold in the AI infrastructure basket.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="6" customHeight="1">
-      <c r="A44" s="45" t="n"/>
-      <c r="B44" s="45" t="n"/>
-    </row>
+          <t>The premier AI data center cooling play and one of the most direct beneficiaries of the AI buildout. Vertiv makes thermal management systems (liquid cooling, air cooling, heat exchangers) along with power distribution infrastructure for data centers. Cooling is not optional — you cannot run a GPU cluster without solving the thermal problem, and as GPU power consumption has exploded from 300W to 700W per chip, existing cooling infrastructure is completely inadequate. Every new AI data center that gets built needs Vertiv's systems. The company has multi-year backlog, growing margins, and is adding capacity to meet demand. A high-conviction hold in the AI infrastructure basket.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A3:Q3"/>
@@ -6412,7 +5436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q46"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6451,7 +5475,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
         </is>
       </c>
     </row>
@@ -6879,266 +5903,78 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="16" customHeight="1">
+    <row r="14" ht="250" customHeight="1">
       <c r="A14" s="43" t="n"/>
       <c r="B14" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Stability and steady compounder — the premier power generation and grid equipment company spun out of GE. GE Vernova makes gas</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="43" t="n"/>
-      <c r="B15" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  turbines, wind turbines, grid software, and electrification equipment. AI data centers are consuming power at a rate that is</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="43" t="n"/>
-      <c r="B16" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  straining the US electrical grid, and new power generation capacity takes years to build. GE Vernova is one of the few companies</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="43" t="n"/>
-      <c r="B17" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  with the scale and installed base to actually supply that new capacity fast. Their gas turbine backlog is multi-year and growing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="43" t="n"/>
-      <c r="B18" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  This is not a speculative bet — it's a high-quality industrial compounder with a very real and durable demand tailwind from AI</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="43" t="n"/>
-      <c r="B19" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  power needs. A core long-term hold.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="6" customHeight="1">
-      <c r="A20" s="45" t="n"/>
-      <c r="B20" s="45" t="n"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="41" t="inlineStr">
+          <t>Stability and steady compounder — the premier power generation and grid equipment company spun out of GE. GE Vernova makes gas turbines, wind turbines, grid software, and electrification equipment. AI data centers are consuming power at a rate that is straining the US electrical grid, and new power generation capacity takes years to build. GE Vernova is one of the few companies with the scale and installed base to actually supply that new capacity fast. Their gas turbine backlog is multi-year and growing. This is not a speculative bet — it's a high-quality industrial compounder with a very real and durable demand tailwind from AI power needs. A core long-term hold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="8" customHeight="1"/>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="41" t="inlineStr">
         <is>
           <t>PWR</t>
         </is>
       </c>
-      <c r="B21" s="42" t="inlineStr">
+      <c r="B16" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  Quanta Services   |   Risk: Medium</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="45" t="n"/>
-      <c r="B22" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Power grid infrastructure and maintenance — a growing bottleneck for the AI buildout. Quanta Services is the largest specialty</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="16" customHeight="1">
+    <row r="17" ht="250" customHeight="1">
+      <c r="A17" s="45" t="n"/>
+      <c r="B17" s="46" t="inlineStr">
+        <is>
+          <t>Power grid infrastructure and maintenance — a growing bottleneck for the AI buildout. Quanta Services is the largest specialty contractor for electric power infrastructure in North America. They build and maintain power lines, substations, and grid connections that are essential to delivering electricity to AI data centers. Every new data center campus needs a grid connection, often requiring new transmission lines and substations — all of which Quanta builds. The company has multi-year visibility through its backlog and framework agreements with utilities. A steady, high-quality compounder that benefits directly and durably from the AI power demand surge. Lower volatility than the semiconductor names with a comparably strong tailwind.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="8" customHeight="1"/>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="41" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="B19" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Bloom Energy   |   Risk: High</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="250" customHeight="1">
+      <c r="A20" s="43" t="n"/>
+      <c r="B20" s="44" t="inlineStr">
+        <is>
+          <t>Moonshot potential if hydrogen and fuel cell technology takes off — and the AI power crisis is accelerating the timeline. Bloom Energy makes solid oxide fuel cells that generate electricity on-site without connecting to the grid. For AI data centers that need reliable, clean, on-site power (especially in areas with grid congestion), Bloom's solution is genuinely compelling. They're already selling to data centers and have partnerships with major tech companies. The bull case: AI power demand is so acute that on-site generation becomes mandatory, and Bloom is uniquely positioned. The bear case: fuel cells are expensive and hydrogen infrastructure is still nascent. Worth holding a position — the upside if they win even a small share of the AI power market is very large.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="8" customHeight="1"/>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="41" t="inlineStr">
+        <is>
+          <t>OKLO</t>
+        </is>
+      </c>
+      <c r="B22" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Oklo Inc   |   Risk: Very High</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="250" customHeight="1">
       <c r="A23" s="45" t="n"/>
       <c r="B23" s="46" t="inlineStr">
         <is>
-          <t xml:space="preserve">  contractor for electric power infrastructure in North America. They build and maintain power lines, substations, and grid</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="45" t="n"/>
-      <c r="B24" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  connections that are essential to delivering electricity to AI data centers. Every new data center campus needs a grid connection,</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="45" t="n"/>
-      <c r="B25" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  often requiring new transmission lines and substations — all of which Quanta builds. The company has multi-year visibility through</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="45" t="n"/>
-      <c r="B26" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  its backlog and framework agreements with utilities. A steady, high-quality compounder that benefits directly and durably from the</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="45" t="n"/>
-      <c r="B27" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  AI power demand surge. Lower volatility than the semiconductor names with a comparably strong tailwind.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="6" customHeight="1">
-      <c r="A28" s="45" t="n"/>
-      <c r="B28" s="45" t="n"/>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="41" t="inlineStr">
-        <is>
-          <t>BE</t>
-        </is>
-      </c>
-      <c r="B29" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Bloom Energy   |   Risk: High</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="43" t="n"/>
-      <c r="B30" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Moonshot potential if hydrogen and fuel cell technology takes off — and the AI power crisis is accelerating the timeline. Bloom</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="43" t="n"/>
-      <c r="B31" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Energy makes solid oxide fuel cells that generate electricity on-site without connecting to the grid. For AI data centers that</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="43" t="n"/>
-      <c r="B32" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  need reliable, clean, on-site power (especially in areas with grid congestion), Bloom's solution is genuinely compelling. They're</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="43" t="n"/>
-      <c r="B33" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  already selling to data centers and have partnerships with major tech companies. The bull case: AI power demand is so acute that</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="43" t="n"/>
-      <c r="B34" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  on-site generation becomes mandatory, and Bloom is uniquely positioned. The bear case: fuel cells are expensive and hydrogen</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="43" t="n"/>
-      <c r="B35" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  infrastructure is still nascent. Worth holding a position — the upside if they win even a small share of the AI power market is</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="43" t="n"/>
-      <c r="B36" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  very large.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="6" customHeight="1">
-      <c r="A37" s="45" t="n"/>
-      <c r="B37" s="45" t="n"/>
-    </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="41" t="inlineStr">
-        <is>
-          <t>OKLO</t>
-        </is>
-      </c>
-      <c r="B38" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Oklo Inc   |   Risk: Very High</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="45" t="n"/>
-      <c r="B39" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Nuclear SMRs and nuclear fuel waste company with massive moonshot potential — but big regulatory and execution risk. Oklo is</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="45" t="n"/>
-      <c r="B40" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  building small modular nuclear reactors (SMRs) that could provide clean, always-on baseload power for AI data centers at scale.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="45" t="n"/>
-      <c r="B41" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Several major tech companies (including Microsoft) have already signed nuclear power agreements, signaling that nuclear is being</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="16" customHeight="1">
-      <c r="A42" s="45" t="n"/>
-      <c r="B42" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  taken seriously as an AI power solution. Oklo also has a fuel recycling angle (using spent nuclear fuel) that could be a</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="16" customHeight="1">
-      <c r="A43" s="45" t="n"/>
-      <c r="B43" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  significant business in itself. The regulatory path is long and uncertain, and Oklo has not yet built a commercial reactor. This</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="16" customHeight="1">
-      <c r="A44" s="45" t="n"/>
-      <c r="B44" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  is a small-% portfolio position — accept that it could go to zero, but the upside if nuclear SMRs get commercially deployed is</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="16" customHeight="1">
-      <c r="A45" s="45" t="n"/>
-      <c r="B45" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  enormous and the valuation reflects very little of that potential today.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="6" customHeight="1">
-      <c r="A46" s="45" t="n"/>
-      <c r="B46" s="45" t="n"/>
-    </row>
+          <t>Nuclear SMRs and nuclear fuel waste company with massive moonshot potential — but big regulatory and execution risk. Oklo is building small modular nuclear reactors (SMRs) that could provide clean, always-on baseload power for AI data centers at scale. Several major tech companies (including Microsoft) have already signed nuclear power agreements, signaling that nuclear is being taken seriously as an AI power solution. Oklo also has a fuel recycling angle (using spent nuclear fuel) that could be a significant business in itself. The regulatory path is long and uncertain, and Oklo has not yet built a commercial reactor. This is a small-% portfolio position — accept that it could go to zero, but the upside if nuclear SMRs get commercially deployed is enormous and the valuation reflects very little of that potential today.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A3:Q3"/>
@@ -7173,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q28"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7212,7 +6048,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
         </is>
       </c>
     </row>
@@ -7506,138 +6342,36 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="16" customHeight="1">
+    <row r="12" ht="250" customHeight="1">
       <c r="A12" s="43" t="n"/>
       <c r="B12" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  The leading Neocloud and one of the most interesting companies in this portfolio. Nebius is a modern Amazon/Google-style company:</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="43" t="n"/>
-      <c r="B13" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  it has a primary product (GPU cloud computing for AI companies that can't get capacity from AWS/Azure/GCP) AND multiple other</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="43" t="n"/>
-      <c r="B14" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  revenue streams that could each become massive independently — Clickhouse (high-performance analytics database used by thousands</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="43" t="n"/>
-      <c r="B15" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  of companies), AV Ride (autonomous vehicle tech), and others. The neocloud thesis: hyperscalers are capacity-constrained and have</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="43" t="n"/>
-      <c r="B16" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  long waitlists for GPU compute, creating a massive opening for alternative cloud providers. NBIS is the best-positioned name to</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="43" t="n"/>
-      <c r="B17" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  fill that gap. I believe this company could become a future Hyperscaler in the same way Amazon AWS or Google Cloud became defining</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="43" t="n"/>
-      <c r="B18" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  infrastructure businesses. High conviction, long-term hold — this is the kind of company you look back on in 10 years and wish you</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="43" t="n"/>
-      <c r="B19" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  owned more of.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="6" customHeight="1">
-      <c r="A20" s="45" t="n"/>
-      <c r="B20" s="45" t="n"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="41" t="inlineStr">
+          <t>The leading Neocloud and one of the most interesting companies in this portfolio. Nebius is a modern Amazon/Google-style company: it has a primary product (GPU cloud computing for AI companies that can't get capacity from AWS/Azure/GCP) AND multiple other revenue streams that could each become massive independently — Clickhouse (high-performance analytics database used by thousands of companies), AV Ride (autonomous vehicle tech), and others. The neocloud thesis: hyperscalers are capacity-constrained and have long waitlists for GPU compute, creating a massive opening for alternative cloud providers. NBIS is the best-positioned name to fill that gap. I believe this company could become a future Hyperscaler in the same way Amazon AWS or Google Cloud became defining infrastructure businesses. High conviction, long-term hold — this is the kind of company you look back on in 10 years and wish you owned more of.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="8" customHeight="1"/>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="41" t="inlineStr">
         <is>
           <t>PLTR</t>
         </is>
       </c>
-      <c r="B21" s="42" t="inlineStr">
+      <c r="B14" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">  Palantir Technologies   |   Risk: Med-High</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="45" t="n"/>
-      <c r="B22" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  So integral to the entire US government AI stack that it is effectively a national security asset. Palantir's software (Gotham for</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="45" t="n"/>
-      <c r="B23" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  government, Foundry for enterprise, AIP for AI) is deeply embedded in the Department of Defense, intelligence agencies, and dozens</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="45" t="n"/>
-      <c r="B24" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  of federal programs. You don't rip out Palantir — agencies build entire workflows on top of it. The AI Platform (AIP) is now being</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="45" t="n"/>
-      <c r="B25" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  adopted by commercial enterprises as well, opening a second growth vector. The $1.5T defense budget and accelerating government AI</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="45" t="n"/>
-      <c r="B26" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  spending is a direct tailwind. Yes, the valuation is demanding, but for a company this strategically embedded, the premium is</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="45" t="n"/>
-      <c r="B27" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  arguably justified. An outlier name outside the data center trade that belongs in a long-term AI portfolio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="6" customHeight="1">
-      <c r="A28" s="45" t="n"/>
-      <c r="B28" s="45" t="n"/>
-    </row>
+    <row r="15" ht="250" customHeight="1">
+      <c r="A15" s="45" t="n"/>
+      <c r="B15" s="46" t="inlineStr">
+        <is>
+          <t>So integral to the entire US government AI stack that it is effectively a national security asset. Palantir's software (Gotham for government, Foundry for enterprise, AIP for AI) is deeply embedded in the Department of Defense, intelligence agencies, and dozens of federal programs. You don't rip out Palantir — agencies build entire workflows on top of it. The AI Platform (AIP) is now being adopted by commercial enterprises as well, opening a second growth vector. The $1.5T defense budget and accelerating government AI spending is a direct tailwind. Yes, the valuation is demanding, but for a company this strategically embedded, the premium is arguably justified. An outlier name outside the data center trade that belongs in a long-term AI portfolio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A3:Q3"/>
@@ -7672,7 +6406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q18"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7711,7 +6445,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 10:46 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
         </is>
       </c>
     </row>
@@ -7938,66 +6672,15 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="16" customHeight="1">
+    <row r="11" ht="250" customHeight="1">
       <c r="A11" s="43" t="n"/>
       <c r="B11" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Drones and defense tech — very speculative but with a massive catalyst behind it. The US government just announced a $1.5 trillion</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="43" t="n"/>
-      <c r="B12" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  defense budget with $56 billion going specifically to drones and counter-drones through the DAWG (Drone and Autonomous Warfare</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="43" t="n"/>
-      <c r="B13" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Group) program. Ondas is one of the few small-cap companies with actual drone technology, recent acquisitions in the space, and</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="43" t="n"/>
-      <c r="B14" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  partnerships that position them to compete for these contracts. Their March 2026 acquisitions and partnerships were specifically</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="43" t="n"/>
-      <c r="B15" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  designed to make them a stronger DAWG program competitor. This is not a guaranteed win — it's a very speculative bet on a small</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="43" t="n"/>
-      <c r="B16" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  company winning government contracts in a highly competitive space. But if they win even a small slice of the $56B drone budget,</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="43" t="n"/>
-      <c r="B17" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  the upside from current levels is enormous. Size it appropriately — this could go to zero or it could 5-10x.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="6" customHeight="1">
-      <c r="A18" s="45" t="n"/>
-      <c r="B18" s="45" t="n"/>
-    </row>
+          <t>Drones and defense tech — very speculative but with a massive catalyst behind it. The US government just announced a $1.5 trillion defense budget with $56 billion going specifically to drones and counter-drones through the DAWG (Drone and Autonomous Warfare Group) program. Ondas is one of the few small-cap companies with actual drone technology, recent acquisitions in the space, and partnerships that position them to compete for these contracts. Their March 2026 acquisitions and partnerships were specifically designed to make them a stronger DAWG program competitor. This is not a guaranteed win — it's a very speculative bet on a small company winning government contracts in a highly competitive space. But if they win even a small slice of the $56B drone budget, the upside from current levels is enormous. Size it appropriately — this could go to zero or it could 5-10x.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A3:Q3"/>

</xml_diff>

<commit_message>
Add hard line breaks to ensure notes are fully visible
Embeds newline characters directly into cell values and dynamically sets row heights to guarantee that all note text is displayed, regardless of viewer limitations.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 007571bf-3a4a-4ecb-8c65-8df6e57061ba
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1071,7 +1071,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1558,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
         </is>
       </c>
     </row>
@@ -1785,11 +1785,28 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="250" customHeight="1">
+    <row r="11" ht="282" customHeight="1">
       <c r="A11" s="43" t="n"/>
       <c r="B11" s="44" t="inlineStr">
         <is>
-          <t>Space economy and space infrastructure — huge future TAM over the next decade and beyond. Rocket Lab is the second most active launch company in the world (after SpaceX) and is the only credible alternative for small and medium satellite launches. Their Electron rocket has an exceptional launch record, and the larger Neutron rocket (in development) is designed to compete with SpaceX's Falcon 9 for medium payloads. The CEO (Peter Beck) is brilliant and has consistently delivered on technical milestones. Near-term catalyst: the SpaceX IPO (expected June 2026) will drive massive media attention to the space economy, and RKLB will benefit as the most investable public proxy. Longer term, Rocket Lab is building a vertically integrated space company (satellites, components, software, launch) which gives them multiple revenue streams. Speculative but with massive compounding upside if they execute over the next 5-10 years.</t>
+          <t>Space economy and space infrastructure — huge future
+TAM over the next decade and beyond. Rocket Lab is the
+second most active launch company in the world (after
+SpaceX) and is the only credible alternative for small
+and medium satellite launches. Their Electron rocket
+has an exceptional launch record, and the larger
+Neutron rocket (in development) is designed to compete
+with SpaceX's Falcon 9 for medium payloads. The CEO
+(Peter Beck) is brilliant and has consistently
+delivered on technical milestones. Near-term catalyst:
+the SpaceX IPO (expected June 2026) will drive massive
+media attention to the space economy, and RKLB will
+benefit as the most investable public proxy. Longer
+term, Rocket Lab is building a vertically integrated
+space company (satellites, components, software,
+launch) which gives them multiple revenue streams.
+Speculative but with massive compounding upside if they
+execute over the next 5-10 years.</t>
         </is>
       </c>
     </row>
@@ -1867,7 +1884,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
         </is>
       </c>
     </row>
@@ -2161,11 +2178,24 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="250" customHeight="1">
+    <row r="12" ht="222" customHeight="1">
       <c r="A12" s="43" t="n"/>
       <c r="B12" s="44" t="inlineStr">
         <is>
-          <t>Under active long-term evaluation. Rubrik is a cybersecurity and data management company focused on data resilience — protecting enterprise data from ransomware, ensuring recoverability, and managing data across hybrid cloud environments. As AI adoption accelerates, the volume and value of enterprise data explodes, making data protection and recovery increasingly critical. Rubrik has a subscription-based revenue model (good for predictability) and is growing fast. The risk: the cybersecurity market is crowded and competitive, and the valuation already prices in significant growth. Watch for: revenue acceleration, margin improvement, and any signs of customer concentration. Add on weakness.</t>
+          <t>Under active long-term evaluation. Rubrik is a
+cybersecurity and data management company focused on
+data resilience — protecting enterprise data from
+ransomware, ensuring recoverability, and managing data
+across hybrid cloud environments. As AI adoption
+accelerates, the volume and value of enterprise data
+explodes, making data protection and recovery
+increasingly critical. Rubrik has a subscription-based
+revenue model (good for predictability) and is growing
+fast. The risk: the cybersecurity market is crowded and
+competitive, and the valuation already prices in
+significant growth. Watch for: revenue acceleration,
+margin improvement, and any signs of customer
+concentration. Add on weakness.</t>
         </is>
       </c>
     </row>
@@ -2182,11 +2212,25 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="250" customHeight="1">
+    <row r="15" ht="237" customHeight="1">
       <c r="A15" s="45" t="n"/>
       <c r="B15" s="46" t="inlineStr">
         <is>
-          <t>Under active long-term evaluation. Novo Nordisk is the global leader in GLP-1 drugs (Ozempic, Wegovy) for diabetes and obesity. The obesity drug market is potentially the largest pharmaceutical market ever — hundreds of millions of people globally are candidates for GLP-1 treatment, and early data suggests these drugs also reduce cardiovascular events, sleep apnea, and other conditions beyond weight loss. Novo has the manufacturing scale, the brand recognition, and the clinical data to dominate this market for years. The stock has pulled back significantly from its highs as competition from Eli Lilly (Mounjaro/Zepbound) has intensified — which creates a potentially attractive entry point. A long-term compounder in healthcare, completely uncorrelated to the AI trade.</t>
+          <t>Under active long-term evaluation. Novo Nordisk is the
+global leader in GLP-1 drugs (Ozempic, Wegovy) for
+diabetes and obesity. The obesity drug market is
+potentially the largest pharmaceutical market ever —
+hundreds of millions of people globally are candidates
+for GLP-1 treatment, and early data suggests these
+drugs also reduce cardiovascular events, sleep apnea,
+and other conditions beyond weight loss. Novo has the
+manufacturing scale, the brand recognition, and the
+clinical data to dominate this market for years. The
+stock has pulled back significantly from its highs as
+competition from Eli Lilly (Mounjaro/Zepbound) has
+intensified — which creates a potentially attractive
+entry point. A long-term compounder in healthcare,
+completely uncorrelated to the AI trade.</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2566,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
         </is>
       </c>
     </row>
@@ -2883,11 +2927,21 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="250" customHeight="1">
+    <row r="13" ht="177" customHeight="1">
       <c r="A13" s="43" t="n"/>
       <c r="B13" s="44" t="inlineStr">
         <is>
-          <t>Next quantum run candidate. The belief: 'Buy IONQ, RGTI, and QBTS — easy 10x within 2 years.' IonQ is the most commercially advanced pure-play quantum computing company, using trapped-ion technology which is considered one of the most promising paths to fault-tolerant quantum computers. They already have paying customers (government, pharma, finance) and are generating real revenue. When the next quantum hype cycle hits, IonQ will be the headline name that institutions pile into. Very speculative — treat as a high-risk asymmetric bet and size position accordingly.</t>
+          <t>Next quantum run candidate. The belief: 'Buy IONQ,
+RGTI, and QBTS — easy 10x within 2 years.' IonQ is the
+most commercially advanced pure-play quantum computing
+company, using trapped-ion technology which is
+considered one of the most promising paths to fault-
+tolerant quantum computers. They already have paying
+customers (government, pharma, finance) and are
+generating real revenue. When the next quantum hype
+cycle hits, IonQ will be the headline name that
+institutions pile into. Very speculative — treat as a
+high-risk asymmetric bet and size position accordingly.</t>
         </is>
       </c>
     </row>
@@ -2904,11 +2958,21 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="250" customHeight="1">
+    <row r="16" ht="177" customHeight="1">
       <c r="A16" s="45" t="n"/>
       <c r="B16" s="46" t="inlineStr">
         <is>
-          <t>Next quantum run candidate alongside IONQ and QBTS. Rigetti builds its own quantum processors and offers cloud-based quantum computing access. It's a smaller, scrappier name than IonQ, which means more volatility but also more upside if they execute. The company has been building out its QPU (quantum processing unit) roadmap and targeting commercial applications in chemistry, logistics, and finance. When the next quantum narrative cycle accelerates, RGTI tends to move fast and hard. Pure asymmetric bet — small position, high conviction on timing.</t>
+          <t>Next quantum run candidate alongside IONQ and QBTS.
+Rigetti builds its own quantum processors and offers
+cloud-based quantum computing access. It's a smaller,
+scrappier name than IonQ, which means more volatility
+but also more upside if they execute. The company has
+been building out its QPU (quantum processing unit)
+roadmap and targeting commercial applications in
+chemistry, logistics, and finance. When the next
+quantum narrative cycle accelerates, RGTI tends to move
+fast and hard. Pure asymmetric bet — small position,
+high conviction on timing.</t>
         </is>
       </c>
     </row>
@@ -2925,11 +2989,21 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="250" customHeight="1">
+    <row r="19" ht="177" customHeight="1">
       <c r="A19" s="43" t="n"/>
       <c r="B19" s="44" t="inlineStr">
         <is>
-          <t>Next quantum run candidate alongside IONQ and RGTI. D-Wave is unique in that it uses quantum annealing rather than gate-based quantum computing, which makes it commercially viable TODAY for specific optimization problems — logistics, scheduling, materials discovery — that classical computers struggle with. It already has real enterprise customers generating recurring revenue. The commercial viability argument is stronger than most quantum names. Easy 10x potential if the next quantum hype cycle materializes. Very speculative — size position accordingly.</t>
+          <t>Next quantum run candidate alongside IONQ and RGTI.
+D-Wave is unique in that it uses quantum annealing
+rather than gate-based quantum computing, which makes
+it commercially viable TODAY for specific optimization
+problems — logistics, scheduling, materials discovery —
+that classical computers struggle with. It already has
+real enterprise customers generating recurring revenue.
+The commercial viability argument is stronger than most
+quantum names. Easy 10x potential if the next quantum
+hype cycle materializes. Very speculative — size
+position accordingly.</t>
         </is>
       </c>
     </row>
@@ -3007,7 +3081,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
         </is>
       </c>
     </row>
@@ -3569,11 +3643,21 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="250" customHeight="1">
+    <row r="16" ht="177" customHeight="1">
       <c r="A16" s="43" t="n"/>
       <c r="B16" s="44" t="inlineStr">
         <is>
-          <t>The AI compute king and the core stability position in this portfolio. NVIDIA doesn't just make GPUs — it has built the dominant software ecosystem (CUDA) that makes its hardware nearly impossible to replace even if competitors close the hardware gap. Every major hyperscaler (Google, Amazon, Microsoft, Meta) depends on NVIDIA for AI training. As AI spending continues to accelerate, NVIDIA captures the most direct revenue from every dollar spent on AI compute. This is a steady compounder that also has massive upside as the AI buildout continues. Hold as a core long-term position.</t>
+          <t>The AI compute king and the core stability position in
+this portfolio. NVIDIA doesn't just make GPUs — it has
+built the dominant software ecosystem (CUDA) that makes
+its hardware nearly impossible to replace even if
+competitors close the hardware gap. Every major
+hyperscaler (Google, Amazon, Microsoft, Meta) depends
+on NVIDIA for AI training. As AI spending continues to
+accelerate, NVIDIA captures the most direct revenue
+from every dollar spent on AI compute. This is a steady
+compounder that also has massive upside as the AI
+buildout continues. Hold as a core long-term position.</t>
         </is>
       </c>
     </row>
@@ -3590,11 +3674,22 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="250" customHeight="1">
+    <row r="19" ht="192" customHeight="1">
       <c r="A19" s="45" t="n"/>
       <c r="B19" s="46" t="inlineStr">
         <is>
-          <t>Stability and steady compounder — one of the most reliable semiconductor businesses in the world. Broadcom makes the networking chips that connect all the GPUs inside hyperscaler data centers. As AI clusters scale to hundreds of thousands of GPUs, the networking infrastructure connecting them becomes more valuable and more complex. Broadcom also has a massive software revenue stream from its VMware acquisition that provides recurring cash flow stability. Management is world-class at capital allocation. This is a core hold that compounds quietly while the AI buildout accelerates.</t>
+          <t>Stability and steady compounder — one of the most
+reliable semiconductor businesses in the world.
+Broadcom makes the networking chips that connect all
+the GPUs inside hyperscaler data centers. As AI
+clusters scale to hundreds of thousands of GPUs, the
+networking infrastructure connecting them becomes more
+valuable and more complex. Broadcom also has a massive
+software revenue stream from its VMware acquisition
+that provides recurring cash flow stability. Management
+is world-class at capital allocation. This is a core
+hold that compounds quietly while the AI buildout
+accelerates.</t>
         </is>
       </c>
     </row>
@@ -3611,11 +3706,22 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="250" customHeight="1">
+    <row r="22" ht="192" customHeight="1">
       <c r="A22" s="43" t="n"/>
       <c r="B22" s="44" t="inlineStr">
         <is>
-          <t>Stability and steady compounder — DRAM equipment leader. Lam Research makes the etch and deposition equipment that builds memory chips (DRAM and NAND). AI requires massive amounts of high-bandwidth memory (HBM), and every HBM chip that gets manufactured requires Lam's tools. This gives Lam direct and durable exposure to the AI memory build-out without the volatility of owning the memory chipmakers directly. The business is highly recurring (installed base + consumables) and grows every time wafer starts increase. A core picks-and-shovels play for the AI infrastructure trade.</t>
+          <t>Stability and steady compounder — DRAM equipment
+leader. Lam Research makes the etch and deposition
+equipment that builds memory chips (DRAM and NAND). AI
+requires massive amounts of high-bandwidth memory
+(HBM), and every HBM chip that gets manufactured
+requires Lam's tools. This gives Lam direct and durable
+exposure to the AI memory build-out without the
+volatility of owning the memory chipmakers directly.
+The business is highly recurring (installed base +
+consumables) and grows every time wafer starts
+increase. A core picks-and-shovels play for the AI
+infrastructure trade.</t>
         </is>
       </c>
     </row>
@@ -3632,11 +3738,22 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="250" customHeight="1">
+    <row r="25" ht="192" customHeight="1">
       <c r="A25" s="45" t="n"/>
       <c r="B25" s="46" t="inlineStr">
         <is>
-          <t>CPU maker deep in the AI infrastructure stack and the only credible challenger to NVIDIA in AI accelerators. AMD's MI300X GPU is winning meaningful enterprise AI workloads, particularly inference, where customers want a cheaper alternative to NVIDIA's H100/H200. On the CPU side, AMD's EPYC chips power a huge share of hyperscaler server infrastructure. The AI narrative is also shifting down-stack into CPU makers — AMD benefits from both trends simultaneously. Risk: NVIDIA's software moat (CUDA) is still wide. But as a compounder and a hedge on NVIDIA dominance, AMD belongs in the portfolio.</t>
+          <t>CPU maker deep in the AI infrastructure stack and the
+only credible challenger to NVIDIA in AI accelerators.
+AMD's MI300X GPU is winning meaningful enterprise AI
+workloads, particularly inference, where customers want
+a cheaper alternative to NVIDIA's H100/H200. On the CPU
+side, AMD's EPYC chips power a huge share of
+hyperscaler server infrastructure. The AI narrative is
+also shifting down-stack into CPU makers — AMD benefits
+from both trends simultaneously. Risk: NVIDIA's
+software moat (CUDA) is still wide. But as a compounder
+and a hedge on NVIDIA dominance, AMD belongs in the
+portfolio.</t>
         </is>
       </c>
     </row>
@@ -3653,11 +3770,24 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="250" customHeight="1">
+    <row r="28" ht="222" customHeight="1">
       <c r="A28" s="43" t="n"/>
       <c r="B28" s="44" t="inlineStr">
         <is>
-          <t>CPU maker in the AI infrastructure stack and the most controversial turnaround story in semiconductors. Intel lost its manufacturing lead to TSMC and its AI accelerator business to NVIDIA and AMD. The thesis here is a turnaround: new management, massive government subsidies via the CHIPS Act, and a path to reclaiming leading-edge manufacturing through its Intel Foundry Services (IFS) division. If the turnaround works, INTC is deeply undervalued. If it doesn't, the downside is meaningful. This is a higher-risk position — size it as a speculative turnaround bet, not a core hold. The AI infrastructure narrative (CPU makers shifting down-stack) gives it a tailwind even without a full recovery.</t>
+          <t>CPU maker in the AI infrastructure stack and the most
+controversial turnaround story in semiconductors. Intel
+lost its manufacturing lead to TSMC and its AI
+accelerator business to NVIDIA and AMD. The thesis here
+is a turnaround: new management, massive government
+subsidies via the CHIPS Act, and a path to reclaiming
+leading-edge manufacturing through its Intel Foundry
+Services (IFS) division. If the turnaround works, INTC
+is deeply undervalued. If it doesn't, the downside is
+meaningful. This is a higher-risk position — size it as
+a speculative turnaround bet, not a core hold. The AI
+infrastructure narrative (CPU makers shifting down-
+stack) gives it a tailwind even without a full
+recovery.</t>
         </is>
       </c>
     </row>
@@ -3674,11 +3804,22 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="250" customHeight="1">
+    <row r="31" ht="192" customHeight="1">
       <c r="A31" s="45" t="n"/>
       <c r="B31" s="46" t="inlineStr">
         <is>
-          <t>The architecture behind nearly every AI chip that isn't an x86 CPU. ARM licenses its instruction set architecture to Apple, Qualcomm, Amazon (Graviton), Google, NVIDIA, and dozens of others. Every time an AI edge chip, smartphone chip, or custom datacenter chip gets designed and sold, ARM earns a royalty. This is a pure royalty business model — no manufacturing risk, no inventory risk — just IP licensing that scales with every chip shipped globally. As AI moves to the edge (phones, cars, robots), ARM's exposure compounds. The royalty rate per chip is also increasing as designs get more complex. A core compounder.</t>
+          <t>The architecture behind nearly every AI chip that isn't
+an x86 CPU. ARM licenses its instruction set
+architecture to Apple, Qualcomm, Amazon (Graviton),
+Google, NVIDIA, and dozens of others. Every time an AI
+edge chip, smartphone chip, or custom datacenter chip
+gets designed and sold, ARM earns a royalty. This is a
+pure royalty business model — no manufacturing risk, no
+inventory risk — just IP licensing that scales with
+every chip shipped globally. As AI moves to the edge
+(phones, cars, robots), ARM's exposure compounds. The
+royalty rate per chip is also increasing as designs get
+more complex. A core compounder.</t>
         </is>
       </c>
     </row>
@@ -3756,7 +3897,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
         </is>
       </c>
     </row>
@@ -4385,11 +4526,24 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="250" customHeight="1">
+    <row r="17" ht="222" customHeight="1">
       <c r="A17" s="43" t="n"/>
       <c r="B17" s="44" t="inlineStr">
         <is>
-          <t>The NVDA-parallel picks-and-shovels bet for AI power. Navitas makes GaN (gallium nitride) power chips that are radically more efficient than traditional silicon-based power delivery. AI data centers are hitting a hard wall on power density — the amount of electricity you can push into a rack is physically limited by current power conversion technology. GaN solves this by converting power more efficiently and at higher frequencies, enabling denser, cooler, more power-efficient data centers. As hyperscalers build out hundreds of gigawatts of AI compute, NVTS stands to be a critical infrastructure supplier. High-risk, asymmetric upside — the kind of bet that looks obvious in hindsight.</t>
+          <t>The NVDA-parallel picks-and-shovels bet for AI power.
+Navitas makes GaN (gallium nitride) power chips that
+are radically more efficient than traditional silicon-
+based power delivery. AI data centers are hitting a
+hard wall on power density — the amount of electricity
+you can push into a rack is physically limited by
+current power conversion technology. GaN solves this by
+converting power more efficiently and at higher
+frequencies, enabling denser, cooler, more power-
+efficient data centers. As hyperscalers build out
+hundreds of gigawatts of AI compute, NVTS stands to be
+a critical infrastructure supplier. High-risk,
+asymmetric upside — the kind of bet that looks obvious
+in hindsight.</t>
         </is>
       </c>
     </row>
@@ -4406,11 +4560,22 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="250" customHeight="1">
+    <row r="20" ht="192" customHeight="1">
       <c r="A20" s="45" t="n"/>
       <c r="B20" s="46" t="inlineStr">
         <is>
-          <t>Classic shovels-in-a-gold-rush setup. AEHR makes specialized semiconductor burn-in and test equipment used to stress-test chips before they ship. As AI chips become more complex and expensive (each H100 costs $30k+), the cost of shipping a defective chip becomes enormous — which means chip manufacturers are investing heavily in advanced testing. More AI chips manufactured = more testing bottleneck demand = more AEHR revenue. The business is lumpy (large equipment orders), which creates volatility, but the long-term tailwind is durable. A pure picks-and-shovels beneficiary of the AI chip production ramp.</t>
+          <t>Classic shovels-in-a-gold-rush setup. AEHR makes
+specialized semiconductor burn-in and test equipment
+used to stress-test chips before they ship. As AI chips
+become more complex and expensive (each H100 costs
+$30k+), the cost of shipping a defective chip becomes
+enormous — which means chip manufacturers are investing
+heavily in advanced testing. More AI chips manufactured
+= more testing bottleneck demand = more AEHR revenue.
+The business is lumpy (large equipment orders), which
+creates volatility, but the long-term tailwind is
+durable. A pure picks-and-shovels beneficiary of the AI
+chip production ramp.</t>
         </is>
       </c>
     </row>
@@ -4427,11 +4592,23 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="250" customHeight="1">
+    <row r="23" ht="207" customHeight="1">
       <c r="A23" s="43" t="n"/>
       <c r="B23" s="44" t="inlineStr">
         <is>
-          <t>One of the cleanest AI infrastructure picks-and-shovels names available. GPUs are useless if the data can't move between them fast enough. Credo makes high-speed SerDes (serializer/deserializer) connectivity chips that are the plumbing inside AI data centers — connecting GPUs to memory, switches, and storage at speeds that match the compute throughput. As AI clusters scale from thousands to hundreds of thousands of GPUs, the interconnect bandwidth requirement explodes. Credo has direct customer relationships with hyperscalers and is already generating real revenue from the AI buildout. Strong execution, growing bookings, and a durable structural tailwind.</t>
+          <t>One of the cleanest AI infrastructure picks-and-shovels
+names available. GPUs are useless if the data can't
+move between them fast enough. Credo makes high-speed
+SerDes (serializer/deserializer) connectivity chips
+that are the plumbing inside AI data centers —
+connecting GPUs to memory, switches, and storage at
+speeds that match the compute throughput. As AI
+clusters scale from thousands to hundreds of thousands
+of GPUs, the interconnect bandwidth requirement
+explodes. Credo has direct customer relationships with
+hyperscalers and is already generating real revenue
+from the AI buildout. Strong execution, growing
+bookings, and a durable structural tailwind.</t>
         </is>
       </c>
     </row>
@@ -4448,11 +4625,23 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="250" customHeight="1">
+    <row r="26" ht="207" customHeight="1">
       <c r="A26" s="45" t="n"/>
       <c r="B26" s="46" t="inlineStr">
         <is>
-          <t>A quiet compounder that is early in its AI rerating narrative. Allegro makes power management and sensing semiconductors used in automotive, industrial, and increasingly AI hardware applications. As AI hardware demands more precise power delivery and thermal sensing, Allegro's chips become more embedded in the data center infrastructure. The automotive exposure (EV power management) provides a separate growth vector. Less hype than the pure-play AI names, which means it hasn't been fully rerated yet — creating a potential catch-up opportunity. More of a steady grower than a moonshot, but with meaningful upside as the narrative broadens.</t>
+          <t>A quiet compounder that is early in its AI rerating
+narrative. Allegro makes power management and sensing
+semiconductors used in automotive, industrial, and
+increasingly AI hardware applications. As AI hardware
+demands more precise power delivery and thermal
+sensing, Allegro's chips become more embedded in the
+data center infrastructure. The automotive exposure (EV
+power management) provides a separate growth vector.
+Less hype than the pure-play AI names, which means it
+hasn't been fully rerated yet — creating a potential
+catch-up opportunity. More of a steady grower than a
+moonshot, but with meaningful upside as the narrative
+broadens.</t>
         </is>
       </c>
     </row>
@@ -4469,11 +4658,23 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="250" customHeight="1">
+    <row r="29" ht="207" customHeight="1">
       <c r="A29" s="43" t="n"/>
       <c r="B29" s="44" t="inlineStr">
         <is>
-          <t>An often-overlooked ADR with cyclical breakout behavior. Himax makes display driver ICs and AI vision chips used in AR/VR devices, automotive displays, and AI edge sensing applications. When AI edge device cycles accelerate — smartphones, AR glasses, smart cameras — Himax tends to move fast. It's historically undervalued relative to its revenue and has a pattern of sharp re-ratings on earnings beats during upcycles. The AR/AI vision chip exposure is genuinely interesting as AI moves from the cloud to the edge. Higher volatility, but the kind of name that can double in a single cycle. Treat as a tactical position sized for the volatility.</t>
+          <t>An often-overlooked ADR with cyclical breakout
+behavior. Himax makes display driver ICs and AI vision
+chips used in AR/VR devices, automotive displays, and
+AI edge sensing applications. When AI edge device
+cycles accelerate — smartphones, AR glasses, smart
+cameras — Himax tends to move fast. It's historically
+undervalued relative to its revenue and has a pattern
+of sharp re-ratings on earnings beats during upcycles.
+The AR/AI vision chip exposure is genuinely interesting
+as AI moves from the cloud to the edge. Higher
+volatility, but the kind of name that can double in a
+single cycle. Treat as a tactical position sized for
+the volatility.</t>
         </is>
       </c>
     </row>
@@ -4490,11 +4691,23 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="250" customHeight="1">
+    <row r="32" ht="207" customHeight="1">
       <c r="A32" s="45" t="n"/>
       <c r="B32" s="46" t="inlineStr">
         <is>
-          <t>Less hype, more industrial AI backbone. MACOM makes RF, microwave, and high-speed analog chips used in data center interconnects, telecom backbones, and defense systems. As AI data centers demand ever-higher bandwidth between racks and buildings, MACOM's optical and RF interconnect chips become critical infrastructure. The telecom angle also gives it exposure to 5G buildout and the long-term bandwidth expansion required to support AI inference at the edge. Not a headline name, but a steady grower with durable end-market demand. The kind of stock that compounds quietly while the hype goes elsewhere, then re-rates when the market catches up.</t>
+          <t>Less hype, more industrial AI backbone. MACOM makes RF,
+microwave, and high-speed analog chips used in data
+center interconnects, telecom backbones, and defense
+systems. As AI data centers demand ever-higher
+bandwidth between racks and buildings, MACOM's optical
+and RF interconnect chips become critical
+infrastructure. The telecom angle also gives it
+exposure to 5G buildout and the long-term bandwidth
+expansion required to support AI inference at the edge.
+Not a headline name, but a steady grower with durable
+end-market demand. The kind of stock that compounds
+quietly while the hype goes elsewhere, then re-rates
+when the market catches up.</t>
         </is>
       </c>
     </row>
@@ -4511,11 +4724,24 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="250" customHeight="1">
+    <row r="35" ht="222" customHeight="1">
       <c r="A35" s="43" t="n"/>
       <c r="B35" s="44" t="inlineStr">
         <is>
-          <t>Pure asymmetric bet — low probability, high upside if they execute. Aeva makes FMCW (frequency-modulated continuous-wave) lidar sensors for autonomous vehicles and robotics. Their approach is technically differentiated — FMCW lidar can detect velocity directly (not just position) and works better in adverse conditions than traditional lidar. The autonomous vehicle and robotics market is massive if it materializes, and Aeva would be a key sensing supplier. Still in early commercialization — revenue is minimal and the path to profitability is long. This is a speculative moonshot, not a core position. Size it as a lottery ticket: accept that it could go to zero, but the upside if robotics/AV take off is 10-20x.</t>
+          <t>Pure asymmetric bet — low probability, high upside if
+they execute. Aeva makes FMCW (frequency-modulated
+continuous-wave) lidar sensors for autonomous vehicles
+and robotics. Their approach is technically
+differentiated — FMCW lidar can detect velocity
+directly (not just position) and works better in
+adverse conditions than traditional lidar. The
+autonomous vehicle and robotics market is massive if it
+materializes, and Aeva would be a key sensing supplier.
+Still in early commercialization — revenue is minimal
+and the path to profitability is long. This is a
+speculative moonshot, not a core position. Size it as a
+lottery ticket: accept that it could go to zero, but
+the upside if robotics/AV take off is 10-20x.</t>
         </is>
       </c>
     </row>
@@ -4593,7 +4819,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
         </is>
       </c>
     </row>
@@ -4820,11 +5046,25 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="250" customHeight="1">
+    <row r="11" ht="237" customHeight="1">
       <c r="A11" s="43" t="n"/>
       <c r="B11" s="44" t="inlineStr">
         <is>
-          <t>King of Photonics — and this could be a genuine moonshot. Lumentum makes the optical components (lasers, transceivers, photonic integrated circuits) that transmit data at the speed of light inside and between AI data centers. As AI clusters scale to hundreds of thousands of GPUs spread across multiple buildings, the optical interconnect becomes the critical bottleneck — you can't run copper cables at those distances and speeds. Lumentum is one of the few companies with the technology and scale to supply this infrastructure. The AI tailwind here is massive and underappreciated. Photonics is the next big narrative after GPUs and power — when the market wakes up to the data movement bottleneck, LITE is the headline name. High conviction, high risk, moonshot potential.</t>
+          <t>King of Photonics — and this could be a genuine
+moonshot. Lumentum makes the optical components
+(lasers, transceivers, photonic integrated circuits)
+that transmit data at the speed of light inside and
+between AI data centers. As AI clusters scale to
+hundreds of thousands of GPUs spread across multiple
+buildings, the optical interconnect becomes the
+critical bottleneck — you can't run copper cables at
+those distances and speeds. Lumentum is one of the few
+companies with the technology and scale to supply this
+infrastructure. The AI tailwind here is massive and
+underappreciated. Photonics is the next big narrative
+after GPUs and power — when the market wakes up to the
+data movement bottleneck, LITE is the headline name.
+High conviction, high risk, moonshot potential.</t>
         </is>
       </c>
     </row>
@@ -4902,7 +5142,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
         </is>
       </c>
     </row>
@@ -5330,11 +5570,23 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="250" customHeight="1">
+    <row r="14" ht="207" customHeight="1">
       <c r="A14" s="43" t="n"/>
       <c r="B14" s="44" t="inlineStr">
         <is>
-          <t>The actual builder and materials company in the AI data center trade. AI data centers are physical buildings requiring massive earthmoving, foundation work, and construction equipment — and Caterpillar is the dominant supplier of that heavy equipment globally. Every hyperscaler campus that Meta, Google, Microsoft, and Amazon builds requires CAT equipment on site. This is a steadier, lower-volatility way to play the AI infrastructure buildout than the semiconductor names. CAT also benefits from infrastructure spending more broadly (roads, bridges, energy projects) which provides diversification. A solid core position — steady compounder with the AI tailwind as a bonus.</t>
+          <t>The actual builder and materials company in the AI data
+center trade. AI data centers are physical buildings
+requiring massive earthmoving, foundation work, and
+construction equipment — and Caterpillar is the
+dominant supplier of that heavy equipment globally.
+Every hyperscaler campus that Meta, Google, Microsoft,
+and Amazon builds requires CAT equipment on site. This
+is a steadier, lower-volatility way to play the AI
+infrastructure buildout than the semiconductor names.
+CAT also benefits from infrastructure spending more
+broadly (roads, bridges, energy projects) which
+provides diversification. A solid core position —
+steady compounder with the AI tailwind as a bonus.</t>
         </is>
       </c>
     </row>
@@ -5351,11 +5603,23 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="250" customHeight="1">
+    <row r="17" ht="207" customHeight="1">
       <c r="A17" s="45" t="n"/>
       <c r="B17" s="46" t="inlineStr">
         <is>
-          <t>Builder AND cooling company — one of the best-positioned picks-and-shovels plays in the AI buildout. Comfort Systems provides HVAC, mechanical, plumbing, and electrical systems for commercial buildings, including AI data centers. Cooling is a MAJOR and growing bottleneck in AI data centers — every GPU cluster generates enormous heat that must be managed. FIX designs and installs the entire MEP (mechanical, electrical, plumbing) system that keeps these facilities running. They have direct contracts with hyperscalers and are seeing demand accelerate as AI data center construction ramps. A quality business with real earnings growth, not a speculative bet.</t>
+          <t>Builder AND cooling company — one of the best-
+positioned picks-and-shovels plays in the AI buildout.
+Comfort Systems provides HVAC, mechanical, plumbing,
+and electrical systems for commercial buildings,
+including AI data centers. Cooling is a MAJOR and
+growing bottleneck in AI data centers — every GPU
+cluster generates enormous heat that must be managed.
+FIX designs and installs the entire MEP (mechanical,
+electrical, plumbing) system that keeps these
+facilities running. They have direct contracts with
+hyperscalers and are seeing demand accelerate as AI
+data center construction ramps. A quality business with
+real earnings growth, not a speculative bet.</t>
         </is>
       </c>
     </row>
@@ -5372,11 +5636,23 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="250" customHeight="1">
+    <row r="20" ht="207" customHeight="1">
       <c r="A20" s="43" t="n"/>
       <c r="B20" s="44" t="inlineStr">
         <is>
-          <t>Electrical infrastructure builder for AI data centers — the company that builds the switchgear, motor control centers, and power distribution equipment that routes electricity inside data centers and industrial facilities. As AI data centers require ever-larger amounts of power (some campus projects exceed 1 GW), the electrical infrastructure to safely distribute that power becomes a critical bottleneck. Powell has a backlog-heavy business model with long-cycle orders, which means revenue visibility is strong. Less volatile than the semiconductor names because of the order backlog and industrial nature of the business. A solid mid-cap infrastructure pick with a genuine AI tailwind.</t>
+          <t>Electrical infrastructure builder for AI data centers —
+the company that builds the switchgear, motor control
+centers, and power distribution equipment that routes
+electricity inside data centers and industrial
+facilities. As AI data centers require ever-larger
+amounts of power (some campus projects exceed 1 GW),
+the electrical infrastructure to safely distribute that
+power becomes a critical bottleneck. Powell has a
+backlog-heavy business model with long-cycle orders,
+which means revenue visibility is strong. Less volatile
+than the semiconductor names because of the order
+backlog and industrial nature of the business. A solid
+mid-cap infrastructure pick with a genuine AI tailwind.</t>
         </is>
       </c>
     </row>
@@ -5393,11 +5669,23 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="250" customHeight="1">
+    <row r="23" ht="207" customHeight="1">
       <c r="A23" s="45" t="n"/>
       <c r="B23" s="46" t="inlineStr">
         <is>
-          <t>The premier AI data center cooling play and one of the most direct beneficiaries of the AI buildout. Vertiv makes thermal management systems (liquid cooling, air cooling, heat exchangers) along with power distribution infrastructure for data centers. Cooling is not optional — you cannot run a GPU cluster without solving the thermal problem, and as GPU power consumption has exploded from 300W to 700W per chip, existing cooling infrastructure is completely inadequate. Every new AI data center that gets built needs Vertiv's systems. The company has multi-year backlog, growing margins, and is adding capacity to meet demand. A high-conviction hold in the AI infrastructure basket.</t>
+          <t>The premier AI data center cooling play and one of the
+most direct beneficiaries of the AI buildout. Vertiv
+makes thermal management systems (liquid cooling, air
+cooling, heat exchangers) along with power distribution
+infrastructure for data centers. Cooling is not
+optional — you cannot run a GPU cluster without solving
+the thermal problem, and as GPU power consumption has
+exploded from 300W to 700W per chip, existing cooling
+infrastructure is completely inadequate. Every new AI
+data center that gets built needs Vertiv's systems. The
+company has multi-year backlog, growing margins, and is
+adding capacity to meet demand. A high-conviction hold
+in the AI infrastructure basket.</t>
         </is>
       </c>
     </row>
@@ -5475,7 +5763,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
         </is>
       </c>
     </row>
@@ -5903,11 +6191,23 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="250" customHeight="1">
+    <row r="14" ht="207" customHeight="1">
       <c r="A14" s="43" t="n"/>
       <c r="B14" s="44" t="inlineStr">
         <is>
-          <t>Stability and steady compounder — the premier power generation and grid equipment company spun out of GE. GE Vernova makes gas turbines, wind turbines, grid software, and electrification equipment. AI data centers are consuming power at a rate that is straining the US electrical grid, and new power generation capacity takes years to build. GE Vernova is one of the few companies with the scale and installed base to actually supply that new capacity fast. Their gas turbine backlog is multi-year and growing. This is not a speculative bet — it's a high-quality industrial compounder with a very real and durable demand tailwind from AI power needs. A core long-term hold.</t>
+          <t>Stability and steady compounder — the premier power
+generation and grid equipment company spun out of GE.
+GE Vernova makes gas turbines, wind turbines, grid
+software, and electrification equipment. AI data
+centers are consuming power at a rate that is straining
+the US electrical grid, and new power generation
+capacity takes years to build. GE Vernova is one of the
+few companies with the scale and installed base to
+actually supply that new capacity fast. Their gas
+turbine backlog is multi-year and growing. This is not
+a speculative bet — it's a high-quality industrial
+compounder with a very real and durable demand tailwind
+from AI power needs. A core long-term hold.</t>
         </is>
       </c>
     </row>
@@ -5924,11 +6224,25 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="250" customHeight="1">
+    <row r="17" ht="237" customHeight="1">
       <c r="A17" s="45" t="n"/>
       <c r="B17" s="46" t="inlineStr">
         <is>
-          <t>Power grid infrastructure and maintenance — a growing bottleneck for the AI buildout. Quanta Services is the largest specialty contractor for electric power infrastructure in North America. They build and maintain power lines, substations, and grid connections that are essential to delivering electricity to AI data centers. Every new data center campus needs a grid connection, often requiring new transmission lines and substations — all of which Quanta builds. The company has multi-year visibility through its backlog and framework agreements with utilities. A steady, high-quality compounder that benefits directly and durably from the AI power demand surge. Lower volatility than the semiconductor names with a comparably strong tailwind.</t>
+          <t>Power grid infrastructure and maintenance — a growing
+bottleneck for the AI buildout. Quanta Services is the
+largest specialty contractor for electric power
+infrastructure in North America. They build and
+maintain power lines, substations, and grid connections
+that are essential to delivering electricity to AI data
+centers. Every new data center campus needs a grid
+connection, often requiring new transmission lines and
+substations — all of which Quanta builds. The company
+has multi-year visibility through its backlog and
+framework agreements with utilities. A steady, high-
+quality compounder that benefits directly and durably
+from the AI power demand surge. Lower volatility than
+the semiconductor names with a comparably strong
+tailwind.</t>
         </is>
       </c>
     </row>
@@ -5945,11 +6259,25 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="250" customHeight="1">
+    <row r="20" ht="237" customHeight="1">
       <c r="A20" s="43" t="n"/>
       <c r="B20" s="44" t="inlineStr">
         <is>
-          <t>Moonshot potential if hydrogen and fuel cell technology takes off — and the AI power crisis is accelerating the timeline. Bloom Energy makes solid oxide fuel cells that generate electricity on-site without connecting to the grid. For AI data centers that need reliable, clean, on-site power (especially in areas with grid congestion), Bloom's solution is genuinely compelling. They're already selling to data centers and have partnerships with major tech companies. The bull case: AI power demand is so acute that on-site generation becomes mandatory, and Bloom is uniquely positioned. The bear case: fuel cells are expensive and hydrogen infrastructure is still nascent. Worth holding a position — the upside if they win even a small share of the AI power market is very large.</t>
+          <t>Moonshot potential if hydrogen and fuel cell technology
+takes off — and the AI power crisis is accelerating the
+timeline. Bloom Energy makes solid oxide fuel cells
+that generate electricity on-site without connecting to
+the grid. For AI data centers that need reliable,
+clean, on-site power (especially in areas with grid
+congestion), Bloom's solution is genuinely compelling.
+They're already selling to data centers and have
+partnerships with major tech companies. The bull case:
+AI power demand is so acute that on-site generation
+becomes mandatory, and Bloom is uniquely positioned.
+The bear case: fuel cells are expensive and hydrogen
+infrastructure is still nascent. Worth holding a
+position — the upside if they win even a small share of
+the AI power market is very large.</t>
         </is>
       </c>
     </row>
@@ -5966,11 +6294,26 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="250" customHeight="1">
+    <row r="23" ht="252" customHeight="1">
       <c r="A23" s="45" t="n"/>
       <c r="B23" s="46" t="inlineStr">
         <is>
-          <t>Nuclear SMRs and nuclear fuel waste company with massive moonshot potential — but big regulatory and execution risk. Oklo is building small modular nuclear reactors (SMRs) that could provide clean, always-on baseload power for AI data centers at scale. Several major tech companies (including Microsoft) have already signed nuclear power agreements, signaling that nuclear is being taken seriously as an AI power solution. Oklo also has a fuel recycling angle (using spent nuclear fuel) that could be a significant business in itself. The regulatory path is long and uncertain, and Oklo has not yet built a commercial reactor. This is a small-% portfolio position — accept that it could go to zero, but the upside if nuclear SMRs get commercially deployed is enormous and the valuation reflects very little of that potential today.</t>
+          <t>Nuclear SMRs and nuclear fuel waste company with
+massive moonshot potential — but big regulatory and
+execution risk. Oklo is building small modular nuclear
+reactors (SMRs) that could provide clean, always-on
+baseload power for AI data centers at scale. Several
+major tech companies (including Microsoft) have already
+signed nuclear power agreements, signaling that nuclear
+is being taken seriously as an AI power solution. Oklo
+also has a fuel recycling angle (using spent nuclear
+fuel) that could be a significant business in itself.
+The regulatory path is long and uncertain, and Oklo has
+not yet built a commercial reactor. This is a small-%
+portfolio position — accept that it could go to zero,
+but the upside if nuclear SMRs get commercially
+deployed is enormous and the valuation reflects very
+little of that potential today.</t>
         </is>
       </c>
     </row>
@@ -6048,7 +6391,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
         </is>
       </c>
     </row>
@@ -6342,11 +6685,28 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="250" customHeight="1">
+    <row r="12" ht="282" customHeight="1">
       <c r="A12" s="43" t="n"/>
       <c r="B12" s="44" t="inlineStr">
         <is>
-          <t>The leading Neocloud and one of the most interesting companies in this portfolio. Nebius is a modern Amazon/Google-style company: it has a primary product (GPU cloud computing for AI companies that can't get capacity from AWS/Azure/GCP) AND multiple other revenue streams that could each become massive independently — Clickhouse (high-performance analytics database used by thousands of companies), AV Ride (autonomous vehicle tech), and others. The neocloud thesis: hyperscalers are capacity-constrained and have long waitlists for GPU compute, creating a massive opening for alternative cloud providers. NBIS is the best-positioned name to fill that gap. I believe this company could become a future Hyperscaler in the same way Amazon AWS or Google Cloud became defining infrastructure businesses. High conviction, long-term hold — this is the kind of company you look back on in 10 years and wish you owned more of.</t>
+          <t>The leading Neocloud and one of the most interesting
+companies in this portfolio. Nebius is a modern
+Amazon/Google-style company: it has a primary product
+(GPU cloud computing for AI companies that can't get
+capacity from AWS/Azure/GCP) AND multiple other revenue
+streams that could each become massive independently —
+Clickhouse (high-performance analytics database used by
+thousands of companies), AV Ride (autonomous vehicle
+tech), and others. The neocloud thesis: hyperscalers
+are capacity-constrained and have long waitlists for
+GPU compute, creating a massive opening for alternative
+cloud providers. NBIS is the best-positioned name to
+fill that gap. I believe this company could become a
+future Hyperscaler in the same way Amazon AWS or Google
+Cloud became defining infrastructure businesses. High
+conviction, long-term hold — this is the kind of
+company you look back on in 10 years and wish you owned
+more of.</t>
         </is>
       </c>
     </row>
@@ -6363,11 +6723,25 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="250" customHeight="1">
+    <row r="15" ht="237" customHeight="1">
       <c r="A15" s="45" t="n"/>
       <c r="B15" s="46" t="inlineStr">
         <is>
-          <t>So integral to the entire US government AI stack that it is effectively a national security asset. Palantir's software (Gotham for government, Foundry for enterprise, AIP for AI) is deeply embedded in the Department of Defense, intelligence agencies, and dozens of federal programs. You don't rip out Palantir — agencies build entire workflows on top of it. The AI Platform (AIP) is now being adopted by commercial enterprises as well, opening a second growth vector. The $1.5T defense budget and accelerating government AI spending is a direct tailwind. Yes, the valuation is demanding, but for a company this strategically embedded, the premium is arguably justified. An outlier name outside the data center trade that belongs in a long-term AI portfolio.</t>
+          <t>So integral to the entire US government AI stack that
+it is effectively a national security asset. Palantir's
+software (Gotham for government, Foundry for
+enterprise, AIP for AI) is deeply embedded in the
+Department of Defense, intelligence agencies, and
+dozens of federal programs. You don't rip out Palantir
+— agencies build entire workflows on top of it. The AI
+Platform (AIP) is now being adopted by commercial
+enterprises as well, opening a second growth vector.
+The $1.5T defense budget and accelerating government AI
+spending is a direct tailwind. Yes, the valuation is
+demanding, but for a company this strategically
+embedded, the premium is arguably justified. An outlier
+name outside the data center trade that belongs in a
+long-term AI portfolio.</t>
         </is>
       </c>
     </row>
@@ -6445,7 +6819,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:01 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
         </is>
       </c>
     </row>
@@ -6672,11 +7046,28 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="250" customHeight="1">
+    <row r="11" ht="282" customHeight="1">
       <c r="A11" s="43" t="n"/>
       <c r="B11" s="44" t="inlineStr">
         <is>
-          <t>Drones and defense tech — very speculative but with a massive catalyst behind it. The US government just announced a $1.5 trillion defense budget with $56 billion going specifically to drones and counter-drones through the DAWG (Drone and Autonomous Warfare Group) program. Ondas is one of the few small-cap companies with actual drone technology, recent acquisitions in the space, and partnerships that position them to compete for these contracts. Their March 2026 acquisitions and partnerships were specifically designed to make them a stronger DAWG program competitor. This is not a guaranteed win — it's a very speculative bet on a small company winning government contracts in a highly competitive space. But if they win even a small slice of the $56B drone budget, the upside from current levels is enormous. Size it appropriately — this could go to zero or it could 5-10x.</t>
+          <t>Drones and defense tech — very speculative but with a
+massive catalyst behind it. The US government just
+announced a $1.5 trillion defense budget with $56
+billion going specifically to drones and counter-drones
+through the DAWG (Drone and Autonomous Warfare Group)
+program. Ondas is one of the few small-cap companies
+with actual drone technology, recent acquisitions in
+the space, and partnerships that position them to
+compete for these contracts. Their March 2026
+acquisitions and partnerships were specifically
+designed to make them a stronger DAWG program
+competitor. This is not a guaranteed win — it's a very
+speculative bet on a small company winning government
+contracts in a highly competitive space. But if they
+win even a small slice of the $56B drone budget, the
+upside from current levels is enormous. Size it
+appropriately — this could go to zero or it could
+5-10x.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add price alerts and Google Sheets export functionality
Adds a new "Price Alert" column with conditional formatting to the Excel tracker and introduces a new script for exporting data to Google Sheets.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 0e261129-5f60-425b-94f8-0a84a3815978
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -31,7 +31,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="+0.00&quot;%&quot;;-0.00&quot;%&quot;;0.00&quot;%&quot;"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -162,6 +162,12 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="007F3F00"/>
       <sz val="10"/>
     </font>
     <font>
@@ -332,7 +338,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="116">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -428,6 +434,9 @@
     <xf numFmtId="10" fontId="0" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -437,6 +446,9 @@
     <xf numFmtId="10" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -450,18 +462,18 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -638,7 +650,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -651,7 +663,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
     <dxf>
       <font>
         <name val="Calibri"/>
@@ -675,6 +687,28 @@
         <patternFill patternType="solid">
           <fgColor rgb="00FFC7CE"/>
           <bgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="00FFFFFF"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FF6600"/>
+          <bgColor rgb="00FF6600"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF0E0"/>
+          <bgColor rgb="00FFF0E0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1071,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:R11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1539,10 +1573,11 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="97" t="inlineStr">
+      <c r="A1" s="99" t="inlineStr">
         <is>
           <t>🚀 Space Economy</t>
         </is>
@@ -1558,107 +1593,113 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="98" t="inlineStr">
+      <c r="A4" s="100" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="98" t="inlineStr">
+      <c r="B4" s="100" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="98" t="inlineStr">
+      <c r="C4" s="100" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="98" t="inlineStr">
+      <c r="D4" s="100" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="98" t="inlineStr">
+      <c r="E4" s="100" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="98" t="inlineStr">
+      <c r="F4" s="100" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="98" t="inlineStr">
+      <c r="G4" s="100" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="98" t="inlineStr">
+      <c r="H4" s="100" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="98" t="inlineStr">
+      <c r="I4" s="100" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="98" t="inlineStr">
+      <c r="J4" s="100" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="98" t="inlineStr">
+      <c r="K4" s="100" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="98" t="inlineStr">
+      <c r="L4" s="100" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="98" t="inlineStr">
+      <c r="M4" s="100" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="98" t="inlineStr">
+      <c r="N4" s="100" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="98" t="inlineStr">
+      <c r="O4" s="100" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="98" t="inlineStr">
+      <c r="P4" s="100" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="98" t="inlineStr">
+      <c r="Q4" s="100" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
         </is>
       </c>
+      <c r="R4" s="100" t="inlineStr">
+        <is>
+          <t>Price
+Alert</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
@@ -1726,68 +1767,73 @@
         <f>IFERROR(P5/E5-1,"")</f>
         <v/>
       </c>
+      <c r="R5" s="33">
+        <f>IF(AND(M5&gt;0,E5&gt;0,O5&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="99" t="inlineStr">
+      <c r="A7" s="101" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H7" s="100">
+      <c r="H7" s="102">
         <f>SUM(H5:H5)</f>
         <v/>
       </c>
-      <c r="I7" s="100">
+      <c r="I7" s="102">
         <f>SUM(I5:I5)</f>
         <v/>
       </c>
-      <c r="J7" s="100">
+      <c r="J7" s="102">
         <f>SUM(J5:J5)</f>
         <v/>
       </c>
-      <c r="K7" s="101">
+      <c r="K7" s="103">
         <f>IFERROR(J7/H7,"")</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="102" t="inlineStr">
+      <c r="A9" s="104" t="inlineStr">
         <is>
           <t>INVESTMENT THESIS &amp; RESEARCH NOTES</t>
         </is>
       </c>
-      <c r="B9" s="103" t="n"/>
-      <c r="C9" s="103" t="n"/>
-      <c r="D9" s="103" t="n"/>
-      <c r="E9" s="103" t="n"/>
-      <c r="F9" s="103" t="n"/>
-      <c r="G9" s="103" t="n"/>
-      <c r="H9" s="103" t="n"/>
-      <c r="I9" s="103" t="n"/>
-      <c r="J9" s="103" t="n"/>
-      <c r="K9" s="103" t="n"/>
-      <c r="L9" s="103" t="n"/>
-      <c r="M9" s="103" t="n"/>
-      <c r="N9" s="103" t="n"/>
-      <c r="O9" s="103" t="n"/>
-      <c r="P9" s="103" t="n"/>
-      <c r="Q9" s="103" t="n"/>
+      <c r="B9" s="105" t="n"/>
+      <c r="C9" s="105" t="n"/>
+      <c r="D9" s="105" t="n"/>
+      <c r="E9" s="105" t="n"/>
+      <c r="F9" s="105" t="n"/>
+      <c r="G9" s="105" t="n"/>
+      <c r="H9" s="105" t="n"/>
+      <c r="I9" s="105" t="n"/>
+      <c r="J9" s="105" t="n"/>
+      <c r="K9" s="105" t="n"/>
+      <c r="L9" s="105" t="n"/>
+      <c r="M9" s="105" t="n"/>
+      <c r="N9" s="105" t="n"/>
+      <c r="O9" s="105" t="n"/>
+      <c r="P9" s="105" t="n"/>
+      <c r="Q9" s="105" t="n"/>
+      <c r="R9" s="105" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="41" t="inlineStr">
+      <c r="A10" s="43" t="inlineStr">
         <is>
           <t>RKLB</t>
         </is>
       </c>
-      <c r="B10" s="42" t="inlineStr">
+      <c r="B10" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rocket Lab USA   |   Risk: High</t>
         </is>
       </c>
     </row>
     <row r="11" ht="282" customHeight="1">
-      <c r="A11" s="43" t="n"/>
-      <c r="B11" s="44" t="inlineStr">
+      <c r="A11" s="45" t="n"/>
+      <c r="B11" s="46" t="inlineStr">
         <is>
           <t>Space economy and space infrastructure — huge future
 TAM over the next decade and beyond. Rocket Lab is the
@@ -1813,9 +1859,9 @@
     <row r="12" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A3:R3"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A1:R1"/>
     <mergeCell ref="A7:G7"/>
   </mergeCells>
   <conditionalFormatting sqref="J5">
@@ -1834,6 +1880,16 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="R5">
+    <cfRule type="expression" priority="5" dxfId="2">
+      <formula>$O5&lt;-0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A5:Q5">
+    <cfRule type="expression" priority="6" dxfId="3">
+      <formula>$O5&lt;-0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1845,7 +1901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:R15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1865,10 +1921,11 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="104" t="inlineStr">
+      <c r="A1" s="106" t="inlineStr">
         <is>
           <t>🔭 Long Term Watchlist</t>
         </is>
@@ -1884,107 +1941,113 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="105" t="inlineStr">
+      <c r="A4" s="107" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="105" t="inlineStr">
+      <c r="B4" s="107" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="105" t="inlineStr">
+      <c r="C4" s="107" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="105" t="inlineStr">
+      <c r="D4" s="107" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="105" t="inlineStr">
+      <c r="E4" s="107" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="105" t="inlineStr">
+      <c r="F4" s="107" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="105" t="inlineStr">
+      <c r="G4" s="107" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="105" t="inlineStr">
+      <c r="H4" s="107" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="105" t="inlineStr">
+      <c r="I4" s="107" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="105" t="inlineStr">
+      <c r="J4" s="107" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="105" t="inlineStr">
+      <c r="K4" s="107" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="105" t="inlineStr">
+      <c r="L4" s="107" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="105" t="inlineStr">
+      <c r="M4" s="107" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="105" t="inlineStr">
+      <c r="N4" s="107" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="105" t="inlineStr">
+      <c r="O4" s="107" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="105" t="inlineStr">
+      <c r="P4" s="107" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="105" t="inlineStr">
+      <c r="Q4" s="107" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
         </is>
       </c>
+      <c r="R4" s="107" t="inlineStr">
+        <is>
+          <t>Price
+Alert</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
@@ -2052,9 +2115,13 @@
         <f>IFERROR(P5/E5-1,"")</f>
         <v/>
       </c>
+      <c r="R5" s="33">
+        <f>IF(AND(M5&gt;0,E5&gt;0,O5&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="33" t="inlineStr">
+      <c r="A6" s="34" t="inlineStr">
         <is>
           <t>NVO</t>
         </is>
@@ -2086,19 +2153,19 @@
       <c r="H6" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="34">
+      <c r="I6" s="35">
         <f>G6*H6</f>
         <v/>
       </c>
-      <c r="J6" s="34">
+      <c r="J6" s="35">
         <f>E6*H6</f>
         <v/>
       </c>
-      <c r="K6" s="34">
+      <c r="K6" s="35">
         <f>J6-I6</f>
         <v/>
       </c>
-      <c r="L6" s="35">
+      <c r="L6" s="36">
         <f>IFERROR(K6/I6,"")</f>
         <v/>
       </c>
@@ -2108,79 +2175,84 @@
       <c r="N6" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="O6" s="35">
+      <c r="O6" s="36">
         <f>IFERROR(E6/M6-1,"")</f>
         <v/>
       </c>
       <c r="P6" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="Q6" s="35">
+      <c r="Q6" s="36">
         <f>IFERROR(P6/E6-1,"")</f>
         <v/>
       </c>
+      <c r="R6" s="37">
+        <f>IF(AND(M6&gt;0,E6&gt;0,O6&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="106" t="inlineStr">
+      <c r="A8" s="108" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H8" s="107">
+      <c r="H8" s="109">
         <f>SUM(H5:H6)</f>
         <v/>
       </c>
-      <c r="I8" s="107">
+      <c r="I8" s="109">
         <f>SUM(I5:I6)</f>
         <v/>
       </c>
-      <c r="J8" s="107">
+      <c r="J8" s="109">
         <f>SUM(J5:J6)</f>
         <v/>
       </c>
-      <c r="K8" s="108">
+      <c r="K8" s="110">
         <f>IFERROR(J8/H8,"")</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="109" t="inlineStr">
+      <c r="A10" s="111" t="inlineStr">
         <is>
           <t>INVESTMENT THESIS &amp; RESEARCH NOTES</t>
         </is>
       </c>
-      <c r="B10" s="110" t="n"/>
-      <c r="C10" s="110" t="n"/>
-      <c r="D10" s="110" t="n"/>
-      <c r="E10" s="110" t="n"/>
-      <c r="F10" s="110" t="n"/>
-      <c r="G10" s="110" t="n"/>
-      <c r="H10" s="110" t="n"/>
-      <c r="I10" s="110" t="n"/>
-      <c r="J10" s="110" t="n"/>
-      <c r="K10" s="110" t="n"/>
-      <c r="L10" s="110" t="n"/>
-      <c r="M10" s="110" t="n"/>
-      <c r="N10" s="110" t="n"/>
-      <c r="O10" s="110" t="n"/>
-      <c r="P10" s="110" t="n"/>
-      <c r="Q10" s="110" t="n"/>
+      <c r="B10" s="112" t="n"/>
+      <c r="C10" s="112" t="n"/>
+      <c r="D10" s="112" t="n"/>
+      <c r="E10" s="112" t="n"/>
+      <c r="F10" s="112" t="n"/>
+      <c r="G10" s="112" t="n"/>
+      <c r="H10" s="112" t="n"/>
+      <c r="I10" s="112" t="n"/>
+      <c r="J10" s="112" t="n"/>
+      <c r="K10" s="112" t="n"/>
+      <c r="L10" s="112" t="n"/>
+      <c r="M10" s="112" t="n"/>
+      <c r="N10" s="112" t="n"/>
+      <c r="O10" s="112" t="n"/>
+      <c r="P10" s="112" t="n"/>
+      <c r="Q10" s="112" t="n"/>
+      <c r="R10" s="112" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="41" t="inlineStr">
+      <c r="A11" s="43" t="inlineStr">
         <is>
           <t>RBRK</t>
         </is>
       </c>
-      <c r="B11" s="42" t="inlineStr">
+      <c r="B11" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rubrik Inc   |   Risk: Med-High</t>
         </is>
       </c>
     </row>
     <row r="12" ht="222" customHeight="1">
-      <c r="A12" s="43" t="n"/>
-      <c r="B12" s="44" t="inlineStr">
+      <c r="A12" s="45" t="n"/>
+      <c r="B12" s="46" t="inlineStr">
         <is>
           <t>Under active long-term evaluation. Rubrik is a
 cybersecurity and data management company focused on
@@ -2201,20 +2273,20 @@
     </row>
     <row r="13" ht="8" customHeight="1"/>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="41" t="inlineStr">
+      <c r="A14" s="43" t="inlineStr">
         <is>
           <t>NVO</t>
         </is>
       </c>
-      <c r="B14" s="42" t="inlineStr">
+      <c r="B14" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Novo Nordisk   |   Risk: Medium</t>
         </is>
       </c>
     </row>
     <row r="15" ht="237" customHeight="1">
-      <c r="A15" s="45" t="n"/>
-      <c r="B15" s="46" t="inlineStr">
+      <c r="A15" s="47" t="n"/>
+      <c r="B15" s="48" t="inlineStr">
         <is>
           <t>Under active long-term evaluation. Novo Nordisk is the
 global leader in GLP-1 drugs (Ozempic, Wegovy) for
@@ -2237,10 +2309,10 @@
     <row r="16" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A3:R3"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A1:R1"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J6">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -2256,6 +2328,16 @@
     </cfRule>
     <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="1">
       <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R5:R6">
+    <cfRule type="expression" priority="5" dxfId="2">
+      <formula>$O5&lt;-0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A5:Q6">
+    <cfRule type="expression" priority="6" dxfId="3">
+      <formula>$O5&lt;-0.2</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2277,14 +2359,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="111" t="inlineStr">
+      <c r="A1" s="113" t="inlineStr">
         <is>
           <t>📝 RESEARCH NOTES &amp; INVESTMENT THESIS</t>
         </is>
       </c>
     </row>
     <row r="2" ht="35" customHeight="1">
-      <c r="A2" s="112" t="inlineStr">
+      <c r="A2" s="114" t="inlineStr">
         <is>
           <t>401k To-Do</t>
         </is>
@@ -2297,7 +2379,7 @@
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="113" t="inlineStr">
+      <c r="A3" s="115" t="inlineStr">
         <is>
           <t>Savings Account</t>
         </is>
@@ -2309,7 +2391,7 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="112" t="inlineStr">
+      <c r="A4" s="114" t="inlineStr">
         <is>
           <t>Research Tools</t>
         </is>
@@ -2321,7 +2403,7 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="113" t="inlineStr">
+      <c r="A5" s="115" t="inlineStr">
         <is>
           <t>Quantum Thesis</t>
         </is>
@@ -2333,7 +2415,7 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="112" t="inlineStr">
+      <c r="A6" s="114" t="inlineStr">
         <is>
           <t>NVTS</t>
         </is>
@@ -2345,7 +2427,7 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="113" t="inlineStr">
+      <c r="A7" s="115" t="inlineStr">
         <is>
           <t>AEHR</t>
         </is>
@@ -2357,7 +2439,7 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="112" t="inlineStr">
+      <c r="A8" s="114" t="inlineStr">
         <is>
           <t>CRDO</t>
         </is>
@@ -2369,7 +2451,7 @@
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="113" t="inlineStr">
+      <c r="A9" s="115" t="inlineStr">
         <is>
           <t>ALGM</t>
         </is>
@@ -2381,7 +2463,7 @@
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="112" t="inlineStr">
+      <c r="A10" s="114" t="inlineStr">
         <is>
           <t>HIMX</t>
         </is>
@@ -2393,7 +2475,7 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="113" t="inlineStr">
+      <c r="A11" s="115" t="inlineStr">
         <is>
           <t>MTSI</t>
         </is>
@@ -2405,7 +2487,7 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="112" t="inlineStr">
+      <c r="A12" s="114" t="inlineStr">
         <is>
           <t>AEVA</t>
         </is>
@@ -2417,7 +2499,7 @@
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="113" t="inlineStr">
+      <c r="A13" s="115" t="inlineStr">
         <is>
           <t>AI Infrastructure</t>
         </is>
@@ -2429,7 +2511,7 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="112" t="inlineStr">
+      <c r="A14" s="114" t="inlineStr">
         <is>
           <t>LITE</t>
         </is>
@@ -2441,7 +2523,7 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="113" t="inlineStr">
+      <c r="A15" s="115" t="inlineStr">
         <is>
           <t>OKLO</t>
         </is>
@@ -2453,7 +2535,7 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="112" t="inlineStr">
+      <c r="A16" s="114" t="inlineStr">
         <is>
           <t>NBIS</t>
         </is>
@@ -2465,7 +2547,7 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="113" t="inlineStr">
+      <c r="A17" s="115" t="inlineStr">
         <is>
           <t>PLTR</t>
         </is>
@@ -2477,7 +2559,7 @@
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="112" t="inlineStr">
+      <c r="A18" s="114" t="inlineStr">
         <is>
           <t>ONDS</t>
         </is>
@@ -2489,7 +2571,7 @@
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="113" t="inlineStr">
+      <c r="A19" s="115" t="inlineStr">
         <is>
           <t>RKLB</t>
         </is>
@@ -2501,7 +2583,7 @@
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="112" t="inlineStr">
+      <c r="A20" s="114" t="inlineStr">
         <is>
           <t>Recommended Portfolio</t>
         </is>
@@ -2527,7 +2609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q19"/>
+  <dimension ref="A1:R19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2547,6 +2629,7 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -2566,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
         </is>
       </c>
     </row>
@@ -2667,6 +2750,12 @@
 Target</t>
         </is>
       </c>
+      <c r="R4" s="26" t="inlineStr">
+        <is>
+          <t>Price
+Alert</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
@@ -2734,9 +2823,13 @@
         <f>IFERROR(P5/E5-1,"")</f>
         <v/>
       </c>
+      <c r="R5" s="33">
+        <f>IF(AND(M5&gt;0,E5&gt;0,O5&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="33" t="inlineStr">
+      <c r="A6" s="34" t="inlineStr">
         <is>
           <t>RGTI</t>
         </is>
@@ -2768,19 +2861,19 @@
       <c r="H6" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="34">
+      <c r="I6" s="35">
         <f>G6*H6</f>
         <v/>
       </c>
-      <c r="J6" s="34">
+      <c r="J6" s="35">
         <f>E6*H6</f>
         <v/>
       </c>
-      <c r="K6" s="34">
+      <c r="K6" s="35">
         <f>J6-I6</f>
         <v/>
       </c>
-      <c r="L6" s="35">
+      <c r="L6" s="36">
         <f>IFERROR(K6/I6,"")</f>
         <v/>
       </c>
@@ -2790,15 +2883,19 @@
       <c r="N6" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="O6" s="35">
+      <c r="O6" s="36">
         <f>IFERROR(E6/M6-1,"")</f>
         <v/>
       </c>
       <c r="P6" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="Q6" s="35">
+      <c r="Q6" s="36">
         <f>IFERROR(P6/E6-1,"")</f>
+        <v/>
+      </c>
+      <c r="R6" s="37">
+        <f>IF(AND(M6&gt;0,E6&gt;0,O6&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
         <v/>
       </c>
     </row>
@@ -2868,68 +2965,73 @@
         <f>IFERROR(P7/E7-1,"")</f>
         <v/>
       </c>
+      <c r="R7" s="33">
+        <f>IF(AND(M7&gt;0,E7&gt;0,O7&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="36" t="inlineStr">
+      <c r="A9" s="38" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H9" s="37">
+      <c r="H9" s="39">
         <f>SUM(H5:H7)</f>
         <v/>
       </c>
-      <c r="I9" s="37">
+      <c r="I9" s="39">
         <f>SUM(I5:I7)</f>
         <v/>
       </c>
-      <c r="J9" s="37">
+      <c r="J9" s="39">
         <f>SUM(J5:J7)</f>
         <v/>
       </c>
-      <c r="K9" s="38">
+      <c r="K9" s="40">
         <f>IFERROR(J9/H9,"")</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="39" t="inlineStr">
+      <c r="A11" s="41" t="inlineStr">
         <is>
           <t>INVESTMENT THESIS &amp; RESEARCH NOTES</t>
         </is>
       </c>
-      <c r="B11" s="40" t="n"/>
-      <c r="C11" s="40" t="n"/>
-      <c r="D11" s="40" t="n"/>
-      <c r="E11" s="40" t="n"/>
-      <c r="F11" s="40" t="n"/>
-      <c r="G11" s="40" t="n"/>
-      <c r="H11" s="40" t="n"/>
-      <c r="I11" s="40" t="n"/>
-      <c r="J11" s="40" t="n"/>
-      <c r="K11" s="40" t="n"/>
-      <c r="L11" s="40" t="n"/>
-      <c r="M11" s="40" t="n"/>
-      <c r="N11" s="40" t="n"/>
-      <c r="O11" s="40" t="n"/>
-      <c r="P11" s="40" t="n"/>
-      <c r="Q11" s="40" t="n"/>
+      <c r="B11" s="42" t="n"/>
+      <c r="C11" s="42" t="n"/>
+      <c r="D11" s="42" t="n"/>
+      <c r="E11" s="42" t="n"/>
+      <c r="F11" s="42" t="n"/>
+      <c r="G11" s="42" t="n"/>
+      <c r="H11" s="42" t="n"/>
+      <c r="I11" s="42" t="n"/>
+      <c r="J11" s="42" t="n"/>
+      <c r="K11" s="42" t="n"/>
+      <c r="L11" s="42" t="n"/>
+      <c r="M11" s="42" t="n"/>
+      <c r="N11" s="42" t="n"/>
+      <c r="O11" s="42" t="n"/>
+      <c r="P11" s="42" t="n"/>
+      <c r="Q11" s="42" t="n"/>
+      <c r="R11" s="42" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="41" t="inlineStr">
+      <c r="A12" s="43" t="inlineStr">
         <is>
           <t>IONQ</t>
         </is>
       </c>
-      <c r="B12" s="42" t="inlineStr">
+      <c r="B12" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  IonQ Inc   |   Risk: Very High</t>
         </is>
       </c>
     </row>
     <row r="13" ht="177" customHeight="1">
-      <c r="A13" s="43" t="n"/>
-      <c r="B13" s="44" t="inlineStr">
+      <c r="A13" s="45" t="n"/>
+      <c r="B13" s="46" t="inlineStr">
         <is>
           <t>Next quantum run candidate. The belief: 'Buy IONQ,
 RGTI, and QBTS — easy 10x within 2 years.' IonQ is the
@@ -2947,20 +3049,20 @@
     </row>
     <row r="14" ht="8" customHeight="1"/>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="41" t="inlineStr">
+      <c r="A15" s="43" t="inlineStr">
         <is>
           <t>RGTI</t>
         </is>
       </c>
-      <c r="B15" s="42" t="inlineStr">
+      <c r="B15" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rigetti Computing   |   Risk: Very High</t>
         </is>
       </c>
     </row>
     <row r="16" ht="177" customHeight="1">
-      <c r="A16" s="45" t="n"/>
-      <c r="B16" s="46" t="inlineStr">
+      <c r="A16" s="47" t="n"/>
+      <c r="B16" s="48" t="inlineStr">
         <is>
           <t>Next quantum run candidate alongside IONQ and QBTS.
 Rigetti builds its own quantum processors and offers
@@ -2978,20 +3080,20 @@
     </row>
     <row r="17" ht="8" customHeight="1"/>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="41" t="inlineStr">
+      <c r="A18" s="43" t="inlineStr">
         <is>
           <t>QBTS</t>
         </is>
       </c>
-      <c r="B18" s="42" t="inlineStr">
+      <c r="B18" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  D-Wave Quantum   |   Risk: Very High</t>
         </is>
       </c>
     </row>
     <row r="19" ht="177" customHeight="1">
-      <c r="A19" s="43" t="n"/>
-      <c r="B19" s="44" t="inlineStr">
+      <c r="A19" s="45" t="n"/>
+      <c r="B19" s="46" t="inlineStr">
         <is>
           <t>Next quantum run candidate alongside IONQ and RGTI.
 D-Wave is unique in that it uses quantum annealing
@@ -3010,9 +3112,9 @@
     <row r="20" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A3:R3"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A1:R1"/>
     <mergeCell ref="A9:G9"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J7">
@@ -3031,6 +3133,16 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="R5:R7">
+    <cfRule type="expression" priority="5" dxfId="2">
+      <formula>$O5&lt;-0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A5:Q7">
+    <cfRule type="expression" priority="6" dxfId="3">
+      <formula>$O5&lt;-0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3042,7 +3154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q31"/>
+  <dimension ref="A1:R31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3062,10 +3174,11 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="47" t="inlineStr">
+      <c r="A1" s="49" t="inlineStr">
         <is>
           <t>🖥️ Semiconductors &amp; Compute</t>
         </is>
@@ -3081,107 +3194,113 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="48" t="inlineStr">
+      <c r="A4" s="50" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="48" t="inlineStr">
+      <c r="B4" s="50" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="48" t="inlineStr">
+      <c r="C4" s="50" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="48" t="inlineStr">
+      <c r="D4" s="50" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="48" t="inlineStr">
+      <c r="E4" s="50" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="48" t="inlineStr">
+      <c r="F4" s="50" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="48" t="inlineStr">
+      <c r="G4" s="50" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="48" t="inlineStr">
+      <c r="H4" s="50" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="48" t="inlineStr">
+      <c r="I4" s="50" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="48" t="inlineStr">
+      <c r="J4" s="50" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="48" t="inlineStr">
+      <c r="K4" s="50" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="48" t="inlineStr">
+      <c r="L4" s="50" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="48" t="inlineStr">
+      <c r="M4" s="50" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="48" t="inlineStr">
+      <c r="N4" s="50" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="48" t="inlineStr">
+      <c r="O4" s="50" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="48" t="inlineStr">
+      <c r="P4" s="50" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="48" t="inlineStr">
+      <c r="Q4" s="50" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
         </is>
       </c>
+      <c r="R4" s="50" t="inlineStr">
+        <is>
+          <t>Price
+Alert</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
@@ -3249,9 +3368,13 @@
         <f>IFERROR(P5/E5-1,"")</f>
         <v/>
       </c>
+      <c r="R5" s="33">
+        <f>IF(AND(M5&gt;0,E5&gt;0,O5&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="33" t="inlineStr">
+      <c r="A6" s="34" t="inlineStr">
         <is>
           <t>AVGO</t>
         </is>
@@ -3274,7 +3397,7 @@
       <c r="E6" s="28" t="n">
         <v>425.44</v>
       </c>
-      <c r="F6" s="49" t="n">
+      <c r="F6" s="51" t="n">
         <v>-1.518517953378183</v>
       </c>
       <c r="G6" s="28" t="n">
@@ -3283,19 +3406,19 @@
       <c r="H6" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="34">
+      <c r="I6" s="35">
         <f>G6*H6</f>
         <v/>
       </c>
-      <c r="J6" s="34">
+      <c r="J6" s="35">
         <f>E6*H6</f>
         <v/>
       </c>
-      <c r="K6" s="34">
+      <c r="K6" s="35">
         <f>J6-I6</f>
         <v/>
       </c>
-      <c r="L6" s="35">
+      <c r="L6" s="36">
         <f>IFERROR(K6/I6,"")</f>
         <v/>
       </c>
@@ -3305,15 +3428,19 @@
       <c r="N6" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="O6" s="35">
+      <c r="O6" s="36">
         <f>IFERROR(E6/M6-1,"")</f>
         <v/>
       </c>
       <c r="P6" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="Q6" s="35">
+      <c r="Q6" s="36">
         <f>IFERROR(P6/E6-1,"")</f>
+        <v/>
+      </c>
+      <c r="R6" s="37">
+        <f>IF(AND(M6&gt;0,E6&gt;0,O6&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
         <v/>
       </c>
     </row>
@@ -3383,9 +3510,13 @@
         <f>IFERROR(P7/E7-1,"")</f>
         <v/>
       </c>
+      <c r="R7" s="33">
+        <f>IF(AND(M7&gt;0,E7&gt;0,O7&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="33" t="inlineStr">
+      <c r="A8" s="34" t="inlineStr">
         <is>
           <t>AMD</t>
         </is>
@@ -3417,19 +3548,19 @@
       <c r="H8" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="34">
+      <c r="I8" s="35">
         <f>G8*H8</f>
         <v/>
       </c>
-      <c r="J8" s="34">
+      <c r="J8" s="35">
         <f>E8*H8</f>
         <v/>
       </c>
-      <c r="K8" s="34">
+      <c r="K8" s="35">
         <f>J8-I8</f>
         <v/>
       </c>
-      <c r="L8" s="35">
+      <c r="L8" s="36">
         <f>IFERROR(K8/I8,"")</f>
         <v/>
       </c>
@@ -3439,15 +3570,19 @@
       <c r="N8" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="O8" s="35">
+      <c r="O8" s="36">
         <f>IFERROR(E8/M8-1,"")</f>
         <v/>
       </c>
       <c r="P8" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="Q8" s="35">
+      <c r="Q8" s="36">
         <f>IFERROR(P8/E8-1,"")</f>
+        <v/>
+      </c>
+      <c r="R8" s="37">
+        <f>IF(AND(M8&gt;0,E8&gt;0,O8&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
         <v/>
       </c>
     </row>
@@ -3475,7 +3610,7 @@
       <c r="E9" s="28" t="n">
         <v>113.01</v>
       </c>
-      <c r="F9" s="49" t="n">
+      <c r="F9" s="51" t="n">
         <v>-0.2999540042077861</v>
       </c>
       <c r="G9" s="28" t="n">
@@ -3517,9 +3652,13 @@
         <f>IFERROR(P9/E9-1,"")</f>
         <v/>
       </c>
+      <c r="R9" s="33">
+        <f>IF(AND(M9&gt;0,E9&gt;0,O9&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="33" t="inlineStr">
+      <c r="A10" s="34" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
@@ -3551,19 +3690,19 @@
       <c r="H10" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="I10" s="34">
+      <c r="I10" s="35">
         <f>G10*H10</f>
         <v/>
       </c>
-      <c r="J10" s="34">
+      <c r="J10" s="35">
         <f>E10*H10</f>
         <v/>
       </c>
-      <c r="K10" s="34">
+      <c r="K10" s="35">
         <f>J10-I10</f>
         <v/>
       </c>
-      <c r="L10" s="35">
+      <c r="L10" s="36">
         <f>IFERROR(K10/I10,"")</f>
         <v/>
       </c>
@@ -3573,79 +3712,84 @@
       <c r="N10" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="O10" s="35">
+      <c r="O10" s="36">
         <f>IFERROR(E10/M10-1,"")</f>
         <v/>
       </c>
       <c r="P10" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="Q10" s="35">
+      <c r="Q10" s="36">
         <f>IFERROR(P10/E10-1,"")</f>
         <v/>
       </c>
+      <c r="R10" s="37">
+        <f>IF(AND(M10&gt;0,E10&gt;0,O10&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="50" t="inlineStr">
+      <c r="A12" s="52" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H12" s="51">
+      <c r="H12" s="53">
         <f>SUM(H5:H10)</f>
         <v/>
       </c>
-      <c r="I12" s="51">
+      <c r="I12" s="53">
         <f>SUM(I5:I10)</f>
         <v/>
       </c>
-      <c r="J12" s="51">
+      <c r="J12" s="53">
         <f>SUM(J5:J10)</f>
         <v/>
       </c>
-      <c r="K12" s="52">
+      <c r="K12" s="54">
         <f>IFERROR(J12/H12,"")</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="53" t="inlineStr">
+      <c r="A14" s="55" t="inlineStr">
         <is>
           <t>INVESTMENT THESIS &amp; RESEARCH NOTES</t>
         </is>
       </c>
-      <c r="B14" s="54" t="n"/>
-      <c r="C14" s="54" t="n"/>
-      <c r="D14" s="54" t="n"/>
-      <c r="E14" s="54" t="n"/>
-      <c r="F14" s="54" t="n"/>
-      <c r="G14" s="54" t="n"/>
-      <c r="H14" s="54" t="n"/>
-      <c r="I14" s="54" t="n"/>
-      <c r="J14" s="54" t="n"/>
-      <c r="K14" s="54" t="n"/>
-      <c r="L14" s="54" t="n"/>
-      <c r="M14" s="54" t="n"/>
-      <c r="N14" s="54" t="n"/>
-      <c r="O14" s="54" t="n"/>
-      <c r="P14" s="54" t="n"/>
-      <c r="Q14" s="54" t="n"/>
+      <c r="B14" s="56" t="n"/>
+      <c r="C14" s="56" t="n"/>
+      <c r="D14" s="56" t="n"/>
+      <c r="E14" s="56" t="n"/>
+      <c r="F14" s="56" t="n"/>
+      <c r="G14" s="56" t="n"/>
+      <c r="H14" s="56" t="n"/>
+      <c r="I14" s="56" t="n"/>
+      <c r="J14" s="56" t="n"/>
+      <c r="K14" s="56" t="n"/>
+      <c r="L14" s="56" t="n"/>
+      <c r="M14" s="56" t="n"/>
+      <c r="N14" s="56" t="n"/>
+      <c r="O14" s="56" t="n"/>
+      <c r="P14" s="56" t="n"/>
+      <c r="Q14" s="56" t="n"/>
+      <c r="R14" s="56" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="41" t="inlineStr">
+      <c r="A15" s="43" t="inlineStr">
         <is>
           <t>NVDA</t>
         </is>
       </c>
-      <c r="B15" s="42" t="inlineStr">
+      <c r="B15" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  NVIDIA Corp   |   Risk: Medium</t>
         </is>
       </c>
     </row>
     <row r="16" ht="177" customHeight="1">
-      <c r="A16" s="43" t="n"/>
-      <c r="B16" s="44" t="inlineStr">
+      <c r="A16" s="45" t="n"/>
+      <c r="B16" s="46" t="inlineStr">
         <is>
           <t>The AI compute king and the core stability position in
 this portfolio. NVIDIA doesn't just make GPUs — it has
@@ -3663,20 +3807,20 @@
     </row>
     <row r="17" ht="8" customHeight="1"/>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="41" t="inlineStr">
+      <c r="A18" s="43" t="inlineStr">
         <is>
           <t>AVGO</t>
         </is>
       </c>
-      <c r="B18" s="42" t="inlineStr">
+      <c r="B18" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Broadcom Inc   |   Risk: Medium</t>
         </is>
       </c>
     </row>
     <row r="19" ht="192" customHeight="1">
-      <c r="A19" s="45" t="n"/>
-      <c r="B19" s="46" t="inlineStr">
+      <c r="A19" s="47" t="n"/>
+      <c r="B19" s="48" t="inlineStr">
         <is>
           <t>Stability and steady compounder — one of the most
 reliable semiconductor businesses in the world.
@@ -3695,20 +3839,20 @@
     </row>
     <row r="20" ht="8" customHeight="1"/>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="41" t="inlineStr">
+      <c r="A21" s="43" t="inlineStr">
         <is>
           <t>LRCX</t>
         </is>
       </c>
-      <c r="B21" s="42" t="inlineStr">
+      <c r="B21" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Lam Research   |   Risk: Medium</t>
         </is>
       </c>
     </row>
     <row r="22" ht="192" customHeight="1">
-      <c r="A22" s="43" t="n"/>
-      <c r="B22" s="44" t="inlineStr">
+      <c r="A22" s="45" t="n"/>
+      <c r="B22" s="46" t="inlineStr">
         <is>
           <t>Stability and steady compounder — DRAM equipment
 leader. Lam Research makes the etch and deposition
@@ -3727,20 +3871,20 @@
     </row>
     <row r="23" ht="8" customHeight="1"/>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="41" t="inlineStr">
+      <c r="A24" s="43" t="inlineStr">
         <is>
           <t>AMD</t>
         </is>
       </c>
-      <c r="B24" s="42" t="inlineStr">
+      <c r="B24" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Advanced Micro Devices   |   Risk: Medium</t>
         </is>
       </c>
     </row>
     <row r="25" ht="192" customHeight="1">
-      <c r="A25" s="45" t="n"/>
-      <c r="B25" s="46" t="inlineStr">
+      <c r="A25" s="47" t="n"/>
+      <c r="B25" s="48" t="inlineStr">
         <is>
           <t>CPU maker deep in the AI infrastructure stack and the
 only credible challenger to NVIDIA in AI accelerators.
@@ -3759,20 +3903,20 @@
     </row>
     <row r="26" ht="8" customHeight="1"/>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="41" t="inlineStr">
+      <c r="A27" s="43" t="inlineStr">
         <is>
           <t>INTC</t>
         </is>
       </c>
-      <c r="B27" s="42" t="inlineStr">
+      <c r="B27" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Intel Corp   |   Risk: Med-High</t>
         </is>
       </c>
     </row>
     <row r="28" ht="222" customHeight="1">
-      <c r="A28" s="43" t="n"/>
-      <c r="B28" s="44" t="inlineStr">
+      <c r="A28" s="45" t="n"/>
+      <c r="B28" s="46" t="inlineStr">
         <is>
           <t>CPU maker in the AI infrastructure stack and the most
 controversial turnaround story in semiconductors. Intel
@@ -3793,20 +3937,20 @@
     </row>
     <row r="29" ht="8" customHeight="1"/>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="41" t="inlineStr">
+      <c r="A30" s="43" t="inlineStr">
         <is>
           <t>ARM</t>
         </is>
       </c>
-      <c r="B30" s="42" t="inlineStr">
+      <c r="B30" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Arm Holdings   |   Risk: Medium</t>
         </is>
       </c>
     </row>
     <row r="31" ht="192" customHeight="1">
-      <c r="A31" s="45" t="n"/>
-      <c r="B31" s="46" t="inlineStr">
+      <c r="A31" s="47" t="n"/>
+      <c r="B31" s="48" t="inlineStr">
         <is>
           <t>The architecture behind nearly every AI chip that isn't
 an x86 CPU. ARM licenses its instruction set
@@ -3826,9 +3970,9 @@
     <row r="32" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A3:R3"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A1:R1"/>
     <mergeCell ref="A12:G12"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J10">
@@ -3847,6 +3991,16 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="R5:R10">
+    <cfRule type="expression" priority="5" dxfId="2">
+      <formula>$O5&lt;-0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A5:Q10">
+    <cfRule type="expression" priority="6" dxfId="3">
+      <formula>$O5&lt;-0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3858,7 +4012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q35"/>
+  <dimension ref="A1:R35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3878,10 +4032,11 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="55" t="inlineStr">
+      <c r="A1" s="57" t="inlineStr">
         <is>
           <t>⚙️ AI Picks &amp; Shovels</t>
         </is>
@@ -3897,107 +4052,113 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="56" t="inlineStr">
+      <c r="A4" s="58" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="56" t="inlineStr">
+      <c r="B4" s="58" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="56" t="inlineStr">
+      <c r="C4" s="58" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="56" t="inlineStr">
+      <c r="D4" s="58" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="56" t="inlineStr">
+      <c r="E4" s="58" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="56" t="inlineStr">
+      <c r="F4" s="58" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="56" t="inlineStr">
+      <c r="G4" s="58" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="56" t="inlineStr">
+      <c r="H4" s="58" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="56" t="inlineStr">
+      <c r="I4" s="58" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="56" t="inlineStr">
+      <c r="J4" s="58" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="56" t="inlineStr">
+      <c r="K4" s="58" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="56" t="inlineStr">
+      <c r="L4" s="58" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="56" t="inlineStr">
+      <c r="M4" s="58" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="56" t="inlineStr">
+      <c r="N4" s="58" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="56" t="inlineStr">
+      <c r="O4" s="58" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="56" t="inlineStr">
+      <c r="P4" s="58" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="56" t="inlineStr">
+      <c r="Q4" s="58" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
         </is>
       </c>
+      <c r="R4" s="58" t="inlineStr">
+        <is>
+          <t>Price
+Alert</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
@@ -4065,9 +4226,13 @@
         <f>IFERROR(P5/E5-1,"")</f>
         <v/>
       </c>
+      <c r="R5" s="33">
+        <f>IF(AND(M5&gt;0,E5&gt;0,O5&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="33" t="inlineStr">
+      <c r="A6" s="34" t="inlineStr">
         <is>
           <t>AEHR</t>
         </is>
@@ -4099,19 +4264,19 @@
       <c r="H6" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="34">
+      <c r="I6" s="35">
         <f>G6*H6</f>
         <v/>
       </c>
-      <c r="J6" s="34">
+      <c r="J6" s="35">
         <f>E6*H6</f>
         <v/>
       </c>
-      <c r="K6" s="34">
+      <c r="K6" s="35">
         <f>J6-I6</f>
         <v/>
       </c>
-      <c r="L6" s="35">
+      <c r="L6" s="36">
         <f>IFERROR(K6/I6,"")</f>
         <v/>
       </c>
@@ -4121,15 +4286,19 @@
       <c r="N6" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="O6" s="35">
+      <c r="O6" s="36">
         <f>IFERROR(E6/M6-1,"")</f>
         <v/>
       </c>
       <c r="P6" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="Q6" s="35">
+      <c r="Q6" s="36">
         <f>IFERROR(P6/E6-1,"")</f>
+        <v/>
+      </c>
+      <c r="R6" s="37">
+        <f>IF(AND(M6&gt;0,E6&gt;0,O6&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
         <v/>
       </c>
     </row>
@@ -4157,7 +4326,7 @@
       <c r="E7" s="28" t="n">
         <v>198.29</v>
       </c>
-      <c r="F7" s="49" t="n">
+      <c r="F7" s="51" t="n">
         <v>-0.1057968331824622</v>
       </c>
       <c r="G7" s="28" t="n">
@@ -4199,9 +4368,13 @@
         <f>IFERROR(P7/E7-1,"")</f>
         <v/>
       </c>
+      <c r="R7" s="33">
+        <f>IF(AND(M7&gt;0,E7&gt;0,O7&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="33" t="inlineStr">
+      <c r="A8" s="34" t="inlineStr">
         <is>
           <t>ALGM</t>
         </is>
@@ -4233,19 +4406,19 @@
       <c r="H8" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="34">
+      <c r="I8" s="35">
         <f>G8*H8</f>
         <v/>
       </c>
-      <c r="J8" s="34">
+      <c r="J8" s="35">
         <f>E8*H8</f>
         <v/>
       </c>
-      <c r="K8" s="34">
+      <c r="K8" s="35">
         <f>J8-I8</f>
         <v/>
       </c>
-      <c r="L8" s="35">
+      <c r="L8" s="36">
         <f>IFERROR(K8/I8,"")</f>
         <v/>
       </c>
@@ -4255,15 +4428,19 @@
       <c r="N8" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="O8" s="35">
+      <c r="O8" s="36">
         <f>IFERROR(E8/M8-1,"")</f>
         <v/>
       </c>
       <c r="P8" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="Q8" s="35">
+      <c r="Q8" s="36">
         <f>IFERROR(P8/E8-1,"")</f>
+        <v/>
+      </c>
+      <c r="R8" s="37">
+        <f>IF(AND(M8&gt;0,E8&gt;0,O8&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
         <v/>
       </c>
     </row>
@@ -4291,7 +4468,7 @@
       <c r="E9" s="28" t="n">
         <v>12.33</v>
       </c>
-      <c r="F9" s="49" t="n">
+      <c r="F9" s="51" t="n">
         <v>-0.2830576327856492</v>
       </c>
       <c r="G9" s="28" t="n">
@@ -4333,9 +4510,13 @@
         <f>IFERROR(P9/E9-1,"")</f>
         <v/>
       </c>
+      <c r="R9" s="33">
+        <f>IF(AND(M9&gt;0,E9&gt;0,O9&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="33" t="inlineStr">
+      <c r="A10" s="34" t="inlineStr">
         <is>
           <t>MTSI</t>
         </is>
@@ -4367,19 +4548,19 @@
       <c r="H10" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="I10" s="34">
+      <c r="I10" s="35">
         <f>G10*H10</f>
         <v/>
       </c>
-      <c r="J10" s="34">
+      <c r="J10" s="35">
         <f>E10*H10</f>
         <v/>
       </c>
-      <c r="K10" s="34">
+      <c r="K10" s="35">
         <f>J10-I10</f>
         <v/>
       </c>
-      <c r="L10" s="35">
+      <c r="L10" s="36">
         <f>IFERROR(K10/I10,"")</f>
         <v/>
       </c>
@@ -4389,15 +4570,19 @@
       <c r="N10" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="O10" s="35">
+      <c r="O10" s="36">
         <f>IFERROR(E10/M10-1,"")</f>
         <v/>
       </c>
       <c r="P10" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="Q10" s="35">
+      <c r="Q10" s="36">
         <f>IFERROR(P10/E10-1,"")</f>
+        <v/>
+      </c>
+      <c r="R10" s="37">
+        <f>IF(AND(M10&gt;0,E10&gt;0,O10&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
         <v/>
       </c>
     </row>
@@ -4467,68 +4652,73 @@
         <f>IFERROR(P11/E11-1,"")</f>
         <v/>
       </c>
+      <c r="R11" s="33">
+        <f>IF(AND(M11&gt;0,E11&gt;0,O11&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="57" t="inlineStr">
+      <c r="A13" s="59" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H13" s="58">
+      <c r="H13" s="60">
         <f>SUM(H5:H11)</f>
         <v/>
       </c>
-      <c r="I13" s="58">
+      <c r="I13" s="60">
         <f>SUM(I5:I11)</f>
         <v/>
       </c>
-      <c r="J13" s="58">
+      <c r="J13" s="60">
         <f>SUM(J5:J11)</f>
         <v/>
       </c>
-      <c r="K13" s="59">
+      <c r="K13" s="61">
         <f>IFERROR(J13/H13,"")</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="60" t="inlineStr">
+      <c r="A15" s="62" t="inlineStr">
         <is>
           <t>INVESTMENT THESIS &amp; RESEARCH NOTES</t>
         </is>
       </c>
-      <c r="B15" s="61" t="n"/>
-      <c r="C15" s="61" t="n"/>
-      <c r="D15" s="61" t="n"/>
-      <c r="E15" s="61" t="n"/>
-      <c r="F15" s="61" t="n"/>
-      <c r="G15" s="61" t="n"/>
-      <c r="H15" s="61" t="n"/>
-      <c r="I15" s="61" t="n"/>
-      <c r="J15" s="61" t="n"/>
-      <c r="K15" s="61" t="n"/>
-      <c r="L15" s="61" t="n"/>
-      <c r="M15" s="61" t="n"/>
-      <c r="N15" s="61" t="n"/>
-      <c r="O15" s="61" t="n"/>
-      <c r="P15" s="61" t="n"/>
-      <c r="Q15" s="61" t="n"/>
+      <c r="B15" s="63" t="n"/>
+      <c r="C15" s="63" t="n"/>
+      <c r="D15" s="63" t="n"/>
+      <c r="E15" s="63" t="n"/>
+      <c r="F15" s="63" t="n"/>
+      <c r="G15" s="63" t="n"/>
+      <c r="H15" s="63" t="n"/>
+      <c r="I15" s="63" t="n"/>
+      <c r="J15" s="63" t="n"/>
+      <c r="K15" s="63" t="n"/>
+      <c r="L15" s="63" t="n"/>
+      <c r="M15" s="63" t="n"/>
+      <c r="N15" s="63" t="n"/>
+      <c r="O15" s="63" t="n"/>
+      <c r="P15" s="63" t="n"/>
+      <c r="Q15" s="63" t="n"/>
+      <c r="R15" s="63" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="41" t="inlineStr">
+      <c r="A16" s="43" t="inlineStr">
         <is>
           <t>NVTS</t>
         </is>
       </c>
-      <c r="B16" s="42" t="inlineStr">
+      <c r="B16" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Navitas Semiconductor   |   Risk: High</t>
         </is>
       </c>
     </row>
     <row r="17" ht="222" customHeight="1">
-      <c r="A17" s="43" t="n"/>
-      <c r="B17" s="44" t="inlineStr">
+      <c r="A17" s="45" t="n"/>
+      <c r="B17" s="46" t="inlineStr">
         <is>
           <t>The NVDA-parallel picks-and-shovels bet for AI power.
 Navitas makes GaN (gallium nitride) power chips that
@@ -4549,20 +4739,20 @@
     </row>
     <row r="18" ht="8" customHeight="1"/>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="41" t="inlineStr">
+      <c r="A19" s="43" t="inlineStr">
         <is>
           <t>AEHR</t>
         </is>
       </c>
-      <c r="B19" s="42" t="inlineStr">
+      <c r="B19" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  AEHR Test Systems   |   Risk: High</t>
         </is>
       </c>
     </row>
     <row r="20" ht="192" customHeight="1">
-      <c r="A20" s="45" t="n"/>
-      <c r="B20" s="46" t="inlineStr">
+      <c r="A20" s="47" t="n"/>
+      <c r="B20" s="48" t="inlineStr">
         <is>
           <t>Classic shovels-in-a-gold-rush setup. AEHR makes
 specialized semiconductor burn-in and test equipment
@@ -4581,20 +4771,20 @@
     </row>
     <row r="21" ht="8" customHeight="1"/>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="41" t="inlineStr">
+      <c r="A22" s="43" t="inlineStr">
         <is>
           <t>CRDO</t>
         </is>
       </c>
-      <c r="B22" s="42" t="inlineStr">
+      <c r="B22" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Credo Technology   |   Risk: High</t>
         </is>
       </c>
     </row>
     <row r="23" ht="207" customHeight="1">
-      <c r="A23" s="43" t="n"/>
-      <c r="B23" s="44" t="inlineStr">
+      <c r="A23" s="45" t="n"/>
+      <c r="B23" s="46" t="inlineStr">
         <is>
           <t>One of the cleanest AI infrastructure picks-and-shovels
 names available. GPUs are useless if the data can't
@@ -4614,20 +4804,20 @@
     </row>
     <row r="24" ht="8" customHeight="1"/>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="41" t="inlineStr">
+      <c r="A25" s="43" t="inlineStr">
         <is>
           <t>ALGM</t>
         </is>
       </c>
-      <c r="B25" s="42" t="inlineStr">
+      <c r="B25" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Allegro MicroSystems   |   Risk: Med-High</t>
         </is>
       </c>
     </row>
     <row r="26" ht="207" customHeight="1">
-      <c r="A26" s="45" t="n"/>
-      <c r="B26" s="46" t="inlineStr">
+      <c r="A26" s="47" t="n"/>
+      <c r="B26" s="48" t="inlineStr">
         <is>
           <t>A quiet compounder that is early in its AI rerating
 narrative. Allegro makes power management and sensing
@@ -4647,20 +4837,20 @@
     </row>
     <row r="27" ht="8" customHeight="1"/>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="41" t="inlineStr">
+      <c r="A28" s="43" t="inlineStr">
         <is>
           <t>HIMX</t>
         </is>
       </c>
-      <c r="B28" s="42" t="inlineStr">
+      <c r="B28" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Himax Technologies   |   Risk: High</t>
         </is>
       </c>
     </row>
     <row r="29" ht="207" customHeight="1">
-      <c r="A29" s="43" t="n"/>
-      <c r="B29" s="44" t="inlineStr">
+      <c r="A29" s="45" t="n"/>
+      <c r="B29" s="46" t="inlineStr">
         <is>
           <t>An often-overlooked ADR with cyclical breakout
 behavior. Himax makes display driver ICs and AI vision
@@ -4680,20 +4870,20 @@
     </row>
     <row r="30" ht="8" customHeight="1"/>
     <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="41" t="inlineStr">
+      <c r="A31" s="43" t="inlineStr">
         <is>
           <t>MTSI</t>
         </is>
       </c>
-      <c r="B31" s="42" t="inlineStr">
+      <c r="B31" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  MACOM Technology   |   Risk: Med-High</t>
         </is>
       </c>
     </row>
     <row r="32" ht="207" customHeight="1">
-      <c r="A32" s="45" t="n"/>
-      <c r="B32" s="46" t="inlineStr">
+      <c r="A32" s="47" t="n"/>
+      <c r="B32" s="48" t="inlineStr">
         <is>
           <t>Less hype, more industrial AI backbone. MACOM makes RF,
 microwave, and high-speed analog chips used in data
@@ -4713,20 +4903,20 @@
     </row>
     <row r="33" ht="8" customHeight="1"/>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="41" t="inlineStr">
+      <c r="A34" s="43" t="inlineStr">
         <is>
           <t>AEVA</t>
         </is>
       </c>
-      <c r="B34" s="42" t="inlineStr">
+      <c r="B34" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Aeva Technologies   |   Risk: Very High</t>
         </is>
       </c>
     </row>
     <row r="35" ht="222" customHeight="1">
-      <c r="A35" s="43" t="n"/>
-      <c r="B35" s="44" t="inlineStr">
+      <c r="A35" s="45" t="n"/>
+      <c r="B35" s="46" t="inlineStr">
         <is>
           <t>Pure asymmetric bet — low probability, high upside if
 they execute. Aeva makes FMCW (frequency-modulated
@@ -4748,10 +4938,10 @@
     <row r="36" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A3:R3"/>
+    <mergeCell ref="A2:R2"/>
     <mergeCell ref="A13:G13"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A1:R1"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J11">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -4769,6 +4959,16 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="R5:R11">
+    <cfRule type="expression" priority="5" dxfId="2">
+      <formula>$O5&lt;-0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A5:Q11">
+    <cfRule type="expression" priority="6" dxfId="3">
+      <formula>$O5&lt;-0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4780,7 +4980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:R11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4800,10 +5000,11 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="62" t="inlineStr">
+      <c r="A1" s="64" t="inlineStr">
         <is>
           <t>💡 Photonics &amp; Optics</t>
         </is>
@@ -4819,107 +5020,113 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="63" t="inlineStr">
+      <c r="A4" s="65" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="63" t="inlineStr">
+      <c r="B4" s="65" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="63" t="inlineStr">
+      <c r="C4" s="65" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="63" t="inlineStr">
+      <c r="D4" s="65" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="63" t="inlineStr">
+      <c r="E4" s="65" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="63" t="inlineStr">
+      <c r="F4" s="65" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="63" t="inlineStr">
+      <c r="G4" s="65" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="63" t="inlineStr">
+      <c r="H4" s="65" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="63" t="inlineStr">
+      <c r="I4" s="65" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="63" t="inlineStr">
+      <c r="J4" s="65" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="63" t="inlineStr">
+      <c r="K4" s="65" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="63" t="inlineStr">
+      <c r="L4" s="65" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="63" t="inlineStr">
+      <c r="M4" s="65" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="63" t="inlineStr">
+      <c r="N4" s="65" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="63" t="inlineStr">
+      <c r="O4" s="65" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="63" t="inlineStr">
+      <c r="P4" s="65" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="63" t="inlineStr">
+      <c r="Q4" s="65" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
         </is>
       </c>
+      <c r="R4" s="65" t="inlineStr">
+        <is>
+          <t>Price
+Alert</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
@@ -4945,7 +5152,7 @@
       <c r="E5" s="28" t="n">
         <v>944.28</v>
       </c>
-      <c r="F5" s="49" t="n">
+      <c r="F5" s="51" t="n">
         <v>-1.642619728464659</v>
       </c>
       <c r="G5" s="28" t="n">
@@ -4987,68 +5194,73 @@
         <f>IFERROR(P5/E5-1,"")</f>
         <v/>
       </c>
+      <c r="R5" s="33">
+        <f>IF(AND(M5&gt;0,E5&gt;0,O5&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="64" t="inlineStr">
+      <c r="A7" s="66" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H7" s="65">
+      <c r="H7" s="67">
         <f>SUM(H5:H5)</f>
         <v/>
       </c>
-      <c r="I7" s="65">
+      <c r="I7" s="67">
         <f>SUM(I5:I5)</f>
         <v/>
       </c>
-      <c r="J7" s="65">
+      <c r="J7" s="67">
         <f>SUM(J5:J5)</f>
         <v/>
       </c>
-      <c r="K7" s="66">
+      <c r="K7" s="68">
         <f>IFERROR(J7/H7,"")</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="67" t="inlineStr">
+      <c r="A9" s="69" t="inlineStr">
         <is>
           <t>INVESTMENT THESIS &amp; RESEARCH NOTES</t>
         </is>
       </c>
-      <c r="B9" s="68" t="n"/>
-      <c r="C9" s="68" t="n"/>
-      <c r="D9" s="68" t="n"/>
-      <c r="E9" s="68" t="n"/>
-      <c r="F9" s="68" t="n"/>
-      <c r="G9" s="68" t="n"/>
-      <c r="H9" s="68" t="n"/>
-      <c r="I9" s="68" t="n"/>
-      <c r="J9" s="68" t="n"/>
-      <c r="K9" s="68" t="n"/>
-      <c r="L9" s="68" t="n"/>
-      <c r="M9" s="68" t="n"/>
-      <c r="N9" s="68" t="n"/>
-      <c r="O9" s="68" t="n"/>
-      <c r="P9" s="68" t="n"/>
-      <c r="Q9" s="68" t="n"/>
+      <c r="B9" s="70" t="n"/>
+      <c r="C9" s="70" t="n"/>
+      <c r="D9" s="70" t="n"/>
+      <c r="E9" s="70" t="n"/>
+      <c r="F9" s="70" t="n"/>
+      <c r="G9" s="70" t="n"/>
+      <c r="H9" s="70" t="n"/>
+      <c r="I9" s="70" t="n"/>
+      <c r="J9" s="70" t="n"/>
+      <c r="K9" s="70" t="n"/>
+      <c r="L9" s="70" t="n"/>
+      <c r="M9" s="70" t="n"/>
+      <c r="N9" s="70" t="n"/>
+      <c r="O9" s="70" t="n"/>
+      <c r="P9" s="70" t="n"/>
+      <c r="Q9" s="70" t="n"/>
+      <c r="R9" s="70" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="41" t="inlineStr">
+      <c r="A10" s="43" t="inlineStr">
         <is>
           <t>LITE</t>
         </is>
       </c>
-      <c r="B10" s="42" t="inlineStr">
+      <c r="B10" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Lumentum Holdings   |   Risk: High</t>
         </is>
       </c>
     </row>
     <row r="11" ht="237" customHeight="1">
-      <c r="A11" s="43" t="n"/>
-      <c r="B11" s="44" t="inlineStr">
+      <c r="A11" s="45" t="n"/>
+      <c r="B11" s="46" t="inlineStr">
         <is>
           <t>King of Photonics — and this could be a genuine
 moonshot. Lumentum makes the optical components
@@ -5071,9 +5283,9 @@
     <row r="12" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A3:R3"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A1:R1"/>
     <mergeCell ref="A7:G7"/>
   </mergeCells>
   <conditionalFormatting sqref="J5">
@@ -5092,6 +5304,16 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="R5">
+    <cfRule type="expression" priority="5" dxfId="2">
+      <formula>$O5&lt;-0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A5:Q5">
+    <cfRule type="expression" priority="6" dxfId="3">
+      <formula>$O5&lt;-0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5103,7 +5325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:R23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5123,10 +5345,11 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="69" t="inlineStr">
+      <c r="A1" s="71" t="inlineStr">
         <is>
           <t>🏗️ DC Builders &amp; Cooling</t>
         </is>
@@ -5142,107 +5365,113 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="70" t="inlineStr">
+      <c r="A4" s="72" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="70" t="inlineStr">
+      <c r="B4" s="72" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="70" t="inlineStr">
+      <c r="C4" s="72" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="70" t="inlineStr">
+      <c r="D4" s="72" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="70" t="inlineStr">
+      <c r="E4" s="72" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="70" t="inlineStr">
+      <c r="F4" s="72" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="70" t="inlineStr">
+      <c r="G4" s="72" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="70" t="inlineStr">
+      <c r="H4" s="72" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="70" t="inlineStr">
+      <c r="I4" s="72" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="70" t="inlineStr">
+      <c r="J4" s="72" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="70" t="inlineStr">
+      <c r="K4" s="72" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="70" t="inlineStr">
+      <c r="L4" s="72" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="70" t="inlineStr">
+      <c r="M4" s="72" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="70" t="inlineStr">
+      <c r="N4" s="72" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="70" t="inlineStr">
+      <c r="O4" s="72" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="70" t="inlineStr">
+      <c r="P4" s="72" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="70" t="inlineStr">
+      <c r="Q4" s="72" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
         </is>
       </c>
+      <c r="R4" s="72" t="inlineStr">
+        <is>
+          <t>Price
+Alert</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
@@ -5310,9 +5539,13 @@
         <f>IFERROR(P5/E5-1,"")</f>
         <v/>
       </c>
+      <c r="R5" s="33">
+        <f>IF(AND(M5&gt;0,E5&gt;0,O5&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="33" t="inlineStr">
+      <c r="A6" s="34" t="inlineStr">
         <is>
           <t>FIX</t>
         </is>
@@ -5344,19 +5577,19 @@
       <c r="H6" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="34">
+      <c r="I6" s="35">
         <f>G6*H6</f>
         <v/>
       </c>
-      <c r="J6" s="34">
+      <c r="J6" s="35">
         <f>E6*H6</f>
         <v/>
       </c>
-      <c r="K6" s="34">
+      <c r="K6" s="35">
         <f>J6-I6</f>
         <v/>
       </c>
-      <c r="L6" s="35">
+      <c r="L6" s="36">
         <f>IFERROR(K6/I6,"")</f>
         <v/>
       </c>
@@ -5366,15 +5599,19 @@
       <c r="N6" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="O6" s="35">
+      <c r="O6" s="36">
         <f>IFERROR(E6/M6-1,"")</f>
         <v/>
       </c>
       <c r="P6" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="Q6" s="35">
+      <c r="Q6" s="36">
         <f>IFERROR(P6/E6-1,"")</f>
+        <v/>
+      </c>
+      <c r="R6" s="37">
+        <f>IF(AND(M6&gt;0,E6&gt;0,O6&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
         <v/>
       </c>
     </row>
@@ -5444,9 +5681,13 @@
         <f>IFERROR(P7/E7-1,"")</f>
         <v/>
       </c>
+      <c r="R7" s="33">
+        <f>IF(AND(M7&gt;0,E7&gt;0,O7&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="33" t="inlineStr">
+      <c r="A8" s="34" t="inlineStr">
         <is>
           <t>VRT</t>
         </is>
@@ -5478,19 +5719,19 @@
       <c r="H8" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="34">
+      <c r="I8" s="35">
         <f>G8*H8</f>
         <v/>
       </c>
-      <c r="J8" s="34">
+      <c r="J8" s="35">
         <f>E8*H8</f>
         <v/>
       </c>
-      <c r="K8" s="34">
+      <c r="K8" s="35">
         <f>J8-I8</f>
         <v/>
       </c>
-      <c r="L8" s="35">
+      <c r="L8" s="36">
         <f>IFERROR(K8/I8,"")</f>
         <v/>
       </c>
@@ -5500,79 +5741,84 @@
       <c r="N8" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="O8" s="35">
+      <c r="O8" s="36">
         <f>IFERROR(E8/M8-1,"")</f>
         <v/>
       </c>
       <c r="P8" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="Q8" s="35">
+      <c r="Q8" s="36">
         <f>IFERROR(P8/E8-1,"")</f>
         <v/>
       </c>
+      <c r="R8" s="37">
+        <f>IF(AND(M8&gt;0,E8&gt;0,O8&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="71" t="inlineStr">
+      <c r="A10" s="73" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H10" s="72">
+      <c r="H10" s="74">
         <f>SUM(H5:H8)</f>
         <v/>
       </c>
-      <c r="I10" s="72">
+      <c r="I10" s="74">
         <f>SUM(I5:I8)</f>
         <v/>
       </c>
-      <c r="J10" s="72">
+      <c r="J10" s="74">
         <f>SUM(J5:J8)</f>
         <v/>
       </c>
-      <c r="K10" s="73">
+      <c r="K10" s="75">
         <f>IFERROR(J10/H10,"")</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="74" t="inlineStr">
+      <c r="A12" s="76" t="inlineStr">
         <is>
           <t>INVESTMENT THESIS &amp; RESEARCH NOTES</t>
         </is>
       </c>
-      <c r="B12" s="75" t="n"/>
-      <c r="C12" s="75" t="n"/>
-      <c r="D12" s="75" t="n"/>
-      <c r="E12" s="75" t="n"/>
-      <c r="F12" s="75" t="n"/>
-      <c r="G12" s="75" t="n"/>
-      <c r="H12" s="75" t="n"/>
-      <c r="I12" s="75" t="n"/>
-      <c r="J12" s="75" t="n"/>
-      <c r="K12" s="75" t="n"/>
-      <c r="L12" s="75" t="n"/>
-      <c r="M12" s="75" t="n"/>
-      <c r="N12" s="75" t="n"/>
-      <c r="O12" s="75" t="n"/>
-      <c r="P12" s="75" t="n"/>
-      <c r="Q12" s="75" t="n"/>
+      <c r="B12" s="77" t="n"/>
+      <c r="C12" s="77" t="n"/>
+      <c r="D12" s="77" t="n"/>
+      <c r="E12" s="77" t="n"/>
+      <c r="F12" s="77" t="n"/>
+      <c r="G12" s="77" t="n"/>
+      <c r="H12" s="77" t="n"/>
+      <c r="I12" s="77" t="n"/>
+      <c r="J12" s="77" t="n"/>
+      <c r="K12" s="77" t="n"/>
+      <c r="L12" s="77" t="n"/>
+      <c r="M12" s="77" t="n"/>
+      <c r="N12" s="77" t="n"/>
+      <c r="O12" s="77" t="n"/>
+      <c r="P12" s="77" t="n"/>
+      <c r="Q12" s="77" t="n"/>
+      <c r="R12" s="77" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="41" t="inlineStr">
+      <c r="A13" s="43" t="inlineStr">
         <is>
           <t>CAT</t>
         </is>
       </c>
-      <c r="B13" s="42" t="inlineStr">
+      <c r="B13" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Caterpillar Inc   |   Risk: Low-Med</t>
         </is>
       </c>
     </row>
     <row r="14" ht="207" customHeight="1">
-      <c r="A14" s="43" t="n"/>
-      <c r="B14" s="44" t="inlineStr">
+      <c r="A14" s="45" t="n"/>
+      <c r="B14" s="46" t="inlineStr">
         <is>
           <t>The actual builder and materials company in the AI data
 center trade. AI data centers are physical buildings
@@ -5592,20 +5838,20 @@
     </row>
     <row r="15" ht="8" customHeight="1"/>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="41" t="inlineStr">
+      <c r="A16" s="43" t="inlineStr">
         <is>
           <t>FIX</t>
         </is>
       </c>
-      <c r="B16" s="42" t="inlineStr">
+      <c r="B16" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Comfort Systems USA   |   Risk: Medium</t>
         </is>
       </c>
     </row>
     <row r="17" ht="207" customHeight="1">
-      <c r="A17" s="45" t="n"/>
-      <c r="B17" s="46" t="inlineStr">
+      <c r="A17" s="47" t="n"/>
+      <c r="B17" s="48" t="inlineStr">
         <is>
           <t>Builder AND cooling company — one of the best-
 positioned picks-and-shovels plays in the AI buildout.
@@ -5625,20 +5871,20 @@
     </row>
     <row r="18" ht="8" customHeight="1"/>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="41" t="inlineStr">
+      <c r="A19" s="43" t="inlineStr">
         <is>
           <t>POWL</t>
         </is>
       </c>
-      <c r="B19" s="42" t="inlineStr">
+      <c r="B19" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Powell Industries   |   Risk: Medium</t>
         </is>
       </c>
     </row>
     <row r="20" ht="207" customHeight="1">
-      <c r="A20" s="43" t="n"/>
-      <c r="B20" s="44" t="inlineStr">
+      <c r="A20" s="45" t="n"/>
+      <c r="B20" s="46" t="inlineStr">
         <is>
           <t>Electrical infrastructure builder for AI data centers —
 the company that builds the switchgear, motor control
@@ -5658,20 +5904,20 @@
     </row>
     <row r="21" ht="8" customHeight="1"/>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="41" t="inlineStr">
+      <c r="A22" s="43" t="inlineStr">
         <is>
           <t>VRT</t>
         </is>
       </c>
-      <c r="B22" s="42" t="inlineStr">
+      <c r="B22" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Vertiv Holdings   |   Risk: Medium</t>
         </is>
       </c>
     </row>
     <row r="23" ht="207" customHeight="1">
-      <c r="A23" s="45" t="n"/>
-      <c r="B23" s="46" t="inlineStr">
+      <c r="A23" s="47" t="n"/>
+      <c r="B23" s="48" t="inlineStr">
         <is>
           <t>The premier AI data center cooling play and one of the
 most direct beneficiaries of the AI buildout. Vertiv
@@ -5692,9 +5938,9 @@
     <row r="24" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A3:R3"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A1:R1"/>
     <mergeCell ref="A10:G10"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J8">
@@ -5713,6 +5959,16 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="R5:R8">
+    <cfRule type="expression" priority="5" dxfId="2">
+      <formula>$O5&lt;-0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A5:Q8">
+    <cfRule type="expression" priority="6" dxfId="3">
+      <formula>$O5&lt;-0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5724,7 +5980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:R23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5744,10 +6000,11 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="76" t="inlineStr">
+      <c r="A1" s="78" t="inlineStr">
         <is>
           <t>⚡ Power &amp; Energy</t>
         </is>
@@ -5763,107 +6020,113 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="77" t="inlineStr">
+      <c r="A4" s="79" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="77" t="inlineStr">
+      <c r="B4" s="79" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="77" t="inlineStr">
+      <c r="C4" s="79" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="77" t="inlineStr">
+      <c r="D4" s="79" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="77" t="inlineStr">
+      <c r="E4" s="79" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="77" t="inlineStr">
+      <c r="F4" s="79" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="77" t="inlineStr">
+      <c r="G4" s="79" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="77" t="inlineStr">
+      <c r="H4" s="79" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="77" t="inlineStr">
+      <c r="I4" s="79" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="77" t="inlineStr">
+      <c r="J4" s="79" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="77" t="inlineStr">
+      <c r="K4" s="79" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="77" t="inlineStr">
+      <c r="L4" s="79" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="77" t="inlineStr">
+      <c r="M4" s="79" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="77" t="inlineStr">
+      <c r="N4" s="79" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="77" t="inlineStr">
+      <c r="O4" s="79" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="77" t="inlineStr">
+      <c r="P4" s="79" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="77" t="inlineStr">
+      <c r="Q4" s="79" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
         </is>
       </c>
+      <c r="R4" s="79" t="inlineStr">
+        <is>
+          <t>Price
+Alert</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
@@ -5931,9 +6194,13 @@
         <f>IFERROR(P5/E5-1,"")</f>
         <v/>
       </c>
+      <c r="R5" s="33">
+        <f>IF(AND(M5&gt;0,E5&gt;0,O5&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="33" t="inlineStr">
+      <c r="A6" s="34" t="inlineStr">
         <is>
           <t>PWR</t>
         </is>
@@ -5965,19 +6232,19 @@
       <c r="H6" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="34">
+      <c r="I6" s="35">
         <f>G6*H6</f>
         <v/>
       </c>
-      <c r="J6" s="34">
+      <c r="J6" s="35">
         <f>E6*H6</f>
         <v/>
       </c>
-      <c r="K6" s="34">
+      <c r="K6" s="35">
         <f>J6-I6</f>
         <v/>
       </c>
-      <c r="L6" s="35">
+      <c r="L6" s="36">
         <f>IFERROR(K6/I6,"")</f>
         <v/>
       </c>
@@ -5987,15 +6254,19 @@
       <c r="N6" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="O6" s="35">
+      <c r="O6" s="36">
         <f>IFERROR(E6/M6-1,"")</f>
         <v/>
       </c>
       <c r="P6" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="Q6" s="35">
+      <c r="Q6" s="36">
         <f>IFERROR(P6/E6-1,"")</f>
+        <v/>
+      </c>
+      <c r="R6" s="37">
+        <f>IF(AND(M6&gt;0,E6&gt;0,O6&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
         <v/>
       </c>
     </row>
@@ -6023,7 +6294,7 @@
       <c r="E7" s="28" t="n">
         <v>285.47</v>
       </c>
-      <c r="F7" s="49" t="n">
+      <c r="F7" s="51" t="n">
         <v>-4.067043441964675</v>
       </c>
       <c r="G7" s="28" t="n">
@@ -6065,9 +6336,13 @@
         <f>IFERROR(P7/E7-1,"")</f>
         <v/>
       </c>
+      <c r="R7" s="33">
+        <f>IF(AND(M7&gt;0,E7&gt;0,O7&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="33" t="inlineStr">
+      <c r="A8" s="34" t="inlineStr">
         <is>
           <t>OKLO</t>
         </is>
@@ -6099,19 +6374,19 @@
       <c r="H8" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="34">
+      <c r="I8" s="35">
         <f>G8*H8</f>
         <v/>
       </c>
-      <c r="J8" s="34">
+      <c r="J8" s="35">
         <f>E8*H8</f>
         <v/>
       </c>
-      <c r="K8" s="34">
+      <c r="K8" s="35">
         <f>J8-I8</f>
         <v/>
       </c>
-      <c r="L8" s="35">
+      <c r="L8" s="36">
         <f>IFERROR(K8/I8,"")</f>
         <v/>
       </c>
@@ -6121,79 +6396,84 @@
       <c r="N8" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="O8" s="35">
+      <c r="O8" s="36">
         <f>IFERROR(E8/M8-1,"")</f>
         <v/>
       </c>
       <c r="P8" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="Q8" s="35">
+      <c r="Q8" s="36">
         <f>IFERROR(P8/E8-1,"")</f>
         <v/>
       </c>
+      <c r="R8" s="37">
+        <f>IF(AND(M8&gt;0,E8&gt;0,O8&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="78" t="inlineStr">
+      <c r="A10" s="80" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H10" s="79">
+      <c r="H10" s="81">
         <f>SUM(H5:H8)</f>
         <v/>
       </c>
-      <c r="I10" s="79">
+      <c r="I10" s="81">
         <f>SUM(I5:I8)</f>
         <v/>
       </c>
-      <c r="J10" s="79">
+      <c r="J10" s="81">
         <f>SUM(J5:J8)</f>
         <v/>
       </c>
-      <c r="K10" s="80">
+      <c r="K10" s="82">
         <f>IFERROR(J10/H10,"")</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="81" t="inlineStr">
+      <c r="A12" s="83" t="inlineStr">
         <is>
           <t>INVESTMENT THESIS &amp; RESEARCH NOTES</t>
         </is>
       </c>
-      <c r="B12" s="82" t="n"/>
-      <c r="C12" s="82" t="n"/>
-      <c r="D12" s="82" t="n"/>
-      <c r="E12" s="82" t="n"/>
-      <c r="F12" s="82" t="n"/>
-      <c r="G12" s="82" t="n"/>
-      <c r="H12" s="82" t="n"/>
-      <c r="I12" s="82" t="n"/>
-      <c r="J12" s="82" t="n"/>
-      <c r="K12" s="82" t="n"/>
-      <c r="L12" s="82" t="n"/>
-      <c r="M12" s="82" t="n"/>
-      <c r="N12" s="82" t="n"/>
-      <c r="O12" s="82" t="n"/>
-      <c r="P12" s="82" t="n"/>
-      <c r="Q12" s="82" t="n"/>
+      <c r="B12" s="84" t="n"/>
+      <c r="C12" s="84" t="n"/>
+      <c r="D12" s="84" t="n"/>
+      <c r="E12" s="84" t="n"/>
+      <c r="F12" s="84" t="n"/>
+      <c r="G12" s="84" t="n"/>
+      <c r="H12" s="84" t="n"/>
+      <c r="I12" s="84" t="n"/>
+      <c r="J12" s="84" t="n"/>
+      <c r="K12" s="84" t="n"/>
+      <c r="L12" s="84" t="n"/>
+      <c r="M12" s="84" t="n"/>
+      <c r="N12" s="84" t="n"/>
+      <c r="O12" s="84" t="n"/>
+      <c r="P12" s="84" t="n"/>
+      <c r="Q12" s="84" t="n"/>
+      <c r="R12" s="84" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="41" t="inlineStr">
+      <c r="A13" s="43" t="inlineStr">
         <is>
           <t>GEV</t>
         </is>
       </c>
-      <c r="B13" s="42" t="inlineStr">
+      <c r="B13" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  GE Vernova   |   Risk: Medium</t>
         </is>
       </c>
     </row>
     <row r="14" ht="207" customHeight="1">
-      <c r="A14" s="43" t="n"/>
-      <c r="B14" s="44" t="inlineStr">
+      <c r="A14" s="45" t="n"/>
+      <c r="B14" s="46" t="inlineStr">
         <is>
           <t>Stability and steady compounder — the premier power
 generation and grid equipment company spun out of GE.
@@ -6213,20 +6493,20 @@
     </row>
     <row r="15" ht="8" customHeight="1"/>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="41" t="inlineStr">
+      <c r="A16" s="43" t="inlineStr">
         <is>
           <t>PWR</t>
         </is>
       </c>
-      <c r="B16" s="42" t="inlineStr">
+      <c r="B16" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Quanta Services   |   Risk: Medium</t>
         </is>
       </c>
     </row>
     <row r="17" ht="237" customHeight="1">
-      <c r="A17" s="45" t="n"/>
-      <c r="B17" s="46" t="inlineStr">
+      <c r="A17" s="47" t="n"/>
+      <c r="B17" s="48" t="inlineStr">
         <is>
           <t>Power grid infrastructure and maintenance — a growing
 bottleneck for the AI buildout. Quanta Services is the
@@ -6248,20 +6528,20 @@
     </row>
     <row r="18" ht="8" customHeight="1"/>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="41" t="inlineStr">
+      <c r="A19" s="43" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="B19" s="42" t="inlineStr">
+      <c r="B19" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Bloom Energy   |   Risk: High</t>
         </is>
       </c>
     </row>
     <row r="20" ht="237" customHeight="1">
-      <c r="A20" s="43" t="n"/>
-      <c r="B20" s="44" t="inlineStr">
+      <c r="A20" s="45" t="n"/>
+      <c r="B20" s="46" t="inlineStr">
         <is>
           <t>Moonshot potential if hydrogen and fuel cell technology
 takes off — and the AI power crisis is accelerating the
@@ -6283,20 +6563,20 @@
     </row>
     <row r="21" ht="8" customHeight="1"/>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="41" t="inlineStr">
+      <c r="A22" s="43" t="inlineStr">
         <is>
           <t>OKLO</t>
         </is>
       </c>
-      <c r="B22" s="42" t="inlineStr">
+      <c r="B22" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Oklo Inc   |   Risk: Very High</t>
         </is>
       </c>
     </row>
     <row r="23" ht="252" customHeight="1">
-      <c r="A23" s="45" t="n"/>
-      <c r="B23" s="46" t="inlineStr">
+      <c r="A23" s="47" t="n"/>
+      <c r="B23" s="48" t="inlineStr">
         <is>
           <t>Nuclear SMRs and nuclear fuel waste company with
 massive moonshot potential — but big regulatory and
@@ -6320,9 +6600,9 @@
     <row r="24" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A3:R3"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A1:R1"/>
     <mergeCell ref="A10:G10"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J8">
@@ -6341,6 +6621,16 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="R5:R8">
+    <cfRule type="expression" priority="5" dxfId="2">
+      <formula>$O5&lt;-0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A5:Q8">
+    <cfRule type="expression" priority="6" dxfId="3">
+      <formula>$O5&lt;-0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6352,7 +6642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:R15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6372,10 +6662,11 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="83" t="inlineStr">
+      <c r="A1" s="85" t="inlineStr">
         <is>
           <t>☁️ Neoclouds &amp; AI Software</t>
         </is>
@@ -6391,107 +6682,113 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="84" t="inlineStr">
+      <c r="A4" s="86" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="84" t="inlineStr">
+      <c r="B4" s="86" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="84" t="inlineStr">
+      <c r="C4" s="86" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="84" t="inlineStr">
+      <c r="D4" s="86" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="84" t="inlineStr">
+      <c r="E4" s="86" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="84" t="inlineStr">
+      <c r="F4" s="86" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="84" t="inlineStr">
+      <c r="G4" s="86" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="84" t="inlineStr">
+      <c r="H4" s="86" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="84" t="inlineStr">
+      <c r="I4" s="86" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="84" t="inlineStr">
+      <c r="J4" s="86" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="84" t="inlineStr">
+      <c r="K4" s="86" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="84" t="inlineStr">
+      <c r="L4" s="86" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="84" t="inlineStr">
+      <c r="M4" s="86" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="84" t="inlineStr">
+      <c r="N4" s="86" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="84" t="inlineStr">
+      <c r="O4" s="86" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="84" t="inlineStr">
+      <c r="P4" s="86" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="84" t="inlineStr">
+      <c r="Q4" s="86" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
         </is>
       </c>
+      <c r="R4" s="86" t="inlineStr">
+        <is>
+          <t>Price
+Alert</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
@@ -6559,9 +6856,13 @@
         <f>IFERROR(P5/E5-1,"")</f>
         <v/>
       </c>
+      <c r="R5" s="33">
+        <f>IF(AND(M5&gt;0,E5&gt;0,O5&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="33" t="inlineStr">
+      <c r="A6" s="34" t="inlineStr">
         <is>
           <t>PLTR</t>
         </is>
@@ -6584,7 +6885,7 @@
       <c r="E6" s="28" t="n">
         <v>133.79</v>
       </c>
-      <c r="F6" s="49" t="n">
+      <c r="F6" s="51" t="n">
         <v>-1.101424241474859</v>
       </c>
       <c r="G6" s="28" t="n">
@@ -6593,19 +6894,19 @@
       <c r="H6" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="34">
+      <c r="I6" s="35">
         <f>G6*H6</f>
         <v/>
       </c>
-      <c r="J6" s="34">
+      <c r="J6" s="35">
         <f>E6*H6</f>
         <v/>
       </c>
-      <c r="K6" s="34">
+      <c r="K6" s="35">
         <f>J6-I6</f>
         <v/>
       </c>
-      <c r="L6" s="35">
+      <c r="L6" s="36">
         <f>IFERROR(K6/I6,"")</f>
         <v/>
       </c>
@@ -6615,79 +6916,84 @@
       <c r="N6" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="O6" s="35">
+      <c r="O6" s="36">
         <f>IFERROR(E6/M6-1,"")</f>
         <v/>
       </c>
       <c r="P6" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="Q6" s="35">
+      <c r="Q6" s="36">
         <f>IFERROR(P6/E6-1,"")</f>
         <v/>
       </c>
+      <c r="R6" s="37">
+        <f>IF(AND(M6&gt;0,E6&gt;0,O6&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="85" t="inlineStr">
+      <c r="A8" s="87" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H8" s="86">
+      <c r="H8" s="88">
         <f>SUM(H5:H6)</f>
         <v/>
       </c>
-      <c r="I8" s="86">
+      <c r="I8" s="88">
         <f>SUM(I5:I6)</f>
         <v/>
       </c>
-      <c r="J8" s="86">
+      <c r="J8" s="88">
         <f>SUM(J5:J6)</f>
         <v/>
       </c>
-      <c r="K8" s="87">
+      <c r="K8" s="89">
         <f>IFERROR(J8/H8,"")</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="88" t="inlineStr">
+      <c r="A10" s="90" t="inlineStr">
         <is>
           <t>INVESTMENT THESIS &amp; RESEARCH NOTES</t>
         </is>
       </c>
-      <c r="B10" s="89" t="n"/>
-      <c r="C10" s="89" t="n"/>
-      <c r="D10" s="89" t="n"/>
-      <c r="E10" s="89" t="n"/>
-      <c r="F10" s="89" t="n"/>
-      <c r="G10" s="89" t="n"/>
-      <c r="H10" s="89" t="n"/>
-      <c r="I10" s="89" t="n"/>
-      <c r="J10" s="89" t="n"/>
-      <c r="K10" s="89" t="n"/>
-      <c r="L10" s="89" t="n"/>
-      <c r="M10" s="89" t="n"/>
-      <c r="N10" s="89" t="n"/>
-      <c r="O10" s="89" t="n"/>
-      <c r="P10" s="89" t="n"/>
-      <c r="Q10" s="89" t="n"/>
+      <c r="B10" s="91" t="n"/>
+      <c r="C10" s="91" t="n"/>
+      <c r="D10" s="91" t="n"/>
+      <c r="E10" s="91" t="n"/>
+      <c r="F10" s="91" t="n"/>
+      <c r="G10" s="91" t="n"/>
+      <c r="H10" s="91" t="n"/>
+      <c r="I10" s="91" t="n"/>
+      <c r="J10" s="91" t="n"/>
+      <c r="K10" s="91" t="n"/>
+      <c r="L10" s="91" t="n"/>
+      <c r="M10" s="91" t="n"/>
+      <c r="N10" s="91" t="n"/>
+      <c r="O10" s="91" t="n"/>
+      <c r="P10" s="91" t="n"/>
+      <c r="Q10" s="91" t="n"/>
+      <c r="R10" s="91" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="41" t="inlineStr">
+      <c r="A11" s="43" t="inlineStr">
         <is>
           <t>NBIS</t>
         </is>
       </c>
-      <c r="B11" s="42" t="inlineStr">
+      <c r="B11" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Nebius Group   |   Risk: High</t>
         </is>
       </c>
     </row>
     <row r="12" ht="282" customHeight="1">
-      <c r="A12" s="43" t="n"/>
-      <c r="B12" s="44" t="inlineStr">
+      <c r="A12" s="45" t="n"/>
+      <c r="B12" s="46" t="inlineStr">
         <is>
           <t>The leading Neocloud and one of the most interesting
 companies in this portfolio. Nebius is a modern
@@ -6712,20 +7018,20 @@
     </row>
     <row r="13" ht="8" customHeight="1"/>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="41" t="inlineStr">
+      <c r="A14" s="43" t="inlineStr">
         <is>
           <t>PLTR</t>
         </is>
       </c>
-      <c r="B14" s="42" t="inlineStr">
+      <c r="B14" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Palantir Technologies   |   Risk: Med-High</t>
         </is>
       </c>
     </row>
     <row r="15" ht="237" customHeight="1">
-      <c r="A15" s="45" t="n"/>
-      <c r="B15" s="46" t="inlineStr">
+      <c r="A15" s="47" t="n"/>
+      <c r="B15" s="48" t="inlineStr">
         <is>
           <t>So integral to the entire US government AI stack that
 it is effectively a national security asset. Palantir's
@@ -6748,10 +7054,10 @@
     <row r="16" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A3:R3"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A1:R1"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J6">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
@@ -6769,6 +7075,16 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="R5:R6">
+    <cfRule type="expression" priority="5" dxfId="2">
+      <formula>$O5&lt;-0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A5:Q6">
+    <cfRule type="expression" priority="6" dxfId="3">
+      <formula>$O5&lt;-0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6780,7 +7096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:R11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6800,10 +7116,11 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="90" t="inlineStr">
+      <c r="A1" s="92" t="inlineStr">
         <is>
           <t>🛡️ Defense &amp; Drones</t>
         </is>
@@ -6819,107 +7136,113 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:05 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="91" t="inlineStr">
+      <c r="A4" s="93" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="91" t="inlineStr">
+      <c r="B4" s="93" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C4" s="91" t="inlineStr">
+      <c r="C4" s="93" t="inlineStr">
         <is>
           <t>Focus / Niche</t>
         </is>
       </c>
-      <c r="D4" s="91" t="inlineStr">
+      <c r="D4" s="93" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="E4" s="91" t="inlineStr">
+      <c r="E4" s="93" t="inlineStr">
         <is>
           <t>Current
 Price</t>
         </is>
       </c>
-      <c r="F4" s="91" t="inlineStr">
+      <c r="F4" s="93" t="inlineStr">
         <is>
           <t>Today's
 +/- %</t>
         </is>
       </c>
-      <c r="G4" s="91" t="inlineStr">
+      <c r="G4" s="93" t="inlineStr">
         <is>
           <t>Purchase
 Price</t>
         </is>
       </c>
-      <c r="H4" s="91" t="inlineStr">
+      <c r="H4" s="93" t="inlineStr">
         <is>
           <t>Shares
 Owned</t>
         </is>
       </c>
-      <c r="I4" s="91" t="inlineStr">
+      <c r="I4" s="93" t="inlineStr">
         <is>
           <t>Total
 Cost</t>
         </is>
       </c>
-      <c r="J4" s="91" t="inlineStr">
+      <c r="J4" s="93" t="inlineStr">
         <is>
           <t>Current
 Value</t>
         </is>
       </c>
-      <c r="K4" s="91" t="inlineStr">
+      <c r="K4" s="93" t="inlineStr">
         <is>
           <t>P&amp;L ($)</t>
         </is>
       </c>
-      <c r="L4" s="91" t="inlineStr">
+      <c r="L4" s="93" t="inlineStr">
         <is>
           <t>P&amp;L (%)</t>
         </is>
       </c>
-      <c r="M4" s="91" t="inlineStr">
+      <c r="M4" s="93" t="inlineStr">
         <is>
           <t>52W
 High</t>
         </is>
       </c>
-      <c r="N4" s="91" t="inlineStr">
+      <c r="N4" s="93" t="inlineStr">
         <is>
           <t>52W
 Low</t>
         </is>
       </c>
-      <c r="O4" s="91" t="inlineStr">
+      <c r="O4" s="93" t="inlineStr">
         <is>
           <t>% from
 52W High</t>
         </is>
       </c>
-      <c r="P4" s="91" t="inlineStr">
+      <c r="P4" s="93" t="inlineStr">
         <is>
           <t>Analyst
 Target</t>
         </is>
       </c>
-      <c r="Q4" s="91" t="inlineStr">
+      <c r="Q4" s="93" t="inlineStr">
         <is>
           <t>Upside to
 Target</t>
         </is>
       </c>
+      <c r="R4" s="93" t="inlineStr">
+        <is>
+          <t>Price
+Alert</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
@@ -6987,68 +7310,73 @@
         <f>IFERROR(P5/E5-1,"")</f>
         <v/>
       </c>
+      <c r="R5" s="33">
+        <f>IF(AND(M5&gt;0,E5&gt;0,O5&lt;-0.2),"▼  BUY ZONE  (-20%+ off high)","")</f>
+        <v/>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="92" t="inlineStr">
+      <c r="A7" s="94" t="inlineStr">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="H7" s="93">
+      <c r="H7" s="95">
         <f>SUM(H5:H5)</f>
         <v/>
       </c>
-      <c r="I7" s="93">
+      <c r="I7" s="95">
         <f>SUM(I5:I5)</f>
         <v/>
       </c>
-      <c r="J7" s="93">
+      <c r="J7" s="95">
         <f>SUM(J5:J5)</f>
         <v/>
       </c>
-      <c r="K7" s="94">
+      <c r="K7" s="96">
         <f>IFERROR(J7/H7,"")</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="95" t="inlineStr">
+      <c r="A9" s="97" t="inlineStr">
         <is>
           <t>INVESTMENT THESIS &amp; RESEARCH NOTES</t>
         </is>
       </c>
-      <c r="B9" s="96" t="n"/>
-      <c r="C9" s="96" t="n"/>
-      <c r="D9" s="96" t="n"/>
-      <c r="E9" s="96" t="n"/>
-      <c r="F9" s="96" t="n"/>
-      <c r="G9" s="96" t="n"/>
-      <c r="H9" s="96" t="n"/>
-      <c r="I9" s="96" t="n"/>
-      <c r="J9" s="96" t="n"/>
-      <c r="K9" s="96" t="n"/>
-      <c r="L9" s="96" t="n"/>
-      <c r="M9" s="96" t="n"/>
-      <c r="N9" s="96" t="n"/>
-      <c r="O9" s="96" t="n"/>
-      <c r="P9" s="96" t="n"/>
-      <c r="Q9" s="96" t="n"/>
+      <c r="B9" s="98" t="n"/>
+      <c r="C9" s="98" t="n"/>
+      <c r="D9" s="98" t="n"/>
+      <c r="E9" s="98" t="n"/>
+      <c r="F9" s="98" t="n"/>
+      <c r="G9" s="98" t="n"/>
+      <c r="H9" s="98" t="n"/>
+      <c r="I9" s="98" t="n"/>
+      <c r="J9" s="98" t="n"/>
+      <c r="K9" s="98" t="n"/>
+      <c r="L9" s="98" t="n"/>
+      <c r="M9" s="98" t="n"/>
+      <c r="N9" s="98" t="n"/>
+      <c r="O9" s="98" t="n"/>
+      <c r="P9" s="98" t="n"/>
+      <c r="Q9" s="98" t="n"/>
+      <c r="R9" s="98" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="41" t="inlineStr">
+      <c r="A10" s="43" t="inlineStr">
         <is>
           <t>ONDS</t>
         </is>
       </c>
-      <c r="B10" s="42" t="inlineStr">
+      <c r="B10" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Ondas Holdings   |   Risk: Very High</t>
         </is>
       </c>
     </row>
     <row r="11" ht="282" customHeight="1">
-      <c r="A11" s="43" t="n"/>
-      <c r="B11" s="44" t="inlineStr">
+      <c r="A11" s="45" t="n"/>
+      <c r="B11" s="46" t="inlineStr">
         <is>
           <t>Drones and defense tech — very speculative but with a
 massive catalyst behind it. The US government just
@@ -7074,9 +7402,9 @@
     <row r="12" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A3:R3"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A1:R1"/>
     <mergeCell ref="A7:G7"/>
   </mergeCells>
   <conditionalFormatting sqref="J5">
@@ -7095,6 +7423,16 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="R5">
+    <cfRule type="expression" priority="5" dxfId="2">
+      <formula>$O5&lt;-0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A5:Q5">
+    <cfRule type="expression" priority="6" dxfId="3">
+      <formula>$O5&lt;-0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update financial tracker to export to Google Sheets and include price alerts
Modify the Excel export to include price alerts and update the Python script to utilize `fetch_live_prices` for Google Sheets export.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: f7984a94-71d9-4e7e-b050-ebaaaa972a66
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1105,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 06, 2026 at 11:13 PM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update financial tracker to a live stock watchlist with news
Refactor Google Sheets export script to use GOOGLEFINANCE formulas for live data and add a news feed sheet populated by yfinance.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: d5c942f1-2d90-4436-a982-60151869e8cc
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1105,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:18 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update financial tracker to fix spreadsheet formatting and data updates
Corrected an issue with argument order in the spreadsheet update function and resolved conflicts between frozen columns and merged cells. Also fixed formatting for the news feed section by removing an unsupported 'italic' parameter.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: aab1ef8a-63d6-47b1-a596-46e57d3ec013
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1105,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:23 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Organize stock data into a dashboard with integrated news feed
Replace the separate news feed tab with a consolidated dashboard that displays a compact stock watchlist by category, analyst ratings, and technical indicators, followed by the news feed.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 5f21a899-cbeb-47e9-b2d4-92a4b614cb2d
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1105,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:29 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Move news feed from dashboard to category tabs
Modify `scripts/export_to_google_sheets.py` to remove the news feed from the dashboard and add it to each respective category tab, below the watchlist. Also updates formatting for the new news section and adjusts the completion message for the dashboard.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 487238c1-c7db-45e4-895b-d5277e8df861
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1105,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add extended hours percentage to the stock tracker dashboard
Add "Ext Hrs %" column to the dashboard, fetching pre/post-market data from yfinance and updating column definitions and formatting in `export_to_google_sheets.py`.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: bec391ea-745e-4b9a-b4bb-e412407623d8
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1105,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:44 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make dashboard category names clickable links to their respective tabs
Update scripts to add hyperlinks to category headers on the dashboard, linking to their respective tabs.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 5be5267f-a673-40fd-9b5c-22e1f5aa1f23
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1105,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:50 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update financial tracker with accurate historical price calculations
Corrected formulas in `scripts/export_to_google_sheets.py` for 1-week, 1-month, 3-month, and YTD percentage changes, and updated `Financial_Stock_Tracker.xlsx`.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: e1cc2471-51a8-4d57-a71c-007fc355409b
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1105,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:53 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve financial tracker by fixing data display and widening columns
Replaced INDEX with QUERY for GOOGLEFINANCE historical price lookups to prevent array spillover and adjusted column widths for better data visibility.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: f2d80463-5c86-4536-85a8-e458f2c13b6e
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1105,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 01:57 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve display of financial data and news headlines
Update the script to adjust row heights, enable text wrapping for better readability of stock data and news headlines, and reposition the published date for news articles.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 8ed4f8d9-bcf7-429b-9dca-5a487e866a5e
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1105,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:01 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adjust spacing for research notes to prevent text clipping
Remove artificial text wrapping and increase row height for research notes to display full text.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: a7ed2dff-078d-44d2-8489-6127ede9d34e
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1105,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:08 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add AI-powered stock impact analysis and hyperlinked articles to financial tracker
Integrate OpenAI API for AI-driven stock impact analysis, convert published dates to EST, and add hyperlinks to news headlines within the financial tracker spreadsheet.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 8bec3621-27bf-4476-b376-bde3c28149b2
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1105,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:13 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix issues with AI analysis display and column widths
Updates the AI model to gpt-4o-mini, widens the "YTD %" column to 130px, and adds header row merges for the news and AI analysis columns.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: b6bccaa9-043a-4b85-a377-5ab59d5da8fb
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1105,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:20 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ensure news articles are relevant to the specific stock
Filter news articles to only include those that mention the stock ticker or company name.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 4cb22f51-f98c-486f-ab33-89cb3f2e32eb
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1105,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:28 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update news timestamps to use 12-hour format with AM/PM
Modify the time formatting in the export script to display news publication times using a 12-hour clock with AM/PM indicators.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: bd8d1c9a-f41a-4890-a329-b7aab1b87323
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1105,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:33 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Organize news headlines by relevance and recency for each stock
Modify `scripts/export_to_google_sheets.py` to sort news articles by relevance and publish timestamp in descending order before appending to `raw_news`, and update `Financial_Stock_Tracker.xlsx`.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: eee76a36-1173-4864-8340-3b6797466249
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1105,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:37 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve news analysis by using article summaries and providing more context
Update the AI analysis function to include article summaries alongside headlines, increasing token limits to accommodate richer context.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 4d1b9236-3747-4293-a93c-9eae13398eb6
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1105,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:39 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add currency formatting to live stock prices on the dashboard
Add CURRENCY format to the Live Price column (C) in the dashboard sheet and adjust row height in scripts/export_to_google_sheets.py.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 525b8429-1f93-4025-90cf-1b8cde742c83
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1105,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:46 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Display live stock prices directly on the dashboard
Replace GOOGLEFINANCE formulas with direct yfinance price data in the dashboard to ensure instant loading and consistent display of all stock prices.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 5ce5ed8e-5eaf-4636-9640-91183932efd8
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1105,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 02:55 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboard category headers to a consistent light purple
Change background color of dashboard category header rows from individual category colors to a fixed light purple hex code.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 3abe7df2-104c-45f1-8d87-f2fa5acd3e0d
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1105,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:00 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboard category headers to a lighter blue color
Change the background color of dashboard category headers to match the subtitle row's light blue ("D9E1F2") and update text color to dark blue for better readability in scripts/export_to_google_sheets.py.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 3606d406-6029-4563-9817-71a98af07e8b
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1105,7 +1105,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 03:15 AM</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:15 AM</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:15 AM</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:15 AM</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:15 AM</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:15 AM</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:15 AM</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:15 AM</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:15 AM</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:15 AM</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:12 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:15 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix historical price tracking by using a more reliable data source
Replace unreliable GOOGLEFINANCE formulas for historical price percentage changes with direct data fetching from yfinance in the watchlist sheets.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: b73d2683-f8c9-4e0d-8d50-598219d52104
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1070,7 +1070,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 03:23 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 03:28 AM</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1534,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:23 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:28 AM</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:23 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:28 AM</t>
         </is>
       </c>
     </row>
@@ -2685,7 +2685,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:23 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:28 AM</t>
         </is>
       </c>
     </row>
@@ -3543,7 +3543,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:23 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:28 AM</t>
         </is>
       </c>
     </row>
@@ -4511,7 +4511,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:23 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:28 AM</t>
         </is>
       </c>
     </row>
@@ -4856,7 +4856,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:23 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:28 AM</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:23 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:28 AM</t>
         </is>
       </c>
     </row>
@@ -6173,7 +6173,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:23 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:28 AM</t>
         </is>
       </c>
     </row>
@@ -6731,7 +6731,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:23 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:28 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace unreliable stock data formulas with direct data retrieval
Modify the script to fetch 52-week high/low, P/E ratio, market cap, and volume directly from yfinance, replacing volatile GOOGLEFINANCE formulas in the spreadsheet.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 8a6043f5-a13c-4c23-a636-73a26a227f4d
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1070,7 +1070,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 03:28 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 03:34 AM</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1534,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:28 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:34 AM</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:28 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:34 AM</t>
         </is>
       </c>
     </row>
@@ -2685,7 +2685,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:28 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:34 AM</t>
         </is>
       </c>
     </row>
@@ -3543,7 +3543,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:28 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:34 AM</t>
         </is>
       </c>
     </row>
@@ -4511,7 +4511,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:28 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:34 AM</t>
         </is>
       </c>
     </row>
@@ -4856,7 +4856,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:28 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:34 AM</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:28 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:34 AM</t>
         </is>
       </c>
     </row>
@@ -6173,7 +6173,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:28 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:34 AM</t>
         </is>
       </c>
     </row>
@@ -6731,7 +6731,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:28 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:34 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove analyst target and upside to target columns from financial tracker
Removes the "Analyst Target" and "Upside to Target" columns from the financial tracking spreadsheet by updating the `WATCH_COLS` definition, removing corresponding data entries in the row builder, and adjusting formatting and legend text in `scripts/export_to_google_sheets.py`.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: ac19fc34-3123-42b5-844e-58d12d03af1c
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1070,7 +1070,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 03:34 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 03:38 AM</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1534,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:34 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:38 AM</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:34 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:38 AM</t>
         </is>
       </c>
     </row>
@@ -2685,7 +2685,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:34 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:38 AM</t>
         </is>
       </c>
     </row>
@@ -3543,7 +3543,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:34 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:38 AM</t>
         </is>
       </c>
     </row>
@@ -4511,7 +4511,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:34 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:38 AM</t>
         </is>
       </c>
     </row>
@@ -4856,7 +4856,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:34 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:38 AM</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:34 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:38 AM</t>
         </is>
       </c>
     </row>
@@ -6173,7 +6173,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:34 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:38 AM</t>
         </is>
       </c>
     </row>
@@ -6731,7 +6731,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:34 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:38 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Format financial data for improved readability
Adds helper functions to format market cap and volume into human-readable strings (e.g., $5.05T, 188.2M) and updates the watchlist sheet to use these formats.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 446703a2-d267-4c78-8ea2-52fa9ec39ac1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 06abc5ec-1518-4c85-91d8-99ecaebba5d9
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Financial_Stock_Tracker.xlsx
+++ b/Financial_Stock_Tracker.xlsx
@@ -1070,7 +1070,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 03:38 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  Green = gain  |  Red = loss  |  📡 Prices fetched: May 07, 2026 at 03:42 AM</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1534,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:38 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:42 AM</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:38 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:42 AM</t>
         </is>
       </c>
     </row>
@@ -2685,7 +2685,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:38 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:42 AM</t>
         </is>
       </c>
     </row>
@@ -3543,7 +3543,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:38 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:42 AM</t>
         </is>
       </c>
     </row>
@@ -4511,7 +4511,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:38 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:42 AM</t>
         </is>
       </c>
     </row>
@@ -4856,7 +4856,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:38 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:42 AM</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:38 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:42 AM</t>
         </is>
       </c>
     </row>
@@ -6173,7 +6173,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:38 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:42 AM</t>
         </is>
       </c>
     </row>
@@ -6731,7 +6731,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:38 AM</t>
+          <t>🟡 Yellow cells = your inputs  |  All other cells auto-calculate  |  📡 Prices fetched: May 07, 2026 at 03:42 AM</t>
         </is>
       </c>
     </row>

</xml_diff>